<commit_message>
Fix invalid Bloomberg field mnemonics in workbook
Verified live on terminal: FUT_CONTRACT_DATE is not a valid field -> replace
with FUT_DLV_DT_FIRST (SR3/SR1 reference-quarter start). Conventions tab: the
USOSFR BGN Curncy rate-quote tickers don't carry leg-level static fields, so
route floating day count / pay freq / payment lag / EOM / compounding / lookback
to DES/SWPM capture and add a USD-SOFR-OIS market-standard reference block; keep
only CRNCY / CALENDAR_CODE / DAY_CNT_DES as BDP pulls. (Bloomberg returns
'#N/A Invalid Field' as text, which IFERROR cannot catch.)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -225,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -290,6 +290,10 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1373,7 +1377,7 @@
       </c>
       <c r="H6" s="20" t="inlineStr">
         <is>
-          <t>FUT_CONTRACT_DATE</t>
+          <t>Ref. start (FUT_DLV_DT_FIRST)</t>
         </is>
       </c>
       <c r="I6" s="20" t="inlineStr">
@@ -1422,7 +1426,7 @@
         <v/>
       </c>
       <c r="H7" s="18">
-        <f>IFERROR(BDP($A7,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A7,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I7" s="18">
@@ -1465,7 +1469,7 @@
         <v/>
       </c>
       <c r="H8" s="24">
-        <f>IFERROR(BDP($A8,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A8,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I8" s="24">
@@ -1508,7 +1512,7 @@
         <v/>
       </c>
       <c r="H9" s="18">
-        <f>IFERROR(BDP($A9,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A9,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I9" s="18">
@@ -1551,7 +1555,7 @@
         <v/>
       </c>
       <c r="H10" s="24">
-        <f>IFERROR(BDP($A10,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A10,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I10" s="24">
@@ -1594,7 +1598,7 @@
         <v/>
       </c>
       <c r="H11" s="18">
-        <f>IFERROR(BDP($A11,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A11,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I11" s="18">
@@ -1637,7 +1641,7 @@
         <v/>
       </c>
       <c r="H12" s="24">
-        <f>IFERROR(BDP($A12,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A12,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I12" s="24">
@@ -1680,7 +1684,7 @@
         <v/>
       </c>
       <c r="H13" s="18">
-        <f>IFERROR(BDP($A13,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A13,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I13" s="18">
@@ -1723,7 +1727,7 @@
         <v/>
       </c>
       <c r="H14" s="24">
-        <f>IFERROR(BDP($A14,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A14,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I14" s="24">
@@ -1766,7 +1770,7 @@
         <v/>
       </c>
       <c r="H15" s="18">
-        <f>IFERROR(BDP($A15,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A15,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I15" s="18">
@@ -1809,7 +1813,7 @@
         <v/>
       </c>
       <c r="H16" s="24">
-        <f>IFERROR(BDP($A16,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A16,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I16" s="24">
@@ -1852,7 +1856,7 @@
         <v/>
       </c>
       <c r="H17" s="18">
-        <f>IFERROR(BDP($A17,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A17,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I17" s="18">
@@ -1895,7 +1899,7 @@
         <v/>
       </c>
       <c r="H18" s="24">
-        <f>IFERROR(BDP($A18,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A18,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I18" s="24">
@@ -1938,7 +1942,7 @@
         <v/>
       </c>
       <c r="H19" s="18">
-        <f>IFERROR(BDP($A19,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A19,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I19" s="18">
@@ -1981,7 +1985,7 @@
         <v/>
       </c>
       <c r="H20" s="24">
-        <f>IFERROR(BDP($A20,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A20,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I20" s="24">
@@ -2024,7 +2028,7 @@
         <v/>
       </c>
       <c r="H21" s="18">
-        <f>IFERROR(BDP($A21,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A21,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I21" s="18">
@@ -2067,7 +2071,7 @@
         <v/>
       </c>
       <c r="H22" s="24">
-        <f>IFERROR(BDP($A22,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A22,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I22" s="24">
@@ -2110,7 +2114,7 @@
         <v/>
       </c>
       <c r="H23" s="18">
-        <f>IFERROR(BDP($A23,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A23,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I23" s="18">
@@ -2153,7 +2157,7 @@
         <v/>
       </c>
       <c r="H24" s="24">
-        <f>IFERROR(BDP($A24,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A24,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I24" s="24">
@@ -2196,7 +2200,7 @@
         <v/>
       </c>
       <c r="H25" s="18">
-        <f>IFERROR(BDP($A25,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A25,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I25" s="18">
@@ -2239,7 +2243,7 @@
         <v/>
       </c>
       <c r="H26" s="24">
-        <f>IFERROR(BDP($A26,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A26,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I26" s="24">
@@ -2307,7 +2311,7 @@
       </c>
       <c r="H31" s="20" t="inlineStr">
         <is>
-          <t>FUT_CONTRACT_DATE</t>
+          <t>Ref. start (FUT_DLV_DT_FIRST)</t>
         </is>
       </c>
       <c r="I31" s="20" t="inlineStr">
@@ -2356,7 +2360,7 @@
         <v/>
       </c>
       <c r="H32" s="18">
-        <f>IFERROR(BDP($A32,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A32,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I32" s="18">
@@ -2399,7 +2403,7 @@
         <v/>
       </c>
       <c r="H33" s="24">
-        <f>IFERROR(BDP($A33,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A33,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I33" s="24">
@@ -2442,7 +2446,7 @@
         <v/>
       </c>
       <c r="H34" s="18">
-        <f>IFERROR(BDP($A34,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A34,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I34" s="18">
@@ -2485,7 +2489,7 @@
         <v/>
       </c>
       <c r="H35" s="24">
-        <f>IFERROR(BDP($A35,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A35,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I35" s="24">
@@ -2528,7 +2532,7 @@
         <v/>
       </c>
       <c r="H36" s="18">
-        <f>IFERROR(BDP($A36,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A36,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I36" s="18">
@@ -2571,7 +2575,7 @@
         <v/>
       </c>
       <c r="H37" s="24">
-        <f>IFERROR(BDP($A37,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A37,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I37" s="24">
@@ -2614,7 +2618,7 @@
         <v/>
       </c>
       <c r="H38" s="18">
-        <f>IFERROR(BDP($A38,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A38,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I38" s="18">
@@ -2657,7 +2661,7 @@
         <v/>
       </c>
       <c r="H39" s="24">
-        <f>IFERROR(BDP($A39,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A39,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I39" s="24">
@@ -2700,7 +2704,7 @@
         <v/>
       </c>
       <c r="H40" s="18">
-        <f>IFERROR(BDP($A40,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A40,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I40" s="18">
@@ -2743,7 +2747,7 @@
         <v/>
       </c>
       <c r="H41" s="24">
-        <f>IFERROR(BDP($A41,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A41,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I41" s="24">
@@ -2786,7 +2790,7 @@
         <v/>
       </c>
       <c r="H42" s="18">
-        <f>IFERROR(BDP($A42,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A42,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I42" s="18">
@@ -2829,7 +2833,7 @@
         <v/>
       </c>
       <c r="H43" s="24">
-        <f>IFERROR(BDP($A43,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A43,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I43" s="24">
@@ -2872,7 +2876,7 @@
         <v/>
       </c>
       <c r="H44" s="18">
-        <f>IFERROR(BDP($A44,"FUT_CONTRACT_DATE"),"")</f>
+        <f>IFERROR(BDP($A44,"FUT_DLV_DT_FIRST"),"")</f>
         <v/>
       </c>
       <c r="I44" s="18">
@@ -4565,7 +4569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4658,24 +4662,28 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>FLOATER_RESET_IDX</t>
-        </is>
-      </c>
-      <c r="C6" s="26">
-        <f>IFERROR(BDP("USOSFRC BGN Curncy","FLOATER_RESET_IDX"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="D6" s="26">
-        <f>IFERROR(BDP("USOSFR1 BGN Curncy","FLOATER_RESET_IDX"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="E6" s="26">
-        <f>IFERROR(BDP("USOSFR5 BGN Curncy","FLOATER_RESET_IDX"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="F6" s="26">
-        <f>IFERROR(BDP("USOSFR30 BGN Curncy","FLOATER_RESET_IDX"),"N/A — use FLDS")</f>
-        <v/>
+          <t>— DES/SWPM manual —</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -4686,24 +4694,28 @@
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>DAYS_TO_SETTLE</t>
-        </is>
-      </c>
-      <c r="C7" s="35">
-        <f>IFERROR(BDP("USOSFRC BGN Curncy","DAYS_TO_SETTLE"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="D7" s="35">
-        <f>IFERROR(BDP("USOSFR1 BGN Curncy","DAYS_TO_SETTLE"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="E7" s="35">
-        <f>IFERROR(BDP("USOSFR5 BGN Curncy","DAYS_TO_SETTLE"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="F7" s="35">
-        <f>IFERROR(BDP("USOSFR30 BGN Curncy","DAYS_TO_SETTLE"),"N/A — use FLDS")</f>
-        <v/>
+          <t>— DES/SWPM manual —</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="D7" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="E7" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="F7" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -4719,22 +4731,22 @@
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="E8" s="26" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
     </row>
@@ -4751,22 +4763,22 @@
       </c>
       <c r="C9" s="35" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="D9" s="35" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
     </row>
@@ -4811,22 +4823,22 @@
       </c>
       <c r="C11" s="35" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="D11" s="35" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
     </row>
@@ -4866,24 +4878,28 @@
       </c>
       <c r="B13" s="34" t="inlineStr">
         <is>
-          <t>CPN_FREQ</t>
-        </is>
-      </c>
-      <c r="C13" s="35">
-        <f>IFERROR(BDP("USOSFRC BGN Curncy","CPN_FREQ"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="D13" s="35">
-        <f>IFERROR(BDP("USOSFR1 BGN Curncy","CPN_FREQ"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="E13" s="35">
-        <f>IFERROR(BDP("USOSFR5 BGN Curncy","CPN_FREQ"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="F13" s="35">
-        <f>IFERROR(BDP("USOSFR30 BGN Curncy","CPN_FREQ"),"N/A — use FLDS")</f>
-        <v/>
+          <t>— DES/SWPM manual —</t>
+        </is>
+      </c>
+      <c r="C13" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="D13" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="E13" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="F13" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -4894,24 +4910,28 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>FLOATING_DAY_COUNT</t>
-        </is>
-      </c>
-      <c r="C14" s="26">
-        <f>IFERROR(BDP("USOSFRC BGN Curncy","FLOATING_DAY_COUNT"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="D14" s="26">
-        <f>IFERROR(BDP("USOSFR1 BGN Curncy","FLOATING_DAY_COUNT"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="E14" s="26">
-        <f>IFERROR(BDP("USOSFR5 BGN Curncy","FLOATING_DAY_COUNT"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="F14" s="26">
-        <f>IFERROR(BDP("USOSFR30 BGN Curncy","FLOATING_DAY_COUNT"),"N/A — use FLDS")</f>
-        <v/>
+          <t>— DES/SWPM manual —</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -4922,24 +4942,28 @@
       </c>
       <c r="B15" s="34" t="inlineStr">
         <is>
-          <t>FLOATING_PAY_FREQ</t>
-        </is>
-      </c>
-      <c r="C15" s="35">
-        <f>IFERROR(BDP("USOSFRC BGN Curncy","FLOATING_PAY_FREQ"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="D15" s="35">
-        <f>IFERROR(BDP("USOSFR1 BGN Curncy","FLOATING_PAY_FREQ"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="E15" s="35">
-        <f>IFERROR(BDP("USOSFR5 BGN Curncy","FLOATING_PAY_FREQ"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="F15" s="35">
-        <f>IFERROR(BDP("USOSFR30 BGN Curncy","FLOATING_PAY_FREQ"),"N/A — use FLDS")</f>
-        <v/>
+          <t>— DES/SWPM manual —</t>
+        </is>
+      </c>
+      <c r="C15" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="D15" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="E15" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="F15" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -4955,22 +4979,22 @@
       </c>
       <c r="C16" s="26" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="E16" s="26" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
     </row>
@@ -4982,24 +5006,28 @@
       </c>
       <c r="B17" s="34" t="inlineStr">
         <is>
-          <t>PAY_LAG</t>
-        </is>
-      </c>
-      <c r="C17" s="35">
-        <f>IFERROR(BDP("USOSFRC BGN Curncy","PAY_LAG"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="D17" s="35">
-        <f>IFERROR(BDP("USOSFR1 BGN Curncy","PAY_LAG"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="E17" s="35">
-        <f>IFERROR(BDP("USOSFR5 BGN Curncy","PAY_LAG"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="F17" s="35">
-        <f>IFERROR(BDP("USOSFR30 BGN Curncy","PAY_LAG"),"N/A — use FLDS")</f>
-        <v/>
+          <t>— DES/SWPM manual —</t>
+        </is>
+      </c>
+      <c r="C17" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="E17" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="F17" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -5015,22 +5043,22 @@
       </c>
       <c r="C18" s="26" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="D18" s="26" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="E18" s="26" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>(read from DES/SWPM)</t>
+          <t>— DES/SWPM —</t>
         </is>
       </c>
     </row>
@@ -5042,39 +5070,272 @@
       </c>
       <c r="B19" s="34" t="inlineStr">
         <is>
-          <t>EOM_ADJ</t>
-        </is>
-      </c>
-      <c r="C19" s="35">
-        <f>IFERROR(BDP("USOSFRC BGN Curncy","EOM_ADJ"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="D19" s="35">
-        <f>IFERROR(BDP("USOSFR1 BGN Curncy","EOM_ADJ"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="E19" s="35">
-        <f>IFERROR(BDP("USOSFR5 BGN Curncy","EOM_ADJ"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-      <c r="F19" s="35">
-        <f>IFERROR(BDP("USOSFR30 BGN Curncy","EOM_ADJ"),"N/A — use FLDS")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>SWPM &lt;GO&gt;: build a representative SOFR OIS for 1Y, 5Y and 30Y and export the cashflow schedule — that gives an authoritative set of pay/accrual dates to test your own date generation against. Field mnemonics above are best-guess and entitlement-dependent: where a cell shows 'N/A — use FLDS', open FLDS &lt;GO&gt; on that security to find the enabled field.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
+          <t>— DES/SWPM manual —</t>
+        </is>
+      </c>
+      <c r="C19" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="E19" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+      <c r="F19" s="35" t="inlineStr">
+        <is>
+          <t>— DES/SWPM —</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>USD SOFR OIS — MARKET-STANDARD CONVENTIONS  (confirm per-trade in DES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Reference index</t>
+        </is>
+      </c>
+      <c r="B22" s="36" t="inlineStr">
+        <is>
+          <t>USD-SOFR (compounded in arrears)</t>
+        </is>
+      </c>
+      <c r="C22" s="37" t="n"/>
+      <c r="D22" s="37" t="n"/>
+      <c r="E22" s="37" t="n"/>
+      <c r="F22" s="37" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Spot / settlement lag</t>
+        </is>
+      </c>
+      <c r="B23" s="36" t="inlineStr">
+        <is>
+          <t>T+2 US business days</t>
+        </is>
+      </c>
+      <c r="C23" s="37" t="n"/>
+      <c r="D23" s="37" t="n"/>
+      <c r="E23" s="37" t="n"/>
+      <c r="F23" s="37" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Effective date rule</t>
+        </is>
+      </c>
+      <c r="B24" s="36" t="inlineStr">
+        <is>
+          <t>Spot (T+2), modified following</t>
+        </is>
+      </c>
+      <c r="C24" s="37" t="n"/>
+      <c r="D24" s="37" t="n"/>
+      <c r="E24" s="37" t="n"/>
+      <c r="F24" s="37" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Maturity date rule</t>
+        </is>
+      </c>
+      <c r="B25" s="36" t="inlineStr">
+        <is>
+          <t>Effective + tenor, modified following</t>
+        </is>
+      </c>
+      <c r="C25" s="37" t="n"/>
+      <c r="D25" s="37" t="n"/>
+      <c r="E25" s="37" t="n"/>
+      <c r="F25" s="37" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Business-day convention</t>
+        </is>
+      </c>
+      <c r="B26" s="36" t="inlineStr">
+        <is>
+          <t>Modified Following</t>
+        </is>
+      </c>
+      <c r="C26" s="37" t="n"/>
+      <c r="D26" s="37" t="n"/>
+      <c r="E26" s="37" t="n"/>
+      <c r="F26" s="37" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>Fixed-leg day count</t>
+        </is>
+      </c>
+      <c r="B27" s="36" t="inlineStr">
+        <is>
+          <t>ACT/360</t>
+        </is>
+      </c>
+      <c r="C27" s="37" t="n"/>
+      <c r="D27" s="37" t="n"/>
+      <c r="E27" s="37" t="n"/>
+      <c r="F27" s="37" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Fixed-leg pay frequency</t>
+        </is>
+      </c>
+      <c r="B28" s="36" t="inlineStr">
+        <is>
+          <t>Annual  (single payment if tenor ≤ 1Y)</t>
+        </is>
+      </c>
+      <c r="C28" s="37" t="n"/>
+      <c r="D28" s="37" t="n"/>
+      <c r="E28" s="37" t="n"/>
+      <c r="F28" s="37" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Floating-leg day count</t>
+        </is>
+      </c>
+      <c r="B29" s="36" t="inlineStr">
+        <is>
+          <t>ACT/360</t>
+        </is>
+      </c>
+      <c r="C29" s="37" t="n"/>
+      <c r="D29" s="37" t="n"/>
+      <c r="E29" s="37" t="n"/>
+      <c r="F29" s="37" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Floating-leg pay frequency</t>
+        </is>
+      </c>
+      <c r="B30" s="36" t="inlineStr">
+        <is>
+          <t>Annual  (single payment if tenor ≤ 1Y)</t>
+        </is>
+      </c>
+      <c r="C30" s="37" t="n"/>
+      <c r="D30" s="37" t="n"/>
+      <c r="E30" s="37" t="n"/>
+      <c r="F30" s="37" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>SOFR compounding method</t>
+        </is>
+      </c>
+      <c r="B31" s="36" t="inlineStr">
+        <is>
+          <t>Daily compounded, ACT/360</t>
+        </is>
+      </c>
+      <c r="C31" s="37" t="n"/>
+      <c r="D31" s="37" t="n"/>
+      <c r="E31" s="37" t="n"/>
+      <c r="F31" s="37" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Payment lag</t>
+        </is>
+      </c>
+      <c r="B32" s="36" t="inlineStr">
+        <is>
+          <t>2 US business days</t>
+        </is>
+      </c>
+      <c r="C32" s="37" t="n"/>
+      <c r="D32" s="37" t="n"/>
+      <c r="E32" s="37" t="n"/>
+      <c r="F32" s="37" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Observation shift / lookback</t>
+        </is>
+      </c>
+      <c r="B33" s="36" t="inlineStr">
+        <is>
+          <t>None (payment-delay convention, 2 bd)</t>
+        </is>
+      </c>
+      <c r="C33" s="37" t="n"/>
+      <c r="D33" s="37" t="n"/>
+      <c r="E33" s="37" t="n"/>
+      <c r="F33" s="37" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>End-of-month treatment</t>
+        </is>
+      </c>
+      <c r="B34" s="36" t="inlineStr">
+        <is>
+          <t>EOM applies</t>
+        </is>
+      </c>
+      <c r="C34" s="37" t="n"/>
+      <c r="D34" s="37" t="n"/>
+      <c r="E34" s="37" t="n"/>
+      <c r="F34" s="37" t="n"/>
+    </row>
+    <row r="36" ht="44" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>SWPM &lt;GO&gt;: build a representative SOFR OIS for 1Y, 5Y and 30Y and export the cashflow schedule — that gives an authoritative set of pay/accrual dates to test your own date generation against. Rows marked '— DES/SWPM —' are leg-level conventions that a rate-quote ticker does not carry; read them from DES &lt;GO&gt; on an actual swap (the market-standard defaults above are the expected values). Where a BDP cell shows 'N/A — use FLDS', open FLDS &lt;GO&gt; to find the enabled field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="17">
+    <mergeCell ref="B30:F30"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="B33:F33"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A21:F22"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="A36:F37"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B27:F27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Make workbook self-contained: add bootstrap methodology to Instructions
The Excel file is the deliverable, so it should explain itself. Adds a
methodology section (three liquid segments + bootstrap order) and the three
conceptual differences from the Lehman 2002 build (single-curve, overnight
compounding, futures convexity) alongside the existing Lehman->modern mapping.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1019,108 +1019,191 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
+          <t>BOOTSTRAP METHODOLOGY  —  one discount curve, three liquid segments</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>Short end (o/n – ~1Y)</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>SOFR fixing + short OIS (1W,1M,3M,6M) anchor P(0,T) at the front — the modern LIBOR-deposit segment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>Mid (~3M – ~5Y)</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>SR3 3M-SOFR futures; implied rate = 100 − price, each covering one 3M IMM reference quarter — the modern Eurodollar-futures segment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>Long end (~2Y – 50Y)</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>SOFR OIS par swaps (mid = (bid+ask)/2) where deep liquidity lives — the modern LIBOR-swap segment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>Bootstrap order</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Left → right: each instrument solves for the next discount-factor pillar given everything already solved to its left (sequential 1-D root find).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>Three differences vs. Lehman 2002 (where 'modern' is not a literal copy):</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>•  Single-curve: the SOFR curve both projects forwards AND discounts. Lehman 2002 was also single-curve (LIBOR did both), so a SOFR OIS build is CLOSER to the paper than a modern LIBOR build would be.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>•  Compounding: SOFR is an overnight rate compounded daily in arrears over each period; LIBOR was a term rate set once. The OIS/futures legs carry a daily-compounding calc LIBOR did not need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>•  Futures convexity: SR3 (like Eurodollar) futures need a small convexity adjustment before the implied rate enters the curve. A first pass can omit it and report the bias against the S490 benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
           <t>TABS IN THIS WORKBOOK</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>1. SOFR_Fixings</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Overnight SOFR fixing — current (BDP) + daily history (BDH).</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="15" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>2. SOFR_Futures</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>SR3 (3M) and SR1 (1M) SOFR futures chains + fields + implied rate = 100 − price.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>3. SOFR_OIS_Quotes</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>Full USOSFR OIS strip (1W–50Y): bid / ask / last + mid. Bootstrap-set flagged.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>4. Bloomberg_S490_Validation</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Bloomberg's own USD SOFR curve (S490) for benchmarking your bootstrap.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="15" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr">
         <is>
           <t>5. Conventions</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>DES/SWPM conventions for representative OIS (spot lag, day counts, compounding, EOM…).</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
         <is>
           <t>DO NOT substitute these (wrong instruments):</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t>•  TSFR1M/3M/6M/12M Index  — Term SOFR benchmarks, NOT overnight-SOFR OIS calibration instruments.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="11" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
         <is>
           <t>•  USISSO02/05/10/30 Index — ICE Swap Rate fixings, NOT the live OIS quote strip needed to bootstrap.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="11" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>•  Use PX midpoint (bid+ask)/2 for construction; use PX_LAST only where bid/ask are unavailable.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
+    <row r="47" ht="28" customHeight="1">
+      <c r="A47" s="11" t="inlineStr">
         <is>
           <t>Licensing: Bloomberg data is licensed and entitlement-dependent — do NOT redistribute pulled values or commit them to a public repository. This template ships formulas only, no data. Some static convention fields may return N/A under your entitlement; use FLDS &lt;GO&gt; on the security to find the enabled mnemonic.</t>
         </is>
       </c>
     </row>
-    <row r="37"/>
+    <row r="48"/>
   </sheetData>
-  <mergeCells count="41">
+  <mergeCells count="50">
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="D13:F13"/>
@@ -1131,37 +1214,46 @@
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="A33:F33"/>
     <mergeCell ref="E20:F20"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="A42:F42"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="D12:F12"/>
     <mergeCell ref="D9:F9"/>
     <mergeCell ref="C22:D22"/>
+    <mergeCell ref="A35:F35"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="D8:F8"/>
-    <mergeCell ref="A36:F37"/>
+    <mergeCell ref="A43:F43"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="D14:F14"/>
-    <mergeCell ref="B29:F29"/>
     <mergeCell ref="C21:D21"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="A44:F44"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="B37:F37"/>
     <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A30:F30"/>
     <mergeCell ref="C17:D17"/>
+    <mergeCell ref="B40:F40"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="D10:F10"/>
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A45:F45"/>
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="E22:F22"/>
+    <mergeCell ref="B36:F36"/>
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="A4:F5"/>
     <mergeCell ref="E18:F18"/>
     <mergeCell ref="B26:F26"/>
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="E21:F21"/>
+    <mergeCell ref="A47:F48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add in-Excel OIS bootstrap tab; fix S490 validation errors
Bootstrap tab: single-curve par-OIS bootstrap from the OIS mid strip,
DF_n = (1 - S_n*A_(n-1))/(1 + S_n*tau_n), producing discount factors, cont.
zero rates (-ln DF / T), simple forwards, and a Delta-z vs S490 paste column.
Recursion validated numerically (all DF > 0, strictly decreasing, zeros track
the par-strip hump). Exact <=10Y; sparse long end uses a labeled pillar-grid
coupon approximation.

S490 fixes: CURVE_DT is an invalid field -> curve date now references VAL_DATE;
CURVE_TENOR_RATES spill columns don't match fixed headers (showed 1900-dates
and date-serials-as-DFs) -> relabeled as a raw dump with General formatting and
routed the real comparison to the Bootstrap tab.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOFR_Fixings" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOFR_Futures" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOFR_OIS_Quotes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloomberg_S490_Validation" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conventions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bootstrap" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloomberg_S490_Validation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conventions" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="VAL_DATE">Instructions!$B$9</definedName>
@@ -28,10 +29,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.00000000"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -225,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -281,9 +283,14 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="11" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -709,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1145,68 +1152,81 @@
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
         <is>
-          <t>4. Bloomberg_S490_Validation</t>
+          <t>4. Bootstrap</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Bloomberg's own USD SOFR curve (S490) for benchmarking your bootstrap.</t>
+          <t>Live single-curve OIS bootstrap → discount factors, zero &amp; forward rates, S490 Δz check.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
         <is>
-          <t>5. Conventions</t>
+          <t>5. Bloomberg_S490_Validation</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
+          <t>Bloomberg's own USD SOFR curve (S490) for benchmarking your bootstrap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>6. Conventions</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
           <t>DES/SWPM conventions for representative OIS (spot lag, day counts, compounding, EOM…).</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="16" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
         <is>
           <t>DO NOT substitute these (wrong instruments):</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="11" t="inlineStr">
-        <is>
-          <t>•  TSFR1M/3M/6M/12M Index  — Term SOFR benchmarks, NOT overnight-SOFR OIS calibration instruments.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>•  USISSO02/05/10/30 Index — ICE Swap Rate fixings, NOT the live OIS quote strip needed to bootstrap.</t>
+          <t>•  TSFR1M/3M/6M/12M Index  — Term SOFR benchmarks, NOT overnight-SOFR OIS calibration instruments.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
         <is>
+          <t>•  USISSO02/05/10/30 Index — ICE Swap Rate fixings, NOT the live OIS quote strip needed to bootstrap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
           <t>•  Use PX midpoint (bid+ask)/2 for construction; use PX_LAST only where bid/ask are unavailable.</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="28" customHeight="1">
-      <c r="A47" s="11" t="inlineStr">
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="11" t="inlineStr">
         <is>
           <t>Licensing: Bloomberg data is licensed and entitlement-dependent — do NOT redistribute pulled values or commit them to a public repository. This template ships formulas only, no data. Some static convention fields may return N/A under your entitlement; use FLDS &lt;GO&gt; on the security to find the enabled mnemonic.</t>
         </is>
       </c>
     </row>
-    <row r="48"/>
+    <row r="49"/>
   </sheetData>
-  <mergeCells count="50">
+  <mergeCells count="51">
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="D13:F13"/>
+    <mergeCell ref="A46:F46"/>
     <mergeCell ref="B25:F25"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="B27:F27"/>
@@ -1215,7 +1235,7 @@
     <mergeCell ref="A33:F33"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="B39:F39"/>
-    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A48:F49"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="D12:F12"/>
@@ -1251,9 +1271,9 @@
     <mergeCell ref="A4:F5"/>
     <mergeCell ref="E18:F18"/>
     <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B41:F41"/>
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="E21:F21"/>
-    <mergeCell ref="A47:F48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4188,6 +4208,1544 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Bootstrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Single-curve OIS bootstrap from the SOFR_OIS_Quotes mid strip → discount factors, zero &amp; forward rates</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Spot (T+2):</t>
+        </is>
+      </c>
+      <c r="B4" s="24">
+        <f>WORKDAY(VAL_DATE,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Par-OIS recursive bootstrap on the quoted tenor grid:  DF_n = (1 − S_n·A_(n-1)) / (1 + S_n·τ_n),  with A_(n-1) = Σ τ_i·DF_i.  Exact for the sub-1Y money-market points and the annual 1Y–10Y section (pillars coincide with coupon dates); the sparse long end (12–50Y) uses the pillar grid AS the coupon schedule — a standard, transparent approximation (the openusdcurve engine does the exact interpolated-annuity build). Par rates are pulled live from the SOFR_OIS_Quotes mid column; paste Bloomberg S490 zero rates into column J for the Δz check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Maturity date</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>T (yrs)</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>τ ACT/360</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>Par rate S (%)</t>
+        </is>
+      </c>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>Annuity Στ·DF (prior)</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>Discount factor</t>
+        </is>
+      </c>
+      <c r="H7" s="20" t="inlineStr">
+        <is>
+          <t>Zero rate (%) cont.</t>
+        </is>
+      </c>
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>Fwd rate (%) simple</t>
+        </is>
+      </c>
+      <c r="J7" s="20" t="inlineStr">
+        <is>
+          <t>S490 zero (%) [paste]</t>
+        </is>
+      </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>Δ vs S490 (bp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>1W</t>
+        </is>
+      </c>
+      <c r="B8" s="18">
+        <f>$B$4+7</f>
+        <v/>
+      </c>
+      <c r="C8" s="31">
+        <f>(B8-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D8" s="21">
+        <f>(B8-$B$4)/360</f>
+        <v/>
+      </c>
+      <c r="E8" s="21">
+        <f>'SOFR_OIS_Quotes'!$G5</f>
+        <v/>
+      </c>
+      <c r="F8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="32">
+        <f>(1-(E8/100)*F8)/(1+(E8/100)*D8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="21">
+        <f>-LN(G8)/C8*100</f>
+        <v/>
+      </c>
+      <c r="I8" s="21">
+        <f>(1/G8-1)/D8*100</f>
+        <v/>
+      </c>
+      <c r="J8" s="33" t="n"/>
+      <c r="K8" s="34">
+        <f>IF(J8="","",(H8-J8)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="B9" s="24">
+        <f>$B$4+14</f>
+        <v/>
+      </c>
+      <c r="C9" s="35">
+        <f>(B9-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D9" s="17">
+        <f>(B9-B8)/360</f>
+        <v/>
+      </c>
+      <c r="E9" s="17">
+        <f>'SOFR_OIS_Quotes'!$G6</f>
+        <v/>
+      </c>
+      <c r="F9" s="17">
+        <f>F8+D8*G8</f>
+        <v/>
+      </c>
+      <c r="G9" s="36">
+        <f>(1-(E9/100)*F9)/(1+(E9/100)*D9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="17">
+        <f>-LN(G9)/C9*100</f>
+        <v/>
+      </c>
+      <c r="I9" s="17">
+        <f>(G8/G9-1)/D9*100</f>
+        <v/>
+      </c>
+      <c r="J9" s="33" t="n"/>
+      <c r="K9" s="37">
+        <f>IF(J9="","",(H9-J9)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>3W</t>
+        </is>
+      </c>
+      <c r="B10" s="18">
+        <f>$B$4+21</f>
+        <v/>
+      </c>
+      <c r="C10" s="31">
+        <f>(B10-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D10" s="21">
+        <f>(B10-B9)/360</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>'SOFR_OIS_Quotes'!$G7</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>F9+D9*G9</f>
+        <v/>
+      </c>
+      <c r="G10" s="32">
+        <f>(1-(E10/100)*F10)/(1+(E10/100)*D10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="21">
+        <f>-LN(G10)/C10*100</f>
+        <v/>
+      </c>
+      <c r="I10" s="21">
+        <f>(G9/G10-1)/D10*100</f>
+        <v/>
+      </c>
+      <c r="J10" s="33" t="n"/>
+      <c r="K10" s="34">
+        <f>IF(J10="","",(H10-J10)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="B11" s="24">
+        <f>EDATE($B$4,1)</f>
+        <v/>
+      </c>
+      <c r="C11" s="35">
+        <f>(B11-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D11" s="17">
+        <f>(B11-B10)/360</f>
+        <v/>
+      </c>
+      <c r="E11" s="17">
+        <f>'SOFR_OIS_Quotes'!$G8</f>
+        <v/>
+      </c>
+      <c r="F11" s="17">
+        <f>F10+D10*G10</f>
+        <v/>
+      </c>
+      <c r="G11" s="36">
+        <f>(1-(E11/100)*F11)/(1+(E11/100)*D11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="17">
+        <f>-LN(G11)/C11*100</f>
+        <v/>
+      </c>
+      <c r="I11" s="17">
+        <f>(G10/G11-1)/D11*100</f>
+        <v/>
+      </c>
+      <c r="J11" s="33" t="n"/>
+      <c r="K11" s="37">
+        <f>IF(J11="","",(H11-J11)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>2M</t>
+        </is>
+      </c>
+      <c r="B12" s="18">
+        <f>EDATE($B$4,2)</f>
+        <v/>
+      </c>
+      <c r="C12" s="31">
+        <f>(B12-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D12" s="21">
+        <f>(B12-B11)/360</f>
+        <v/>
+      </c>
+      <c r="E12" s="21">
+        <f>'SOFR_OIS_Quotes'!$G9</f>
+        <v/>
+      </c>
+      <c r="F12" s="21">
+        <f>F11+D11*G11</f>
+        <v/>
+      </c>
+      <c r="G12" s="32">
+        <f>(1-(E12/100)*F12)/(1+(E12/100)*D12)</f>
+        <v/>
+      </c>
+      <c r="H12" s="21">
+        <f>-LN(G12)/C12*100</f>
+        <v/>
+      </c>
+      <c r="I12" s="21">
+        <f>(G11/G12-1)/D12*100</f>
+        <v/>
+      </c>
+      <c r="J12" s="33" t="n"/>
+      <c r="K12" s="34">
+        <f>IF(J12="","",(H12-J12)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>3M</t>
+        </is>
+      </c>
+      <c r="B13" s="24">
+        <f>EDATE($B$4,3)</f>
+        <v/>
+      </c>
+      <c r="C13" s="35">
+        <f>(B13-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D13" s="17">
+        <f>(B13-B12)/360</f>
+        <v/>
+      </c>
+      <c r="E13" s="17">
+        <f>'SOFR_OIS_Quotes'!$G10</f>
+        <v/>
+      </c>
+      <c r="F13" s="17">
+        <f>F12+D12*G12</f>
+        <v/>
+      </c>
+      <c r="G13" s="36">
+        <f>(1-(E13/100)*F13)/(1+(E13/100)*D13)</f>
+        <v/>
+      </c>
+      <c r="H13" s="17">
+        <f>-LN(G13)/C13*100</f>
+        <v/>
+      </c>
+      <c r="I13" s="17">
+        <f>(G12/G13-1)/D13*100</f>
+        <v/>
+      </c>
+      <c r="J13" s="33" t="n"/>
+      <c r="K13" s="37">
+        <f>IF(J13="","",(H13-J13)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>4M</t>
+        </is>
+      </c>
+      <c r="B14" s="18">
+        <f>EDATE($B$4,4)</f>
+        <v/>
+      </c>
+      <c r="C14" s="31">
+        <f>(B14-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D14" s="21">
+        <f>(B14-B13)/360</f>
+        <v/>
+      </c>
+      <c r="E14" s="21">
+        <f>'SOFR_OIS_Quotes'!$G11</f>
+        <v/>
+      </c>
+      <c r="F14" s="21">
+        <f>F13+D13*G13</f>
+        <v/>
+      </c>
+      <c r="G14" s="32">
+        <f>(1-(E14/100)*F14)/(1+(E14/100)*D14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="21">
+        <f>-LN(G14)/C14*100</f>
+        <v/>
+      </c>
+      <c r="I14" s="21">
+        <f>(G13/G14-1)/D14*100</f>
+        <v/>
+      </c>
+      <c r="J14" s="33" t="n"/>
+      <c r="K14" s="34">
+        <f>IF(J14="","",(H14-J14)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>5M</t>
+        </is>
+      </c>
+      <c r="B15" s="24">
+        <f>EDATE($B$4,5)</f>
+        <v/>
+      </c>
+      <c r="C15" s="35">
+        <f>(B15-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D15" s="17">
+        <f>(B15-B14)/360</f>
+        <v/>
+      </c>
+      <c r="E15" s="17">
+        <f>'SOFR_OIS_Quotes'!$G12</f>
+        <v/>
+      </c>
+      <c r="F15" s="17">
+        <f>F14+D14*G14</f>
+        <v/>
+      </c>
+      <c r="G15" s="36">
+        <f>(1-(E15/100)*F15)/(1+(E15/100)*D15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="17">
+        <f>-LN(G15)/C15*100</f>
+        <v/>
+      </c>
+      <c r="I15" s="17">
+        <f>(G14/G15-1)/D15*100</f>
+        <v/>
+      </c>
+      <c r="J15" s="33" t="n"/>
+      <c r="K15" s="37">
+        <f>IF(J15="","",(H15-J15)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>6M</t>
+        </is>
+      </c>
+      <c r="B16" s="18">
+        <f>EDATE($B$4,6)</f>
+        <v/>
+      </c>
+      <c r="C16" s="31">
+        <f>(B16-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D16" s="21">
+        <f>(B16-B15)/360</f>
+        <v/>
+      </c>
+      <c r="E16" s="21">
+        <f>'SOFR_OIS_Quotes'!$G13</f>
+        <v/>
+      </c>
+      <c r="F16" s="21">
+        <f>F15+D15*G15</f>
+        <v/>
+      </c>
+      <c r="G16" s="32">
+        <f>(1-(E16/100)*F16)/(1+(E16/100)*D16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="21">
+        <f>-LN(G16)/C16*100</f>
+        <v/>
+      </c>
+      <c r="I16" s="21">
+        <f>(G15/G16-1)/D16*100</f>
+        <v/>
+      </c>
+      <c r="J16" s="33" t="n"/>
+      <c r="K16" s="34">
+        <f>IF(J16="","",(H16-J16)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>7M</t>
+        </is>
+      </c>
+      <c r="B17" s="24">
+        <f>EDATE($B$4,7)</f>
+        <v/>
+      </c>
+      <c r="C17" s="35">
+        <f>(B17-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D17" s="17">
+        <f>(B17-B16)/360</f>
+        <v/>
+      </c>
+      <c r="E17" s="17">
+        <f>'SOFR_OIS_Quotes'!$G14</f>
+        <v/>
+      </c>
+      <c r="F17" s="17">
+        <f>F16+D16*G16</f>
+        <v/>
+      </c>
+      <c r="G17" s="36">
+        <f>(1-(E17/100)*F17)/(1+(E17/100)*D17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="17">
+        <f>-LN(G17)/C17*100</f>
+        <v/>
+      </c>
+      <c r="I17" s="17">
+        <f>(G16/G17-1)/D17*100</f>
+        <v/>
+      </c>
+      <c r="J17" s="33" t="n"/>
+      <c r="K17" s="37">
+        <f>IF(J17="","",(H17-J17)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>8M</t>
+        </is>
+      </c>
+      <c r="B18" s="18">
+        <f>EDATE($B$4,8)</f>
+        <v/>
+      </c>
+      <c r="C18" s="31">
+        <f>(B18-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D18" s="21">
+        <f>(B18-B17)/360</f>
+        <v/>
+      </c>
+      <c r="E18" s="21">
+        <f>'SOFR_OIS_Quotes'!$G15</f>
+        <v/>
+      </c>
+      <c r="F18" s="21">
+        <f>F17+D17*G17</f>
+        <v/>
+      </c>
+      <c r="G18" s="32">
+        <f>(1-(E18/100)*F18)/(1+(E18/100)*D18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="21">
+        <f>-LN(G18)/C18*100</f>
+        <v/>
+      </c>
+      <c r="I18" s="21">
+        <f>(G17/G18-1)/D18*100</f>
+        <v/>
+      </c>
+      <c r="J18" s="33" t="n"/>
+      <c r="K18" s="34">
+        <f>IF(J18="","",(H18-J18)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>9M</t>
+        </is>
+      </c>
+      <c r="B19" s="24">
+        <f>EDATE($B$4,9)</f>
+        <v/>
+      </c>
+      <c r="C19" s="35">
+        <f>(B19-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D19" s="17">
+        <f>(B19-B18)/360</f>
+        <v/>
+      </c>
+      <c r="E19" s="17">
+        <f>'SOFR_OIS_Quotes'!$G16</f>
+        <v/>
+      </c>
+      <c r="F19" s="17">
+        <f>F18+D18*G18</f>
+        <v/>
+      </c>
+      <c r="G19" s="36">
+        <f>(1-(E19/100)*F19)/(1+(E19/100)*D19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="17">
+        <f>-LN(G19)/C19*100</f>
+        <v/>
+      </c>
+      <c r="I19" s="17">
+        <f>(G18/G19-1)/D19*100</f>
+        <v/>
+      </c>
+      <c r="J19" s="33" t="n"/>
+      <c r="K19" s="37">
+        <f>IF(J19="","",(H19-J19)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>10M</t>
+        </is>
+      </c>
+      <c r="B20" s="18">
+        <f>EDATE($B$4,10)</f>
+        <v/>
+      </c>
+      <c r="C20" s="31">
+        <f>(B20-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D20" s="21">
+        <f>(B20-B19)/360</f>
+        <v/>
+      </c>
+      <c r="E20" s="21">
+        <f>'SOFR_OIS_Quotes'!$G17</f>
+        <v/>
+      </c>
+      <c r="F20" s="21">
+        <f>F19+D19*G19</f>
+        <v/>
+      </c>
+      <c r="G20" s="32">
+        <f>(1-(E20/100)*F20)/(1+(E20/100)*D20)</f>
+        <v/>
+      </c>
+      <c r="H20" s="21">
+        <f>-LN(G20)/C20*100</f>
+        <v/>
+      </c>
+      <c r="I20" s="21">
+        <f>(G19/G20-1)/D20*100</f>
+        <v/>
+      </c>
+      <c r="J20" s="33" t="n"/>
+      <c r="K20" s="34">
+        <f>IF(J20="","",(H20-J20)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>11M</t>
+        </is>
+      </c>
+      <c r="B21" s="24">
+        <f>EDATE($B$4,11)</f>
+        <v/>
+      </c>
+      <c r="C21" s="35">
+        <f>(B21-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D21" s="17">
+        <f>(B21-B20)/360</f>
+        <v/>
+      </c>
+      <c r="E21" s="17">
+        <f>'SOFR_OIS_Quotes'!$G18</f>
+        <v/>
+      </c>
+      <c r="F21" s="17">
+        <f>F20+D20*G20</f>
+        <v/>
+      </c>
+      <c r="G21" s="36">
+        <f>(1-(E21/100)*F21)/(1+(E21/100)*D21)</f>
+        <v/>
+      </c>
+      <c r="H21" s="17">
+        <f>-LN(G21)/C21*100</f>
+        <v/>
+      </c>
+      <c r="I21" s="17">
+        <f>(G20/G21-1)/D21*100</f>
+        <v/>
+      </c>
+      <c r="J21" s="33" t="n"/>
+      <c r="K21" s="37">
+        <f>IF(J21="","",(H21-J21)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>1Y</t>
+        </is>
+      </c>
+      <c r="B22" s="18">
+        <f>EDATE($B$4,12)</f>
+        <v/>
+      </c>
+      <c r="C22" s="31">
+        <f>(B22-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D22" s="21">
+        <f>(B22-B21)/360</f>
+        <v/>
+      </c>
+      <c r="E22" s="21">
+        <f>'SOFR_OIS_Quotes'!$G19</f>
+        <v/>
+      </c>
+      <c r="F22" s="21">
+        <f>F21+D21*G21</f>
+        <v/>
+      </c>
+      <c r="G22" s="32">
+        <f>(1-(E22/100)*F22)/(1+(E22/100)*D22)</f>
+        <v/>
+      </c>
+      <c r="H22" s="21">
+        <f>-LN(G22)/C22*100</f>
+        <v/>
+      </c>
+      <c r="I22" s="21">
+        <f>(G21/G22-1)/D22*100</f>
+        <v/>
+      </c>
+      <c r="J22" s="33" t="n"/>
+      <c r="K22" s="34">
+        <f>IF(J22="","",(H22-J22)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>18M</t>
+        </is>
+      </c>
+      <c r="B23" s="24">
+        <f>EDATE($B$4,18)</f>
+        <v/>
+      </c>
+      <c r="C23" s="35">
+        <f>(B23-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D23" s="17">
+        <f>(B23-B22)/360</f>
+        <v/>
+      </c>
+      <c r="E23" s="17">
+        <f>'SOFR_OIS_Quotes'!$G20</f>
+        <v/>
+      </c>
+      <c r="F23" s="17">
+        <f>F22+D22*G22</f>
+        <v/>
+      </c>
+      <c r="G23" s="36">
+        <f>(1-(E23/100)*F23)/(1+(E23/100)*D23)</f>
+        <v/>
+      </c>
+      <c r="H23" s="17">
+        <f>-LN(G23)/C23*100</f>
+        <v/>
+      </c>
+      <c r="I23" s="17">
+        <f>(G22/G23-1)/D23*100</f>
+        <v/>
+      </c>
+      <c r="J23" s="33" t="n"/>
+      <c r="K23" s="37">
+        <f>IF(J23="","",(H23-J23)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="B24" s="18">
+        <f>EDATE($B$4,24)</f>
+        <v/>
+      </c>
+      <c r="C24" s="31">
+        <f>(B24-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D24" s="21">
+        <f>(B24-B23)/360</f>
+        <v/>
+      </c>
+      <c r="E24" s="21">
+        <f>'SOFR_OIS_Quotes'!$G21</f>
+        <v/>
+      </c>
+      <c r="F24" s="21">
+        <f>F23+D23*G23</f>
+        <v/>
+      </c>
+      <c r="G24" s="32">
+        <f>(1-(E24/100)*F24)/(1+(E24/100)*D24)</f>
+        <v/>
+      </c>
+      <c r="H24" s="21">
+        <f>-LN(G24)/C24*100</f>
+        <v/>
+      </c>
+      <c r="I24" s="21">
+        <f>(G23/G24-1)/D24*100</f>
+        <v/>
+      </c>
+      <c r="J24" s="33" t="n"/>
+      <c r="K24" s="34">
+        <f>IF(J24="","",(H24-J24)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="B25" s="24">
+        <f>EDATE($B$4,36)</f>
+        <v/>
+      </c>
+      <c r="C25" s="35">
+        <f>(B25-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D25" s="17">
+        <f>(B25-B24)/360</f>
+        <v/>
+      </c>
+      <c r="E25" s="17">
+        <f>'SOFR_OIS_Quotes'!$G22</f>
+        <v/>
+      </c>
+      <c r="F25" s="17">
+        <f>F24+D24*G24</f>
+        <v/>
+      </c>
+      <c r="G25" s="36">
+        <f>(1-(E25/100)*F25)/(1+(E25/100)*D25)</f>
+        <v/>
+      </c>
+      <c r="H25" s="17">
+        <f>-LN(G25)/C25*100</f>
+        <v/>
+      </c>
+      <c r="I25" s="17">
+        <f>(G24/G25-1)/D25*100</f>
+        <v/>
+      </c>
+      <c r="J25" s="33" t="n"/>
+      <c r="K25" s="37">
+        <f>IF(J25="","",(H25-J25)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>4Y</t>
+        </is>
+      </c>
+      <c r="B26" s="18">
+        <f>EDATE($B$4,48)</f>
+        <v/>
+      </c>
+      <c r="C26" s="31">
+        <f>(B26-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D26" s="21">
+        <f>(B26-B25)/360</f>
+        <v/>
+      </c>
+      <c r="E26" s="21">
+        <f>'SOFR_OIS_Quotes'!$G23</f>
+        <v/>
+      </c>
+      <c r="F26" s="21">
+        <f>F25+D25*G25</f>
+        <v/>
+      </c>
+      <c r="G26" s="32">
+        <f>(1-(E26/100)*F26)/(1+(E26/100)*D26)</f>
+        <v/>
+      </c>
+      <c r="H26" s="21">
+        <f>-LN(G26)/C26*100</f>
+        <v/>
+      </c>
+      <c r="I26" s="21">
+        <f>(G25/G26-1)/D26*100</f>
+        <v/>
+      </c>
+      <c r="J26" s="33" t="n"/>
+      <c r="K26" s="34">
+        <f>IF(J26="","",(H26-J26)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>5Y</t>
+        </is>
+      </c>
+      <c r="B27" s="24">
+        <f>EDATE($B$4,60)</f>
+        <v/>
+      </c>
+      <c r="C27" s="35">
+        <f>(B27-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D27" s="17">
+        <f>(B27-B26)/360</f>
+        <v/>
+      </c>
+      <c r="E27" s="17">
+        <f>'SOFR_OIS_Quotes'!$G24</f>
+        <v/>
+      </c>
+      <c r="F27" s="17">
+        <f>F26+D26*G26</f>
+        <v/>
+      </c>
+      <c r="G27" s="36">
+        <f>(1-(E27/100)*F27)/(1+(E27/100)*D27)</f>
+        <v/>
+      </c>
+      <c r="H27" s="17">
+        <f>-LN(G27)/C27*100</f>
+        <v/>
+      </c>
+      <c r="I27" s="17">
+        <f>(G26/G27-1)/D27*100</f>
+        <v/>
+      </c>
+      <c r="J27" s="33" t="n"/>
+      <c r="K27" s="37">
+        <f>IF(J27="","",(H27-J27)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>6Y</t>
+        </is>
+      </c>
+      <c r="B28" s="18">
+        <f>EDATE($B$4,72)</f>
+        <v/>
+      </c>
+      <c r="C28" s="31">
+        <f>(B28-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D28" s="21">
+        <f>(B28-B27)/360</f>
+        <v/>
+      </c>
+      <c r="E28" s="21">
+        <f>'SOFR_OIS_Quotes'!$G25</f>
+        <v/>
+      </c>
+      <c r="F28" s="21">
+        <f>F27+D27*G27</f>
+        <v/>
+      </c>
+      <c r="G28" s="32">
+        <f>(1-(E28/100)*F28)/(1+(E28/100)*D28)</f>
+        <v/>
+      </c>
+      <c r="H28" s="21">
+        <f>-LN(G28)/C28*100</f>
+        <v/>
+      </c>
+      <c r="I28" s="21">
+        <f>(G27/G28-1)/D28*100</f>
+        <v/>
+      </c>
+      <c r="J28" s="33" t="n"/>
+      <c r="K28" s="34">
+        <f>IF(J28="","",(H28-J28)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>7Y</t>
+        </is>
+      </c>
+      <c r="B29" s="24">
+        <f>EDATE($B$4,84)</f>
+        <v/>
+      </c>
+      <c r="C29" s="35">
+        <f>(B29-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D29" s="17">
+        <f>(B29-B28)/360</f>
+        <v/>
+      </c>
+      <c r="E29" s="17">
+        <f>'SOFR_OIS_Quotes'!$G26</f>
+        <v/>
+      </c>
+      <c r="F29" s="17">
+        <f>F28+D28*G28</f>
+        <v/>
+      </c>
+      <c r="G29" s="36">
+        <f>(1-(E29/100)*F29)/(1+(E29/100)*D29)</f>
+        <v/>
+      </c>
+      <c r="H29" s="17">
+        <f>-LN(G29)/C29*100</f>
+        <v/>
+      </c>
+      <c r="I29" s="17">
+        <f>(G28/G29-1)/D29*100</f>
+        <v/>
+      </c>
+      <c r="J29" s="33" t="n"/>
+      <c r="K29" s="37">
+        <f>IF(J29="","",(H29-J29)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>8Y</t>
+        </is>
+      </c>
+      <c r="B30" s="18">
+        <f>EDATE($B$4,96)</f>
+        <v/>
+      </c>
+      <c r="C30" s="31">
+        <f>(B30-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D30" s="21">
+        <f>(B30-B29)/360</f>
+        <v/>
+      </c>
+      <c r="E30" s="21">
+        <f>'SOFR_OIS_Quotes'!$G27</f>
+        <v/>
+      </c>
+      <c r="F30" s="21">
+        <f>F29+D29*G29</f>
+        <v/>
+      </c>
+      <c r="G30" s="32">
+        <f>(1-(E30/100)*F30)/(1+(E30/100)*D30)</f>
+        <v/>
+      </c>
+      <c r="H30" s="21">
+        <f>-LN(G30)/C30*100</f>
+        <v/>
+      </c>
+      <c r="I30" s="21">
+        <f>(G29/G30-1)/D30*100</f>
+        <v/>
+      </c>
+      <c r="J30" s="33" t="n"/>
+      <c r="K30" s="34">
+        <f>IF(J30="","",(H30-J30)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="inlineStr">
+        <is>
+          <t>9Y</t>
+        </is>
+      </c>
+      <c r="B31" s="24">
+        <f>EDATE($B$4,108)</f>
+        <v/>
+      </c>
+      <c r="C31" s="35">
+        <f>(B31-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D31" s="17">
+        <f>(B31-B30)/360</f>
+        <v/>
+      </c>
+      <c r="E31" s="17">
+        <f>'SOFR_OIS_Quotes'!$G28</f>
+        <v/>
+      </c>
+      <c r="F31" s="17">
+        <f>F30+D30*G30</f>
+        <v/>
+      </c>
+      <c r="G31" s="36">
+        <f>(1-(E31/100)*F31)/(1+(E31/100)*D31)</f>
+        <v/>
+      </c>
+      <c r="H31" s="17">
+        <f>-LN(G31)/C31*100</f>
+        <v/>
+      </c>
+      <c r="I31" s="17">
+        <f>(G30/G31-1)/D31*100</f>
+        <v/>
+      </c>
+      <c r="J31" s="33" t="n"/>
+      <c r="K31" s="37">
+        <f>IF(J31="","",(H31-J31)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="B32" s="18">
+        <f>EDATE($B$4,120)</f>
+        <v/>
+      </c>
+      <c r="C32" s="31">
+        <f>(B32-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D32" s="21">
+        <f>(B32-B31)/360</f>
+        <v/>
+      </c>
+      <c r="E32" s="21">
+        <f>'SOFR_OIS_Quotes'!$G29</f>
+        <v/>
+      </c>
+      <c r="F32" s="21">
+        <f>F31+D31*G31</f>
+        <v/>
+      </c>
+      <c r="G32" s="32">
+        <f>(1-(E32/100)*F32)/(1+(E32/100)*D32)</f>
+        <v/>
+      </c>
+      <c r="H32" s="21">
+        <f>-LN(G32)/C32*100</f>
+        <v/>
+      </c>
+      <c r="I32" s="21">
+        <f>(G31/G32-1)/D32*100</f>
+        <v/>
+      </c>
+      <c r="J32" s="33" t="n"/>
+      <c r="K32" s="34">
+        <f>IF(J32="","",(H32-J32)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t>12Y</t>
+        </is>
+      </c>
+      <c r="B33" s="24">
+        <f>EDATE($B$4,144)</f>
+        <v/>
+      </c>
+      <c r="C33" s="35">
+        <f>(B33-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D33" s="17">
+        <f>(B33-B32)/360</f>
+        <v/>
+      </c>
+      <c r="E33" s="17">
+        <f>'SOFR_OIS_Quotes'!$G30</f>
+        <v/>
+      </c>
+      <c r="F33" s="17">
+        <f>F32+D32*G32</f>
+        <v/>
+      </c>
+      <c r="G33" s="36">
+        <f>(1-(E33/100)*F33)/(1+(E33/100)*D33)</f>
+        <v/>
+      </c>
+      <c r="H33" s="17">
+        <f>-LN(G33)/C33*100</f>
+        <v/>
+      </c>
+      <c r="I33" s="17">
+        <f>(G32/G33-1)/D33*100</f>
+        <v/>
+      </c>
+      <c r="J33" s="33" t="n"/>
+      <c r="K33" s="37">
+        <f>IF(J33="","",(H33-J33)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>15Y</t>
+        </is>
+      </c>
+      <c r="B34" s="18">
+        <f>EDATE($B$4,180)</f>
+        <v/>
+      </c>
+      <c r="C34" s="31">
+        <f>(B34-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D34" s="21">
+        <f>(B34-B33)/360</f>
+        <v/>
+      </c>
+      <c r="E34" s="21">
+        <f>'SOFR_OIS_Quotes'!$G31</f>
+        <v/>
+      </c>
+      <c r="F34" s="21">
+        <f>F33+D33*G33</f>
+        <v/>
+      </c>
+      <c r="G34" s="32">
+        <f>(1-(E34/100)*F34)/(1+(E34/100)*D34)</f>
+        <v/>
+      </c>
+      <c r="H34" s="21">
+        <f>-LN(G34)/C34*100</f>
+        <v/>
+      </c>
+      <c r="I34" s="21">
+        <f>(G33/G34-1)/D34*100</f>
+        <v/>
+      </c>
+      <c r="J34" s="33" t="n"/>
+      <c r="K34" s="34">
+        <f>IF(J34="","",(H34-J34)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="23" t="inlineStr">
+        <is>
+          <t>20Y</t>
+        </is>
+      </c>
+      <c r="B35" s="24">
+        <f>EDATE($B$4,240)</f>
+        <v/>
+      </c>
+      <c r="C35" s="35">
+        <f>(B35-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D35" s="17">
+        <f>(B35-B34)/360</f>
+        <v/>
+      </c>
+      <c r="E35" s="17">
+        <f>'SOFR_OIS_Quotes'!$G32</f>
+        <v/>
+      </c>
+      <c r="F35" s="17">
+        <f>F34+D34*G34</f>
+        <v/>
+      </c>
+      <c r="G35" s="36">
+        <f>(1-(E35/100)*F35)/(1+(E35/100)*D35)</f>
+        <v/>
+      </c>
+      <c r="H35" s="17">
+        <f>-LN(G35)/C35*100</f>
+        <v/>
+      </c>
+      <c r="I35" s="17">
+        <f>(G34/G35-1)/D35*100</f>
+        <v/>
+      </c>
+      <c r="J35" s="33" t="n"/>
+      <c r="K35" s="37">
+        <f>IF(J35="","",(H35-J35)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>25Y</t>
+        </is>
+      </c>
+      <c r="B36" s="18">
+        <f>EDATE($B$4,300)</f>
+        <v/>
+      </c>
+      <c r="C36" s="31">
+        <f>(B36-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D36" s="21">
+        <f>(B36-B35)/360</f>
+        <v/>
+      </c>
+      <c r="E36" s="21">
+        <f>'SOFR_OIS_Quotes'!$G33</f>
+        <v/>
+      </c>
+      <c r="F36" s="21">
+        <f>F35+D35*G35</f>
+        <v/>
+      </c>
+      <c r="G36" s="32">
+        <f>(1-(E36/100)*F36)/(1+(E36/100)*D36)</f>
+        <v/>
+      </c>
+      <c r="H36" s="21">
+        <f>-LN(G36)/C36*100</f>
+        <v/>
+      </c>
+      <c r="I36" s="21">
+        <f>(G35/G36-1)/D36*100</f>
+        <v/>
+      </c>
+      <c r="J36" s="33" t="n"/>
+      <c r="K36" s="34">
+        <f>IF(J36="","",(H36-J36)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="23" t="inlineStr">
+        <is>
+          <t>30Y</t>
+        </is>
+      </c>
+      <c r="B37" s="24">
+        <f>EDATE($B$4,360)</f>
+        <v/>
+      </c>
+      <c r="C37" s="35">
+        <f>(B37-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D37" s="17">
+        <f>(B37-B36)/360</f>
+        <v/>
+      </c>
+      <c r="E37" s="17">
+        <f>'SOFR_OIS_Quotes'!$G34</f>
+        <v/>
+      </c>
+      <c r="F37" s="17">
+        <f>F36+D36*G36</f>
+        <v/>
+      </c>
+      <c r="G37" s="36">
+        <f>(1-(E37/100)*F37)/(1+(E37/100)*D37)</f>
+        <v/>
+      </c>
+      <c r="H37" s="17">
+        <f>-LN(G37)/C37*100</f>
+        <v/>
+      </c>
+      <c r="I37" s="17">
+        <f>(G36/G37-1)/D37*100</f>
+        <v/>
+      </c>
+      <c r="J37" s="33" t="n"/>
+      <c r="K37" s="37">
+        <f>IF(J37="","",(H37-J37)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>40Y</t>
+        </is>
+      </c>
+      <c r="B38" s="18">
+        <f>EDATE($B$4,480)</f>
+        <v/>
+      </c>
+      <c r="C38" s="31">
+        <f>(B38-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D38" s="21">
+        <f>(B38-B37)/360</f>
+        <v/>
+      </c>
+      <c r="E38" s="21">
+        <f>'SOFR_OIS_Quotes'!$G35</f>
+        <v/>
+      </c>
+      <c r="F38" s="21">
+        <f>F37+D37*G37</f>
+        <v/>
+      </c>
+      <c r="G38" s="32">
+        <f>(1-(E38/100)*F38)/(1+(E38/100)*D38)</f>
+        <v/>
+      </c>
+      <c r="H38" s="21">
+        <f>-LN(G38)/C38*100</f>
+        <v/>
+      </c>
+      <c r="I38" s="21">
+        <f>(G37/G38-1)/D38*100</f>
+        <v/>
+      </c>
+      <c r="J38" s="33" t="n"/>
+      <c r="K38" s="34">
+        <f>IF(J38="","",(H38-J38)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="23" t="inlineStr">
+        <is>
+          <t>50Y</t>
+        </is>
+      </c>
+      <c r="B39" s="24">
+        <f>EDATE($B$4,600)</f>
+        <v/>
+      </c>
+      <c r="C39" s="35">
+        <f>(B39-$B$4)/365</f>
+        <v/>
+      </c>
+      <c r="D39" s="17">
+        <f>(B39-B38)/360</f>
+        <v/>
+      </c>
+      <c r="E39" s="17">
+        <f>'SOFR_OIS_Quotes'!$G36</f>
+        <v/>
+      </c>
+      <c r="F39" s="17">
+        <f>F38+D38*G38</f>
+        <v/>
+      </c>
+      <c r="G39" s="36">
+        <f>(1-(E39/100)*F39)/(1+(E39/100)*D39)</f>
+        <v/>
+      </c>
+      <c r="H39" s="17">
+        <f>-LN(G39)/C39*100</f>
+        <v/>
+      </c>
+      <c r="I39" s="17">
+        <f>(G38/G39-1)/D39*100</f>
+        <v/>
+      </c>
+      <c r="J39" s="33" t="n"/>
+      <c r="K39" s="37">
+        <f>IF(J39="","",(H39-J39)*100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="40" customHeight="1">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>Discount factor is the deliverable curve P(0,T). Zero rate is continuously-compounded (ACT/365): z = −ln(DF)/T. Forward is the simple rate over each pillar interval. Yellow column J is for pasting the Bloomberg S490 zero rates; Δ (bp) then shows your bootstrap vs Bloomberg — the validation the Lehman paper does against the dealer curve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A41:K42"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A5:K6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4231,417 +5789,393 @@
           <t>Curve date</t>
         </is>
       </c>
-      <c r="B5" s="31">
-        <f>IFERROR(BDP(S490_TKR,"CURVE_DT"),VAL_DATE)</f>
+      <c r="B5" s="38">
+        <f>VAL_DATE</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Primary pull: the anchor cell A8 holds =BDS(S490_TKR,"CURVE_TENOR_RATES"), which spills Tenor + par rate. Zero rate, discount factor and forward rate are best exported from the curve screen (type YCSW0490 &lt;GO&gt;, or SWDF), because they are not all returned by a single BDS field under every entitlement — paste them into columns E:G alongside the spilled tenors. Compare your bootstrap's P(0,T), zero and forward against these.</t>
+          <t>The anchor cell A8 holds =BDS(S490_TKR,"CURVE_TENOR_RATES") and spills raw below in Bloomberg's own column order (typically tenor, curve member, maturity, mid rate). It is NOT pre-labeled, because forcing headers/date-formats mis-aligned the columns. Bloomberg's zero rates / discount factors are best read from the curve screen (YCSW0490 &lt;GO&gt;, or SWDF). The actual bootstrap + comparison lives on the Bootstrap tab: paste S490 zero rates into its column J to get Δz in bp.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="inlineStr">
         <is>
-          <t>Tenor</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>Curve date</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>Maturity date</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>Market/par rate (%)</t>
-        </is>
-      </c>
-      <c r="E7" s="20" t="inlineStr">
-        <is>
-          <t>Zero rate (%)</t>
-        </is>
-      </c>
-      <c r="F7" s="20" t="inlineStr">
-        <is>
-          <t>Discount factor</t>
-        </is>
-      </c>
-      <c r="G7" s="20" t="inlineStr">
-        <is>
-          <t>Forward rate (%)</t>
-        </is>
-      </c>
+          <t>Raw CURVE_TENOR_RATES dump — Bloomberg-defined column order; verify on terminal, then paste S490 zero rates into the Bootstrap tab (column J) for the Δz check</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr"/>
+      <c r="C7" s="20" t="inlineStr"/>
+      <c r="D7" s="20" t="inlineStr"/>
+      <c r="E7" s="20" t="inlineStr"/>
+      <c r="F7" s="20" t="inlineStr"/>
+      <c r="G7" s="20" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="8">
         <f>BDS(S490_TKR,"CURVE_TENOR_RATES")</f>
         <v/>
       </c>
-      <c r="B8" s="18" t="n"/>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="21" t="n"/>
-      <c r="E8" s="21" t="n"/>
-      <c r="F8" s="32" t="n"/>
-      <c r="G8" s="21" t="n"/>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="23" t="n"/>
-      <c r="B9" s="24" t="n"/>
-      <c r="C9" s="24" t="n"/>
-      <c r="D9" s="17" t="n"/>
-      <c r="E9" s="17" t="n"/>
-      <c r="F9" s="33" t="n"/>
-      <c r="G9" s="17" t="n"/>
+      <c r="B9" s="23" t="n"/>
+      <c r="C9" s="23" t="n"/>
+      <c r="D9" s="23" t="n"/>
+      <c r="E9" s="23" t="n"/>
+      <c r="F9" s="23" t="n"/>
+      <c r="G9" s="23" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n"/>
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="21" t="n"/>
-      <c r="E10" s="21" t="n"/>
-      <c r="F10" s="32" t="n"/>
-      <c r="G10" s="21" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="23" t="n"/>
-      <c r="B11" s="24" t="n"/>
-      <c r="C11" s="24" t="n"/>
-      <c r="D11" s="17" t="n"/>
-      <c r="E11" s="17" t="n"/>
-      <c r="F11" s="33" t="n"/>
-      <c r="G11" s="17" t="n"/>
+      <c r="B11" s="23" t="n"/>
+      <c r="C11" s="23" t="n"/>
+      <c r="D11" s="23" t="n"/>
+      <c r="E11" s="23" t="n"/>
+      <c r="F11" s="23" t="n"/>
+      <c r="G11" s="23" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n"/>
-      <c r="B12" s="18" t="n"/>
-      <c r="C12" s="18" t="n"/>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="21" t="n"/>
-      <c r="F12" s="32" t="n"/>
-      <c r="G12" s="21" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="23" t="n"/>
-      <c r="B13" s="24" t="n"/>
-      <c r="C13" s="24" t="n"/>
-      <c r="D13" s="17" t="n"/>
-      <c r="E13" s="17" t="n"/>
-      <c r="F13" s="33" t="n"/>
-      <c r="G13" s="17" t="n"/>
+      <c r="B13" s="23" t="n"/>
+      <c r="C13" s="23" t="n"/>
+      <c r="D13" s="23" t="n"/>
+      <c r="E13" s="23" t="n"/>
+      <c r="F13" s="23" t="n"/>
+      <c r="G13" s="23" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n"/>
-      <c r="B14" s="18" t="n"/>
-      <c r="C14" s="18" t="n"/>
-      <c r="D14" s="21" t="n"/>
-      <c r="E14" s="21" t="n"/>
-      <c r="F14" s="32" t="n"/>
-      <c r="G14" s="21" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="23" t="n"/>
-      <c r="B15" s="24" t="n"/>
-      <c r="C15" s="24" t="n"/>
-      <c r="D15" s="17" t="n"/>
-      <c r="E15" s="17" t="n"/>
-      <c r="F15" s="33" t="n"/>
-      <c r="G15" s="17" t="n"/>
+      <c r="B15" s="23" t="n"/>
+      <c r="C15" s="23" t="n"/>
+      <c r="D15" s="23" t="n"/>
+      <c r="E15" s="23" t="n"/>
+      <c r="F15" s="23" t="n"/>
+      <c r="G15" s="23" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n"/>
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="21" t="n"/>
-      <c r="E16" s="21" t="n"/>
-      <c r="F16" s="32" t="n"/>
-      <c r="G16" s="21" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="23" t="n"/>
-      <c r="B17" s="24" t="n"/>
-      <c r="C17" s="24" t="n"/>
-      <c r="D17" s="17" t="n"/>
-      <c r="E17" s="17" t="n"/>
-      <c r="F17" s="33" t="n"/>
-      <c r="G17" s="17" t="n"/>
+      <c r="B17" s="23" t="n"/>
+      <c r="C17" s="23" t="n"/>
+      <c r="D17" s="23" t="n"/>
+      <c r="E17" s="23" t="n"/>
+      <c r="F17" s="23" t="n"/>
+      <c r="G17" s="23" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n"/>
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="21" t="n"/>
-      <c r="E18" s="21" t="n"/>
-      <c r="F18" s="32" t="n"/>
-      <c r="G18" s="21" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="8" t="n"/>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="23" t="n"/>
-      <c r="B19" s="24" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="17" t="n"/>
-      <c r="E19" s="17" t="n"/>
-      <c r="F19" s="33" t="n"/>
-      <c r="G19" s="17" t="n"/>
+      <c r="B19" s="23" t="n"/>
+      <c r="C19" s="23" t="n"/>
+      <c r="D19" s="23" t="n"/>
+      <c r="E19" s="23" t="n"/>
+      <c r="F19" s="23" t="n"/>
+      <c r="G19" s="23" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n"/>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="21" t="n"/>
-      <c r="E20" s="21" t="n"/>
-      <c r="F20" s="32" t="n"/>
-      <c r="G20" s="21" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="23" t="n"/>
-      <c r="B21" s="24" t="n"/>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="17" t="n"/>
-      <c r="E21" s="17" t="n"/>
-      <c r="F21" s="33" t="n"/>
-      <c r="G21" s="17" t="n"/>
+      <c r="B21" s="23" t="n"/>
+      <c r="C21" s="23" t="n"/>
+      <c r="D21" s="23" t="n"/>
+      <c r="E21" s="23" t="n"/>
+      <c r="F21" s="23" t="n"/>
+      <c r="G21" s="23" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n"/>
-      <c r="B22" s="18" t="n"/>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="21" t="n"/>
-      <c r="E22" s="21" t="n"/>
-      <c r="F22" s="32" t="n"/>
-      <c r="G22" s="21" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="23" t="n"/>
-      <c r="B23" s="24" t="n"/>
-      <c r="C23" s="24" t="n"/>
-      <c r="D23" s="17" t="n"/>
-      <c r="E23" s="17" t="n"/>
-      <c r="F23" s="33" t="n"/>
-      <c r="G23" s="17" t="n"/>
+      <c r="B23" s="23" t="n"/>
+      <c r="C23" s="23" t="n"/>
+      <c r="D23" s="23" t="n"/>
+      <c r="E23" s="23" t="n"/>
+      <c r="F23" s="23" t="n"/>
+      <c r="G23" s="23" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n"/>
-      <c r="B24" s="18" t="n"/>
-      <c r="C24" s="18" t="n"/>
-      <c r="D24" s="21" t="n"/>
-      <c r="E24" s="21" t="n"/>
-      <c r="F24" s="32" t="n"/>
-      <c r="G24" s="21" t="n"/>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="23" t="n"/>
-      <c r="B25" s="24" t="n"/>
-      <c r="C25" s="24" t="n"/>
-      <c r="D25" s="17" t="n"/>
-      <c r="E25" s="17" t="n"/>
-      <c r="F25" s="33" t="n"/>
-      <c r="G25" s="17" t="n"/>
+      <c r="B25" s="23" t="n"/>
+      <c r="C25" s="23" t="n"/>
+      <c r="D25" s="23" t="n"/>
+      <c r="E25" s="23" t="n"/>
+      <c r="F25" s="23" t="n"/>
+      <c r="G25" s="23" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n"/>
-      <c r="B26" s="18" t="n"/>
-      <c r="C26" s="18" t="n"/>
-      <c r="D26" s="21" t="n"/>
-      <c r="E26" s="21" t="n"/>
-      <c r="F26" s="32" t="n"/>
-      <c r="G26" s="21" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="8" t="n"/>
+      <c r="E26" s="8" t="n"/>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="23" t="n"/>
-      <c r="B27" s="24" t="n"/>
-      <c r="C27" s="24" t="n"/>
-      <c r="D27" s="17" t="n"/>
-      <c r="E27" s="17" t="n"/>
-      <c r="F27" s="33" t="n"/>
-      <c r="G27" s="17" t="n"/>
+      <c r="B27" s="23" t="n"/>
+      <c r="C27" s="23" t="n"/>
+      <c r="D27" s="23" t="n"/>
+      <c r="E27" s="23" t="n"/>
+      <c r="F27" s="23" t="n"/>
+      <c r="G27" s="23" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="n"/>
-      <c r="B28" s="18" t="n"/>
-      <c r="C28" s="18" t="n"/>
-      <c r="D28" s="21" t="n"/>
-      <c r="E28" s="21" t="n"/>
-      <c r="F28" s="32" t="n"/>
-      <c r="G28" s="21" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="8" t="n"/>
+      <c r="E28" s="8" t="n"/>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="8" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="23" t="n"/>
-      <c r="B29" s="24" t="n"/>
-      <c r="C29" s="24" t="n"/>
-      <c r="D29" s="17" t="n"/>
-      <c r="E29" s="17" t="n"/>
-      <c r="F29" s="33" t="n"/>
-      <c r="G29" s="17" t="n"/>
+      <c r="B29" s="23" t="n"/>
+      <c r="C29" s="23" t="n"/>
+      <c r="D29" s="23" t="n"/>
+      <c r="E29" s="23" t="n"/>
+      <c r="F29" s="23" t="n"/>
+      <c r="G29" s="23" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n"/>
-      <c r="B30" s="18" t="n"/>
-      <c r="C30" s="18" t="n"/>
-      <c r="D30" s="21" t="n"/>
-      <c r="E30" s="21" t="n"/>
-      <c r="F30" s="32" t="n"/>
-      <c r="G30" s="21" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="8" t="n"/>
+      <c r="G30" s="8" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="23" t="n"/>
-      <c r="B31" s="24" t="n"/>
-      <c r="C31" s="24" t="n"/>
-      <c r="D31" s="17" t="n"/>
-      <c r="E31" s="17" t="n"/>
-      <c r="F31" s="33" t="n"/>
-      <c r="G31" s="17" t="n"/>
+      <c r="B31" s="23" t="n"/>
+      <c r="C31" s="23" t="n"/>
+      <c r="D31" s="23" t="n"/>
+      <c r="E31" s="23" t="n"/>
+      <c r="F31" s="23" t="n"/>
+      <c r="G31" s="23" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n"/>
-      <c r="B32" s="18" t="n"/>
-      <c r="C32" s="18" t="n"/>
-      <c r="D32" s="21" t="n"/>
-      <c r="E32" s="21" t="n"/>
-      <c r="F32" s="32" t="n"/>
-      <c r="G32" s="21" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="8" t="n"/>
+      <c r="F32" s="8" t="n"/>
+      <c r="G32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="23" t="n"/>
-      <c r="B33" s="24" t="n"/>
-      <c r="C33" s="24" t="n"/>
-      <c r="D33" s="17" t="n"/>
-      <c r="E33" s="17" t="n"/>
-      <c r="F33" s="33" t="n"/>
-      <c r="G33" s="17" t="n"/>
+      <c r="B33" s="23" t="n"/>
+      <c r="C33" s="23" t="n"/>
+      <c r="D33" s="23" t="n"/>
+      <c r="E33" s="23" t="n"/>
+      <c r="F33" s="23" t="n"/>
+      <c r="G33" s="23" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n"/>
-      <c r="B34" s="18" t="n"/>
-      <c r="C34" s="18" t="n"/>
-      <c r="D34" s="21" t="n"/>
-      <c r="E34" s="21" t="n"/>
-      <c r="F34" s="32" t="n"/>
-      <c r="G34" s="21" t="n"/>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="8" t="n"/>
+      <c r="D34" s="8" t="n"/>
+      <c r="E34" s="8" t="n"/>
+      <c r="F34" s="8" t="n"/>
+      <c r="G34" s="8" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="23" t="n"/>
-      <c r="B35" s="24" t="n"/>
-      <c r="C35" s="24" t="n"/>
-      <c r="D35" s="17" t="n"/>
-      <c r="E35" s="17" t="n"/>
-      <c r="F35" s="33" t="n"/>
-      <c r="G35" s="17" t="n"/>
+      <c r="B35" s="23" t="n"/>
+      <c r="C35" s="23" t="n"/>
+      <c r="D35" s="23" t="n"/>
+      <c r="E35" s="23" t="n"/>
+      <c r="F35" s="23" t="n"/>
+      <c r="G35" s="23" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n"/>
-      <c r="B36" s="18" t="n"/>
-      <c r="C36" s="18" t="n"/>
-      <c r="D36" s="21" t="n"/>
-      <c r="E36" s="21" t="n"/>
-      <c r="F36" s="32" t="n"/>
-      <c r="G36" s="21" t="n"/>
+      <c r="B36" s="8" t="n"/>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="8" t="n"/>
+      <c r="E36" s="8" t="n"/>
+      <c r="F36" s="8" t="n"/>
+      <c r="G36" s="8" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="23" t="n"/>
-      <c r="B37" s="24" t="n"/>
-      <c r="C37" s="24" t="n"/>
-      <c r="D37" s="17" t="n"/>
-      <c r="E37" s="17" t="n"/>
-      <c r="F37" s="33" t="n"/>
-      <c r="G37" s="17" t="n"/>
+      <c r="B37" s="23" t="n"/>
+      <c r="C37" s="23" t="n"/>
+      <c r="D37" s="23" t="n"/>
+      <c r="E37" s="23" t="n"/>
+      <c r="F37" s="23" t="n"/>
+      <c r="G37" s="23" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n"/>
-      <c r="B38" s="18" t="n"/>
-      <c r="C38" s="18" t="n"/>
-      <c r="D38" s="21" t="n"/>
-      <c r="E38" s="21" t="n"/>
-      <c r="F38" s="32" t="n"/>
-      <c r="G38" s="21" t="n"/>
+      <c r="B38" s="8" t="n"/>
+      <c r="C38" s="8" t="n"/>
+      <c r="D38" s="8" t="n"/>
+      <c r="E38" s="8" t="n"/>
+      <c r="F38" s="8" t="n"/>
+      <c r="G38" s="8" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="23" t="n"/>
-      <c r="B39" s="24" t="n"/>
-      <c r="C39" s="24" t="n"/>
-      <c r="D39" s="17" t="n"/>
-      <c r="E39" s="17" t="n"/>
-      <c r="F39" s="33" t="n"/>
-      <c r="G39" s="17" t="n"/>
+      <c r="B39" s="23" t="n"/>
+      <c r="C39" s="23" t="n"/>
+      <c r="D39" s="23" t="n"/>
+      <c r="E39" s="23" t="n"/>
+      <c r="F39" s="23" t="n"/>
+      <c r="G39" s="23" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n"/>
-      <c r="B40" s="18" t="n"/>
-      <c r="C40" s="18" t="n"/>
-      <c r="D40" s="21" t="n"/>
-      <c r="E40" s="21" t="n"/>
-      <c r="F40" s="32" t="n"/>
-      <c r="G40" s="21" t="n"/>
+      <c r="B40" s="8" t="n"/>
+      <c r="C40" s="8" t="n"/>
+      <c r="D40" s="8" t="n"/>
+      <c r="E40" s="8" t="n"/>
+      <c r="F40" s="8" t="n"/>
+      <c r="G40" s="8" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="23" t="n"/>
-      <c r="B41" s="24" t="n"/>
-      <c r="C41" s="24" t="n"/>
-      <c r="D41" s="17" t="n"/>
-      <c r="E41" s="17" t="n"/>
-      <c r="F41" s="33" t="n"/>
-      <c r="G41" s="17" t="n"/>
+      <c r="B41" s="23" t="n"/>
+      <c r="C41" s="23" t="n"/>
+      <c r="D41" s="23" t="n"/>
+      <c r="E41" s="23" t="n"/>
+      <c r="F41" s="23" t="n"/>
+      <c r="G41" s="23" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n"/>
-      <c r="B42" s="18" t="n"/>
-      <c r="C42" s="18" t="n"/>
-      <c r="D42" s="21" t="n"/>
-      <c r="E42" s="21" t="n"/>
-      <c r="F42" s="32" t="n"/>
-      <c r="G42" s="21" t="n"/>
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="23" t="n"/>
-      <c r="B43" s="24" t="n"/>
-      <c r="C43" s="24" t="n"/>
-      <c r="D43" s="17" t="n"/>
-      <c r="E43" s="17" t="n"/>
-      <c r="F43" s="33" t="n"/>
-      <c r="G43" s="17" t="n"/>
+      <c r="B43" s="23" t="n"/>
+      <c r="C43" s="23" t="n"/>
+      <c r="D43" s="23" t="n"/>
+      <c r="E43" s="23" t="n"/>
+      <c r="F43" s="23" t="n"/>
+      <c r="G43" s="23" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n"/>
-      <c r="B44" s="18" t="n"/>
-      <c r="C44" s="18" t="n"/>
-      <c r="D44" s="21" t="n"/>
-      <c r="E44" s="21" t="n"/>
-      <c r="F44" s="32" t="n"/>
-      <c r="G44" s="21" t="n"/>
+      <c r="B44" s="8" t="n"/>
+      <c r="C44" s="8" t="n"/>
+      <c r="D44" s="8" t="n"/>
+      <c r="E44" s="8" t="n"/>
+      <c r="F44" s="8" t="n"/>
+      <c r="G44" s="8" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="23" t="n"/>
-      <c r="B45" s="24" t="n"/>
-      <c r="C45" s="24" t="n"/>
-      <c r="D45" s="17" t="n"/>
-      <c r="E45" s="17" t="n"/>
-      <c r="F45" s="33" t="n"/>
-      <c r="G45" s="17" t="n"/>
+      <c r="B45" s="23" t="n"/>
+      <c r="C45" s="23" t="n"/>
+      <c r="D45" s="23" t="n"/>
+      <c r="E45" s="23" t="n"/>
+      <c r="F45" s="23" t="n"/>
+      <c r="G45" s="23" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n"/>
-      <c r="B46" s="18" t="n"/>
-      <c r="C46" s="18" t="n"/>
-      <c r="D46" s="21" t="n"/>
-      <c r="E46" s="21" t="n"/>
-      <c r="F46" s="32" t="n"/>
-      <c r="G46" s="21" t="n"/>
+      <c r="B46" s="8" t="n"/>
+      <c r="C46" s="8" t="n"/>
+      <c r="D46" s="8" t="n"/>
+      <c r="E46" s="8" t="n"/>
+      <c r="F46" s="8" t="n"/>
+      <c r="G46" s="8" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="23" t="n"/>
-      <c r="B47" s="24" t="n"/>
-      <c r="C47" s="24" t="n"/>
-      <c r="D47" s="17" t="n"/>
-      <c r="E47" s="17" t="n"/>
-      <c r="F47" s="33" t="n"/>
-      <c r="G47" s="17" t="n"/>
+      <c r="B47" s="23" t="n"/>
+      <c r="C47" s="23" t="n"/>
+      <c r="D47" s="23" t="n"/>
+      <c r="E47" s="23" t="n"/>
+      <c r="F47" s="23" t="n"/>
+      <c r="G47" s="23" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -4655,7 +6189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4724,24 +6258,24 @@
           <t>Currency</t>
         </is>
       </c>
-      <c r="B5" s="34" t="inlineStr">
+      <c r="B5" s="39" t="inlineStr">
         <is>
           <t>CRNCY</t>
         </is>
       </c>
-      <c r="C5" s="35">
+      <c r="C5" s="40">
         <f>IFERROR(BDP("USOSFRC BGN Curncy","CRNCY"),"N/A — use FLDS")</f>
         <v/>
       </c>
-      <c r="D5" s="35">
+      <c r="D5" s="40">
         <f>IFERROR(BDP("USOSFR1 BGN Curncy","CRNCY"),"N/A — use FLDS")</f>
         <v/>
       </c>
-      <c r="E5" s="35">
+      <c r="E5" s="40">
         <f>IFERROR(BDP("USOSFR5 BGN Curncy","CRNCY"),"N/A — use FLDS")</f>
         <v/>
       </c>
-      <c r="F5" s="35">
+      <c r="F5" s="40">
         <f>IFERROR(BDP("USOSFR30 BGN Curncy","CRNCY"),"N/A — use FLDS")</f>
         <v/>
       </c>
@@ -4784,27 +6318,27 @@
           <t>Spot / settlement lag</t>
         </is>
       </c>
-      <c r="B7" s="34" t="inlineStr">
+      <c r="B7" s="39" t="inlineStr">
         <is>
           <t>— DES/SWPM manual —</t>
         </is>
       </c>
-      <c r="C7" s="35" t="inlineStr">
+      <c r="C7" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="D7" s="35" t="inlineStr">
+      <c r="D7" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="E7" s="35" t="inlineStr">
+      <c r="E7" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="F7" s="35" t="inlineStr">
+      <c r="F7" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
@@ -4848,27 +6382,27 @@
           <t>Maturity date rule</t>
         </is>
       </c>
-      <c r="B9" s="34" t="inlineStr">
+      <c r="B9" s="39" t="inlineStr">
         <is>
           <t>— DES/SWPM manual —</t>
         </is>
       </c>
-      <c r="C9" s="35" t="inlineStr">
+      <c r="C9" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="D9" s="35" t="inlineStr">
+      <c r="D9" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="E9" s="35" t="inlineStr">
+      <c r="E9" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="F9" s="35" t="inlineStr">
+      <c r="F9" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
@@ -4908,27 +6442,27 @@
           <t>Business-day convention</t>
         </is>
       </c>
-      <c r="B11" s="34" t="inlineStr">
+      <c r="B11" s="39" t="inlineStr">
         <is>
           <t>— DES/SWPM manual —</t>
         </is>
       </c>
-      <c r="C11" s="35" t="inlineStr">
+      <c r="C11" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="D11" s="35" t="inlineStr">
+      <c r="D11" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="E11" s="35" t="inlineStr">
+      <c r="E11" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="F11" s="35" t="inlineStr">
+      <c r="F11" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
@@ -4968,27 +6502,27 @@
           <t>Fixed-leg pay frequency</t>
         </is>
       </c>
-      <c r="B13" s="34" t="inlineStr">
+      <c r="B13" s="39" t="inlineStr">
         <is>
           <t>— DES/SWPM manual —</t>
         </is>
       </c>
-      <c r="C13" s="35" t="inlineStr">
+      <c r="C13" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="D13" s="35" t="inlineStr">
+      <c r="D13" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="E13" s="35" t="inlineStr">
+      <c r="E13" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="F13" s="35" t="inlineStr">
+      <c r="F13" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
@@ -5032,27 +6566,27 @@
           <t>Floating-leg pay frequency</t>
         </is>
       </c>
-      <c r="B15" s="34" t="inlineStr">
+      <c r="B15" s="39" t="inlineStr">
         <is>
           <t>— DES/SWPM manual —</t>
         </is>
       </c>
-      <c r="C15" s="35" t="inlineStr">
+      <c r="C15" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="D15" s="35" t="inlineStr">
+      <c r="D15" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="E15" s="35" t="inlineStr">
+      <c r="E15" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="F15" s="35" t="inlineStr">
+      <c r="F15" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
@@ -5096,27 +6630,27 @@
           <t>Payment lag</t>
         </is>
       </c>
-      <c r="B17" s="34" t="inlineStr">
+      <c r="B17" s="39" t="inlineStr">
         <is>
           <t>— DES/SWPM manual —</t>
         </is>
       </c>
-      <c r="C17" s="35" t="inlineStr">
+      <c r="C17" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="D17" s="35" t="inlineStr">
+      <c r="D17" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="E17" s="35" t="inlineStr">
+      <c r="E17" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="F17" s="35" t="inlineStr">
+      <c r="F17" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
@@ -5160,27 +6694,27 @@
           <t>End-of-month treatment</t>
         </is>
       </c>
-      <c r="B19" s="34" t="inlineStr">
+      <c r="B19" s="39" t="inlineStr">
         <is>
           <t>— DES/SWPM manual —</t>
         </is>
       </c>
-      <c r="C19" s="35" t="inlineStr">
+      <c r="C19" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="D19" s="35" t="inlineStr">
+      <c r="D19" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="E19" s="35" t="inlineStr">
+      <c r="E19" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
       </c>
-      <c r="F19" s="35" t="inlineStr">
+      <c r="F19" s="40" t="inlineStr">
         <is>
           <t>— DES/SWPM —</t>
         </is>
@@ -5199,15 +6733,15 @@
           <t>Reference index</t>
         </is>
       </c>
-      <c r="B22" s="36" t="inlineStr">
+      <c r="B22" s="41" t="inlineStr">
         <is>
           <t>USD-SOFR (compounded in arrears)</t>
         </is>
       </c>
-      <c r="C22" s="37" t="n"/>
-      <c r="D22" s="37" t="n"/>
-      <c r="E22" s="37" t="n"/>
-      <c r="F22" s="37" t="n"/>
+      <c r="C22" s="42" t="n"/>
+      <c r="D22" s="42" t="n"/>
+      <c r="E22" s="42" t="n"/>
+      <c r="F22" s="42" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -5215,15 +6749,15 @@
           <t>Spot / settlement lag</t>
         </is>
       </c>
-      <c r="B23" s="36" t="inlineStr">
+      <c r="B23" s="41" t="inlineStr">
         <is>
           <t>T+2 US business days</t>
         </is>
       </c>
-      <c r="C23" s="37" t="n"/>
-      <c r="D23" s="37" t="n"/>
-      <c r="E23" s="37" t="n"/>
-      <c r="F23" s="37" t="n"/>
+      <c r="C23" s="42" t="n"/>
+      <c r="D23" s="42" t="n"/>
+      <c r="E23" s="42" t="n"/>
+      <c r="F23" s="42" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -5231,15 +6765,15 @@
           <t>Effective date rule</t>
         </is>
       </c>
-      <c r="B24" s="36" t="inlineStr">
+      <c r="B24" s="41" t="inlineStr">
         <is>
           <t>Spot (T+2), modified following</t>
         </is>
       </c>
-      <c r="C24" s="37" t="n"/>
-      <c r="D24" s="37" t="n"/>
-      <c r="E24" s="37" t="n"/>
-      <c r="F24" s="37" t="n"/>
+      <c r="C24" s="42" t="n"/>
+      <c r="D24" s="42" t="n"/>
+      <c r="E24" s="42" t="n"/>
+      <c r="F24" s="42" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -5247,15 +6781,15 @@
           <t>Maturity date rule</t>
         </is>
       </c>
-      <c r="B25" s="36" t="inlineStr">
+      <c r="B25" s="41" t="inlineStr">
         <is>
           <t>Effective + tenor, modified following</t>
         </is>
       </c>
-      <c r="C25" s="37" t="n"/>
-      <c r="D25" s="37" t="n"/>
-      <c r="E25" s="37" t="n"/>
-      <c r="F25" s="37" t="n"/>
+      <c r="C25" s="42" t="n"/>
+      <c r="D25" s="42" t="n"/>
+      <c r="E25" s="42" t="n"/>
+      <c r="F25" s="42" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -5263,15 +6797,15 @@
           <t>Business-day convention</t>
         </is>
       </c>
-      <c r="B26" s="36" t="inlineStr">
+      <c r="B26" s="41" t="inlineStr">
         <is>
           <t>Modified Following</t>
         </is>
       </c>
-      <c r="C26" s="37" t="n"/>
-      <c r="D26" s="37" t="n"/>
-      <c r="E26" s="37" t="n"/>
-      <c r="F26" s="37" t="n"/>
+      <c r="C26" s="42" t="n"/>
+      <c r="D26" s="42" t="n"/>
+      <c r="E26" s="42" t="n"/>
+      <c r="F26" s="42" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -5279,15 +6813,15 @@
           <t>Fixed-leg day count</t>
         </is>
       </c>
-      <c r="B27" s="36" t="inlineStr">
+      <c r="B27" s="41" t="inlineStr">
         <is>
           <t>ACT/360</t>
         </is>
       </c>
-      <c r="C27" s="37" t="n"/>
-      <c r="D27" s="37" t="n"/>
-      <c r="E27" s="37" t="n"/>
-      <c r="F27" s="37" t="n"/>
+      <c r="C27" s="42" t="n"/>
+      <c r="D27" s="42" t="n"/>
+      <c r="E27" s="42" t="n"/>
+      <c r="F27" s="42" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -5295,15 +6829,15 @@
           <t>Fixed-leg pay frequency</t>
         </is>
       </c>
-      <c r="B28" s="36" t="inlineStr">
+      <c r="B28" s="41" t="inlineStr">
         <is>
           <t>Annual  (single payment if tenor ≤ 1Y)</t>
         </is>
       </c>
-      <c r="C28" s="37" t="n"/>
-      <c r="D28" s="37" t="n"/>
-      <c r="E28" s="37" t="n"/>
-      <c r="F28" s="37" t="n"/>
+      <c r="C28" s="42" t="n"/>
+      <c r="D28" s="42" t="n"/>
+      <c r="E28" s="42" t="n"/>
+      <c r="F28" s="42" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -5311,15 +6845,15 @@
           <t>Floating-leg day count</t>
         </is>
       </c>
-      <c r="B29" s="36" t="inlineStr">
+      <c r="B29" s="41" t="inlineStr">
         <is>
           <t>ACT/360</t>
         </is>
       </c>
-      <c r="C29" s="37" t="n"/>
-      <c r="D29" s="37" t="n"/>
-      <c r="E29" s="37" t="n"/>
-      <c r="F29" s="37" t="n"/>
+      <c r="C29" s="42" t="n"/>
+      <c r="D29" s="42" t="n"/>
+      <c r="E29" s="42" t="n"/>
+      <c r="F29" s="42" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -5327,15 +6861,15 @@
           <t>Floating-leg pay frequency</t>
         </is>
       </c>
-      <c r="B30" s="36" t="inlineStr">
+      <c r="B30" s="41" t="inlineStr">
         <is>
           <t>Annual  (single payment if tenor ≤ 1Y)</t>
         </is>
       </c>
-      <c r="C30" s="37" t="n"/>
-      <c r="D30" s="37" t="n"/>
-      <c r="E30" s="37" t="n"/>
-      <c r="F30" s="37" t="n"/>
+      <c r="C30" s="42" t="n"/>
+      <c r="D30" s="42" t="n"/>
+      <c r="E30" s="42" t="n"/>
+      <c r="F30" s="42" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
@@ -5343,15 +6877,15 @@
           <t>SOFR compounding method</t>
         </is>
       </c>
-      <c r="B31" s="36" t="inlineStr">
+      <c r="B31" s="41" t="inlineStr">
         <is>
           <t>Daily compounded, ACT/360</t>
         </is>
       </c>
-      <c r="C31" s="37" t="n"/>
-      <c r="D31" s="37" t="n"/>
-      <c r="E31" s="37" t="n"/>
-      <c r="F31" s="37" t="n"/>
+      <c r="C31" s="42" t="n"/>
+      <c r="D31" s="42" t="n"/>
+      <c r="E31" s="42" t="n"/>
+      <c r="F31" s="42" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
@@ -5359,15 +6893,15 @@
           <t>Payment lag</t>
         </is>
       </c>
-      <c r="B32" s="36" t="inlineStr">
+      <c r="B32" s="41" t="inlineStr">
         <is>
           <t>2 US business days</t>
         </is>
       </c>
-      <c r="C32" s="37" t="n"/>
-      <c r="D32" s="37" t="n"/>
-      <c r="E32" s="37" t="n"/>
-      <c r="F32" s="37" t="n"/>
+      <c r="C32" s="42" t="n"/>
+      <c r="D32" s="42" t="n"/>
+      <c r="E32" s="42" t="n"/>
+      <c r="F32" s="42" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
@@ -5375,15 +6909,15 @@
           <t>Observation shift / lookback</t>
         </is>
       </c>
-      <c r="B33" s="36" t="inlineStr">
+      <c r="B33" s="41" t="inlineStr">
         <is>
           <t>None (payment-delay convention, 2 bd)</t>
         </is>
       </c>
-      <c r="C33" s="37" t="n"/>
-      <c r="D33" s="37" t="n"/>
-      <c r="E33" s="37" t="n"/>
-      <c r="F33" s="37" t="n"/>
+      <c r="C33" s="42" t="n"/>
+      <c r="D33" s="42" t="n"/>
+      <c r="E33" s="42" t="n"/>
+      <c r="F33" s="42" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
@@ -5391,15 +6925,15 @@
           <t>End-of-month treatment</t>
         </is>
       </c>
-      <c r="B34" s="36" t="inlineStr">
+      <c r="B34" s="41" t="inlineStr">
         <is>
           <t>EOM applies</t>
         </is>
       </c>
-      <c r="C34" s="37" t="n"/>
-      <c r="D34" s="37" t="n"/>
-      <c r="E34" s="37" t="n"/>
-      <c r="F34" s="37" t="n"/>
+      <c r="C34" s="42" t="n"/>
+      <c r="D34" s="42" t="n"/>
+      <c r="E34" s="42" t="n"/>
+      <c r="F34" s="42" t="n"/>
     </row>
     <row r="36" ht="44" customHeight="1">
       <c r="A36" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Fix Excel 'problem with content' — remove orphaned cell comments
The workbook shipped comment1-3.xml + VML drawings, but the worksheets had no
<legacyDrawing> element and the sheet .rels were empty — nothing linked the
comment parts to the sheets (an openpyxl linkage quirk, aggravated by creating
sheets at explicit indexes after comments were added). Excel flagged the
inconsistent package and offered to repair.

Removed all cell comments (they duplicated the visible on-sheet notes, so no
info lost). Verified: no comment/vml parts remain, Content_Types no longer
declares them, all sheet XML well-formed, workbook round-trips, formulas intact.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -405,56 +405,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>template</author>
-  </authors>
-  <commentList>
-    <comment ref="A12" authorId="0" shapeId="0">
-      <text>
-        <t>Array (spilling) formula. In Excel with Bloomberg it fills Date + PX_LAST down this block. If your Excel is pre-dynamic-array, it may need Ctrl+Shift+Enter across A:B.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>template</author>
-  </authors>
-  <commentList>
-    <comment ref="A7" authorId="0" shapeId="0">
-      <text>
-        <t>Spilling chain. Fills contract tickers down this column in Excel+Bloomberg.</t>
-      </text>
-    </comment>
-    <comment ref="A32" authorId="0" shapeId="0">
-      <text>
-        <t>Spilling chain. Fills contract tickers down this column in Excel+Bloomberg.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>template</author>
-  </authors>
-  <commentList>
-    <comment ref="A8" authorId="0" shapeId="0">
-      <text>
-        <t>Spilling: Tenor in col A, par/market rate in col B (or D depending on Bloomberg's return order — verify and align). Fill zero/DF/forward from the curve screen.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1425,7 +1375,6 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -3042,7 +2991,6 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -8883,7 +8831,6 @@
     <mergeCell ref="B4:D4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fix Excel 'Removed Records: Formula' — notes starting with '='
Two Swap_Pricer note strings began with '=' ('= Effective + Tenor.' and
'= Fixed - Float ...'). openpyxl stores any string starting with '=' as a
FORMULA, so Excel tried to parse the prose as a formula, failed, and stripped
it (the sheet6.xml 'Removed Records: Formula' repair). Rewrote both as plain
text. Validated the whole workbook through the 'formulas' Excel-formula
compiler — all formulas now compile with zero errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -6144,9 +6144,10 @@
         <f>EDATE(B8,12*B9)</f>
         <v/>
       </c>
-      <c r="C10" s="32">
-        <f> Effective + Tenor.</f>
-        <v/>
+      <c r="C10" s="32" t="inlineStr">
+        <is>
+          <t>Effective + Tenor.</t>
+        </is>
       </c>
       <c r="K10" s="17">
         <f>Bootstrap!B11</f>
@@ -6520,9 +6521,10 @@
         <f>B26+B27</f>
         <v/>
       </c>
-      <c r="C28" s="32">
-        <f> Fixed − Float (notionals cancel). ≈ 0 at par coupon.</f>
-        <v/>
+      <c r="C28" s="32" t="inlineStr">
+        <is>
+          <t>Fixed − Float (notionals cancel); ≈ 0 at par coupon.</t>
+        </is>
       </c>
       <c r="K28" s="17">
         <f>Bootstrap!B29</f>

</xml_diff>

<commit_message>
Rebuild Bootstrap as three segments (short OIS / SR3 futures / OIS swaps)
Per the Zhou 2002 structure with cutovers at 1Y and 5Y (no overlap):
- SHORT o/n-1Y: single-payment SOFR OIS.
- MIDDLE 1Y-5Y: 18M/2Y/3Y/4Y/5Y DFs now come from an SR3 futures chain (new
  helper block, cols O-W) that discounts each contract's forward from the OIS
  1Y DF, counting only the portion beyond 1Y (tau_eff) so pre-1Y contracts pass
  through and there's no overlap. Convexity column (bp, default 0) included.
- LONG 5Y-50Y: annual SOFR OIS swaps built off the futures-derived 5Y point.

Swap_Pricer curve reference unchanged (same pillar table). Validated: futures
mid DFs monotonic and within a few bp of pure-OIS; whole workbook compiles
through the formulas engine with zero errors; no orphaned parts.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -130,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -182,17 +182,18 @@
     <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -4228,7 +4229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M42"/>
+  <dimension ref="A1:Z42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4244,6 +4245,17 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4256,7 +4268,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Single-curve OIS bootstrap from the SOFR_OIS_Quotes mid strip → discount factors, zero &amp; forward rates</t>
+          <t>Three-segment USD curve (Zhou 2002): short OIS (≤1Y) · SR3 futures (1Y–5Y) · OIS swaps (5Y–50Y)</t>
         </is>
       </c>
     </row>
@@ -4274,11 +4286,22 @@
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Proper single-curve OIS bootstrap that respects the payment convention: OIS ≤ 1Y pay a SINGLE coupon at maturity → DF = 1/(1 + S·τ0); OIS ≥ 18M pay ANNUAL coupons → DF = (1 − S·A_prior)/(1 + S·τcoupon), where A_prior = Σ τ·DF over prior annual coupon dates (column I accumulates these; sub-annual and 18M rows add 0 so only annual pillars enter the annuity). Exact through 10Y; the sparse long end (12–50Y) uses the pillar grid as the coupon schedule. Every input reprices to par to ~0 bp. Par rates pull live from SOFR_OIS_Quotes; paste S490 zeros into column L for the Δz check.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6"/>
+          <t>SHORT (o/n–1Y): single-payment SOFR OIS, DF = 1/(1+S·τ0).  MIDDLE (1Y–5Y): the DF at 18M/2Y/3Y/4Y/5Y is interpolated off the SR3 futures chain (helper block cols O–W), which discounts each contract's forward rate forward from the OIS 1Y DF — so 18M/2Y…5Y here are driven by FUTURES, not the OIS pars (col E is shown only for reference).  LONG (5Y–50Y): annual SOFR OIS swaps, DF = (1−S·A_prior)/(1+S·τcoupon), with the annuity (col I) built from the short + futures DFs. Cutovers at 1Y and 5Y mean nothing overlaps. Paste S490 zeros into column L for the Δz check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>MIDDLE SEGMENT — SR3 futures chain (1Y→5Y)</t>
+        </is>
+      </c>
+      <c r="Y6" s="4" t="inlineStr">
+        <is>
+          <t>Mid interp grid</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
@@ -4343,6 +4366,61 @@
       <c r="M7" s="19" t="inlineStr">
         <is>
           <t>Δ vs S490 (bp)</t>
+        </is>
+      </c>
+      <c r="O7" s="19" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+      <c r="P7" s="19" t="inlineStr">
+        <is>
+          <t>Fut start</t>
+        </is>
+      </c>
+      <c r="Q7" s="19" t="inlineStr">
+        <is>
+          <t>Fut end</t>
+        </is>
+      </c>
+      <c r="R7" s="19" t="inlineStr">
+        <is>
+          <t>τ eff (post-1Y)</t>
+        </is>
+      </c>
+      <c r="S7" s="19" t="inlineStr">
+        <is>
+          <t>Implied %</t>
+        </is>
+      </c>
+      <c r="T7" s="19" t="inlineStr">
+        <is>
+          <t>Convexity bp</t>
+        </is>
+      </c>
+      <c r="U7" s="19" t="inlineStr">
+        <is>
+          <t>Fwd</t>
+        </is>
+      </c>
+      <c r="V7" s="19" t="inlineStr">
+        <is>
+          <t>DF before</t>
+        </is>
+      </c>
+      <c r="W7" s="19" t="inlineStr">
+        <is>
+          <t>DF after</t>
+        </is>
+      </c>
+      <c r="Y7" s="19" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="Z7" s="19" t="inlineStr">
+        <is>
+          <t>DF</t>
         </is>
       </c>
     </row>
@@ -4392,6 +4470,49 @@
         <f>IF(L8="","",(J8-L8)*100)</f>
         <v/>
       </c>
+      <c r="O8" s="6">
+        <f>'SOFR_Futures'!A7</f>
+        <v/>
+      </c>
+      <c r="P8" s="17">
+        <f>'SOFR_Futures'!H7</f>
+        <v/>
+      </c>
+      <c r="Q8" s="17">
+        <f>'SOFR_Futures'!H8</f>
+        <v/>
+      </c>
+      <c r="R8" s="16">
+        <f>MAX(0,(Q8-MAX(P8,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S8" s="16">
+        <f>'SOFR_Futures'!F7</f>
+        <v/>
+      </c>
+      <c r="T8" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="32">
+        <f>(S8-T8/100)/100</f>
+        <v/>
+      </c>
+      <c r="V8" s="33">
+        <f>$H$22</f>
+        <v/>
+      </c>
+      <c r="W8" s="33">
+        <f>V8/(1+U8*R8)</f>
+        <v/>
+      </c>
+      <c r="Y8" s="17">
+        <f>$B$22</f>
+        <v/>
+      </c>
+      <c r="Z8" s="33">
+        <f>$H$22</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -4440,6 +4561,49 @@
         <f>IF(L9="","",(J9-L9)*100)</f>
         <v/>
       </c>
+      <c r="O9" s="6">
+        <f>'SOFR_Futures'!A8</f>
+        <v/>
+      </c>
+      <c r="P9" s="17">
+        <f>'SOFR_Futures'!H8</f>
+        <v/>
+      </c>
+      <c r="Q9" s="17">
+        <f>'SOFR_Futures'!H9</f>
+        <v/>
+      </c>
+      <c r="R9" s="16">
+        <f>MAX(0,(Q9-MAX(P9,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S9" s="16">
+        <f>'SOFR_Futures'!F8</f>
+        <v/>
+      </c>
+      <c r="T9" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="32">
+        <f>(S9-T9/100)/100</f>
+        <v/>
+      </c>
+      <c r="V9" s="33">
+        <f>W8</f>
+        <v/>
+      </c>
+      <c r="W9" s="33">
+        <f>V9/(1+U9*R9)</f>
+        <v/>
+      </c>
+      <c r="Y9" s="17">
+        <f>MAX(Q8,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z9" s="33">
+        <f>W8</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -4488,6 +4652,49 @@
         <f>IF(L10="","",(J10-L10)*100)</f>
         <v/>
       </c>
+      <c r="O10" s="6">
+        <f>'SOFR_Futures'!A9</f>
+        <v/>
+      </c>
+      <c r="P10" s="17">
+        <f>'SOFR_Futures'!H9</f>
+        <v/>
+      </c>
+      <c r="Q10" s="17">
+        <f>'SOFR_Futures'!H10</f>
+        <v/>
+      </c>
+      <c r="R10" s="16">
+        <f>MAX(0,(Q10-MAX(P10,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S10" s="16">
+        <f>'SOFR_Futures'!F9</f>
+        <v/>
+      </c>
+      <c r="T10" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="32">
+        <f>(S10-T10/100)/100</f>
+        <v/>
+      </c>
+      <c r="V10" s="33">
+        <f>W9</f>
+        <v/>
+      </c>
+      <c r="W10" s="33">
+        <f>V10/(1+U10*R10)</f>
+        <v/>
+      </c>
+      <c r="Y10" s="17">
+        <f>MAX(Q9,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z10" s="33">
+        <f>W9</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -4536,6 +4743,49 @@
         <f>IF(L11="","",(J11-L11)*100)</f>
         <v/>
       </c>
+      <c r="O11" s="6">
+        <f>'SOFR_Futures'!A10</f>
+        <v/>
+      </c>
+      <c r="P11" s="17">
+        <f>'SOFR_Futures'!H10</f>
+        <v/>
+      </c>
+      <c r="Q11" s="17">
+        <f>'SOFR_Futures'!H11</f>
+        <v/>
+      </c>
+      <c r="R11" s="16">
+        <f>MAX(0,(Q11-MAX(P11,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S11" s="16">
+        <f>'SOFR_Futures'!F10</f>
+        <v/>
+      </c>
+      <c r="T11" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="32">
+        <f>(S11-T11/100)/100</f>
+        <v/>
+      </c>
+      <c r="V11" s="33">
+        <f>W10</f>
+        <v/>
+      </c>
+      <c r="W11" s="33">
+        <f>V11/(1+U11*R11)</f>
+        <v/>
+      </c>
+      <c r="Y11" s="17">
+        <f>MAX(Q10,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z11" s="33">
+        <f>W10</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -4584,6 +4834,49 @@
         <f>IF(L12="","",(J12-L12)*100)</f>
         <v/>
       </c>
+      <c r="O12" s="6">
+        <f>'SOFR_Futures'!A11</f>
+        <v/>
+      </c>
+      <c r="P12" s="17">
+        <f>'SOFR_Futures'!H11</f>
+        <v/>
+      </c>
+      <c r="Q12" s="17">
+        <f>'SOFR_Futures'!H12</f>
+        <v/>
+      </c>
+      <c r="R12" s="16">
+        <f>MAX(0,(Q12-MAX(P12,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S12" s="16">
+        <f>'SOFR_Futures'!F11</f>
+        <v/>
+      </c>
+      <c r="T12" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="32">
+        <f>(S12-T12/100)/100</f>
+        <v/>
+      </c>
+      <c r="V12" s="33">
+        <f>W11</f>
+        <v/>
+      </c>
+      <c r="W12" s="33">
+        <f>V12/(1+U12*R12)</f>
+        <v/>
+      </c>
+      <c r="Y12" s="17">
+        <f>MAX(Q11,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z12" s="33">
+        <f>W11</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -4632,6 +4925,49 @@
         <f>IF(L13="","",(J13-L13)*100)</f>
         <v/>
       </c>
+      <c r="O13" s="6">
+        <f>'SOFR_Futures'!A12</f>
+        <v/>
+      </c>
+      <c r="P13" s="17">
+        <f>'SOFR_Futures'!H12</f>
+        <v/>
+      </c>
+      <c r="Q13" s="17">
+        <f>'SOFR_Futures'!H13</f>
+        <v/>
+      </c>
+      <c r="R13" s="16">
+        <f>MAX(0,(Q13-MAX(P13,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S13" s="16">
+        <f>'SOFR_Futures'!F12</f>
+        <v/>
+      </c>
+      <c r="T13" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="32">
+        <f>(S13-T13/100)/100</f>
+        <v/>
+      </c>
+      <c r="V13" s="33">
+        <f>W12</f>
+        <v/>
+      </c>
+      <c r="W13" s="33">
+        <f>V13/(1+U13*R13)</f>
+        <v/>
+      </c>
+      <c r="Y13" s="17">
+        <f>MAX(Q12,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z13" s="33">
+        <f>W12</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -4680,6 +5016,49 @@
         <f>IF(L14="","",(J14-L14)*100)</f>
         <v/>
       </c>
+      <c r="O14" s="6">
+        <f>'SOFR_Futures'!A13</f>
+        <v/>
+      </c>
+      <c r="P14" s="17">
+        <f>'SOFR_Futures'!H13</f>
+        <v/>
+      </c>
+      <c r="Q14" s="17">
+        <f>'SOFR_Futures'!H14</f>
+        <v/>
+      </c>
+      <c r="R14" s="16">
+        <f>MAX(0,(Q14-MAX(P14,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S14" s="16">
+        <f>'SOFR_Futures'!F13</f>
+        <v/>
+      </c>
+      <c r="T14" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="32">
+        <f>(S14-T14/100)/100</f>
+        <v/>
+      </c>
+      <c r="V14" s="33">
+        <f>W13</f>
+        <v/>
+      </c>
+      <c r="W14" s="33">
+        <f>V14/(1+U14*R14)</f>
+        <v/>
+      </c>
+      <c r="Y14" s="17">
+        <f>MAX(Q13,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z14" s="33">
+        <f>W13</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -4728,6 +5107,49 @@
         <f>IF(L15="","",(J15-L15)*100)</f>
         <v/>
       </c>
+      <c r="O15" s="6">
+        <f>'SOFR_Futures'!A14</f>
+        <v/>
+      </c>
+      <c r="P15" s="17">
+        <f>'SOFR_Futures'!H14</f>
+        <v/>
+      </c>
+      <c r="Q15" s="17">
+        <f>'SOFR_Futures'!H15</f>
+        <v/>
+      </c>
+      <c r="R15" s="16">
+        <f>MAX(0,(Q15-MAX(P15,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S15" s="16">
+        <f>'SOFR_Futures'!F14</f>
+        <v/>
+      </c>
+      <c r="T15" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="32">
+        <f>(S15-T15/100)/100</f>
+        <v/>
+      </c>
+      <c r="V15" s="33">
+        <f>W14</f>
+        <v/>
+      </c>
+      <c r="W15" s="33">
+        <f>V15/(1+U15*R15)</f>
+        <v/>
+      </c>
+      <c r="Y15" s="17">
+        <f>MAX(Q14,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z15" s="33">
+        <f>W14</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -4776,6 +5198,49 @@
         <f>IF(L16="","",(J16-L16)*100)</f>
         <v/>
       </c>
+      <c r="O16" s="6">
+        <f>'SOFR_Futures'!A15</f>
+        <v/>
+      </c>
+      <c r="P16" s="17">
+        <f>'SOFR_Futures'!H15</f>
+        <v/>
+      </c>
+      <c r="Q16" s="17">
+        <f>'SOFR_Futures'!H16</f>
+        <v/>
+      </c>
+      <c r="R16" s="16">
+        <f>MAX(0,(Q16-MAX(P16,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S16" s="16">
+        <f>'SOFR_Futures'!F15</f>
+        <v/>
+      </c>
+      <c r="T16" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="32">
+        <f>(S16-T16/100)/100</f>
+        <v/>
+      </c>
+      <c r="V16" s="33">
+        <f>W15</f>
+        <v/>
+      </c>
+      <c r="W16" s="33">
+        <f>V16/(1+U16*R16)</f>
+        <v/>
+      </c>
+      <c r="Y16" s="17">
+        <f>MAX(Q15,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z16" s="33">
+        <f>W15</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -4824,6 +5289,49 @@
         <f>IF(L17="","",(J17-L17)*100)</f>
         <v/>
       </c>
+      <c r="O17" s="6">
+        <f>'SOFR_Futures'!A16</f>
+        <v/>
+      </c>
+      <c r="P17" s="17">
+        <f>'SOFR_Futures'!H16</f>
+        <v/>
+      </c>
+      <c r="Q17" s="17">
+        <f>'SOFR_Futures'!H17</f>
+        <v/>
+      </c>
+      <c r="R17" s="16">
+        <f>MAX(0,(Q17-MAX(P17,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S17" s="16">
+        <f>'SOFR_Futures'!F16</f>
+        <v/>
+      </c>
+      <c r="T17" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" s="32">
+        <f>(S17-T17/100)/100</f>
+        <v/>
+      </c>
+      <c r="V17" s="33">
+        <f>W16</f>
+        <v/>
+      </c>
+      <c r="W17" s="33">
+        <f>V17/(1+U17*R17)</f>
+        <v/>
+      </c>
+      <c r="Y17" s="17">
+        <f>MAX(Q16,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z17" s="33">
+        <f>W16</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -4872,6 +5380,49 @@
         <f>IF(L18="","",(J18-L18)*100)</f>
         <v/>
       </c>
+      <c r="O18" s="6">
+        <f>'SOFR_Futures'!A17</f>
+        <v/>
+      </c>
+      <c r="P18" s="17">
+        <f>'SOFR_Futures'!H17</f>
+        <v/>
+      </c>
+      <c r="Q18" s="17">
+        <f>'SOFR_Futures'!H18</f>
+        <v/>
+      </c>
+      <c r="R18" s="16">
+        <f>MAX(0,(Q18-MAX(P18,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S18" s="16">
+        <f>'SOFR_Futures'!F17</f>
+        <v/>
+      </c>
+      <c r="T18" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" s="32">
+        <f>(S18-T18/100)/100</f>
+        <v/>
+      </c>
+      <c r="V18" s="33">
+        <f>W17</f>
+        <v/>
+      </c>
+      <c r="W18" s="33">
+        <f>V18/(1+U18*R18)</f>
+        <v/>
+      </c>
+      <c r="Y18" s="17">
+        <f>MAX(Q17,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z18" s="33">
+        <f>W17</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -4920,6 +5471,49 @@
         <f>IF(L19="","",(J19-L19)*100)</f>
         <v/>
       </c>
+      <c r="O19" s="6">
+        <f>'SOFR_Futures'!A18</f>
+        <v/>
+      </c>
+      <c r="P19" s="17">
+        <f>'SOFR_Futures'!H18</f>
+        <v/>
+      </c>
+      <c r="Q19" s="17">
+        <f>'SOFR_Futures'!H19</f>
+        <v/>
+      </c>
+      <c r="R19" s="16">
+        <f>MAX(0,(Q19-MAX(P19,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S19" s="16">
+        <f>'SOFR_Futures'!F18</f>
+        <v/>
+      </c>
+      <c r="T19" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="32">
+        <f>(S19-T19/100)/100</f>
+        <v/>
+      </c>
+      <c r="V19" s="33">
+        <f>W18</f>
+        <v/>
+      </c>
+      <c r="W19" s="33">
+        <f>V19/(1+U19*R19)</f>
+        <v/>
+      </c>
+      <c r="Y19" s="17">
+        <f>MAX(Q18,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z19" s="33">
+        <f>W18</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -4968,6 +5562,49 @@
         <f>IF(L20="","",(J20-L20)*100)</f>
         <v/>
       </c>
+      <c r="O20" s="6">
+        <f>'SOFR_Futures'!A19</f>
+        <v/>
+      </c>
+      <c r="P20" s="17">
+        <f>'SOFR_Futures'!H19</f>
+        <v/>
+      </c>
+      <c r="Q20" s="17">
+        <f>'SOFR_Futures'!H20</f>
+        <v/>
+      </c>
+      <c r="R20" s="16">
+        <f>MAX(0,(Q20-MAX(P20,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S20" s="16">
+        <f>'SOFR_Futures'!F19</f>
+        <v/>
+      </c>
+      <c r="T20" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" s="32">
+        <f>(S20-T20/100)/100</f>
+        <v/>
+      </c>
+      <c r="V20" s="33">
+        <f>W19</f>
+        <v/>
+      </c>
+      <c r="W20" s="33">
+        <f>V20/(1+U20*R20)</f>
+        <v/>
+      </c>
+      <c r="Y20" s="17">
+        <f>MAX(Q19,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z20" s="33">
+        <f>W19</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -5016,6 +5653,49 @@
         <f>IF(L21="","",(J21-L21)*100)</f>
         <v/>
       </c>
+      <c r="O21" s="6">
+        <f>'SOFR_Futures'!A20</f>
+        <v/>
+      </c>
+      <c r="P21" s="17">
+        <f>'SOFR_Futures'!H20</f>
+        <v/>
+      </c>
+      <c r="Q21" s="17">
+        <f>'SOFR_Futures'!H21</f>
+        <v/>
+      </c>
+      <c r="R21" s="16">
+        <f>MAX(0,(Q21-MAX(P21,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S21" s="16">
+        <f>'SOFR_Futures'!F20</f>
+        <v/>
+      </c>
+      <c r="T21" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" s="32">
+        <f>(S21-T21/100)/100</f>
+        <v/>
+      </c>
+      <c r="V21" s="33">
+        <f>W20</f>
+        <v/>
+      </c>
+      <c r="W21" s="33">
+        <f>V21/(1+U21*R21)</f>
+        <v/>
+      </c>
+      <c r="Y21" s="17">
+        <f>MAX(Q20,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z21" s="33">
+        <f>W20</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -5068,6 +5748,49 @@
         <f>IF(L22="","",(J22-L22)*100)</f>
         <v/>
       </c>
+      <c r="O22" s="6">
+        <f>'SOFR_Futures'!A21</f>
+        <v/>
+      </c>
+      <c r="P22" s="17">
+        <f>'SOFR_Futures'!H21</f>
+        <v/>
+      </c>
+      <c r="Q22" s="17">
+        <f>'SOFR_Futures'!H22</f>
+        <v/>
+      </c>
+      <c r="R22" s="16">
+        <f>MAX(0,(Q22-MAX(P22,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S22" s="16">
+        <f>'SOFR_Futures'!F21</f>
+        <v/>
+      </c>
+      <c r="T22" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" s="32">
+        <f>(S22-T22/100)/100</f>
+        <v/>
+      </c>
+      <c r="V22" s="33">
+        <f>W21</f>
+        <v/>
+      </c>
+      <c r="W22" s="33">
+        <f>V22/(1+U22*R22)</f>
+        <v/>
+      </c>
+      <c r="Y22" s="17">
+        <f>MAX(Q21,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z22" s="33">
+        <f>W21</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -5100,7 +5823,7 @@
         <v/>
       </c>
       <c r="H23" s="28">
-        <f>(1-(E23/100)*G23)/(1+(E23/100)*F23)</f>
+        <f>IFERROR(INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1)))^((B23-INDEX($Y$8:$Y$28,MATCH(B23,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B23,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B23,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1)))</f>
         <v/>
       </c>
       <c r="I23" s="16" t="n">
@@ -5119,6 +5842,49 @@
         <f>IF(L23="","",(J23-L23)*100)</f>
         <v/>
       </c>
+      <c r="O23" s="6">
+        <f>'SOFR_Futures'!A22</f>
+        <v/>
+      </c>
+      <c r="P23" s="17">
+        <f>'SOFR_Futures'!H22</f>
+        <v/>
+      </c>
+      <c r="Q23" s="17">
+        <f>'SOFR_Futures'!H23</f>
+        <v/>
+      </c>
+      <c r="R23" s="16">
+        <f>MAX(0,(Q23-MAX(P23,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S23" s="16">
+        <f>'SOFR_Futures'!F22</f>
+        <v/>
+      </c>
+      <c r="T23" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" s="32">
+        <f>(S23-T23/100)/100</f>
+        <v/>
+      </c>
+      <c r="V23" s="33">
+        <f>W22</f>
+        <v/>
+      </c>
+      <c r="W23" s="33">
+        <f>V23/(1+U23*R23)</f>
+        <v/>
+      </c>
+      <c r="Y23" s="17">
+        <f>MAX(Q22,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z23" s="33">
+        <f>W22</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -5151,7 +5917,7 @@
         <v/>
       </c>
       <c r="H24" s="28">
-        <f>(1-(E24/100)*G24)/(1+(E24/100)*F24)</f>
+        <f>IFERROR(INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1)))^((B24-INDEX($Y$8:$Y$28,MATCH(B24,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B24,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B24,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1)))</f>
         <v/>
       </c>
       <c r="I24" s="16">
@@ -5171,6 +5937,49 @@
         <f>IF(L24="","",(J24-L24)*100)</f>
         <v/>
       </c>
+      <c r="O24" s="6">
+        <f>'SOFR_Futures'!A23</f>
+        <v/>
+      </c>
+      <c r="P24" s="17">
+        <f>'SOFR_Futures'!H23</f>
+        <v/>
+      </c>
+      <c r="Q24" s="17">
+        <f>'SOFR_Futures'!H24</f>
+        <v/>
+      </c>
+      <c r="R24" s="16">
+        <f>MAX(0,(Q24-MAX(P24,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S24" s="16">
+        <f>'SOFR_Futures'!F23</f>
+        <v/>
+      </c>
+      <c r="T24" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U24" s="32">
+        <f>(S24-T24/100)/100</f>
+        <v/>
+      </c>
+      <c r="V24" s="33">
+        <f>W23</f>
+        <v/>
+      </c>
+      <c r="W24" s="33">
+        <f>V24/(1+U24*R24)</f>
+        <v/>
+      </c>
+      <c r="Y24" s="17">
+        <f>MAX(Q23,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z24" s="33">
+        <f>W23</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -5203,7 +6012,7 @@
         <v/>
       </c>
       <c r="H25" s="28">
-        <f>(1-(E25/100)*G25)/(1+(E25/100)*F25)</f>
+        <f>IFERROR(INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1)))^((B25-INDEX($Y$8:$Y$28,MATCH(B25,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B25,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B25,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1)))</f>
         <v/>
       </c>
       <c r="I25" s="16">
@@ -5223,6 +6032,49 @@
         <f>IF(L25="","",(J25-L25)*100)</f>
         <v/>
       </c>
+      <c r="O25" s="6">
+        <f>'SOFR_Futures'!A24</f>
+        <v/>
+      </c>
+      <c r="P25" s="17">
+        <f>'SOFR_Futures'!H24</f>
+        <v/>
+      </c>
+      <c r="Q25" s="17">
+        <f>'SOFR_Futures'!H25</f>
+        <v/>
+      </c>
+      <c r="R25" s="16">
+        <f>MAX(0,(Q25-MAX(P25,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S25" s="16">
+        <f>'SOFR_Futures'!F24</f>
+        <v/>
+      </c>
+      <c r="T25" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U25" s="32">
+        <f>(S25-T25/100)/100</f>
+        <v/>
+      </c>
+      <c r="V25" s="33">
+        <f>W24</f>
+        <v/>
+      </c>
+      <c r="W25" s="33">
+        <f>V25/(1+U25*R25)</f>
+        <v/>
+      </c>
+      <c r="Y25" s="17">
+        <f>MAX(Q24,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z25" s="33">
+        <f>W24</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -5255,7 +6107,7 @@
         <v/>
       </c>
       <c r="H26" s="28">
-        <f>(1-(E26/100)*G26)/(1+(E26/100)*F26)</f>
+        <f>IFERROR(INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1)))^((B26-INDEX($Y$8:$Y$28,MATCH(B26,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B26,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B26,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1)))</f>
         <v/>
       </c>
       <c r="I26" s="16">
@@ -5275,6 +6127,49 @@
         <f>IF(L26="","",(J26-L26)*100)</f>
         <v/>
       </c>
+      <c r="O26" s="6">
+        <f>'SOFR_Futures'!A25</f>
+        <v/>
+      </c>
+      <c r="P26" s="17">
+        <f>'SOFR_Futures'!H25</f>
+        <v/>
+      </c>
+      <c r="Q26" s="17">
+        <f>'SOFR_Futures'!H26</f>
+        <v/>
+      </c>
+      <c r="R26" s="16">
+        <f>MAX(0,(Q26-MAX(P26,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S26" s="16">
+        <f>'SOFR_Futures'!F25</f>
+        <v/>
+      </c>
+      <c r="T26" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U26" s="32">
+        <f>(S26-T26/100)/100</f>
+        <v/>
+      </c>
+      <c r="V26" s="33">
+        <f>W25</f>
+        <v/>
+      </c>
+      <c r="W26" s="33">
+        <f>V26/(1+U26*R26)</f>
+        <v/>
+      </c>
+      <c r="Y26" s="17">
+        <f>MAX(Q25,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z26" s="33">
+        <f>W25</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -5307,7 +6202,7 @@
         <v/>
       </c>
       <c r="H27" s="28">
-        <f>(1-(E27/100)*G27)/(1+(E27/100)*F27)</f>
+        <f>IFERROR(INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1)))^((B27-INDEX($Y$8:$Y$28,MATCH(B27,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B27,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B27,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1)))</f>
         <v/>
       </c>
       <c r="I27" s="16">
@@ -5327,6 +6222,49 @@
         <f>IF(L27="","",(J27-L27)*100)</f>
         <v/>
       </c>
+      <c r="O27" s="6">
+        <f>'SOFR_Futures'!A26</f>
+        <v/>
+      </c>
+      <c r="P27" s="17">
+        <f>'SOFR_Futures'!H26</f>
+        <v/>
+      </c>
+      <c r="Q27" s="17">
+        <f>EDATE(P27,3)</f>
+        <v/>
+      </c>
+      <c r="R27" s="16">
+        <f>MAX(0,(Q27-MAX(P27,$B$22))/360)</f>
+        <v/>
+      </c>
+      <c r="S27" s="16">
+        <f>'SOFR_Futures'!F26</f>
+        <v/>
+      </c>
+      <c r="T27" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" s="32">
+        <f>(S27-T27/100)/100</f>
+        <v/>
+      </c>
+      <c r="V27" s="33">
+        <f>W26</f>
+        <v/>
+      </c>
+      <c r="W27" s="33">
+        <f>V27/(1+U27*R27)</f>
+        <v/>
+      </c>
+      <c r="Y27" s="17">
+        <f>MAX(Q26,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z27" s="33">
+        <f>W26</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -5379,6 +6317,14 @@
         <f>IF(L28="","",(J28-L28)*100)</f>
         <v/>
       </c>
+      <c r="Y28" s="17">
+        <f>MAX(Q27,$B$22)</f>
+        <v/>
+      </c>
+      <c r="Z28" s="33">
+        <f>W27</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -5955,14 +6901,16 @@
     <row r="41" ht="44" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>Column H (Discount factor) is the deliverable curve P(0,T). Zero rate is continuously-compounded (ACT/365): z = −ln(DF)/T. Column I (Ann.add) is τ·DF booked only at annual coupon dates, so column G sums exactly the coupons each swap actually pays. Yellow column L takes pasted Bloomberg S490 zeros; Δ (bp) is your bootstrap vs Bloomberg — the dealer-curve validation from the Lehman paper. The Swap_Pricer tab values any SOFR OIS off this curve.</t>
+          <t>THREE SEGMENTS (Zhou 2002 structure):  SHORT o/n–1Y = single-payment SOFR OIS  (DF=1/(1+S·τ0));  MIDDLE 1Y–5Y = SR3 futures chained from the 1Y DF (helper block to the right, cols O–W);  LONG 5Y–50Y = annual SOFR OIS swaps built off the futures-derived 5Y point. No overlap — each maturity is covered once. Column H is the curve P(0,T); zero z=−ln(DF)/T. The futures convexity column (T) defaults to 0 — enter an adjustment in bp to correct futures→forward. Paste S490 zeros into column L for the Δz check; the Swap_Pricer values any OIS off this curve.</t>
         </is>
       </c>
     </row>
     <row r="42"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
+    <mergeCell ref="O6:W6"/>
     <mergeCell ref="A5:M6"/>
+    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="A41:M42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6024,12 +6972,12 @@
           <t>Direction (Leg 1 = Fixed)</t>
         </is>
       </c>
-      <c r="B5" s="31" t="inlineStr">
+      <c r="B5" s="34" t="inlineStr">
         <is>
           <t>Receive fixed</t>
         </is>
       </c>
-      <c r="C5" s="32" t="inlineStr">
+      <c r="C5" s="35" t="inlineStr">
         <is>
           <t>Type "Receive fixed" or "Pay fixed". Sets the sign of the net NPV.</t>
         </is>
@@ -6051,10 +6999,10 @@
           <t>Notional</t>
         </is>
       </c>
-      <c r="B6" s="33" t="n">
+      <c r="B6" s="36" t="n">
         <v>10000000</v>
       </c>
-      <c r="C6" s="32" t="inlineStr">
+      <c r="C6" s="35" t="inlineStr">
         <is>
           <t>Both legs, USD.</t>
         </is>
@@ -6063,7 +7011,7 @@
         <f>Bootstrap!$B$4</f>
         <v/>
       </c>
-      <c r="L6" s="34" t="n">
+      <c r="L6" s="33" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6082,7 +7030,7 @@
         <f>Bootstrap!B8</f>
         <v/>
       </c>
-      <c r="L7" s="34">
+      <c r="L7" s="33">
         <f>Bootstrap!H8</f>
         <v/>
       </c>
@@ -6093,11 +7041,11 @@
           <t>Effective date</t>
         </is>
       </c>
-      <c r="B8" s="35">
+      <c r="B8" s="37">
         <f>Bootstrap!$B$4</f>
         <v/>
       </c>
-      <c r="C8" s="32" t="inlineStr">
+      <c r="C8" s="35" t="inlineStr">
         <is>
           <t>Defaults to curve spot (T+2). Overtype for a forward-start swap.</t>
         </is>
@@ -6106,7 +7054,7 @@
         <f>Bootstrap!B9</f>
         <v/>
       </c>
-      <c r="L8" s="34">
+      <c r="L8" s="33">
         <f>Bootstrap!H9</f>
         <v/>
       </c>
@@ -6117,10 +7065,10 @@
           <t>Tenor (years)</t>
         </is>
       </c>
-      <c r="B9" s="36" t="n">
+      <c r="B9" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="32" t="inlineStr">
+      <c r="C9" s="35" t="inlineStr">
         <is>
           <t>Whole years; drives the annual coupon schedule below.</t>
         </is>
@@ -6129,7 +7077,7 @@
         <f>Bootstrap!B10</f>
         <v/>
       </c>
-      <c r="L9" s="34">
+      <c r="L9" s="33">
         <f>Bootstrap!H10</f>
         <v/>
       </c>
@@ -6144,7 +7092,7 @@
         <f>EDATE(B8,12*B9)</f>
         <v/>
       </c>
-      <c r="C10" s="32" t="inlineStr">
+      <c r="C10" s="35" t="inlineStr">
         <is>
           <t>Effective + Tenor.</t>
         </is>
@@ -6153,7 +7101,7 @@
         <f>Bootstrap!B11</f>
         <v/>
       </c>
-      <c r="L10" s="34">
+      <c r="L10" s="33">
         <f>Bootstrap!H11</f>
         <v/>
       </c>
@@ -6164,11 +7112,11 @@
           <t>Fixed coupon (%)</t>
         </is>
       </c>
-      <c r="B11" s="37">
+      <c r="B11" s="39">
         <f>B25</f>
         <v/>
       </c>
-      <c r="C11" s="32" t="inlineStr">
+      <c r="C11" s="35" t="inlineStr">
         <is>
           <t>Defaults to the Par coupon (row 25) → NPV ≈ 0. Overtype to value an off-market coupon.</t>
         </is>
@@ -6177,7 +7125,7 @@
         <f>Bootstrap!B12</f>
         <v/>
       </c>
-      <c r="L11" s="34">
+      <c r="L11" s="33">
         <f>Bootstrap!H12</f>
         <v/>
       </c>
@@ -6197,7 +7145,7 @@
         <f>Bootstrap!B13</f>
         <v/>
       </c>
-      <c r="L12" s="34">
+      <c r="L12" s="33">
         <f>Bootstrap!H13</f>
         <v/>
       </c>
@@ -6217,7 +7165,7 @@
         <f>Bootstrap!B14</f>
         <v/>
       </c>
-      <c r="L13" s="34">
+      <c r="L13" s="33">
         <f>Bootstrap!H14</f>
         <v/>
       </c>
@@ -6237,7 +7185,7 @@
         <f>Bootstrap!B15</f>
         <v/>
       </c>
-      <c r="L14" s="34">
+      <c r="L14" s="33">
         <f>Bootstrap!H15</f>
         <v/>
       </c>
@@ -6252,7 +7200,7 @@
         <f>VAL_DATE</f>
         <v/>
       </c>
-      <c r="C15" s="32" t="inlineStr">
+      <c r="C15" s="35" t="inlineStr">
         <is>
           <t>Curve is discounted from spot = Bootstrap!B4.</t>
         </is>
@@ -6261,7 +7209,7 @@
         <f>Bootstrap!B16</f>
         <v/>
       </c>
-      <c r="L15" s="34">
+      <c r="L15" s="33">
         <f>Bootstrap!H16</f>
         <v/>
       </c>
@@ -6272,7 +7220,7 @@
           <t>Direction sign (+recv / −pay)</t>
         </is>
       </c>
-      <c r="B16" s="38">
+      <c r="B16" s="40">
         <f>IF($B$5="Receive fixed",1,-1)</f>
         <v/>
       </c>
@@ -6280,7 +7228,7 @@
         <f>Bootstrap!B17</f>
         <v/>
       </c>
-      <c r="L16" s="34">
+      <c r="L16" s="33">
         <f>Bootstrap!H17</f>
         <v/>
       </c>
@@ -6290,7 +7238,7 @@
         <f>Bootstrap!B18</f>
         <v/>
       </c>
-      <c r="L17" s="34">
+      <c r="L17" s="33">
         <f>Bootstrap!H18</f>
         <v/>
       </c>
@@ -6305,7 +7253,7 @@
         <f>Bootstrap!B19</f>
         <v/>
       </c>
-      <c r="L18" s="34">
+      <c r="L18" s="33">
         <f>Bootstrap!H19</f>
         <v/>
       </c>
@@ -6316,11 +7264,11 @@
           <t>DF(effective)</t>
         </is>
       </c>
-      <c r="B19" s="34">
+      <c r="B19" s="33">
         <f>IFERROR(INDEX($L$6:$L$38,MATCH($B$8,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH($B$8,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH($B$8,$K$6:$K$38,1)))^(($B$8-INDEX($K$6:$K$38,MATCH($B$8,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH($B$8,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH($B$8,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH($B$8,$K$6:$K$38,1)))</f>
         <v/>
       </c>
-      <c r="C19" s="32" t="inlineStr">
+      <c r="C19" s="35" t="inlineStr">
         <is>
           <t>Interpolated from the curve.</t>
         </is>
@@ -6329,7 +7277,7 @@
         <f>Bootstrap!B20</f>
         <v/>
       </c>
-      <c r="L19" s="34">
+      <c r="L19" s="33">
         <f>Bootstrap!H20</f>
         <v/>
       </c>
@@ -6340,7 +7288,7 @@
           <t>DF(maturity)</t>
         </is>
       </c>
-      <c r="B20" s="34">
+      <c r="B20" s="33">
         <f>IFERROR(INDEX($L$6:$L$38,MATCH($B$10,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH($B$10,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH($B$10,$K$6:$K$38,1)))^(($B$10-INDEX($K$6:$K$38,MATCH($B$10,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH($B$10,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH($B$10,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH($B$10,$K$6:$K$38,1)))</f>
         <v/>
       </c>
@@ -6348,7 +7296,7 @@
         <f>Bootstrap!B21</f>
         <v/>
       </c>
-      <c r="L20" s="34">
+      <c r="L20" s="33">
         <f>Bootstrap!H21</f>
         <v/>
       </c>
@@ -6359,11 +7307,11 @@
           <t>Fixed annuity  Στ·DF</t>
         </is>
       </c>
-      <c r="B21" s="39">
+      <c r="B21" s="32">
         <f>SUM(H36:H85)</f>
         <v/>
       </c>
-      <c r="C21" s="32" t="inlineStr">
+      <c r="C21" s="35" t="inlineStr">
         <is>
           <t>Sum of τ·DF over the fixed coupon dates.</t>
         </is>
@@ -6372,7 +7320,7 @@
         <f>Bootstrap!B22</f>
         <v/>
       </c>
-      <c r="L21" s="34">
+      <c r="L21" s="33">
         <f>Bootstrap!H22</f>
         <v/>
       </c>
@@ -6383,7 +7331,7 @@
           <t>Fixed leg PV (coupons)</t>
         </is>
       </c>
-      <c r="B22" s="40">
+      <c r="B22" s="41">
         <f>SUM(G36:G85)</f>
         <v/>
       </c>
@@ -6391,7 +7339,7 @@
         <f>Bootstrap!B23</f>
         <v/>
       </c>
-      <c r="L22" s="34">
+      <c r="L22" s="33">
         <f>Bootstrap!H23</f>
         <v/>
       </c>
@@ -6402,11 +7350,11 @@
           <t>Float leg PV</t>
         </is>
       </c>
-      <c r="B23" s="40">
+      <c r="B23" s="41">
         <f>B6*(B19-B20)</f>
         <v/>
       </c>
-      <c r="C23" s="32" t="inlineStr">
+      <c r="C23" s="35" t="inlineStr">
         <is>
           <t>Single-curve SOFR float leg telescopes to N·(DF_eff − DF_mat).</t>
         </is>
@@ -6415,7 +7363,7 @@
         <f>Bootstrap!B24</f>
         <v/>
       </c>
-      <c r="L23" s="34">
+      <c r="L23" s="33">
         <f>Bootstrap!H24</f>
         <v/>
       </c>
@@ -6426,11 +7374,11 @@
           <t>Notional PV @ maturity</t>
         </is>
       </c>
-      <c r="B24" s="40">
+      <c r="B24" s="41">
         <f>B6*B20</f>
         <v/>
       </c>
-      <c r="C24" s="32" t="inlineStr">
+      <c r="C24" s="35" t="inlineStr">
         <is>
           <t>For the SWPM-style leg display only.</t>
         </is>
@@ -6439,7 +7387,7 @@
         <f>Bootstrap!B25</f>
         <v/>
       </c>
-      <c r="L24" s="34">
+      <c r="L24" s="33">
         <f>Bootstrap!H25</f>
         <v/>
       </c>
@@ -6450,11 +7398,11 @@
           <t>Par coupon (%)</t>
         </is>
       </c>
-      <c r="B25" s="39">
+      <c r="B25" s="32">
         <f>(B19-B20)/B21*100</f>
         <v/>
       </c>
-      <c r="C25" s="32" t="inlineStr">
+      <c r="C25" s="35" t="inlineStr">
         <is>
           <t>Coupon that sets NPV = 0:  (DF_eff − DF_mat) / annuity.</t>
         </is>
@@ -6463,7 +7411,7 @@
         <f>Bootstrap!B26</f>
         <v/>
       </c>
-      <c r="L25" s="34">
+      <c r="L25" s="33">
         <f>Bootstrap!H26</f>
         <v/>
       </c>
@@ -6474,11 +7422,11 @@
           <t>Leg 1 NPV  (fixed + notional)</t>
         </is>
       </c>
-      <c r="B26" s="40">
+      <c r="B26" s="41">
         <f>B16*(B22+B24)</f>
         <v/>
       </c>
-      <c r="C26" s="32" t="inlineStr">
+      <c r="C26" s="35" t="inlineStr">
         <is>
           <t>SWPM shows each leg incl. a notional redemption.</t>
         </is>
@@ -6487,7 +7435,7 @@
         <f>Bootstrap!B27</f>
         <v/>
       </c>
-      <c r="L26" s="34">
+      <c r="L26" s="33">
         <f>Bootstrap!H27</f>
         <v/>
       </c>
@@ -6498,7 +7446,7 @@
           <t>Leg 2 NPV  (float + notional)</t>
         </is>
       </c>
-      <c r="B27" s="40">
+      <c r="B27" s="41">
         <f>-B16*(B23+B24)</f>
         <v/>
       </c>
@@ -6506,7 +7454,7 @@
         <f>Bootstrap!B28</f>
         <v/>
       </c>
-      <c r="L27" s="34">
+      <c r="L27" s="33">
         <f>Bootstrap!H28</f>
         <v/>
       </c>
@@ -6517,11 +7465,11 @@
           <t>Net swap NPV</t>
         </is>
       </c>
-      <c r="B28" s="41">
+      <c r="B28" s="42">
         <f>B26+B27</f>
         <v/>
       </c>
-      <c r="C28" s="32" t="inlineStr">
+      <c r="C28" s="35" t="inlineStr">
         <is>
           <t>Fixed − Float (notionals cancel); ≈ 0 at par coupon.</t>
         </is>
@@ -6530,7 +7478,7 @@
         <f>Bootstrap!B29</f>
         <v/>
       </c>
-      <c r="L28" s="34">
+      <c r="L28" s="33">
         <f>Bootstrap!H29</f>
         <v/>
       </c>
@@ -6541,11 +7489,11 @@
           <t>PV01 / DV01  (per 1bp)</t>
         </is>
       </c>
-      <c r="B29" s="40">
+      <c r="B29" s="41">
         <f>B6*B21*0.0001</f>
         <v/>
       </c>
-      <c r="C29" s="32" t="inlineStr">
+      <c r="C29" s="35" t="inlineStr">
         <is>
           <t>Annuity × notional × 1bp.</t>
         </is>
@@ -6554,7 +7502,7 @@
         <f>Bootstrap!B30</f>
         <v/>
       </c>
-      <c r="L29" s="34">
+      <c r="L29" s="33">
         <f>Bootstrap!H30</f>
         <v/>
       </c>
@@ -6565,14 +7513,14 @@
           <t>Accrued (at inception)</t>
         </is>
       </c>
-      <c r="B30" s="40" t="n">
+      <c r="B30" s="41" t="n">
         <v>0</v>
       </c>
       <c r="K30" s="17">
         <f>Bootstrap!B31</f>
         <v/>
       </c>
-      <c r="L30" s="34">
+      <c r="L30" s="33">
         <f>Bootstrap!H31</f>
         <v/>
       </c>
@@ -6582,7 +7530,7 @@
         <f>Bootstrap!B32</f>
         <v/>
       </c>
-      <c r="L31" s="34">
+      <c r="L31" s="33">
         <f>Bootstrap!H32</f>
         <v/>
       </c>
@@ -6597,7 +7545,7 @@
         <f>Bootstrap!B33</f>
         <v/>
       </c>
-      <c r="L32" s="34">
+      <c r="L32" s="33">
         <f>Bootstrap!H33</f>
         <v/>
       </c>
@@ -6607,7 +7555,7 @@
         <f>Bootstrap!B34</f>
         <v/>
       </c>
-      <c r="L33" s="34">
+      <c r="L33" s="33">
         <f>Bootstrap!H34</f>
         <v/>
       </c>
@@ -6617,7 +7565,7 @@
         <f>Bootstrap!B35</f>
         <v/>
       </c>
-      <c r="L34" s="34">
+      <c r="L34" s="33">
         <f>Bootstrap!H35</f>
         <v/>
       </c>
@@ -6667,13 +7615,13 @@
         <f>Bootstrap!B36</f>
         <v/>
       </c>
-      <c r="L35" s="34">
+      <c r="L35" s="33">
         <f>Bootstrap!H36</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="38">
+      <c r="A36" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -6689,19 +7637,19 @@
         <f>IF(A36&lt;=$B$9,(B36-C36)/360,"")</f>
         <v/>
       </c>
-      <c r="E36" s="34">
+      <c r="E36" s="33">
         <f>IF(A36&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B36,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B36,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B36,$K$6:$K$38,1)))^((B36-INDEX($K$6:$K$38,MATCH(B36,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B36,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B36,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B36,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F36" s="40">
+      <c r="F36" s="41">
         <f>IF(A36&lt;=$B$9,$B$6*$B$11/100*D36,"")</f>
         <v/>
       </c>
-      <c r="G36" s="40">
+      <c r="G36" s="41">
         <f>IF(A36&lt;=$B$9,F36*E36,"")</f>
         <v/>
       </c>
-      <c r="H36" s="39">
+      <c r="H36" s="32">
         <f>IF(A36&lt;=$B$9,D36*E36,"")</f>
         <v/>
       </c>
@@ -6709,13 +7657,13 @@
         <f>Bootstrap!B37</f>
         <v/>
       </c>
-      <c r="L36" s="34">
+      <c r="L36" s="33">
         <f>Bootstrap!H37</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="38">
+      <c r="A37" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -6731,19 +7679,19 @@
         <f>IF(A37&lt;=$B$9,(B37-C37)/360,"")</f>
         <v/>
       </c>
-      <c r="E37" s="34">
+      <c r="E37" s="33">
         <f>IF(A37&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B37,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B37,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B37,$K$6:$K$38,1)))^((B37-INDEX($K$6:$K$38,MATCH(B37,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B37,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B37,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B37,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F37" s="40">
+      <c r="F37" s="41">
         <f>IF(A37&lt;=$B$9,$B$6*$B$11/100*D37,"")</f>
         <v/>
       </c>
-      <c r="G37" s="40">
+      <c r="G37" s="41">
         <f>IF(A37&lt;=$B$9,F37*E37,"")</f>
         <v/>
       </c>
-      <c r="H37" s="39">
+      <c r="H37" s="32">
         <f>IF(A37&lt;=$B$9,D37*E37,"")</f>
         <v/>
       </c>
@@ -6751,13 +7699,13 @@
         <f>Bootstrap!B38</f>
         <v/>
       </c>
-      <c r="L37" s="34">
+      <c r="L37" s="33">
         <f>Bootstrap!H38</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="38">
+      <c r="A38" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -6773,19 +7721,19 @@
         <f>IF(A38&lt;=$B$9,(B38-C38)/360,"")</f>
         <v/>
       </c>
-      <c r="E38" s="34">
+      <c r="E38" s="33">
         <f>IF(A38&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B38,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B38,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B38,$K$6:$K$38,1)))^((B38-INDEX($K$6:$K$38,MATCH(B38,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B38,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B38,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B38,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F38" s="40">
+      <c r="F38" s="41">
         <f>IF(A38&lt;=$B$9,$B$6*$B$11/100*D38,"")</f>
         <v/>
       </c>
-      <c r="G38" s="40">
+      <c r="G38" s="41">
         <f>IF(A38&lt;=$B$9,F38*E38,"")</f>
         <v/>
       </c>
-      <c r="H38" s="39">
+      <c r="H38" s="32">
         <f>IF(A38&lt;=$B$9,D38*E38,"")</f>
         <v/>
       </c>
@@ -6793,13 +7741,13 @@
         <f>Bootstrap!B39</f>
         <v/>
       </c>
-      <c r="L38" s="34">
+      <c r="L38" s="33">
         <f>Bootstrap!H39</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="38">
+      <c r="A39" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -6815,19 +7763,19 @@
         <f>IF(A39&lt;=$B$9,(B39-C39)/360,"")</f>
         <v/>
       </c>
-      <c r="E39" s="34">
+      <c r="E39" s="33">
         <f>IF(A39&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B39,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B39,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B39,$K$6:$K$38,1)))^((B39-INDEX($K$6:$K$38,MATCH(B39,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B39,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B39,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B39,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F39" s="40">
+      <c r="F39" s="41">
         <f>IF(A39&lt;=$B$9,$B$6*$B$11/100*D39,"")</f>
         <v/>
       </c>
-      <c r="G39" s="40">
+      <c r="G39" s="41">
         <f>IF(A39&lt;=$B$9,F39*E39,"")</f>
         <v/>
       </c>
-      <c r="H39" s="39">
+      <c r="H39" s="32">
         <f>IF(A39&lt;=$B$9,D39*E39,"")</f>
         <v/>
       </c>
@@ -6838,7 +7786,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="38">
+      <c r="A40" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -6854,25 +7802,25 @@
         <f>IF(A40&lt;=$B$9,(B40-C40)/360,"")</f>
         <v/>
       </c>
-      <c r="E40" s="34">
+      <c r="E40" s="33">
         <f>IF(A40&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B40,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B40,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B40,$K$6:$K$38,1)))^((B40-INDEX($K$6:$K$38,MATCH(B40,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B40,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B40,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B40,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F40" s="40">
+      <c r="F40" s="41">
         <f>IF(A40&lt;=$B$9,$B$6*$B$11/100*D40,"")</f>
         <v/>
       </c>
-      <c r="G40" s="40">
+      <c r="G40" s="41">
         <f>IF(A40&lt;=$B$9,F40*E40,"")</f>
         <v/>
       </c>
-      <c r="H40" s="39">
+      <c r="H40" s="32">
         <f>IF(A40&lt;=$B$9,D40*E40,"")</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="38">
+      <c r="A41" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -6888,25 +7836,25 @@
         <f>IF(A41&lt;=$B$9,(B41-C41)/360,"")</f>
         <v/>
       </c>
-      <c r="E41" s="34">
+      <c r="E41" s="33">
         <f>IF(A41&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B41,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B41,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B41,$K$6:$K$38,1)))^((B41-INDEX($K$6:$K$38,MATCH(B41,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B41,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B41,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B41,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F41" s="40">
+      <c r="F41" s="41">
         <f>IF(A41&lt;=$B$9,$B$6*$B$11/100*D41,"")</f>
         <v/>
       </c>
-      <c r="G41" s="40">
+      <c r="G41" s="41">
         <f>IF(A41&lt;=$B$9,F41*E41,"")</f>
         <v/>
       </c>
-      <c r="H41" s="39">
+      <c r="H41" s="32">
         <f>IF(A41&lt;=$B$9,D41*E41,"")</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="38">
+      <c r="A42" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -6922,25 +7870,25 @@
         <f>IF(A42&lt;=$B$9,(B42-C42)/360,"")</f>
         <v/>
       </c>
-      <c r="E42" s="34">
+      <c r="E42" s="33">
         <f>IF(A42&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B42,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B42,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B42,$K$6:$K$38,1)))^((B42-INDEX($K$6:$K$38,MATCH(B42,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B42,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B42,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B42,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F42" s="40">
+      <c r="F42" s="41">
         <f>IF(A42&lt;=$B$9,$B$6*$B$11/100*D42,"")</f>
         <v/>
       </c>
-      <c r="G42" s="40">
+      <c r="G42" s="41">
         <f>IF(A42&lt;=$B$9,F42*E42,"")</f>
         <v/>
       </c>
-      <c r="H42" s="39">
+      <c r="H42" s="32">
         <f>IF(A42&lt;=$B$9,D42*E42,"")</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="38">
+      <c r="A43" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -6956,25 +7904,25 @@
         <f>IF(A43&lt;=$B$9,(B43-C43)/360,"")</f>
         <v/>
       </c>
-      <c r="E43" s="34">
+      <c r="E43" s="33">
         <f>IF(A43&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B43,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B43,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B43,$K$6:$K$38,1)))^((B43-INDEX($K$6:$K$38,MATCH(B43,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B43,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B43,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B43,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F43" s="40">
+      <c r="F43" s="41">
         <f>IF(A43&lt;=$B$9,$B$6*$B$11/100*D43,"")</f>
         <v/>
       </c>
-      <c r="G43" s="40">
+      <c r="G43" s="41">
         <f>IF(A43&lt;=$B$9,F43*E43,"")</f>
         <v/>
       </c>
-      <c r="H43" s="39">
+      <c r="H43" s="32">
         <f>IF(A43&lt;=$B$9,D43*E43,"")</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="38">
+      <c r="A44" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -6990,25 +7938,25 @@
         <f>IF(A44&lt;=$B$9,(B44-C44)/360,"")</f>
         <v/>
       </c>
-      <c r="E44" s="34">
+      <c r="E44" s="33">
         <f>IF(A44&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B44,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B44,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B44,$K$6:$K$38,1)))^((B44-INDEX($K$6:$K$38,MATCH(B44,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B44,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B44,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B44,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F44" s="40">
+      <c r="F44" s="41">
         <f>IF(A44&lt;=$B$9,$B$6*$B$11/100*D44,"")</f>
         <v/>
       </c>
-      <c r="G44" s="40">
+      <c r="G44" s="41">
         <f>IF(A44&lt;=$B$9,F44*E44,"")</f>
         <v/>
       </c>
-      <c r="H44" s="39">
+      <c r="H44" s="32">
         <f>IF(A44&lt;=$B$9,D44*E44,"")</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="38">
+      <c r="A45" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7024,25 +7972,25 @@
         <f>IF(A45&lt;=$B$9,(B45-C45)/360,"")</f>
         <v/>
       </c>
-      <c r="E45" s="34">
+      <c r="E45" s="33">
         <f>IF(A45&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B45,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B45,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B45,$K$6:$K$38,1)))^((B45-INDEX($K$6:$K$38,MATCH(B45,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B45,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B45,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B45,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F45" s="40">
+      <c r="F45" s="41">
         <f>IF(A45&lt;=$B$9,$B$6*$B$11/100*D45,"")</f>
         <v/>
       </c>
-      <c r="G45" s="40">
+      <c r="G45" s="41">
         <f>IF(A45&lt;=$B$9,F45*E45,"")</f>
         <v/>
       </c>
-      <c r="H45" s="39">
+      <c r="H45" s="32">
         <f>IF(A45&lt;=$B$9,D45*E45,"")</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="38">
+      <c r="A46" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7058,25 +8006,25 @@
         <f>IF(A46&lt;=$B$9,(B46-C46)/360,"")</f>
         <v/>
       </c>
-      <c r="E46" s="34">
+      <c r="E46" s="33">
         <f>IF(A46&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B46,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B46,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B46,$K$6:$K$38,1)))^((B46-INDEX($K$6:$K$38,MATCH(B46,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B46,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B46,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B46,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F46" s="40">
+      <c r="F46" s="41">
         <f>IF(A46&lt;=$B$9,$B$6*$B$11/100*D46,"")</f>
         <v/>
       </c>
-      <c r="G46" s="40">
+      <c r="G46" s="41">
         <f>IF(A46&lt;=$B$9,F46*E46,"")</f>
         <v/>
       </c>
-      <c r="H46" s="39">
+      <c r="H46" s="32">
         <f>IF(A46&lt;=$B$9,D46*E46,"")</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="38">
+      <c r="A47" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7092,25 +8040,25 @@
         <f>IF(A47&lt;=$B$9,(B47-C47)/360,"")</f>
         <v/>
       </c>
-      <c r="E47" s="34">
+      <c r="E47" s="33">
         <f>IF(A47&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B47,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B47,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B47,$K$6:$K$38,1)))^((B47-INDEX($K$6:$K$38,MATCH(B47,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B47,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B47,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B47,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F47" s="40">
+      <c r="F47" s="41">
         <f>IF(A47&lt;=$B$9,$B$6*$B$11/100*D47,"")</f>
         <v/>
       </c>
-      <c r="G47" s="40">
+      <c r="G47" s="41">
         <f>IF(A47&lt;=$B$9,F47*E47,"")</f>
         <v/>
       </c>
-      <c r="H47" s="39">
+      <c r="H47" s="32">
         <f>IF(A47&lt;=$B$9,D47*E47,"")</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="38">
+      <c r="A48" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7126,25 +8074,25 @@
         <f>IF(A48&lt;=$B$9,(B48-C48)/360,"")</f>
         <v/>
       </c>
-      <c r="E48" s="34">
+      <c r="E48" s="33">
         <f>IF(A48&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B48,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B48,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B48,$K$6:$K$38,1)))^((B48-INDEX($K$6:$K$38,MATCH(B48,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B48,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B48,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B48,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F48" s="40">
+      <c r="F48" s="41">
         <f>IF(A48&lt;=$B$9,$B$6*$B$11/100*D48,"")</f>
         <v/>
       </c>
-      <c r="G48" s="40">
+      <c r="G48" s="41">
         <f>IF(A48&lt;=$B$9,F48*E48,"")</f>
         <v/>
       </c>
-      <c r="H48" s="39">
+      <c r="H48" s="32">
         <f>IF(A48&lt;=$B$9,D48*E48,"")</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="38">
+      <c r="A49" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7160,25 +8108,25 @@
         <f>IF(A49&lt;=$B$9,(B49-C49)/360,"")</f>
         <v/>
       </c>
-      <c r="E49" s="34">
+      <c r="E49" s="33">
         <f>IF(A49&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B49,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B49,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B49,$K$6:$K$38,1)))^((B49-INDEX($K$6:$K$38,MATCH(B49,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B49,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B49,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B49,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F49" s="40">
+      <c r="F49" s="41">
         <f>IF(A49&lt;=$B$9,$B$6*$B$11/100*D49,"")</f>
         <v/>
       </c>
-      <c r="G49" s="40">
+      <c r="G49" s="41">
         <f>IF(A49&lt;=$B$9,F49*E49,"")</f>
         <v/>
       </c>
-      <c r="H49" s="39">
+      <c r="H49" s="32">
         <f>IF(A49&lt;=$B$9,D49*E49,"")</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="38">
+      <c r="A50" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7194,25 +8142,25 @@
         <f>IF(A50&lt;=$B$9,(B50-C50)/360,"")</f>
         <v/>
       </c>
-      <c r="E50" s="34">
+      <c r="E50" s="33">
         <f>IF(A50&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B50,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B50,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B50,$K$6:$K$38,1)))^((B50-INDEX($K$6:$K$38,MATCH(B50,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B50,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B50,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B50,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F50" s="40">
+      <c r="F50" s="41">
         <f>IF(A50&lt;=$B$9,$B$6*$B$11/100*D50,"")</f>
         <v/>
       </c>
-      <c r="G50" s="40">
+      <c r="G50" s="41">
         <f>IF(A50&lt;=$B$9,F50*E50,"")</f>
         <v/>
       </c>
-      <c r="H50" s="39">
+      <c r="H50" s="32">
         <f>IF(A50&lt;=$B$9,D50*E50,"")</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="38">
+      <c r="A51" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7228,25 +8176,25 @@
         <f>IF(A51&lt;=$B$9,(B51-C51)/360,"")</f>
         <v/>
       </c>
-      <c r="E51" s="34">
+      <c r="E51" s="33">
         <f>IF(A51&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B51,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B51,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B51,$K$6:$K$38,1)))^((B51-INDEX($K$6:$K$38,MATCH(B51,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B51,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B51,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B51,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F51" s="40">
+      <c r="F51" s="41">
         <f>IF(A51&lt;=$B$9,$B$6*$B$11/100*D51,"")</f>
         <v/>
       </c>
-      <c r="G51" s="40">
+      <c r="G51" s="41">
         <f>IF(A51&lt;=$B$9,F51*E51,"")</f>
         <v/>
       </c>
-      <c r="H51" s="39">
+      <c r="H51" s="32">
         <f>IF(A51&lt;=$B$9,D51*E51,"")</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="38">
+      <c r="A52" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7262,25 +8210,25 @@
         <f>IF(A52&lt;=$B$9,(B52-C52)/360,"")</f>
         <v/>
       </c>
-      <c r="E52" s="34">
+      <c r="E52" s="33">
         <f>IF(A52&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B52,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B52,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B52,$K$6:$K$38,1)))^((B52-INDEX($K$6:$K$38,MATCH(B52,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B52,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B52,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B52,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F52" s="40">
+      <c r="F52" s="41">
         <f>IF(A52&lt;=$B$9,$B$6*$B$11/100*D52,"")</f>
         <v/>
       </c>
-      <c r="G52" s="40">
+      <c r="G52" s="41">
         <f>IF(A52&lt;=$B$9,F52*E52,"")</f>
         <v/>
       </c>
-      <c r="H52" s="39">
+      <c r="H52" s="32">
         <f>IF(A52&lt;=$B$9,D52*E52,"")</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="38">
+      <c r="A53" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7296,25 +8244,25 @@
         <f>IF(A53&lt;=$B$9,(B53-C53)/360,"")</f>
         <v/>
       </c>
-      <c r="E53" s="34">
+      <c r="E53" s="33">
         <f>IF(A53&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B53,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B53,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B53,$K$6:$K$38,1)))^((B53-INDEX($K$6:$K$38,MATCH(B53,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B53,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B53,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B53,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F53" s="40">
+      <c r="F53" s="41">
         <f>IF(A53&lt;=$B$9,$B$6*$B$11/100*D53,"")</f>
         <v/>
       </c>
-      <c r="G53" s="40">
+      <c r="G53" s="41">
         <f>IF(A53&lt;=$B$9,F53*E53,"")</f>
         <v/>
       </c>
-      <c r="H53" s="39">
+      <c r="H53" s="32">
         <f>IF(A53&lt;=$B$9,D53*E53,"")</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="38">
+      <c r="A54" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7330,25 +8278,25 @@
         <f>IF(A54&lt;=$B$9,(B54-C54)/360,"")</f>
         <v/>
       </c>
-      <c r="E54" s="34">
+      <c r="E54" s="33">
         <f>IF(A54&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B54,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B54,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B54,$K$6:$K$38,1)))^((B54-INDEX($K$6:$K$38,MATCH(B54,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B54,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B54,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B54,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F54" s="40">
+      <c r="F54" s="41">
         <f>IF(A54&lt;=$B$9,$B$6*$B$11/100*D54,"")</f>
         <v/>
       </c>
-      <c r="G54" s="40">
+      <c r="G54" s="41">
         <f>IF(A54&lt;=$B$9,F54*E54,"")</f>
         <v/>
       </c>
-      <c r="H54" s="39">
+      <c r="H54" s="32">
         <f>IF(A54&lt;=$B$9,D54*E54,"")</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="38">
+      <c r="A55" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7364,25 +8312,25 @@
         <f>IF(A55&lt;=$B$9,(B55-C55)/360,"")</f>
         <v/>
       </c>
-      <c r="E55" s="34">
+      <c r="E55" s="33">
         <f>IF(A55&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B55,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B55,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B55,$K$6:$K$38,1)))^((B55-INDEX($K$6:$K$38,MATCH(B55,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B55,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B55,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B55,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F55" s="40">
+      <c r="F55" s="41">
         <f>IF(A55&lt;=$B$9,$B$6*$B$11/100*D55,"")</f>
         <v/>
       </c>
-      <c r="G55" s="40">
+      <c r="G55" s="41">
         <f>IF(A55&lt;=$B$9,F55*E55,"")</f>
         <v/>
       </c>
-      <c r="H55" s="39">
+      <c r="H55" s="32">
         <f>IF(A55&lt;=$B$9,D55*E55,"")</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="38">
+      <c r="A56" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7398,25 +8346,25 @@
         <f>IF(A56&lt;=$B$9,(B56-C56)/360,"")</f>
         <v/>
       </c>
-      <c r="E56" s="34">
+      <c r="E56" s="33">
         <f>IF(A56&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B56,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B56,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B56,$K$6:$K$38,1)))^((B56-INDEX($K$6:$K$38,MATCH(B56,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B56,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B56,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B56,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F56" s="40">
+      <c r="F56" s="41">
         <f>IF(A56&lt;=$B$9,$B$6*$B$11/100*D56,"")</f>
         <v/>
       </c>
-      <c r="G56" s="40">
+      <c r="G56" s="41">
         <f>IF(A56&lt;=$B$9,F56*E56,"")</f>
         <v/>
       </c>
-      <c r="H56" s="39">
+      <c r="H56" s="32">
         <f>IF(A56&lt;=$B$9,D56*E56,"")</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="38">
+      <c r="A57" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7432,25 +8380,25 @@
         <f>IF(A57&lt;=$B$9,(B57-C57)/360,"")</f>
         <v/>
       </c>
-      <c r="E57" s="34">
+      <c r="E57" s="33">
         <f>IF(A57&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B57,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B57,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B57,$K$6:$K$38,1)))^((B57-INDEX($K$6:$K$38,MATCH(B57,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B57,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B57,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B57,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F57" s="40">
+      <c r="F57" s="41">
         <f>IF(A57&lt;=$B$9,$B$6*$B$11/100*D57,"")</f>
         <v/>
       </c>
-      <c r="G57" s="40">
+      <c r="G57" s="41">
         <f>IF(A57&lt;=$B$9,F57*E57,"")</f>
         <v/>
       </c>
-      <c r="H57" s="39">
+      <c r="H57" s="32">
         <f>IF(A57&lt;=$B$9,D57*E57,"")</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="38">
+      <c r="A58" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7466,25 +8414,25 @@
         <f>IF(A58&lt;=$B$9,(B58-C58)/360,"")</f>
         <v/>
       </c>
-      <c r="E58" s="34">
+      <c r="E58" s="33">
         <f>IF(A58&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B58,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B58,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B58,$K$6:$K$38,1)))^((B58-INDEX($K$6:$K$38,MATCH(B58,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B58,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B58,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B58,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F58" s="40">
+      <c r="F58" s="41">
         <f>IF(A58&lt;=$B$9,$B$6*$B$11/100*D58,"")</f>
         <v/>
       </c>
-      <c r="G58" s="40">
+      <c r="G58" s="41">
         <f>IF(A58&lt;=$B$9,F58*E58,"")</f>
         <v/>
       </c>
-      <c r="H58" s="39">
+      <c r="H58" s="32">
         <f>IF(A58&lt;=$B$9,D58*E58,"")</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="38">
+      <c r="A59" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7500,25 +8448,25 @@
         <f>IF(A59&lt;=$B$9,(B59-C59)/360,"")</f>
         <v/>
       </c>
-      <c r="E59" s="34">
+      <c r="E59" s="33">
         <f>IF(A59&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B59,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B59,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B59,$K$6:$K$38,1)))^((B59-INDEX($K$6:$K$38,MATCH(B59,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B59,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B59,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B59,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F59" s="40">
+      <c r="F59" s="41">
         <f>IF(A59&lt;=$B$9,$B$6*$B$11/100*D59,"")</f>
         <v/>
       </c>
-      <c r="G59" s="40">
+      <c r="G59" s="41">
         <f>IF(A59&lt;=$B$9,F59*E59,"")</f>
         <v/>
       </c>
-      <c r="H59" s="39">
+      <c r="H59" s="32">
         <f>IF(A59&lt;=$B$9,D59*E59,"")</f>
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="38">
+      <c r="A60" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7534,25 +8482,25 @@
         <f>IF(A60&lt;=$B$9,(B60-C60)/360,"")</f>
         <v/>
       </c>
-      <c r="E60" s="34">
+      <c r="E60" s="33">
         <f>IF(A60&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B60,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B60,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B60,$K$6:$K$38,1)))^((B60-INDEX($K$6:$K$38,MATCH(B60,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B60,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B60,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B60,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F60" s="40">
+      <c r="F60" s="41">
         <f>IF(A60&lt;=$B$9,$B$6*$B$11/100*D60,"")</f>
         <v/>
       </c>
-      <c r="G60" s="40">
+      <c r="G60" s="41">
         <f>IF(A60&lt;=$B$9,F60*E60,"")</f>
         <v/>
       </c>
-      <c r="H60" s="39">
+      <c r="H60" s="32">
         <f>IF(A60&lt;=$B$9,D60*E60,"")</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="38">
+      <c r="A61" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7568,25 +8516,25 @@
         <f>IF(A61&lt;=$B$9,(B61-C61)/360,"")</f>
         <v/>
       </c>
-      <c r="E61" s="34">
+      <c r="E61" s="33">
         <f>IF(A61&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B61,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B61,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B61,$K$6:$K$38,1)))^((B61-INDEX($K$6:$K$38,MATCH(B61,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B61,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B61,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B61,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F61" s="40">
+      <c r="F61" s="41">
         <f>IF(A61&lt;=$B$9,$B$6*$B$11/100*D61,"")</f>
         <v/>
       </c>
-      <c r="G61" s="40">
+      <c r="G61" s="41">
         <f>IF(A61&lt;=$B$9,F61*E61,"")</f>
         <v/>
       </c>
-      <c r="H61" s="39">
+      <c r="H61" s="32">
         <f>IF(A61&lt;=$B$9,D61*E61,"")</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="38">
+      <c r="A62" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7602,25 +8550,25 @@
         <f>IF(A62&lt;=$B$9,(B62-C62)/360,"")</f>
         <v/>
       </c>
-      <c r="E62" s="34">
+      <c r="E62" s="33">
         <f>IF(A62&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B62,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B62,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B62,$K$6:$K$38,1)))^((B62-INDEX($K$6:$K$38,MATCH(B62,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B62,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B62,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B62,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F62" s="40">
+      <c r="F62" s="41">
         <f>IF(A62&lt;=$B$9,$B$6*$B$11/100*D62,"")</f>
         <v/>
       </c>
-      <c r="G62" s="40">
+      <c r="G62" s="41">
         <f>IF(A62&lt;=$B$9,F62*E62,"")</f>
         <v/>
       </c>
-      <c r="H62" s="39">
+      <c r="H62" s="32">
         <f>IF(A62&lt;=$B$9,D62*E62,"")</f>
         <v/>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="38">
+      <c r="A63" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7636,25 +8584,25 @@
         <f>IF(A63&lt;=$B$9,(B63-C63)/360,"")</f>
         <v/>
       </c>
-      <c r="E63" s="34">
+      <c r="E63" s="33">
         <f>IF(A63&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B63,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B63,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B63,$K$6:$K$38,1)))^((B63-INDEX($K$6:$K$38,MATCH(B63,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B63,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B63,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B63,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F63" s="40">
+      <c r="F63" s="41">
         <f>IF(A63&lt;=$B$9,$B$6*$B$11/100*D63,"")</f>
         <v/>
       </c>
-      <c r="G63" s="40">
+      <c r="G63" s="41">
         <f>IF(A63&lt;=$B$9,F63*E63,"")</f>
         <v/>
       </c>
-      <c r="H63" s="39">
+      <c r="H63" s="32">
         <f>IF(A63&lt;=$B$9,D63*E63,"")</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="38">
+      <c r="A64" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7670,25 +8618,25 @@
         <f>IF(A64&lt;=$B$9,(B64-C64)/360,"")</f>
         <v/>
       </c>
-      <c r="E64" s="34">
+      <c r="E64" s="33">
         <f>IF(A64&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B64,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B64,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B64,$K$6:$K$38,1)))^((B64-INDEX($K$6:$K$38,MATCH(B64,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B64,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B64,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B64,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F64" s="40">
+      <c r="F64" s="41">
         <f>IF(A64&lt;=$B$9,$B$6*$B$11/100*D64,"")</f>
         <v/>
       </c>
-      <c r="G64" s="40">
+      <c r="G64" s="41">
         <f>IF(A64&lt;=$B$9,F64*E64,"")</f>
         <v/>
       </c>
-      <c r="H64" s="39">
+      <c r="H64" s="32">
         <f>IF(A64&lt;=$B$9,D64*E64,"")</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="38">
+      <c r="A65" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7704,25 +8652,25 @@
         <f>IF(A65&lt;=$B$9,(B65-C65)/360,"")</f>
         <v/>
       </c>
-      <c r="E65" s="34">
+      <c r="E65" s="33">
         <f>IF(A65&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B65,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B65,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B65,$K$6:$K$38,1)))^((B65-INDEX($K$6:$K$38,MATCH(B65,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B65,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B65,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B65,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F65" s="40">
+      <c r="F65" s="41">
         <f>IF(A65&lt;=$B$9,$B$6*$B$11/100*D65,"")</f>
         <v/>
       </c>
-      <c r="G65" s="40">
+      <c r="G65" s="41">
         <f>IF(A65&lt;=$B$9,F65*E65,"")</f>
         <v/>
       </c>
-      <c r="H65" s="39">
+      <c r="H65" s="32">
         <f>IF(A65&lt;=$B$9,D65*E65,"")</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="38">
+      <c r="A66" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7738,25 +8686,25 @@
         <f>IF(A66&lt;=$B$9,(B66-C66)/360,"")</f>
         <v/>
       </c>
-      <c r="E66" s="34">
+      <c r="E66" s="33">
         <f>IF(A66&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B66,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B66,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B66,$K$6:$K$38,1)))^((B66-INDEX($K$6:$K$38,MATCH(B66,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B66,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B66,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B66,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F66" s="40">
+      <c r="F66" s="41">
         <f>IF(A66&lt;=$B$9,$B$6*$B$11/100*D66,"")</f>
         <v/>
       </c>
-      <c r="G66" s="40">
+      <c r="G66" s="41">
         <f>IF(A66&lt;=$B$9,F66*E66,"")</f>
         <v/>
       </c>
-      <c r="H66" s="39">
+      <c r="H66" s="32">
         <f>IF(A66&lt;=$B$9,D66*E66,"")</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="38">
+      <c r="A67" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7772,25 +8720,25 @@
         <f>IF(A67&lt;=$B$9,(B67-C67)/360,"")</f>
         <v/>
       </c>
-      <c r="E67" s="34">
+      <c r="E67" s="33">
         <f>IF(A67&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B67,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B67,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B67,$K$6:$K$38,1)))^((B67-INDEX($K$6:$K$38,MATCH(B67,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B67,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B67,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B67,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F67" s="40">
+      <c r="F67" s="41">
         <f>IF(A67&lt;=$B$9,$B$6*$B$11/100*D67,"")</f>
         <v/>
       </c>
-      <c r="G67" s="40">
+      <c r="G67" s="41">
         <f>IF(A67&lt;=$B$9,F67*E67,"")</f>
         <v/>
       </c>
-      <c r="H67" s="39">
+      <c r="H67" s="32">
         <f>IF(A67&lt;=$B$9,D67*E67,"")</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="38">
+      <c r="A68" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7806,25 +8754,25 @@
         <f>IF(A68&lt;=$B$9,(B68-C68)/360,"")</f>
         <v/>
       </c>
-      <c r="E68" s="34">
+      <c r="E68" s="33">
         <f>IF(A68&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B68,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B68,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B68,$K$6:$K$38,1)))^((B68-INDEX($K$6:$K$38,MATCH(B68,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B68,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B68,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B68,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F68" s="40">
+      <c r="F68" s="41">
         <f>IF(A68&lt;=$B$9,$B$6*$B$11/100*D68,"")</f>
         <v/>
       </c>
-      <c r="G68" s="40">
+      <c r="G68" s="41">
         <f>IF(A68&lt;=$B$9,F68*E68,"")</f>
         <v/>
       </c>
-      <c r="H68" s="39">
+      <c r="H68" s="32">
         <f>IF(A68&lt;=$B$9,D68*E68,"")</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="38">
+      <c r="A69" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7840,25 +8788,25 @@
         <f>IF(A69&lt;=$B$9,(B69-C69)/360,"")</f>
         <v/>
       </c>
-      <c r="E69" s="34">
+      <c r="E69" s="33">
         <f>IF(A69&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B69,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B69,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B69,$K$6:$K$38,1)))^((B69-INDEX($K$6:$K$38,MATCH(B69,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B69,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B69,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B69,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F69" s="40">
+      <c r="F69" s="41">
         <f>IF(A69&lt;=$B$9,$B$6*$B$11/100*D69,"")</f>
         <v/>
       </c>
-      <c r="G69" s="40">
+      <c r="G69" s="41">
         <f>IF(A69&lt;=$B$9,F69*E69,"")</f>
         <v/>
       </c>
-      <c r="H69" s="39">
+      <c r="H69" s="32">
         <f>IF(A69&lt;=$B$9,D69*E69,"")</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="38">
+      <c r="A70" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7874,25 +8822,25 @@
         <f>IF(A70&lt;=$B$9,(B70-C70)/360,"")</f>
         <v/>
       </c>
-      <c r="E70" s="34">
+      <c r="E70" s="33">
         <f>IF(A70&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B70,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B70,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B70,$K$6:$K$38,1)))^((B70-INDEX($K$6:$K$38,MATCH(B70,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B70,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B70,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B70,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F70" s="40">
+      <c r="F70" s="41">
         <f>IF(A70&lt;=$B$9,$B$6*$B$11/100*D70,"")</f>
         <v/>
       </c>
-      <c r="G70" s="40">
+      <c r="G70" s="41">
         <f>IF(A70&lt;=$B$9,F70*E70,"")</f>
         <v/>
       </c>
-      <c r="H70" s="39">
+      <c r="H70" s="32">
         <f>IF(A70&lt;=$B$9,D70*E70,"")</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="38">
+      <c r="A71" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7908,25 +8856,25 @@
         <f>IF(A71&lt;=$B$9,(B71-C71)/360,"")</f>
         <v/>
       </c>
-      <c r="E71" s="34">
+      <c r="E71" s="33">
         <f>IF(A71&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B71,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B71,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B71,$K$6:$K$38,1)))^((B71-INDEX($K$6:$K$38,MATCH(B71,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B71,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B71,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B71,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F71" s="40">
+      <c r="F71" s="41">
         <f>IF(A71&lt;=$B$9,$B$6*$B$11/100*D71,"")</f>
         <v/>
       </c>
-      <c r="G71" s="40">
+      <c r="G71" s="41">
         <f>IF(A71&lt;=$B$9,F71*E71,"")</f>
         <v/>
       </c>
-      <c r="H71" s="39">
+      <c r="H71" s="32">
         <f>IF(A71&lt;=$B$9,D71*E71,"")</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="38">
+      <c r="A72" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7942,25 +8890,25 @@
         <f>IF(A72&lt;=$B$9,(B72-C72)/360,"")</f>
         <v/>
       </c>
-      <c r="E72" s="34">
+      <c r="E72" s="33">
         <f>IF(A72&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B72,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B72,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B72,$K$6:$K$38,1)))^((B72-INDEX($K$6:$K$38,MATCH(B72,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B72,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B72,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B72,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F72" s="40">
+      <c r="F72" s="41">
         <f>IF(A72&lt;=$B$9,$B$6*$B$11/100*D72,"")</f>
         <v/>
       </c>
-      <c r="G72" s="40">
+      <c r="G72" s="41">
         <f>IF(A72&lt;=$B$9,F72*E72,"")</f>
         <v/>
       </c>
-      <c r="H72" s="39">
+      <c r="H72" s="32">
         <f>IF(A72&lt;=$B$9,D72*E72,"")</f>
         <v/>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="38">
+      <c r="A73" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -7976,25 +8924,25 @@
         <f>IF(A73&lt;=$B$9,(B73-C73)/360,"")</f>
         <v/>
       </c>
-      <c r="E73" s="34">
+      <c r="E73" s="33">
         <f>IF(A73&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B73,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B73,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B73,$K$6:$K$38,1)))^((B73-INDEX($K$6:$K$38,MATCH(B73,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B73,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B73,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B73,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F73" s="40">
+      <c r="F73" s="41">
         <f>IF(A73&lt;=$B$9,$B$6*$B$11/100*D73,"")</f>
         <v/>
       </c>
-      <c r="G73" s="40">
+      <c r="G73" s="41">
         <f>IF(A73&lt;=$B$9,F73*E73,"")</f>
         <v/>
       </c>
-      <c r="H73" s="39">
+      <c r="H73" s="32">
         <f>IF(A73&lt;=$B$9,D73*E73,"")</f>
         <v/>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="38">
+      <c r="A74" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -8010,25 +8958,25 @@
         <f>IF(A74&lt;=$B$9,(B74-C74)/360,"")</f>
         <v/>
       </c>
-      <c r="E74" s="34">
+      <c r="E74" s="33">
         <f>IF(A74&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B74,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B74,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B74,$K$6:$K$38,1)))^((B74-INDEX($K$6:$K$38,MATCH(B74,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B74,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B74,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B74,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F74" s="40">
+      <c r="F74" s="41">
         <f>IF(A74&lt;=$B$9,$B$6*$B$11/100*D74,"")</f>
         <v/>
       </c>
-      <c r="G74" s="40">
+      <c r="G74" s="41">
         <f>IF(A74&lt;=$B$9,F74*E74,"")</f>
         <v/>
       </c>
-      <c r="H74" s="39">
+      <c r="H74" s="32">
         <f>IF(A74&lt;=$B$9,D74*E74,"")</f>
         <v/>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="38">
+      <c r="A75" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -8044,25 +8992,25 @@
         <f>IF(A75&lt;=$B$9,(B75-C75)/360,"")</f>
         <v/>
       </c>
-      <c r="E75" s="34">
+      <c r="E75" s="33">
         <f>IF(A75&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B75,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B75,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B75,$K$6:$K$38,1)))^((B75-INDEX($K$6:$K$38,MATCH(B75,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B75,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B75,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B75,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F75" s="40">
+      <c r="F75" s="41">
         <f>IF(A75&lt;=$B$9,$B$6*$B$11/100*D75,"")</f>
         <v/>
       </c>
-      <c r="G75" s="40">
+      <c r="G75" s="41">
         <f>IF(A75&lt;=$B$9,F75*E75,"")</f>
         <v/>
       </c>
-      <c r="H75" s="39">
+      <c r="H75" s="32">
         <f>IF(A75&lt;=$B$9,D75*E75,"")</f>
         <v/>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="38">
+      <c r="A76" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -8078,25 +9026,25 @@
         <f>IF(A76&lt;=$B$9,(B76-C76)/360,"")</f>
         <v/>
       </c>
-      <c r="E76" s="34">
+      <c r="E76" s="33">
         <f>IF(A76&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B76,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B76,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B76,$K$6:$K$38,1)))^((B76-INDEX($K$6:$K$38,MATCH(B76,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B76,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B76,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B76,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F76" s="40">
+      <c r="F76" s="41">
         <f>IF(A76&lt;=$B$9,$B$6*$B$11/100*D76,"")</f>
         <v/>
       </c>
-      <c r="G76" s="40">
+      <c r="G76" s="41">
         <f>IF(A76&lt;=$B$9,F76*E76,"")</f>
         <v/>
       </c>
-      <c r="H76" s="39">
+      <c r="H76" s="32">
         <f>IF(A76&lt;=$B$9,D76*E76,"")</f>
         <v/>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="38">
+      <c r="A77" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -8112,25 +9060,25 @@
         <f>IF(A77&lt;=$B$9,(B77-C77)/360,"")</f>
         <v/>
       </c>
-      <c r="E77" s="34">
+      <c r="E77" s="33">
         <f>IF(A77&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B77,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B77,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B77,$K$6:$K$38,1)))^((B77-INDEX($K$6:$K$38,MATCH(B77,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B77,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B77,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B77,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F77" s="40">
+      <c r="F77" s="41">
         <f>IF(A77&lt;=$B$9,$B$6*$B$11/100*D77,"")</f>
         <v/>
       </c>
-      <c r="G77" s="40">
+      <c r="G77" s="41">
         <f>IF(A77&lt;=$B$9,F77*E77,"")</f>
         <v/>
       </c>
-      <c r="H77" s="39">
+      <c r="H77" s="32">
         <f>IF(A77&lt;=$B$9,D77*E77,"")</f>
         <v/>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="38">
+      <c r="A78" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -8146,25 +9094,25 @@
         <f>IF(A78&lt;=$B$9,(B78-C78)/360,"")</f>
         <v/>
       </c>
-      <c r="E78" s="34">
+      <c r="E78" s="33">
         <f>IF(A78&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B78,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B78,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B78,$K$6:$K$38,1)))^((B78-INDEX($K$6:$K$38,MATCH(B78,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B78,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B78,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B78,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F78" s="40">
+      <c r="F78" s="41">
         <f>IF(A78&lt;=$B$9,$B$6*$B$11/100*D78,"")</f>
         <v/>
       </c>
-      <c r="G78" s="40">
+      <c r="G78" s="41">
         <f>IF(A78&lt;=$B$9,F78*E78,"")</f>
         <v/>
       </c>
-      <c r="H78" s="39">
+      <c r="H78" s="32">
         <f>IF(A78&lt;=$B$9,D78*E78,"")</f>
         <v/>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="38">
+      <c r="A79" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -8180,25 +9128,25 @@
         <f>IF(A79&lt;=$B$9,(B79-C79)/360,"")</f>
         <v/>
       </c>
-      <c r="E79" s="34">
+      <c r="E79" s="33">
         <f>IF(A79&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B79,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B79,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B79,$K$6:$K$38,1)))^((B79-INDEX($K$6:$K$38,MATCH(B79,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B79,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B79,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B79,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F79" s="40">
+      <c r="F79" s="41">
         <f>IF(A79&lt;=$B$9,$B$6*$B$11/100*D79,"")</f>
         <v/>
       </c>
-      <c r="G79" s="40">
+      <c r="G79" s="41">
         <f>IF(A79&lt;=$B$9,F79*E79,"")</f>
         <v/>
       </c>
-      <c r="H79" s="39">
+      <c r="H79" s="32">
         <f>IF(A79&lt;=$B$9,D79*E79,"")</f>
         <v/>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="38">
+      <c r="A80" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -8214,25 +9162,25 @@
         <f>IF(A80&lt;=$B$9,(B80-C80)/360,"")</f>
         <v/>
       </c>
-      <c r="E80" s="34">
+      <c r="E80" s="33">
         <f>IF(A80&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B80,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B80,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B80,$K$6:$K$38,1)))^((B80-INDEX($K$6:$K$38,MATCH(B80,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B80,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B80,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B80,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F80" s="40">
+      <c r="F80" s="41">
         <f>IF(A80&lt;=$B$9,$B$6*$B$11/100*D80,"")</f>
         <v/>
       </c>
-      <c r="G80" s="40">
+      <c r="G80" s="41">
         <f>IF(A80&lt;=$B$9,F80*E80,"")</f>
         <v/>
       </c>
-      <c r="H80" s="39">
+      <c r="H80" s="32">
         <f>IF(A80&lt;=$B$9,D80*E80,"")</f>
         <v/>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="38">
+      <c r="A81" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -8248,25 +9196,25 @@
         <f>IF(A81&lt;=$B$9,(B81-C81)/360,"")</f>
         <v/>
       </c>
-      <c r="E81" s="34">
+      <c r="E81" s="33">
         <f>IF(A81&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B81,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B81,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B81,$K$6:$K$38,1)))^((B81-INDEX($K$6:$K$38,MATCH(B81,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B81,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B81,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B81,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F81" s="40">
+      <c r="F81" s="41">
         <f>IF(A81&lt;=$B$9,$B$6*$B$11/100*D81,"")</f>
         <v/>
       </c>
-      <c r="G81" s="40">
+      <c r="G81" s="41">
         <f>IF(A81&lt;=$B$9,F81*E81,"")</f>
         <v/>
       </c>
-      <c r="H81" s="39">
+      <c r="H81" s="32">
         <f>IF(A81&lt;=$B$9,D81*E81,"")</f>
         <v/>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="38">
+      <c r="A82" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -8282,25 +9230,25 @@
         <f>IF(A82&lt;=$B$9,(B82-C82)/360,"")</f>
         <v/>
       </c>
-      <c r="E82" s="34">
+      <c r="E82" s="33">
         <f>IF(A82&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B82,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B82,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B82,$K$6:$K$38,1)))^((B82-INDEX($K$6:$K$38,MATCH(B82,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B82,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B82,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B82,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F82" s="40">
+      <c r="F82" s="41">
         <f>IF(A82&lt;=$B$9,$B$6*$B$11/100*D82,"")</f>
         <v/>
       </c>
-      <c r="G82" s="40">
+      <c r="G82" s="41">
         <f>IF(A82&lt;=$B$9,F82*E82,"")</f>
         <v/>
       </c>
-      <c r="H82" s="39">
+      <c r="H82" s="32">
         <f>IF(A82&lt;=$B$9,D82*E82,"")</f>
         <v/>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="38">
+      <c r="A83" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -8316,25 +9264,25 @@
         <f>IF(A83&lt;=$B$9,(B83-C83)/360,"")</f>
         <v/>
       </c>
-      <c r="E83" s="34">
+      <c r="E83" s="33">
         <f>IF(A83&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B83,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B83,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B83,$K$6:$K$38,1)))^((B83-INDEX($K$6:$K$38,MATCH(B83,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B83,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B83,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B83,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F83" s="40">
+      <c r="F83" s="41">
         <f>IF(A83&lt;=$B$9,$B$6*$B$11/100*D83,"")</f>
         <v/>
       </c>
-      <c r="G83" s="40">
+      <c r="G83" s="41">
         <f>IF(A83&lt;=$B$9,F83*E83,"")</f>
         <v/>
       </c>
-      <c r="H83" s="39">
+      <c r="H83" s="32">
         <f>IF(A83&lt;=$B$9,D83*E83,"")</f>
         <v/>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="38">
+      <c r="A84" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -8350,25 +9298,25 @@
         <f>IF(A84&lt;=$B$9,(B84-C84)/360,"")</f>
         <v/>
       </c>
-      <c r="E84" s="34">
+      <c r="E84" s="33">
         <f>IF(A84&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B84,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B84,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B84,$K$6:$K$38,1)))^((B84-INDEX($K$6:$K$38,MATCH(B84,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B84,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B84,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B84,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F84" s="40">
+      <c r="F84" s="41">
         <f>IF(A84&lt;=$B$9,$B$6*$B$11/100*D84,"")</f>
         <v/>
       </c>
-      <c r="G84" s="40">
+      <c r="G84" s="41">
         <f>IF(A84&lt;=$B$9,F84*E84,"")</f>
         <v/>
       </c>
-      <c r="H84" s="39">
+      <c r="H84" s="32">
         <f>IF(A84&lt;=$B$9,D84*E84,"")</f>
         <v/>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="38">
+      <c r="A85" s="40">
         <f>ROW()-35</f>
         <v/>
       </c>
@@ -8384,19 +9332,19 @@
         <f>IF(A85&lt;=$B$9,(B85-C85)/360,"")</f>
         <v/>
       </c>
-      <c r="E85" s="34">
+      <c r="E85" s="33">
         <f>IF(A85&lt;=$B$9,IFERROR(INDEX($L$6:$L$38,MATCH(B85,$K$6:$K$38,1))*(INDEX($L$6:$L$38,MATCH(B85,$K$6:$K$38,1)+1)/INDEX($L$6:$L$38,MATCH(B85,$K$6:$K$38,1)))^((B85-INDEX($K$6:$K$38,MATCH(B85,$K$6:$K$38,1)))/(INDEX($K$6:$K$38,MATCH(B85,$K$6:$K$38,1)+1)-INDEX($K$6:$K$38,MATCH(B85,$K$6:$K$38,1)))),INDEX($L$6:$L$38,MATCH(B85,$K$6:$K$38,1))),"")</f>
         <v/>
       </c>
-      <c r="F85" s="40">
+      <c r="F85" s="41">
         <f>IF(A85&lt;=$B$9,$B$6*$B$11/100*D85,"")</f>
         <v/>
       </c>
-      <c r="G85" s="40">
+      <c r="G85" s="41">
         <f>IF(A85&lt;=$B$9,F85*E85,"")</f>
         <v/>
       </c>
-      <c r="H85" s="39">
+      <c r="H85" s="32">
         <f>IF(A85&lt;=$B$9,D85*E85,"")</f>
         <v/>
       </c>
@@ -8477,7 +9425,7 @@
           <t>Curve date</t>
         </is>
       </c>
-      <c r="B5" s="42">
+      <c r="B5" s="43">
         <f>VAL_DATE</f>
         <v/>
       </c>
@@ -9418,7 +10366,7 @@
           <t>Reference index</t>
         </is>
       </c>
-      <c r="B22" s="43" t="inlineStr">
+      <c r="B22" s="44" t="inlineStr">
         <is>
           <t>USD-SOFR (compounded in arrears)</t>
         </is>
@@ -9434,7 +10382,7 @@
           <t>Spot / settlement lag</t>
         </is>
       </c>
-      <c r="B23" s="43" t="inlineStr">
+      <c r="B23" s="44" t="inlineStr">
         <is>
           <t>T+2 US business days</t>
         </is>
@@ -9450,7 +10398,7 @@
           <t>Effective date rule</t>
         </is>
       </c>
-      <c r="B24" s="43" t="inlineStr">
+      <c r="B24" s="44" t="inlineStr">
         <is>
           <t>Spot (T+2), modified following</t>
         </is>
@@ -9466,7 +10414,7 @@
           <t>Maturity date rule</t>
         </is>
       </c>
-      <c r="B25" s="43" t="inlineStr">
+      <c r="B25" s="44" t="inlineStr">
         <is>
           <t>Effective + tenor, modified following</t>
         </is>
@@ -9482,7 +10430,7 @@
           <t>Business-day convention</t>
         </is>
       </c>
-      <c r="B26" s="43" t="inlineStr">
+      <c r="B26" s="44" t="inlineStr">
         <is>
           <t>Modified Following</t>
         </is>
@@ -9498,7 +10446,7 @@
           <t>Fixed-leg day count</t>
         </is>
       </c>
-      <c r="B27" s="43" t="inlineStr">
+      <c r="B27" s="44" t="inlineStr">
         <is>
           <t>ACT/360</t>
         </is>
@@ -9514,7 +10462,7 @@
           <t>Fixed-leg pay frequency</t>
         </is>
       </c>
-      <c r="B28" s="43" t="inlineStr">
+      <c r="B28" s="44" t="inlineStr">
         <is>
           <t>Annual  (single payment if tenor ≤ 1Y)</t>
         </is>
@@ -9530,7 +10478,7 @@
           <t>Floating-leg day count</t>
         </is>
       </c>
-      <c r="B29" s="43" t="inlineStr">
+      <c r="B29" s="44" t="inlineStr">
         <is>
           <t>ACT/360</t>
         </is>
@@ -9546,7 +10494,7 @@
           <t>Floating-leg pay frequency</t>
         </is>
       </c>
-      <c r="B30" s="43" t="inlineStr">
+      <c r="B30" s="44" t="inlineStr">
         <is>
           <t>Annual  (single payment if tenor ≤ 1Y)</t>
         </is>
@@ -9562,7 +10510,7 @@
           <t>SOFR compounding method</t>
         </is>
       </c>
-      <c r="B31" s="43" t="inlineStr">
+      <c r="B31" s="44" t="inlineStr">
         <is>
           <t>Daily compounded, ACT/360</t>
         </is>
@@ -9578,7 +10526,7 @@
           <t>Payment lag</t>
         </is>
       </c>
-      <c r="B32" s="43" t="inlineStr">
+      <c r="B32" s="44" t="inlineStr">
         <is>
           <t>2 US business days</t>
         </is>
@@ -9594,7 +10542,7 @@
           <t>Observation shift / lookback</t>
         </is>
       </c>
-      <c r="B33" s="43" t="inlineStr">
+      <c r="B33" s="44" t="inlineStr">
         <is>
           <t>None (payment-delay convention, 2 bd)</t>
         </is>
@@ -9610,7 +10558,7 @@
           <t>End-of-month treatment</t>
         </is>
       </c>
-      <c r="B34" s="43" t="inlineStr">
+      <c r="B34" s="44" t="inlineStr">
         <is>
           <t>EOM applies</t>
         </is>

</xml_diff>

<commit_message>
Add Fwd_Interp tab: Zhou 2002 forward interpolation (V1 flat, V2 quadratic)
Both variants reprice the bootstrapped pillar DFs identically (shared segment
integral). V1 = piecewise-flat instantaneous forward (step curve, Lehman's
default). V2 = piecewise-quadratic f(x)=a+bx+cx², continuous across pillars via
a shared node forward, still exact-repricing. Key insight: because the bootstrap
already fixes each segment integral, a/b/c are CLOSED-FORM from (f_left, f_right,
integral) — no solver, so it works in cell formulas. reprice-check column
(quad integral - segment integral ~ 0) proves DFs preserved. Validated: closed
form reproduces integrals to machine precision; whole workbook compiles clean.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Swap_Pricer" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloomberg_S490_Validation" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conventions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fwd_Interp" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="VAL_DATE">Instructions!$B$9</definedName>
@@ -30,12 +31,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.00000000"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="0.000000"/>
+    <numFmt numFmtId="169" formatCode="0.0000%"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -130,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -200,6 +202,11 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -565,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1032,44 +1039,56 @@
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="15" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>7. Fwd_Interp</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Zhou 2002 forward interpolation: V1 piecewise-flat vs V2 piecewise-quadratic forwards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>DO NOT substitute these (wrong instruments):</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="9" t="inlineStr">
-        <is>
-          <t>•  TSFR1M/3M/6M/12M Index  — Term SOFR benchmarks, NOT overnight-SOFR OIS calibration instruments.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>•  USISSO02/05/10/30 Index — ICE Swap Rate fixings, NOT the live OIS quote strip needed to bootstrap.</t>
+          <t>•  TSFR1M/3M/6M/12M Index  — Term SOFR benchmarks, NOT overnight-SOFR OIS calibration instruments.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
+          <t>•  USISSO02/05/10/30 Index — ICE Swap Rate fixings, NOT the live OIS quote strip needed to bootstrap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
           <t>•  Use PX midpoint (bid+ask)/2 for construction; use PX_LAST only where bid/ask are unavailable.</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="28" customHeight="1">
-      <c r="A48" s="9" t="inlineStr">
+    <row r="49" ht="28" customHeight="1">
+      <c r="A49" s="9" t="inlineStr">
         <is>
           <t>Licensing: Bloomberg data is licensed and entitlement-dependent — do NOT redistribute pulled values or commit them to a public repository. This template ships formulas only, no data. Some static convention fields may return N/A under your entitlement; use FLDS &lt;GO&gt; on the security to find the enabled mnemonic.</t>
         </is>
       </c>
     </row>
-    <row r="49"/>
+    <row r="50"/>
   </sheetData>
-  <mergeCells count="49">
+  <mergeCells count="50">
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="D13:F13"/>
@@ -1081,7 +1100,9 @@
     <mergeCell ref="A33:F33"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="B39:F39"/>
-    <mergeCell ref="A48:F49"/>
+    <mergeCell ref="A47:F47"/>
+    <mergeCell ref="A49:F50"/>
+    <mergeCell ref="B42:F42"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="D12:F12"/>
@@ -1090,7 +1111,6 @@
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="D8:F8"/>
-    <mergeCell ref="A43:F43"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="C21:D21"/>
@@ -10596,4 +10616,1737 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Fwd_Interp</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Zhou 2002 forward interpolation — V1 piecewise-flat vs V2 piecewise-quadratic instantaneous forwards</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="70" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Both variants reprice the pillar DFs IDENTICALLY (same segment integral ∫f = −ln(DF_i/DF_(i-1))). V1 (Flat fwd) holds the instantaneous forward CONSTANT over each segment → a step curve; simplest &amp; most stable — Lehman's default. V2 makes the forward piecewise-QUADRATIC f(x)=a+bx+cx², CONTINUOUS across pillars (adjacent segments share the Node fwd) while still repricing exactly. a,b,c are closed-form from (f_left=node at left pillar, f_right=node at right pillar, ∫f) — no solver needed. Node fwd = average of the two adjacent flat forwards. 'reprice check' = ∫quad − ∫f ≈ 0 confirms V2 preserves every DF. The difference is intra-segment: compare Flat fwd (V1) vs V2 fwd @ mid — largest across the wide long-end gaps (10Y→15Y→20Y→30Y), which is exactly what V2 smooths.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>Pillar</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>T (yrs)</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Δ (yrs)</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>∫f (integral)</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>Flat fwd (V1)</t>
+        </is>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>Node fwd</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="I7" s="19" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="J7" s="19" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="K7" s="19" t="inlineStr">
+        <is>
+          <t>V2 fwd @ mid</t>
+        </is>
+      </c>
+      <c r="L7" s="19" t="inlineStr">
+        <is>
+          <t>reprice check</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Spot</t>
+        </is>
+      </c>
+      <c r="B8" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="47">
+        <f>F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6">
+        <f>'Bootstrap'!A8</f>
+        <v/>
+      </c>
+      <c r="B9" s="27">
+        <f>'Bootstrap'!C8</f>
+        <v/>
+      </c>
+      <c r="C9" s="33">
+        <f>'Bootstrap'!H8</f>
+        <v/>
+      </c>
+      <c r="D9" s="27">
+        <f>B9-B8</f>
+        <v/>
+      </c>
+      <c r="E9" s="32">
+        <f>-LN(C9/C8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="48">
+        <f>E9/D9</f>
+        <v/>
+      </c>
+      <c r="G9" s="48">
+        <f>(F9+F10)/2</f>
+        <v/>
+      </c>
+      <c r="H9" s="48">
+        <f>G8</f>
+        <v/>
+      </c>
+      <c r="I9" s="32">
+        <f>(G9-G8)/D9-J9*D9</f>
+        <v/>
+      </c>
+      <c r="J9" s="32">
+        <f>3*(G9-G8)/D9^2-6*(E9-G8*D9)/D9^3</f>
+        <v/>
+      </c>
+      <c r="K9" s="48">
+        <f>H9+I9*D9/2+J9*D9^2/4</f>
+        <v/>
+      </c>
+      <c r="L9" s="49">
+        <f>H9*D9+I9*D9^2/2+J9*D9^3/3-E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6">
+        <f>'Bootstrap'!A9</f>
+        <v/>
+      </c>
+      <c r="B10" s="27">
+        <f>'Bootstrap'!C9</f>
+        <v/>
+      </c>
+      <c r="C10" s="33">
+        <f>'Bootstrap'!H9</f>
+        <v/>
+      </c>
+      <c r="D10" s="27">
+        <f>B10-B9</f>
+        <v/>
+      </c>
+      <c r="E10" s="32">
+        <f>-LN(C10/C9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="48">
+        <f>E10/D10</f>
+        <v/>
+      </c>
+      <c r="G10" s="48">
+        <f>(F10+F11)/2</f>
+        <v/>
+      </c>
+      <c r="H10" s="48">
+        <f>G9</f>
+        <v/>
+      </c>
+      <c r="I10" s="32">
+        <f>(G10-G9)/D10-J10*D10</f>
+        <v/>
+      </c>
+      <c r="J10" s="32">
+        <f>3*(G10-G9)/D10^2-6*(E10-G9*D10)/D10^3</f>
+        <v/>
+      </c>
+      <c r="K10" s="48">
+        <f>H10+I10*D10/2+J10*D10^2/4</f>
+        <v/>
+      </c>
+      <c r="L10" s="49">
+        <f>H10*D10+I10*D10^2/2+J10*D10^3/3-E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6">
+        <f>'Bootstrap'!A10</f>
+        <v/>
+      </c>
+      <c r="B11" s="27">
+        <f>'Bootstrap'!C10</f>
+        <v/>
+      </c>
+      <c r="C11" s="33">
+        <f>'Bootstrap'!H10</f>
+        <v/>
+      </c>
+      <c r="D11" s="27">
+        <f>B11-B10</f>
+        <v/>
+      </c>
+      <c r="E11" s="32">
+        <f>-LN(C11/C10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="48">
+        <f>E11/D11</f>
+        <v/>
+      </c>
+      <c r="G11" s="48">
+        <f>(F11+F12)/2</f>
+        <v/>
+      </c>
+      <c r="H11" s="48">
+        <f>G10</f>
+        <v/>
+      </c>
+      <c r="I11" s="32">
+        <f>(G11-G10)/D11-J11*D11</f>
+        <v/>
+      </c>
+      <c r="J11" s="32">
+        <f>3*(G11-G10)/D11^2-6*(E11-G10*D11)/D11^3</f>
+        <v/>
+      </c>
+      <c r="K11" s="48">
+        <f>H11+I11*D11/2+J11*D11^2/4</f>
+        <v/>
+      </c>
+      <c r="L11" s="49">
+        <f>H11*D11+I11*D11^2/2+J11*D11^3/3-E11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6">
+        <f>'Bootstrap'!A11</f>
+        <v/>
+      </c>
+      <c r="B12" s="27">
+        <f>'Bootstrap'!C11</f>
+        <v/>
+      </c>
+      <c r="C12" s="33">
+        <f>'Bootstrap'!H11</f>
+        <v/>
+      </c>
+      <c r="D12" s="27">
+        <f>B12-B11</f>
+        <v/>
+      </c>
+      <c r="E12" s="32">
+        <f>-LN(C12/C11)</f>
+        <v/>
+      </c>
+      <c r="F12" s="48">
+        <f>E12/D12</f>
+        <v/>
+      </c>
+      <c r="G12" s="48">
+        <f>(F12+F13)/2</f>
+        <v/>
+      </c>
+      <c r="H12" s="48">
+        <f>G11</f>
+        <v/>
+      </c>
+      <c r="I12" s="32">
+        <f>(G12-G11)/D12-J12*D12</f>
+        <v/>
+      </c>
+      <c r="J12" s="32">
+        <f>3*(G12-G11)/D12^2-6*(E12-G11*D12)/D12^3</f>
+        <v/>
+      </c>
+      <c r="K12" s="48">
+        <f>H12+I12*D12/2+J12*D12^2/4</f>
+        <v/>
+      </c>
+      <c r="L12" s="49">
+        <f>H12*D12+I12*D12^2/2+J12*D12^3/3-E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6">
+        <f>'Bootstrap'!A12</f>
+        <v/>
+      </c>
+      <c r="B13" s="27">
+        <f>'Bootstrap'!C12</f>
+        <v/>
+      </c>
+      <c r="C13" s="33">
+        <f>'Bootstrap'!H12</f>
+        <v/>
+      </c>
+      <c r="D13" s="27">
+        <f>B13-B12</f>
+        <v/>
+      </c>
+      <c r="E13" s="32">
+        <f>-LN(C13/C12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="48">
+        <f>E13/D13</f>
+        <v/>
+      </c>
+      <c r="G13" s="48">
+        <f>(F13+F14)/2</f>
+        <v/>
+      </c>
+      <c r="H13" s="48">
+        <f>G12</f>
+        <v/>
+      </c>
+      <c r="I13" s="32">
+        <f>(G13-G12)/D13-J13*D13</f>
+        <v/>
+      </c>
+      <c r="J13" s="32">
+        <f>3*(G13-G12)/D13^2-6*(E13-G12*D13)/D13^3</f>
+        <v/>
+      </c>
+      <c r="K13" s="48">
+        <f>H13+I13*D13/2+J13*D13^2/4</f>
+        <v/>
+      </c>
+      <c r="L13" s="49">
+        <f>H13*D13+I13*D13^2/2+J13*D13^3/3-E13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6">
+        <f>'Bootstrap'!A13</f>
+        <v/>
+      </c>
+      <c r="B14" s="27">
+        <f>'Bootstrap'!C13</f>
+        <v/>
+      </c>
+      <c r="C14" s="33">
+        <f>'Bootstrap'!H13</f>
+        <v/>
+      </c>
+      <c r="D14" s="27">
+        <f>B14-B13</f>
+        <v/>
+      </c>
+      <c r="E14" s="32">
+        <f>-LN(C14/C13)</f>
+        <v/>
+      </c>
+      <c r="F14" s="48">
+        <f>E14/D14</f>
+        <v/>
+      </c>
+      <c r="G14" s="48">
+        <f>(F14+F15)/2</f>
+        <v/>
+      </c>
+      <c r="H14" s="48">
+        <f>G13</f>
+        <v/>
+      </c>
+      <c r="I14" s="32">
+        <f>(G14-G13)/D14-J14*D14</f>
+        <v/>
+      </c>
+      <c r="J14" s="32">
+        <f>3*(G14-G13)/D14^2-6*(E14-G13*D14)/D14^3</f>
+        <v/>
+      </c>
+      <c r="K14" s="48">
+        <f>H14+I14*D14/2+J14*D14^2/4</f>
+        <v/>
+      </c>
+      <c r="L14" s="49">
+        <f>H14*D14+I14*D14^2/2+J14*D14^3/3-E14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6">
+        <f>'Bootstrap'!A14</f>
+        <v/>
+      </c>
+      <c r="B15" s="27">
+        <f>'Bootstrap'!C14</f>
+        <v/>
+      </c>
+      <c r="C15" s="33">
+        <f>'Bootstrap'!H14</f>
+        <v/>
+      </c>
+      <c r="D15" s="27">
+        <f>B15-B14</f>
+        <v/>
+      </c>
+      <c r="E15" s="32">
+        <f>-LN(C15/C14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="48">
+        <f>E15/D15</f>
+        <v/>
+      </c>
+      <c r="G15" s="48">
+        <f>(F15+F16)/2</f>
+        <v/>
+      </c>
+      <c r="H15" s="48">
+        <f>G14</f>
+        <v/>
+      </c>
+      <c r="I15" s="32">
+        <f>(G15-G14)/D15-J15*D15</f>
+        <v/>
+      </c>
+      <c r="J15" s="32">
+        <f>3*(G15-G14)/D15^2-6*(E15-G14*D15)/D15^3</f>
+        <v/>
+      </c>
+      <c r="K15" s="48">
+        <f>H15+I15*D15/2+J15*D15^2/4</f>
+        <v/>
+      </c>
+      <c r="L15" s="49">
+        <f>H15*D15+I15*D15^2/2+J15*D15^3/3-E15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6">
+        <f>'Bootstrap'!A15</f>
+        <v/>
+      </c>
+      <c r="B16" s="27">
+        <f>'Bootstrap'!C15</f>
+        <v/>
+      </c>
+      <c r="C16" s="33">
+        <f>'Bootstrap'!H15</f>
+        <v/>
+      </c>
+      <c r="D16" s="27">
+        <f>B16-B15</f>
+        <v/>
+      </c>
+      <c r="E16" s="32">
+        <f>-LN(C16/C15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="48">
+        <f>E16/D16</f>
+        <v/>
+      </c>
+      <c r="G16" s="48">
+        <f>(F16+F17)/2</f>
+        <v/>
+      </c>
+      <c r="H16" s="48">
+        <f>G15</f>
+        <v/>
+      </c>
+      <c r="I16" s="32">
+        <f>(G16-G15)/D16-J16*D16</f>
+        <v/>
+      </c>
+      <c r="J16" s="32">
+        <f>3*(G16-G15)/D16^2-6*(E16-G15*D16)/D16^3</f>
+        <v/>
+      </c>
+      <c r="K16" s="48">
+        <f>H16+I16*D16/2+J16*D16^2/4</f>
+        <v/>
+      </c>
+      <c r="L16" s="49">
+        <f>H16*D16+I16*D16^2/2+J16*D16^3/3-E16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6">
+        <f>'Bootstrap'!A16</f>
+        <v/>
+      </c>
+      <c r="B17" s="27">
+        <f>'Bootstrap'!C16</f>
+        <v/>
+      </c>
+      <c r="C17" s="33">
+        <f>'Bootstrap'!H16</f>
+        <v/>
+      </c>
+      <c r="D17" s="27">
+        <f>B17-B16</f>
+        <v/>
+      </c>
+      <c r="E17" s="32">
+        <f>-LN(C17/C16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="48">
+        <f>E17/D17</f>
+        <v/>
+      </c>
+      <c r="G17" s="48">
+        <f>(F17+F18)/2</f>
+        <v/>
+      </c>
+      <c r="H17" s="48">
+        <f>G16</f>
+        <v/>
+      </c>
+      <c r="I17" s="32">
+        <f>(G17-G16)/D17-J17*D17</f>
+        <v/>
+      </c>
+      <c r="J17" s="32">
+        <f>3*(G17-G16)/D17^2-6*(E17-G16*D17)/D17^3</f>
+        <v/>
+      </c>
+      <c r="K17" s="48">
+        <f>H17+I17*D17/2+J17*D17^2/4</f>
+        <v/>
+      </c>
+      <c r="L17" s="49">
+        <f>H17*D17+I17*D17^2/2+J17*D17^3/3-E17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6">
+        <f>'Bootstrap'!A17</f>
+        <v/>
+      </c>
+      <c r="B18" s="27">
+        <f>'Bootstrap'!C17</f>
+        <v/>
+      </c>
+      <c r="C18" s="33">
+        <f>'Bootstrap'!H17</f>
+        <v/>
+      </c>
+      <c r="D18" s="27">
+        <f>B18-B17</f>
+        <v/>
+      </c>
+      <c r="E18" s="32">
+        <f>-LN(C18/C17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="48">
+        <f>E18/D18</f>
+        <v/>
+      </c>
+      <c r="G18" s="48">
+        <f>(F18+F19)/2</f>
+        <v/>
+      </c>
+      <c r="H18" s="48">
+        <f>G17</f>
+        <v/>
+      </c>
+      <c r="I18" s="32">
+        <f>(G18-G17)/D18-J18*D18</f>
+        <v/>
+      </c>
+      <c r="J18" s="32">
+        <f>3*(G18-G17)/D18^2-6*(E18-G17*D18)/D18^3</f>
+        <v/>
+      </c>
+      <c r="K18" s="48">
+        <f>H18+I18*D18/2+J18*D18^2/4</f>
+        <v/>
+      </c>
+      <c r="L18" s="49">
+        <f>H18*D18+I18*D18^2/2+J18*D18^3/3-E18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6">
+        <f>'Bootstrap'!A18</f>
+        <v/>
+      </c>
+      <c r="B19" s="27">
+        <f>'Bootstrap'!C18</f>
+        <v/>
+      </c>
+      <c r="C19" s="33">
+        <f>'Bootstrap'!H18</f>
+        <v/>
+      </c>
+      <c r="D19" s="27">
+        <f>B19-B18</f>
+        <v/>
+      </c>
+      <c r="E19" s="32">
+        <f>-LN(C19/C18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="48">
+        <f>E19/D19</f>
+        <v/>
+      </c>
+      <c r="G19" s="48">
+        <f>(F19+F20)/2</f>
+        <v/>
+      </c>
+      <c r="H19" s="48">
+        <f>G18</f>
+        <v/>
+      </c>
+      <c r="I19" s="32">
+        <f>(G19-G18)/D19-J19*D19</f>
+        <v/>
+      </c>
+      <c r="J19" s="32">
+        <f>3*(G19-G18)/D19^2-6*(E19-G18*D19)/D19^3</f>
+        <v/>
+      </c>
+      <c r="K19" s="48">
+        <f>H19+I19*D19/2+J19*D19^2/4</f>
+        <v/>
+      </c>
+      <c r="L19" s="49">
+        <f>H19*D19+I19*D19^2/2+J19*D19^3/3-E19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6">
+        <f>'Bootstrap'!A19</f>
+        <v/>
+      </c>
+      <c r="B20" s="27">
+        <f>'Bootstrap'!C19</f>
+        <v/>
+      </c>
+      <c r="C20" s="33">
+        <f>'Bootstrap'!H19</f>
+        <v/>
+      </c>
+      <c r="D20" s="27">
+        <f>B20-B19</f>
+        <v/>
+      </c>
+      <c r="E20" s="32">
+        <f>-LN(C20/C19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="48">
+        <f>E20/D20</f>
+        <v/>
+      </c>
+      <c r="G20" s="48">
+        <f>(F20+F21)/2</f>
+        <v/>
+      </c>
+      <c r="H20" s="48">
+        <f>G19</f>
+        <v/>
+      </c>
+      <c r="I20" s="32">
+        <f>(G20-G19)/D20-J20*D20</f>
+        <v/>
+      </c>
+      <c r="J20" s="32">
+        <f>3*(G20-G19)/D20^2-6*(E20-G19*D20)/D20^3</f>
+        <v/>
+      </c>
+      <c r="K20" s="48">
+        <f>H20+I20*D20/2+J20*D20^2/4</f>
+        <v/>
+      </c>
+      <c r="L20" s="49">
+        <f>H20*D20+I20*D20^2/2+J20*D20^3/3-E20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6">
+        <f>'Bootstrap'!A20</f>
+        <v/>
+      </c>
+      <c r="B21" s="27">
+        <f>'Bootstrap'!C20</f>
+        <v/>
+      </c>
+      <c r="C21" s="33">
+        <f>'Bootstrap'!H20</f>
+        <v/>
+      </c>
+      <c r="D21" s="27">
+        <f>B21-B20</f>
+        <v/>
+      </c>
+      <c r="E21" s="32">
+        <f>-LN(C21/C20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="48">
+        <f>E21/D21</f>
+        <v/>
+      </c>
+      <c r="G21" s="48">
+        <f>(F21+F22)/2</f>
+        <v/>
+      </c>
+      <c r="H21" s="48">
+        <f>G20</f>
+        <v/>
+      </c>
+      <c r="I21" s="32">
+        <f>(G21-G20)/D21-J21*D21</f>
+        <v/>
+      </c>
+      <c r="J21" s="32">
+        <f>3*(G21-G20)/D21^2-6*(E21-G20*D21)/D21^3</f>
+        <v/>
+      </c>
+      <c r="K21" s="48">
+        <f>H21+I21*D21/2+J21*D21^2/4</f>
+        <v/>
+      </c>
+      <c r="L21" s="49">
+        <f>H21*D21+I21*D21^2/2+J21*D21^3/3-E21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6">
+        <f>'Bootstrap'!A21</f>
+        <v/>
+      </c>
+      <c r="B22" s="27">
+        <f>'Bootstrap'!C21</f>
+        <v/>
+      </c>
+      <c r="C22" s="33">
+        <f>'Bootstrap'!H21</f>
+        <v/>
+      </c>
+      <c r="D22" s="27">
+        <f>B22-B21</f>
+        <v/>
+      </c>
+      <c r="E22" s="32">
+        <f>-LN(C22/C21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="48">
+        <f>E22/D22</f>
+        <v/>
+      </c>
+      <c r="G22" s="48">
+        <f>(F22+F23)/2</f>
+        <v/>
+      </c>
+      <c r="H22" s="48">
+        <f>G21</f>
+        <v/>
+      </c>
+      <c r="I22" s="32">
+        <f>(G22-G21)/D22-J22*D22</f>
+        <v/>
+      </c>
+      <c r="J22" s="32">
+        <f>3*(G22-G21)/D22^2-6*(E22-G21*D22)/D22^3</f>
+        <v/>
+      </c>
+      <c r="K22" s="48">
+        <f>H22+I22*D22/2+J22*D22^2/4</f>
+        <v/>
+      </c>
+      <c r="L22" s="49">
+        <f>H22*D22+I22*D22^2/2+J22*D22^3/3-E22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6">
+        <f>'Bootstrap'!A22</f>
+        <v/>
+      </c>
+      <c r="B23" s="27">
+        <f>'Bootstrap'!C22</f>
+        <v/>
+      </c>
+      <c r="C23" s="33">
+        <f>'Bootstrap'!H22</f>
+        <v/>
+      </c>
+      <c r="D23" s="27">
+        <f>B23-B22</f>
+        <v/>
+      </c>
+      <c r="E23" s="32">
+        <f>-LN(C23/C22)</f>
+        <v/>
+      </c>
+      <c r="F23" s="48">
+        <f>E23/D23</f>
+        <v/>
+      </c>
+      <c r="G23" s="48">
+        <f>(F23+F24)/2</f>
+        <v/>
+      </c>
+      <c r="H23" s="48">
+        <f>G22</f>
+        <v/>
+      </c>
+      <c r="I23" s="32">
+        <f>(G23-G22)/D23-J23*D23</f>
+        <v/>
+      </c>
+      <c r="J23" s="32">
+        <f>3*(G23-G22)/D23^2-6*(E23-G22*D23)/D23^3</f>
+        <v/>
+      </c>
+      <c r="K23" s="48">
+        <f>H23+I23*D23/2+J23*D23^2/4</f>
+        <v/>
+      </c>
+      <c r="L23" s="49">
+        <f>H23*D23+I23*D23^2/2+J23*D23^3/3-E23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6">
+        <f>'Bootstrap'!A23</f>
+        <v/>
+      </c>
+      <c r="B24" s="27">
+        <f>'Bootstrap'!C23</f>
+        <v/>
+      </c>
+      <c r="C24" s="33">
+        <f>'Bootstrap'!H23</f>
+        <v/>
+      </c>
+      <c r="D24" s="27">
+        <f>B24-B23</f>
+        <v/>
+      </c>
+      <c r="E24" s="32">
+        <f>-LN(C24/C23)</f>
+        <v/>
+      </c>
+      <c r="F24" s="48">
+        <f>E24/D24</f>
+        <v/>
+      </c>
+      <c r="G24" s="48">
+        <f>(F24+F25)/2</f>
+        <v/>
+      </c>
+      <c r="H24" s="48">
+        <f>G23</f>
+        <v/>
+      </c>
+      <c r="I24" s="32">
+        <f>(G24-G23)/D24-J24*D24</f>
+        <v/>
+      </c>
+      <c r="J24" s="32">
+        <f>3*(G24-G23)/D24^2-6*(E24-G23*D24)/D24^3</f>
+        <v/>
+      </c>
+      <c r="K24" s="48">
+        <f>H24+I24*D24/2+J24*D24^2/4</f>
+        <v/>
+      </c>
+      <c r="L24" s="49">
+        <f>H24*D24+I24*D24^2/2+J24*D24^3/3-E24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6">
+        <f>'Bootstrap'!A24</f>
+        <v/>
+      </c>
+      <c r="B25" s="27">
+        <f>'Bootstrap'!C24</f>
+        <v/>
+      </c>
+      <c r="C25" s="33">
+        <f>'Bootstrap'!H24</f>
+        <v/>
+      </c>
+      <c r="D25" s="27">
+        <f>B25-B24</f>
+        <v/>
+      </c>
+      <c r="E25" s="32">
+        <f>-LN(C25/C24)</f>
+        <v/>
+      </c>
+      <c r="F25" s="48">
+        <f>E25/D25</f>
+        <v/>
+      </c>
+      <c r="G25" s="48">
+        <f>(F25+F26)/2</f>
+        <v/>
+      </c>
+      <c r="H25" s="48">
+        <f>G24</f>
+        <v/>
+      </c>
+      <c r="I25" s="32">
+        <f>(G25-G24)/D25-J25*D25</f>
+        <v/>
+      </c>
+      <c r="J25" s="32">
+        <f>3*(G25-G24)/D25^2-6*(E25-G24*D25)/D25^3</f>
+        <v/>
+      </c>
+      <c r="K25" s="48">
+        <f>H25+I25*D25/2+J25*D25^2/4</f>
+        <v/>
+      </c>
+      <c r="L25" s="49">
+        <f>H25*D25+I25*D25^2/2+J25*D25^3/3-E25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6">
+        <f>'Bootstrap'!A25</f>
+        <v/>
+      </c>
+      <c r="B26" s="27">
+        <f>'Bootstrap'!C25</f>
+        <v/>
+      </c>
+      <c r="C26" s="33">
+        <f>'Bootstrap'!H25</f>
+        <v/>
+      </c>
+      <c r="D26" s="27">
+        <f>B26-B25</f>
+        <v/>
+      </c>
+      <c r="E26" s="32">
+        <f>-LN(C26/C25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="48">
+        <f>E26/D26</f>
+        <v/>
+      </c>
+      <c r="G26" s="48">
+        <f>(F26+F27)/2</f>
+        <v/>
+      </c>
+      <c r="H26" s="48">
+        <f>G25</f>
+        <v/>
+      </c>
+      <c r="I26" s="32">
+        <f>(G26-G25)/D26-J26*D26</f>
+        <v/>
+      </c>
+      <c r="J26" s="32">
+        <f>3*(G26-G25)/D26^2-6*(E26-G25*D26)/D26^3</f>
+        <v/>
+      </c>
+      <c r="K26" s="48">
+        <f>H26+I26*D26/2+J26*D26^2/4</f>
+        <v/>
+      </c>
+      <c r="L26" s="49">
+        <f>H26*D26+I26*D26^2/2+J26*D26^3/3-E26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6">
+        <f>'Bootstrap'!A26</f>
+        <v/>
+      </c>
+      <c r="B27" s="27">
+        <f>'Bootstrap'!C26</f>
+        <v/>
+      </c>
+      <c r="C27" s="33">
+        <f>'Bootstrap'!H26</f>
+        <v/>
+      </c>
+      <c r="D27" s="27">
+        <f>B27-B26</f>
+        <v/>
+      </c>
+      <c r="E27" s="32">
+        <f>-LN(C27/C26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="48">
+        <f>E27/D27</f>
+        <v/>
+      </c>
+      <c r="G27" s="48">
+        <f>(F27+F28)/2</f>
+        <v/>
+      </c>
+      <c r="H27" s="48">
+        <f>G26</f>
+        <v/>
+      </c>
+      <c r="I27" s="32">
+        <f>(G27-G26)/D27-J27*D27</f>
+        <v/>
+      </c>
+      <c r="J27" s="32">
+        <f>3*(G27-G26)/D27^2-6*(E27-G26*D27)/D27^3</f>
+        <v/>
+      </c>
+      <c r="K27" s="48">
+        <f>H27+I27*D27/2+J27*D27^2/4</f>
+        <v/>
+      </c>
+      <c r="L27" s="49">
+        <f>H27*D27+I27*D27^2/2+J27*D27^3/3-E27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6">
+        <f>'Bootstrap'!A27</f>
+        <v/>
+      </c>
+      <c r="B28" s="27">
+        <f>'Bootstrap'!C27</f>
+        <v/>
+      </c>
+      <c r="C28" s="33">
+        <f>'Bootstrap'!H27</f>
+        <v/>
+      </c>
+      <c r="D28" s="27">
+        <f>B28-B27</f>
+        <v/>
+      </c>
+      <c r="E28" s="32">
+        <f>-LN(C28/C27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="48">
+        <f>E28/D28</f>
+        <v/>
+      </c>
+      <c r="G28" s="48">
+        <f>(F28+F29)/2</f>
+        <v/>
+      </c>
+      <c r="H28" s="48">
+        <f>G27</f>
+        <v/>
+      </c>
+      <c r="I28" s="32">
+        <f>(G28-G27)/D28-J28*D28</f>
+        <v/>
+      </c>
+      <c r="J28" s="32">
+        <f>3*(G28-G27)/D28^2-6*(E28-G27*D28)/D28^3</f>
+        <v/>
+      </c>
+      <c r="K28" s="48">
+        <f>H28+I28*D28/2+J28*D28^2/4</f>
+        <v/>
+      </c>
+      <c r="L28" s="49">
+        <f>H28*D28+I28*D28^2/2+J28*D28^3/3-E28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6">
+        <f>'Bootstrap'!A28</f>
+        <v/>
+      </c>
+      <c r="B29" s="27">
+        <f>'Bootstrap'!C28</f>
+        <v/>
+      </c>
+      <c r="C29" s="33">
+        <f>'Bootstrap'!H28</f>
+        <v/>
+      </c>
+      <c r="D29" s="27">
+        <f>B29-B28</f>
+        <v/>
+      </c>
+      <c r="E29" s="32">
+        <f>-LN(C29/C28)</f>
+        <v/>
+      </c>
+      <c r="F29" s="48">
+        <f>E29/D29</f>
+        <v/>
+      </c>
+      <c r="G29" s="48">
+        <f>(F29+F30)/2</f>
+        <v/>
+      </c>
+      <c r="H29" s="48">
+        <f>G28</f>
+        <v/>
+      </c>
+      <c r="I29" s="32">
+        <f>(G29-G28)/D29-J29*D29</f>
+        <v/>
+      </c>
+      <c r="J29" s="32">
+        <f>3*(G29-G28)/D29^2-6*(E29-G28*D29)/D29^3</f>
+        <v/>
+      </c>
+      <c r="K29" s="48">
+        <f>H29+I29*D29/2+J29*D29^2/4</f>
+        <v/>
+      </c>
+      <c r="L29" s="49">
+        <f>H29*D29+I29*D29^2/2+J29*D29^3/3-E29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6">
+        <f>'Bootstrap'!A29</f>
+        <v/>
+      </c>
+      <c r="B30" s="27">
+        <f>'Bootstrap'!C29</f>
+        <v/>
+      </c>
+      <c r="C30" s="33">
+        <f>'Bootstrap'!H29</f>
+        <v/>
+      </c>
+      <c r="D30" s="27">
+        <f>B30-B29</f>
+        <v/>
+      </c>
+      <c r="E30" s="32">
+        <f>-LN(C30/C29)</f>
+        <v/>
+      </c>
+      <c r="F30" s="48">
+        <f>E30/D30</f>
+        <v/>
+      </c>
+      <c r="G30" s="48">
+        <f>(F30+F31)/2</f>
+        <v/>
+      </c>
+      <c r="H30" s="48">
+        <f>G29</f>
+        <v/>
+      </c>
+      <c r="I30" s="32">
+        <f>(G30-G29)/D30-J30*D30</f>
+        <v/>
+      </c>
+      <c r="J30" s="32">
+        <f>3*(G30-G29)/D30^2-6*(E30-G29*D30)/D30^3</f>
+        <v/>
+      </c>
+      <c r="K30" s="48">
+        <f>H30+I30*D30/2+J30*D30^2/4</f>
+        <v/>
+      </c>
+      <c r="L30" s="49">
+        <f>H30*D30+I30*D30^2/2+J30*D30^3/3-E30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6">
+        <f>'Bootstrap'!A30</f>
+        <v/>
+      </c>
+      <c r="B31" s="27">
+        <f>'Bootstrap'!C30</f>
+        <v/>
+      </c>
+      <c r="C31" s="33">
+        <f>'Bootstrap'!H30</f>
+        <v/>
+      </c>
+      <c r="D31" s="27">
+        <f>B31-B30</f>
+        <v/>
+      </c>
+      <c r="E31" s="32">
+        <f>-LN(C31/C30)</f>
+        <v/>
+      </c>
+      <c r="F31" s="48">
+        <f>E31/D31</f>
+        <v/>
+      </c>
+      <c r="G31" s="48">
+        <f>(F31+F32)/2</f>
+        <v/>
+      </c>
+      <c r="H31" s="48">
+        <f>G30</f>
+        <v/>
+      </c>
+      <c r="I31" s="32">
+        <f>(G31-G30)/D31-J31*D31</f>
+        <v/>
+      </c>
+      <c r="J31" s="32">
+        <f>3*(G31-G30)/D31^2-6*(E31-G30*D31)/D31^3</f>
+        <v/>
+      </c>
+      <c r="K31" s="48">
+        <f>H31+I31*D31/2+J31*D31^2/4</f>
+        <v/>
+      </c>
+      <c r="L31" s="49">
+        <f>H31*D31+I31*D31^2/2+J31*D31^3/3-E31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6">
+        <f>'Bootstrap'!A31</f>
+        <v/>
+      </c>
+      <c r="B32" s="27">
+        <f>'Bootstrap'!C31</f>
+        <v/>
+      </c>
+      <c r="C32" s="33">
+        <f>'Bootstrap'!H31</f>
+        <v/>
+      </c>
+      <c r="D32" s="27">
+        <f>B32-B31</f>
+        <v/>
+      </c>
+      <c r="E32" s="32">
+        <f>-LN(C32/C31)</f>
+        <v/>
+      </c>
+      <c r="F32" s="48">
+        <f>E32/D32</f>
+        <v/>
+      </c>
+      <c r="G32" s="48">
+        <f>(F32+F33)/2</f>
+        <v/>
+      </c>
+      <c r="H32" s="48">
+        <f>G31</f>
+        <v/>
+      </c>
+      <c r="I32" s="32">
+        <f>(G32-G31)/D32-J32*D32</f>
+        <v/>
+      </c>
+      <c r="J32" s="32">
+        <f>3*(G32-G31)/D32^2-6*(E32-G31*D32)/D32^3</f>
+        <v/>
+      </c>
+      <c r="K32" s="48">
+        <f>H32+I32*D32/2+J32*D32^2/4</f>
+        <v/>
+      </c>
+      <c r="L32" s="49">
+        <f>H32*D32+I32*D32^2/2+J32*D32^3/3-E32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6">
+        <f>'Bootstrap'!A32</f>
+        <v/>
+      </c>
+      <c r="B33" s="27">
+        <f>'Bootstrap'!C32</f>
+        <v/>
+      </c>
+      <c r="C33" s="33">
+        <f>'Bootstrap'!H32</f>
+        <v/>
+      </c>
+      <c r="D33" s="27">
+        <f>B33-B32</f>
+        <v/>
+      </c>
+      <c r="E33" s="32">
+        <f>-LN(C33/C32)</f>
+        <v/>
+      </c>
+      <c r="F33" s="48">
+        <f>E33/D33</f>
+        <v/>
+      </c>
+      <c r="G33" s="48">
+        <f>(F33+F34)/2</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>G32</f>
+        <v/>
+      </c>
+      <c r="I33" s="32">
+        <f>(G33-G32)/D33-J33*D33</f>
+        <v/>
+      </c>
+      <c r="J33" s="32">
+        <f>3*(G33-G32)/D33^2-6*(E33-G32*D33)/D33^3</f>
+        <v/>
+      </c>
+      <c r="K33" s="48">
+        <f>H33+I33*D33/2+J33*D33^2/4</f>
+        <v/>
+      </c>
+      <c r="L33" s="49">
+        <f>H33*D33+I33*D33^2/2+J33*D33^3/3-E33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6">
+        <f>'Bootstrap'!A33</f>
+        <v/>
+      </c>
+      <c r="B34" s="27">
+        <f>'Bootstrap'!C33</f>
+        <v/>
+      </c>
+      <c r="C34" s="33">
+        <f>'Bootstrap'!H33</f>
+        <v/>
+      </c>
+      <c r="D34" s="27">
+        <f>B34-B33</f>
+        <v/>
+      </c>
+      <c r="E34" s="32">
+        <f>-LN(C34/C33)</f>
+        <v/>
+      </c>
+      <c r="F34" s="48">
+        <f>E34/D34</f>
+        <v/>
+      </c>
+      <c r="G34" s="48">
+        <f>(F34+F35)/2</f>
+        <v/>
+      </c>
+      <c r="H34" s="48">
+        <f>G33</f>
+        <v/>
+      </c>
+      <c r="I34" s="32">
+        <f>(G34-G33)/D34-J34*D34</f>
+        <v/>
+      </c>
+      <c r="J34" s="32">
+        <f>3*(G34-G33)/D34^2-6*(E34-G33*D34)/D34^3</f>
+        <v/>
+      </c>
+      <c r="K34" s="48">
+        <f>H34+I34*D34/2+J34*D34^2/4</f>
+        <v/>
+      </c>
+      <c r="L34" s="49">
+        <f>H34*D34+I34*D34^2/2+J34*D34^3/3-E34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6">
+        <f>'Bootstrap'!A34</f>
+        <v/>
+      </c>
+      <c r="B35" s="27">
+        <f>'Bootstrap'!C34</f>
+        <v/>
+      </c>
+      <c r="C35" s="33">
+        <f>'Bootstrap'!H34</f>
+        <v/>
+      </c>
+      <c r="D35" s="27">
+        <f>B35-B34</f>
+        <v/>
+      </c>
+      <c r="E35" s="32">
+        <f>-LN(C35/C34)</f>
+        <v/>
+      </c>
+      <c r="F35" s="48">
+        <f>E35/D35</f>
+        <v/>
+      </c>
+      <c r="G35" s="48">
+        <f>(F35+F36)/2</f>
+        <v/>
+      </c>
+      <c r="H35" s="48">
+        <f>G34</f>
+        <v/>
+      </c>
+      <c r="I35" s="32">
+        <f>(G35-G34)/D35-J35*D35</f>
+        <v/>
+      </c>
+      <c r="J35" s="32">
+        <f>3*(G35-G34)/D35^2-6*(E35-G34*D35)/D35^3</f>
+        <v/>
+      </c>
+      <c r="K35" s="48">
+        <f>H35+I35*D35/2+J35*D35^2/4</f>
+        <v/>
+      </c>
+      <c r="L35" s="49">
+        <f>H35*D35+I35*D35^2/2+J35*D35^3/3-E35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6">
+        <f>'Bootstrap'!A35</f>
+        <v/>
+      </c>
+      <c r="B36" s="27">
+        <f>'Bootstrap'!C35</f>
+        <v/>
+      </c>
+      <c r="C36" s="33">
+        <f>'Bootstrap'!H35</f>
+        <v/>
+      </c>
+      <c r="D36" s="27">
+        <f>B36-B35</f>
+        <v/>
+      </c>
+      <c r="E36" s="32">
+        <f>-LN(C36/C35)</f>
+        <v/>
+      </c>
+      <c r="F36" s="48">
+        <f>E36/D36</f>
+        <v/>
+      </c>
+      <c r="G36" s="48">
+        <f>(F36+F37)/2</f>
+        <v/>
+      </c>
+      <c r="H36" s="48">
+        <f>G35</f>
+        <v/>
+      </c>
+      <c r="I36" s="32">
+        <f>(G36-G35)/D36-J36*D36</f>
+        <v/>
+      </c>
+      <c r="J36" s="32">
+        <f>3*(G36-G35)/D36^2-6*(E36-G35*D36)/D36^3</f>
+        <v/>
+      </c>
+      <c r="K36" s="48">
+        <f>H36+I36*D36/2+J36*D36^2/4</f>
+        <v/>
+      </c>
+      <c r="L36" s="49">
+        <f>H36*D36+I36*D36^2/2+J36*D36^3/3-E36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6">
+        <f>'Bootstrap'!A36</f>
+        <v/>
+      </c>
+      <c r="B37" s="27">
+        <f>'Bootstrap'!C36</f>
+        <v/>
+      </c>
+      <c r="C37" s="33">
+        <f>'Bootstrap'!H36</f>
+        <v/>
+      </c>
+      <c r="D37" s="27">
+        <f>B37-B36</f>
+        <v/>
+      </c>
+      <c r="E37" s="32">
+        <f>-LN(C37/C36)</f>
+        <v/>
+      </c>
+      <c r="F37" s="48">
+        <f>E37/D37</f>
+        <v/>
+      </c>
+      <c r="G37" s="48">
+        <f>(F37+F38)/2</f>
+        <v/>
+      </c>
+      <c r="H37" s="48">
+        <f>G36</f>
+        <v/>
+      </c>
+      <c r="I37" s="32">
+        <f>(G37-G36)/D37-J37*D37</f>
+        <v/>
+      </c>
+      <c r="J37" s="32">
+        <f>3*(G37-G36)/D37^2-6*(E37-G36*D37)/D37^3</f>
+        <v/>
+      </c>
+      <c r="K37" s="48">
+        <f>H37+I37*D37/2+J37*D37^2/4</f>
+        <v/>
+      </c>
+      <c r="L37" s="49">
+        <f>H37*D37+I37*D37^2/2+J37*D37^3/3-E37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6">
+        <f>'Bootstrap'!A37</f>
+        <v/>
+      </c>
+      <c r="B38" s="27">
+        <f>'Bootstrap'!C37</f>
+        <v/>
+      </c>
+      <c r="C38" s="33">
+        <f>'Bootstrap'!H37</f>
+        <v/>
+      </c>
+      <c r="D38" s="27">
+        <f>B38-B37</f>
+        <v/>
+      </c>
+      <c r="E38" s="32">
+        <f>-LN(C38/C37)</f>
+        <v/>
+      </c>
+      <c r="F38" s="48">
+        <f>E38/D38</f>
+        <v/>
+      </c>
+      <c r="G38" s="48">
+        <f>(F38+F39)/2</f>
+        <v/>
+      </c>
+      <c r="H38" s="48">
+        <f>G37</f>
+        <v/>
+      </c>
+      <c r="I38" s="32">
+        <f>(G38-G37)/D38-J38*D38</f>
+        <v/>
+      </c>
+      <c r="J38" s="32">
+        <f>3*(G38-G37)/D38^2-6*(E38-G37*D38)/D38^3</f>
+        <v/>
+      </c>
+      <c r="K38" s="48">
+        <f>H38+I38*D38/2+J38*D38^2/4</f>
+        <v/>
+      </c>
+      <c r="L38" s="49">
+        <f>H38*D38+I38*D38^2/2+J38*D38^3/3-E38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6">
+        <f>'Bootstrap'!A38</f>
+        <v/>
+      </c>
+      <c r="B39" s="27">
+        <f>'Bootstrap'!C38</f>
+        <v/>
+      </c>
+      <c r="C39" s="33">
+        <f>'Bootstrap'!H38</f>
+        <v/>
+      </c>
+      <c r="D39" s="27">
+        <f>B39-B38</f>
+        <v/>
+      </c>
+      <c r="E39" s="32">
+        <f>-LN(C39/C38)</f>
+        <v/>
+      </c>
+      <c r="F39" s="48">
+        <f>E39/D39</f>
+        <v/>
+      </c>
+      <c r="G39" s="48">
+        <f>(F39+F40)/2</f>
+        <v/>
+      </c>
+      <c r="H39" s="48">
+        <f>G38</f>
+        <v/>
+      </c>
+      <c r="I39" s="32">
+        <f>(G39-G38)/D39-J39*D39</f>
+        <v/>
+      </c>
+      <c r="J39" s="32">
+        <f>3*(G39-G38)/D39^2-6*(E39-G38*D39)/D39^3</f>
+        <v/>
+      </c>
+      <c r="K39" s="48">
+        <f>H39+I39*D39/2+J39*D39^2/4</f>
+        <v/>
+      </c>
+      <c r="L39" s="49">
+        <f>H39*D39+I39*D39^2/2+J39*D39^3/3-E39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6">
+        <f>'Bootstrap'!A39</f>
+        <v/>
+      </c>
+      <c r="B40" s="27">
+        <f>'Bootstrap'!C39</f>
+        <v/>
+      </c>
+      <c r="C40" s="33">
+        <f>'Bootstrap'!H39</f>
+        <v/>
+      </c>
+      <c r="D40" s="27">
+        <f>B40-B39</f>
+        <v/>
+      </c>
+      <c r="E40" s="32">
+        <f>-LN(C40/C39)</f>
+        <v/>
+      </c>
+      <c r="F40" s="48">
+        <f>E40/D40</f>
+        <v/>
+      </c>
+      <c r="G40" s="48">
+        <f>F40</f>
+        <v/>
+      </c>
+      <c r="H40" s="48">
+        <f>G39</f>
+        <v/>
+      </c>
+      <c r="I40" s="32">
+        <f>(G40-G39)/D40-J40*D40</f>
+        <v/>
+      </c>
+      <c r="J40" s="32">
+        <f>3*(G40-G39)/D40^2-6*(E40-G39*D40)/D40^3</f>
+        <v/>
+      </c>
+      <c r="K40" s="48">
+        <f>H40+I40*D40/2+J40*D40^2/4</f>
+        <v/>
+      </c>
+      <c r="L40" s="49">
+        <f>H40*D40+I40*D40^2/2+J40*D40^3/3-E40</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A4:L6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add DF-source column; replace tau/sigma glyphs with ASCII
- Bootstrap tab: new 'DF source' column (N) labels each pillar 'short OIS' /
  'SR3 futures' / 'OIS swap', so it's unambiguous which instrument builds each
  segment (the futures drive 18M-5Y; col E OIS pars are reference only).
- Replace every tau glyph with 'tau' and the two sigma glyphs with 'Sum'
  across all headers/notes, per request.
Regenerated; formulas compile clean, no orphaned parts.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -4265,6 +4265,7 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
@@ -4306,7 +4307,7 @@
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>SHORT (o/n–1Y): single-payment SOFR OIS, DF = 1/(1+S·τ0).  MIDDLE (1Y–5Y): the DF at 18M/2Y/3Y/4Y/5Y is interpolated off the SR3 futures chain (helper block cols O–W), which discounts each contract's forward rate forward from the OIS 1Y DF — so 18M/2Y…5Y here are driven by FUTURES, not the OIS pars (col E is shown only for reference).  LONG (5Y–50Y): annual SOFR OIS swaps, DF = (1−S·A_prior)/(1+S·τcoupon), with the annuity (col I) built from the short + futures DFs. Cutovers at 1Y and 5Y mean nothing overlaps. Paste S490 zeros into column L for the Δz check.</t>
+          <t>SHORT (o/n–1Y): single-payment SOFR OIS, DF = 1/(1+S·tau0).  MIDDLE (1Y–5Y): the DF at 18M/2Y/3Y/4Y/5Y is interpolated off the SR3 futures chain (helper block cols O–W), which discounts each contract's forward rate forward from the OIS 1Y DF — so 18M/2Y…5Y here are driven by FUTURES, not the OIS pars (col E is shown only for reference).  LONG (5Y–50Y): annual SOFR OIS swaps, DF = (1−S·A_prior)/(1+S·taucoupon), with the annuity (col I) built from the short + futures DFs. Cutovers at 1Y and 5Y mean nothing overlaps. Paste S490 zeros into column L for the Δz check.</t>
         </is>
       </c>
     </row>
@@ -4340,7 +4341,7 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>τ0 spot→mat</t>
+          <t>tau0 spot→mat</t>
         </is>
       </c>
       <c r="E7" s="19" t="inlineStr">
@@ -4350,7 +4351,7 @@
       </c>
       <c r="F7" s="19" t="inlineStr">
         <is>
-          <t>τ coupon</t>
+          <t>tau coupon</t>
         </is>
       </c>
       <c r="G7" s="19" t="inlineStr">
@@ -4365,7 +4366,7 @@
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
-          <t>Ann.add τ·DF</t>
+          <t>Ann.add tau·DF</t>
         </is>
       </c>
       <c r="J7" s="19" t="inlineStr">
@@ -4388,6 +4389,11 @@
           <t>Δ vs S490 (bp)</t>
         </is>
       </c>
+      <c r="N7" s="19" t="inlineStr">
+        <is>
+          <t>DF source</t>
+        </is>
+      </c>
       <c r="O7" s="19" t="inlineStr">
         <is>
           <t>Contract</t>
@@ -4405,7 +4411,7 @@
       </c>
       <c r="R7" s="19" t="inlineStr">
         <is>
-          <t>τ eff (post-1Y)</t>
+          <t>tau eff (post-1Y)</t>
         </is>
       </c>
       <c r="S7" s="19" t="inlineStr">
@@ -4490,6 +4496,11 @@
         <f>IF(L8="","",(J8-L8)*100)</f>
         <v/>
       </c>
+      <c r="N8" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O8" s="6">
         <f>'SOFR_Futures'!A7</f>
         <v/>
@@ -4581,6 +4592,11 @@
         <f>IF(L9="","",(J9-L9)*100)</f>
         <v/>
       </c>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O9" s="6">
         <f>'SOFR_Futures'!A8</f>
         <v/>
@@ -4672,6 +4688,11 @@
         <f>IF(L10="","",(J10-L10)*100)</f>
         <v/>
       </c>
+      <c r="N10" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O10" s="6">
         <f>'SOFR_Futures'!A9</f>
         <v/>
@@ -4763,6 +4784,11 @@
         <f>IF(L11="","",(J11-L11)*100)</f>
         <v/>
       </c>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O11" s="6">
         <f>'SOFR_Futures'!A10</f>
         <v/>
@@ -4854,6 +4880,11 @@
         <f>IF(L12="","",(J12-L12)*100)</f>
         <v/>
       </c>
+      <c r="N12" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O12" s="6">
         <f>'SOFR_Futures'!A11</f>
         <v/>
@@ -4945,6 +4976,11 @@
         <f>IF(L13="","",(J13-L13)*100)</f>
         <v/>
       </c>
+      <c r="N13" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O13" s="6">
         <f>'SOFR_Futures'!A12</f>
         <v/>
@@ -5036,6 +5072,11 @@
         <f>IF(L14="","",(J14-L14)*100)</f>
         <v/>
       </c>
+      <c r="N14" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O14" s="6">
         <f>'SOFR_Futures'!A13</f>
         <v/>
@@ -5127,6 +5168,11 @@
         <f>IF(L15="","",(J15-L15)*100)</f>
         <v/>
       </c>
+      <c r="N15" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O15" s="6">
         <f>'SOFR_Futures'!A14</f>
         <v/>
@@ -5218,6 +5264,11 @@
         <f>IF(L16="","",(J16-L16)*100)</f>
         <v/>
       </c>
+      <c r="N16" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O16" s="6">
         <f>'SOFR_Futures'!A15</f>
         <v/>
@@ -5309,6 +5360,11 @@
         <f>IF(L17="","",(J17-L17)*100)</f>
         <v/>
       </c>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O17" s="6">
         <f>'SOFR_Futures'!A16</f>
         <v/>
@@ -5400,6 +5456,11 @@
         <f>IF(L18="","",(J18-L18)*100)</f>
         <v/>
       </c>
+      <c r="N18" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O18" s="6">
         <f>'SOFR_Futures'!A17</f>
         <v/>
@@ -5491,6 +5552,11 @@
         <f>IF(L19="","",(J19-L19)*100)</f>
         <v/>
       </c>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O19" s="6">
         <f>'SOFR_Futures'!A18</f>
         <v/>
@@ -5582,6 +5648,11 @@
         <f>IF(L20="","",(J20-L20)*100)</f>
         <v/>
       </c>
+      <c r="N20" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O20" s="6">
         <f>'SOFR_Futures'!A19</f>
         <v/>
@@ -5673,6 +5744,11 @@
         <f>IF(L21="","",(J21-L21)*100)</f>
         <v/>
       </c>
+      <c r="N21" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O21" s="6">
         <f>'SOFR_Futures'!A20</f>
         <v/>
@@ -5768,6 +5844,11 @@
         <f>IF(L22="","",(J22-L22)*100)</f>
         <v/>
       </c>
+      <c r="N22" s="6" t="inlineStr">
+        <is>
+          <t>short OIS</t>
+        </is>
+      </c>
       <c r="O22" s="6">
         <f>'SOFR_Futures'!A21</f>
         <v/>
@@ -5862,6 +5943,11 @@
         <f>IF(L23="","",(J23-L23)*100)</f>
         <v/>
       </c>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
+          <t>SR3 futures</t>
+        </is>
+      </c>
       <c r="O23" s="6">
         <f>'SOFR_Futures'!A22</f>
         <v/>
@@ -5957,6 +6043,11 @@
         <f>IF(L24="","",(J24-L24)*100)</f>
         <v/>
       </c>
+      <c r="N24" s="6" t="inlineStr">
+        <is>
+          <t>SR3 futures</t>
+        </is>
+      </c>
       <c r="O24" s="6">
         <f>'SOFR_Futures'!A23</f>
         <v/>
@@ -6052,6 +6143,11 @@
         <f>IF(L25="","",(J25-L25)*100)</f>
         <v/>
       </c>
+      <c r="N25" s="6" t="inlineStr">
+        <is>
+          <t>SR3 futures</t>
+        </is>
+      </c>
       <c r="O25" s="6">
         <f>'SOFR_Futures'!A24</f>
         <v/>
@@ -6147,6 +6243,11 @@
         <f>IF(L26="","",(J26-L26)*100)</f>
         <v/>
       </c>
+      <c r="N26" s="6" t="inlineStr">
+        <is>
+          <t>SR3 futures</t>
+        </is>
+      </c>
       <c r="O26" s="6">
         <f>'SOFR_Futures'!A25</f>
         <v/>
@@ -6242,6 +6343,11 @@
         <f>IF(L27="","",(J27-L27)*100)</f>
         <v/>
       </c>
+      <c r="N27" s="6" t="inlineStr">
+        <is>
+          <t>SR3 futures</t>
+        </is>
+      </c>
       <c r="O27" s="6">
         <f>'SOFR_Futures'!A26</f>
         <v/>
@@ -6337,6 +6443,11 @@
         <f>IF(L28="","",(J28-L28)*100)</f>
         <v/>
       </c>
+      <c r="N28" s="6" t="inlineStr">
+        <is>
+          <t>OIS swap</t>
+        </is>
+      </c>
       <c r="Y28" s="17">
         <f>MAX(Q27,$B$22)</f>
         <v/>
@@ -6397,6 +6508,11 @@
         <f>IF(L29="","",(J29-L29)*100)</f>
         <v/>
       </c>
+      <c r="N29" s="6" t="inlineStr">
+        <is>
+          <t>OIS swap</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -6449,6 +6565,11 @@
         <f>IF(L30="","",(J30-L30)*100)</f>
         <v/>
       </c>
+      <c r="N30" s="6" t="inlineStr">
+        <is>
+          <t>OIS swap</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -6501,6 +6622,11 @@
         <f>IF(L31="","",(J31-L31)*100)</f>
         <v/>
       </c>
+      <c r="N31" s="6" t="inlineStr">
+        <is>
+          <t>OIS swap</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -6553,6 +6679,11 @@
         <f>IF(L32="","",(J32-L32)*100)</f>
         <v/>
       </c>
+      <c r="N32" s="6" t="inlineStr">
+        <is>
+          <t>OIS swap</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -6605,6 +6736,11 @@
         <f>IF(L33="","",(J33-L33)*100)</f>
         <v/>
       </c>
+      <c r="N33" s="6" t="inlineStr">
+        <is>
+          <t>OIS swap</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -6657,6 +6793,11 @@
         <f>IF(L34="","",(J34-L34)*100)</f>
         <v/>
       </c>
+      <c r="N34" s="6" t="inlineStr">
+        <is>
+          <t>OIS swap</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -6709,6 +6850,11 @@
         <f>IF(L35="","",(J35-L35)*100)</f>
         <v/>
       </c>
+      <c r="N35" s="6" t="inlineStr">
+        <is>
+          <t>OIS swap</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -6761,6 +6907,11 @@
         <f>IF(L36="","",(J36-L36)*100)</f>
         <v/>
       </c>
+      <c r="N36" s="6" t="inlineStr">
+        <is>
+          <t>OIS swap</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -6813,6 +6964,11 @@
         <f>IF(L37="","",(J37-L37)*100)</f>
         <v/>
       </c>
+      <c r="N37" s="6" t="inlineStr">
+        <is>
+          <t>OIS swap</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -6865,6 +7021,11 @@
         <f>IF(L38="","",(J38-L38)*100)</f>
         <v/>
       </c>
+      <c r="N38" s="6" t="inlineStr">
+        <is>
+          <t>OIS swap</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -6917,11 +7078,16 @@
         <f>IF(L39="","",(J39-L39)*100)</f>
         <v/>
       </c>
+      <c r="N39" s="6" t="inlineStr">
+        <is>
+          <t>OIS swap</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="44" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>THREE SEGMENTS (Zhou 2002 structure):  SHORT o/n–1Y = single-payment SOFR OIS  (DF=1/(1+S·τ0));  MIDDLE 1Y–5Y = SR3 futures chained from the 1Y DF (helper block to the right, cols O–W);  LONG 5Y–50Y = annual SOFR OIS swaps built off the futures-derived 5Y point. No overlap — each maturity is covered once. Column H is the curve P(0,T); zero z=−ln(DF)/T. The futures convexity column (T) defaults to 0 — enter an adjustment in bp to correct futures→forward. Paste S490 zeros into column L for the Δz check; the Swap_Pricer values any OIS off this curve.</t>
+          <t>THREE SEGMENTS (Zhou 2002 structure):  SHORT o/n–1Y = single-payment SOFR OIS  (DF=1/(1+S·tau0));  MIDDLE 1Y–5Y = SR3 futures chained from the 1Y DF (helper block to the right, cols O–W);  LONG 5Y–50Y = annual SOFR OIS swaps built off the futures-derived 5Y point. No overlap — each maturity is covered once. Column H is the curve P(0,T); zero z=−ln(DF)/T. The futures convexity column (T) defaults to 0 — enter an adjustment in bp to correct futures→forward. Paste S490 zeros into column L for the Δz check; the Swap_Pricer values any OIS off this curve.</t>
         </is>
       </c>
     </row>
@@ -6929,9 +7095,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="O6:W6"/>
-    <mergeCell ref="A5:M6"/>
     <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="A41:M42"/>
+    <mergeCell ref="A5:N6"/>
+    <mergeCell ref="A41:N42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7324,7 +7490,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Fixed annuity  Στ·DF</t>
+          <t>Fixed annuity  Sum tau·DF</t>
         </is>
       </c>
       <c r="B21" s="32">
@@ -7333,7 +7499,7 @@
       </c>
       <c r="C21" s="35" t="inlineStr">
         <is>
-          <t>Sum of τ·DF over the fixed coupon dates.</t>
+          <t>Sum of tau·DF over the fixed coupon dates.</t>
         </is>
       </c>
       <c r="K21" s="17">
@@ -7608,7 +7774,7 @@
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>τ ACT/360</t>
+          <t>tau ACT/360</t>
         </is>
       </c>
       <c r="E35" s="19" t="inlineStr">
@@ -7628,7 +7794,7 @@
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>τ·DF</t>
+          <t>tau·DF</t>
         </is>
       </c>
       <c r="K35" s="17">

</xml_diff>

<commit_message>
Make IFERROR fallbacks loud: 'ERROR PLZ FIX' instead of blank
Replace the silent/blank IFERROR fallbacks on the Bloomberg-pull and derived
cells (fixings, OIS bid/ask/mid, futures fields + implied rate, conventions,
S490 name/BDH) with a loud 'ERROR PLZ FIX' so a failed pull is visible instead
of hidden. Left the two interpolation IFERRORs untouched — their fallback is a
valid boundary discount factor (INDEX(...)), not an error. Formulas compile
clean; no orphaned parts.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -1695,19 +1695,19 @@
         </is>
       </c>
       <c r="C5" s="22">
-        <f>IFERROR(BDP("USOSFRC BGN Curncy","CRNCY"),"N/A — use FLDS")</f>
+        <f>IFERROR(BDP("USOSFRC BGN Curncy","CRNCY"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D5" s="22">
-        <f>IFERROR(BDP("USOSFR1 BGN Curncy","CRNCY"),"N/A — use FLDS")</f>
+        <f>IFERROR(BDP("USOSFR1 BGN Curncy","CRNCY"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E5" s="22">
-        <f>IFERROR(BDP("USOSFR5 BGN Curncy","CRNCY"),"N/A — use FLDS")</f>
+        <f>IFERROR(BDP("USOSFR5 BGN Curncy","CRNCY"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F5" s="22">
-        <f>IFERROR(BDP("USOSFR30 BGN Curncy","CRNCY"),"N/A — use FLDS")</f>
+        <f>IFERROR(BDP("USOSFR30 BGN Curncy","CRNCY"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
@@ -1851,19 +1851,19 @@
         </is>
       </c>
       <c r="C10" s="22">
-        <f>IFERROR(BDP("USOSFRC BGN Curncy","CALENDAR_CODE"),"N/A — use FLDS")</f>
+        <f>IFERROR(BDP("USOSFRC BGN Curncy","CALENDAR_CODE"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D10" s="22">
-        <f>IFERROR(BDP("USOSFR1 BGN Curncy","CALENDAR_CODE"),"N/A — use FLDS")</f>
+        <f>IFERROR(BDP("USOSFR1 BGN Curncy","CALENDAR_CODE"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>IFERROR(BDP("USOSFR5 BGN Curncy","CALENDAR_CODE"),"N/A — use FLDS")</f>
+        <f>IFERROR(BDP("USOSFR5 BGN Curncy","CALENDAR_CODE"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>IFERROR(BDP("USOSFR30 BGN Curncy","CALENDAR_CODE"),"N/A — use FLDS")</f>
+        <f>IFERROR(BDP("USOSFR30 BGN Curncy","CALENDAR_CODE"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
@@ -1911,19 +1911,19 @@
         </is>
       </c>
       <c r="C12" s="22">
-        <f>IFERROR(BDP("USOSFRC BGN Curncy","DAY_CNT_DES"),"N/A — use FLDS")</f>
+        <f>IFERROR(BDP("USOSFRC BGN Curncy","DAY_CNT_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D12" s="22">
-        <f>IFERROR(BDP("USOSFR1 BGN Curncy","DAY_CNT_DES"),"N/A — use FLDS")</f>
+        <f>IFERROR(BDP("USOSFR1 BGN Curncy","DAY_CNT_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>IFERROR(BDP("USOSFR5 BGN Curncy","DAY_CNT_DES"),"N/A — use FLDS")</f>
+        <f>IFERROR(BDP("USOSFR5 BGN Curncy","DAY_CNT_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>IFERROR(BDP("USOSFR30 BGN Curncy","DAY_CNT_DES"),"N/A — use FLDS")</f>
+        <f>IFERROR(BDP("USOSFR30 BGN Curncy","DAY_CNT_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
@@ -4230,11 +4230,11 @@
         </is>
       </c>
       <c r="C6" s="17">
-        <f>IFERROR(BDP(SOFR_TKR,"PX_LAST"),"open in Bloomberg")</f>
+        <f>IFERROR(BDP(SOFR_TKR,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D6" s="18">
-        <f>IFERROR(BDP(SOFR_TKR,"LAST_UPDATE_DT"),"—")</f>
+        <f>IFERROR(BDP(SOFR_TKR,"LAST_UPDATE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
     </row>
     <row r="12">
       <c r="A12" s="19">
-        <f>IFERROR(BDH(SOFR_TKR,"PX_LAST",TEXT(HIST_START,"mm/dd/yyyy"),TEXT(HIST_END,"mm/dd/yyyy")),"open in Bloomberg")</f>
+        <f>IFERROR(BDH(SOFR_TKR,"PX_LAST",TEXT(HIST_START,"mm/dd/yyyy"),TEXT(HIST_END,"mm/dd/yyyy")),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
@@ -4393,860 +4393,860 @@
         <v/>
       </c>
       <c r="B7" s="6">
-        <f>IFERROR(BDP($A7,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A7,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C7" s="17">
-        <f>IFERROR(BDP($A7,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A7,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D7" s="17">
-        <f>IFERROR(BDP($A7,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A7,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E7" s="17">
-        <f>IFERROR(BDP($A7,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A7,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F7" s="17">
-        <f>IFERROR(100-C7,"")</f>
+        <f>IFERROR(100-C7,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G7" s="6">
-        <f>IFERROR(BDP($A7,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A7,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H7" s="18">
-        <f>IFERROR(BDP($A7,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A7,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I7" s="18">
-        <f>IFERROR(BDP($A7,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A7,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J7" s="21">
-        <f>IFERROR(BDP($A7,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A7,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K7" s="21">
-        <f>IFERROR(BDP($A7,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A7,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n"/>
       <c r="B8" s="6">
-        <f>IFERROR(BDP($A8,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A8,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C8" s="17">
-        <f>IFERROR(BDP($A8,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A8,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D8" s="17">
-        <f>IFERROR(BDP($A8,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A8,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E8" s="17">
-        <f>IFERROR(BDP($A8,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A8,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F8" s="17">
-        <f>IFERROR(100-C8,"")</f>
+        <f>IFERROR(100-C8,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G8" s="6">
-        <f>IFERROR(BDP($A8,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A8,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H8" s="18">
-        <f>IFERROR(BDP($A8,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A8,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I8" s="18">
-        <f>IFERROR(BDP($A8,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A8,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J8" s="21">
-        <f>IFERROR(BDP($A8,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A8,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K8" s="21">
-        <f>IFERROR(BDP($A8,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A8,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
       <c r="B9" s="6">
-        <f>IFERROR(BDP($A9,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A9,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C9" s="17">
-        <f>IFERROR(BDP($A9,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A9,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D9" s="17">
-        <f>IFERROR(BDP($A9,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A9,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E9" s="17">
-        <f>IFERROR(BDP($A9,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A9,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F9" s="17">
-        <f>IFERROR(100-C9,"")</f>
+        <f>IFERROR(100-C9,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G9" s="6">
-        <f>IFERROR(BDP($A9,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A9,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H9" s="18">
-        <f>IFERROR(BDP($A9,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A9,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I9" s="18">
-        <f>IFERROR(BDP($A9,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A9,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J9" s="21">
-        <f>IFERROR(BDP($A9,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A9,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K9" s="21">
-        <f>IFERROR(BDP($A9,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A9,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
       <c r="B10" s="6">
-        <f>IFERROR(BDP($A10,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A10,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C10" s="17">
-        <f>IFERROR(BDP($A10,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A10,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D10" s="17">
-        <f>IFERROR(BDP($A10,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A10,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E10" s="17">
-        <f>IFERROR(BDP($A10,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A10,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F10" s="17">
-        <f>IFERROR(100-C10,"")</f>
+        <f>IFERROR(100-C10,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G10" s="6">
-        <f>IFERROR(BDP($A10,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A10,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H10" s="18">
-        <f>IFERROR(BDP($A10,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A10,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I10" s="18">
-        <f>IFERROR(BDP($A10,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A10,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J10" s="21">
-        <f>IFERROR(BDP($A10,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A10,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K10" s="21">
-        <f>IFERROR(BDP($A10,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A10,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
       <c r="B11" s="6">
-        <f>IFERROR(BDP($A11,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A11,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C11" s="17">
-        <f>IFERROR(BDP($A11,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A11,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D11" s="17">
-        <f>IFERROR(BDP($A11,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A11,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E11" s="17">
-        <f>IFERROR(BDP($A11,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A11,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F11" s="17">
-        <f>IFERROR(100-C11,"")</f>
+        <f>IFERROR(100-C11,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G11" s="6">
-        <f>IFERROR(BDP($A11,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A11,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H11" s="18">
-        <f>IFERROR(BDP($A11,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A11,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I11" s="18">
-        <f>IFERROR(BDP($A11,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A11,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J11" s="21">
-        <f>IFERROR(BDP($A11,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A11,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K11" s="21">
-        <f>IFERROR(BDP($A11,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A11,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n"/>
       <c r="B12" s="6">
-        <f>IFERROR(BDP($A12,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A12,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C12" s="17">
-        <f>IFERROR(BDP($A12,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A12,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D12" s="17">
-        <f>IFERROR(BDP($A12,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A12,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E12" s="17">
-        <f>IFERROR(BDP($A12,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A12,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F12" s="17">
-        <f>IFERROR(100-C12,"")</f>
+        <f>IFERROR(100-C12,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G12" s="6">
-        <f>IFERROR(BDP($A12,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A12,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H12" s="18">
-        <f>IFERROR(BDP($A12,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A12,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I12" s="18">
-        <f>IFERROR(BDP($A12,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A12,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J12" s="21">
-        <f>IFERROR(BDP($A12,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A12,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K12" s="21">
-        <f>IFERROR(BDP($A12,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A12,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
       <c r="B13" s="6">
-        <f>IFERROR(BDP($A13,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A13,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C13" s="17">
-        <f>IFERROR(BDP($A13,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A13,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D13" s="17">
-        <f>IFERROR(BDP($A13,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A13,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E13" s="17">
-        <f>IFERROR(BDP($A13,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A13,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F13" s="17">
-        <f>IFERROR(100-C13,"")</f>
+        <f>IFERROR(100-C13,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G13" s="6">
-        <f>IFERROR(BDP($A13,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A13,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H13" s="18">
-        <f>IFERROR(BDP($A13,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A13,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I13" s="18">
-        <f>IFERROR(BDP($A13,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A13,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J13" s="21">
-        <f>IFERROR(BDP($A13,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A13,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K13" s="21">
-        <f>IFERROR(BDP($A13,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A13,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
       <c r="B14" s="6">
-        <f>IFERROR(BDP($A14,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A14,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C14" s="17">
-        <f>IFERROR(BDP($A14,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A14,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D14" s="17">
-        <f>IFERROR(BDP($A14,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A14,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E14" s="17">
-        <f>IFERROR(BDP($A14,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A14,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F14" s="17">
-        <f>IFERROR(100-C14,"")</f>
+        <f>IFERROR(100-C14,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G14" s="6">
-        <f>IFERROR(BDP($A14,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A14,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H14" s="18">
-        <f>IFERROR(BDP($A14,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A14,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I14" s="18">
-        <f>IFERROR(BDP($A14,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A14,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J14" s="21">
-        <f>IFERROR(BDP($A14,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A14,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K14" s="21">
-        <f>IFERROR(BDP($A14,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A14,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
       <c r="B15" s="6">
-        <f>IFERROR(BDP($A15,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A15,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C15" s="17">
-        <f>IFERROR(BDP($A15,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A15,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D15" s="17">
-        <f>IFERROR(BDP($A15,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A15,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E15" s="17">
-        <f>IFERROR(BDP($A15,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A15,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F15" s="17">
-        <f>IFERROR(100-C15,"")</f>
+        <f>IFERROR(100-C15,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G15" s="6">
-        <f>IFERROR(BDP($A15,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A15,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H15" s="18">
-        <f>IFERROR(BDP($A15,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A15,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I15" s="18">
-        <f>IFERROR(BDP($A15,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A15,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J15" s="21">
-        <f>IFERROR(BDP($A15,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A15,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K15" s="21">
-        <f>IFERROR(BDP($A15,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A15,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
       <c r="B16" s="6">
-        <f>IFERROR(BDP($A16,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A16,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C16" s="17">
-        <f>IFERROR(BDP($A16,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A16,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D16" s="17">
-        <f>IFERROR(BDP($A16,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A16,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E16" s="17">
-        <f>IFERROR(BDP($A16,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A16,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F16" s="17">
-        <f>IFERROR(100-C16,"")</f>
+        <f>IFERROR(100-C16,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G16" s="6">
-        <f>IFERROR(BDP($A16,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A16,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H16" s="18">
-        <f>IFERROR(BDP($A16,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A16,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I16" s="18">
-        <f>IFERROR(BDP($A16,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A16,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J16" s="21">
-        <f>IFERROR(BDP($A16,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A16,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K16" s="21">
-        <f>IFERROR(BDP($A16,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A16,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
       <c r="B17" s="6">
-        <f>IFERROR(BDP($A17,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A17,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C17" s="17">
-        <f>IFERROR(BDP($A17,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A17,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D17" s="17">
-        <f>IFERROR(BDP($A17,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A17,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E17" s="17">
-        <f>IFERROR(BDP($A17,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A17,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F17" s="17">
-        <f>IFERROR(100-C17,"")</f>
+        <f>IFERROR(100-C17,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G17" s="6">
-        <f>IFERROR(BDP($A17,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A17,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H17" s="18">
-        <f>IFERROR(BDP($A17,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A17,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I17" s="18">
-        <f>IFERROR(BDP($A17,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A17,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J17" s="21">
-        <f>IFERROR(BDP($A17,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A17,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K17" s="21">
-        <f>IFERROR(BDP($A17,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A17,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
       <c r="B18" s="6">
-        <f>IFERROR(BDP($A18,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A18,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C18" s="17">
-        <f>IFERROR(BDP($A18,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A18,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D18" s="17">
-        <f>IFERROR(BDP($A18,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A18,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E18" s="17">
-        <f>IFERROR(BDP($A18,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A18,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F18" s="17">
-        <f>IFERROR(100-C18,"")</f>
+        <f>IFERROR(100-C18,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G18" s="6">
-        <f>IFERROR(BDP($A18,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A18,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H18" s="18">
-        <f>IFERROR(BDP($A18,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A18,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I18" s="18">
-        <f>IFERROR(BDP($A18,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A18,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J18" s="21">
-        <f>IFERROR(BDP($A18,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A18,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K18" s="21">
-        <f>IFERROR(BDP($A18,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A18,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="6">
-        <f>IFERROR(BDP($A19,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A19,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C19" s="17">
-        <f>IFERROR(BDP($A19,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A19,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D19" s="17">
-        <f>IFERROR(BDP($A19,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A19,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E19" s="17">
-        <f>IFERROR(BDP($A19,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A19,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F19" s="17">
-        <f>IFERROR(100-C19,"")</f>
+        <f>IFERROR(100-C19,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G19" s="6">
-        <f>IFERROR(BDP($A19,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A19,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H19" s="18">
-        <f>IFERROR(BDP($A19,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A19,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I19" s="18">
-        <f>IFERROR(BDP($A19,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A19,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J19" s="21">
-        <f>IFERROR(BDP($A19,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A19,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K19" s="21">
-        <f>IFERROR(BDP($A19,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A19,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n"/>
       <c r="B20" s="6">
-        <f>IFERROR(BDP($A20,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A20,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C20" s="17">
-        <f>IFERROR(BDP($A20,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A20,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D20" s="17">
-        <f>IFERROR(BDP($A20,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A20,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E20" s="17">
-        <f>IFERROR(BDP($A20,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A20,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F20" s="17">
-        <f>IFERROR(100-C20,"")</f>
+        <f>IFERROR(100-C20,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G20" s="6">
-        <f>IFERROR(BDP($A20,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A20,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H20" s="18">
-        <f>IFERROR(BDP($A20,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A20,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I20" s="18">
-        <f>IFERROR(BDP($A20,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A20,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J20" s="21">
-        <f>IFERROR(BDP($A20,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A20,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K20" s="21">
-        <f>IFERROR(BDP($A20,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A20,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n"/>
       <c r="B21" s="6">
-        <f>IFERROR(BDP($A21,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A21,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C21" s="17">
-        <f>IFERROR(BDP($A21,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A21,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D21" s="17">
-        <f>IFERROR(BDP($A21,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A21,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E21" s="17">
-        <f>IFERROR(BDP($A21,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A21,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F21" s="17">
-        <f>IFERROR(100-C21,"")</f>
+        <f>IFERROR(100-C21,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G21" s="6">
-        <f>IFERROR(BDP($A21,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A21,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H21" s="18">
-        <f>IFERROR(BDP($A21,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A21,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I21" s="18">
-        <f>IFERROR(BDP($A21,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A21,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J21" s="21">
-        <f>IFERROR(BDP($A21,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A21,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K21" s="21">
-        <f>IFERROR(BDP($A21,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A21,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n"/>
       <c r="B22" s="6">
-        <f>IFERROR(BDP($A22,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A22,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C22" s="17">
-        <f>IFERROR(BDP($A22,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A22,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D22" s="17">
-        <f>IFERROR(BDP($A22,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A22,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E22" s="17">
-        <f>IFERROR(BDP($A22,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A22,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F22" s="17">
-        <f>IFERROR(100-C22,"")</f>
+        <f>IFERROR(100-C22,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G22" s="6">
-        <f>IFERROR(BDP($A22,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A22,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H22" s="18">
-        <f>IFERROR(BDP($A22,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A22,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I22" s="18">
-        <f>IFERROR(BDP($A22,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A22,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J22" s="21">
-        <f>IFERROR(BDP($A22,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A22,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K22" s="21">
-        <f>IFERROR(BDP($A22,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A22,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="6">
-        <f>IFERROR(BDP($A23,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A23,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C23" s="17">
-        <f>IFERROR(BDP($A23,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A23,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D23" s="17">
-        <f>IFERROR(BDP($A23,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A23,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E23" s="17">
-        <f>IFERROR(BDP($A23,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A23,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F23" s="17">
-        <f>IFERROR(100-C23,"")</f>
+        <f>IFERROR(100-C23,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G23" s="6">
-        <f>IFERROR(BDP($A23,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A23,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H23" s="18">
-        <f>IFERROR(BDP($A23,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A23,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I23" s="18">
-        <f>IFERROR(BDP($A23,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A23,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J23" s="21">
-        <f>IFERROR(BDP($A23,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A23,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K23" s="21">
-        <f>IFERROR(BDP($A23,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A23,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n"/>
       <c r="B24" s="6">
-        <f>IFERROR(BDP($A24,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A24,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C24" s="17">
-        <f>IFERROR(BDP($A24,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A24,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D24" s="17">
-        <f>IFERROR(BDP($A24,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A24,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E24" s="17">
-        <f>IFERROR(BDP($A24,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A24,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F24" s="17">
-        <f>IFERROR(100-C24,"")</f>
+        <f>IFERROR(100-C24,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G24" s="6">
-        <f>IFERROR(BDP($A24,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A24,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H24" s="18">
-        <f>IFERROR(BDP($A24,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A24,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I24" s="18">
-        <f>IFERROR(BDP($A24,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A24,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J24" s="21">
-        <f>IFERROR(BDP($A24,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A24,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K24" s="21">
-        <f>IFERROR(BDP($A24,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A24,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="6">
-        <f>IFERROR(BDP($A25,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A25,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C25" s="17">
-        <f>IFERROR(BDP($A25,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A25,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D25" s="17">
-        <f>IFERROR(BDP($A25,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A25,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E25" s="17">
-        <f>IFERROR(BDP($A25,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A25,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F25" s="17">
-        <f>IFERROR(100-C25,"")</f>
+        <f>IFERROR(100-C25,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G25" s="6">
-        <f>IFERROR(BDP($A25,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A25,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H25" s="18">
-        <f>IFERROR(BDP($A25,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A25,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I25" s="18">
-        <f>IFERROR(BDP($A25,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A25,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J25" s="21">
-        <f>IFERROR(BDP($A25,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A25,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K25" s="21">
-        <f>IFERROR(BDP($A25,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A25,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="6">
-        <f>IFERROR(BDP($A26,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A26,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C26" s="17">
-        <f>IFERROR(BDP($A26,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A26,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D26" s="17">
-        <f>IFERROR(BDP($A26,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A26,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E26" s="17">
-        <f>IFERROR(BDP($A26,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A26,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F26" s="17">
-        <f>IFERROR(100-C26,"")</f>
+        <f>IFERROR(100-C26,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G26" s="6">
-        <f>IFERROR(BDP($A26,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A26,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H26" s="18">
-        <f>IFERROR(BDP($A26,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A26,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I26" s="18">
-        <f>IFERROR(BDP($A26,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A26,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J26" s="21">
-        <f>IFERROR(BDP($A26,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A26,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K26" s="21">
-        <f>IFERROR(BDP($A26,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A26,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
@@ -5327,559 +5327,559 @@
         <v/>
       </c>
       <c r="B32" s="6">
-        <f>IFERROR(BDP($A32,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A32,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C32" s="17">
-        <f>IFERROR(BDP($A32,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A32,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D32" s="17">
-        <f>IFERROR(BDP($A32,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A32,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E32" s="17">
-        <f>IFERROR(BDP($A32,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A32,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F32" s="17">
-        <f>IFERROR(100-C32,"")</f>
+        <f>IFERROR(100-C32,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G32" s="6">
-        <f>IFERROR(BDP($A32,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A32,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H32" s="18">
-        <f>IFERROR(BDP($A32,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A32,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I32" s="18">
-        <f>IFERROR(BDP($A32,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A32,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J32" s="21">
-        <f>IFERROR(BDP($A32,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A32,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K32" s="21">
-        <f>IFERROR(BDP($A32,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A32,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="6">
-        <f>IFERROR(BDP($A33,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A33,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C33" s="17">
-        <f>IFERROR(BDP($A33,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A33,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D33" s="17">
-        <f>IFERROR(BDP($A33,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A33,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E33" s="17">
-        <f>IFERROR(BDP($A33,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A33,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F33" s="17">
-        <f>IFERROR(100-C33,"")</f>
+        <f>IFERROR(100-C33,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G33" s="6">
-        <f>IFERROR(BDP($A33,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A33,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H33" s="18">
-        <f>IFERROR(BDP($A33,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A33,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I33" s="18">
-        <f>IFERROR(BDP($A33,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A33,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J33" s="21">
-        <f>IFERROR(BDP($A33,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A33,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K33" s="21">
-        <f>IFERROR(BDP($A33,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A33,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n"/>
       <c r="B34" s="6">
-        <f>IFERROR(BDP($A34,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A34,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C34" s="17">
-        <f>IFERROR(BDP($A34,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A34,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D34" s="17">
-        <f>IFERROR(BDP($A34,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A34,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E34" s="17">
-        <f>IFERROR(BDP($A34,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A34,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F34" s="17">
-        <f>IFERROR(100-C34,"")</f>
+        <f>IFERROR(100-C34,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G34" s="6">
-        <f>IFERROR(BDP($A34,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A34,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H34" s="18">
-        <f>IFERROR(BDP($A34,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A34,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I34" s="18">
-        <f>IFERROR(BDP($A34,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A34,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J34" s="21">
-        <f>IFERROR(BDP($A34,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A34,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K34" s="21">
-        <f>IFERROR(BDP($A34,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A34,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="6">
-        <f>IFERROR(BDP($A35,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A35,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C35" s="17">
-        <f>IFERROR(BDP($A35,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A35,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D35" s="17">
-        <f>IFERROR(BDP($A35,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A35,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E35" s="17">
-        <f>IFERROR(BDP($A35,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A35,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F35" s="17">
-        <f>IFERROR(100-C35,"")</f>
+        <f>IFERROR(100-C35,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G35" s="6">
-        <f>IFERROR(BDP($A35,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A35,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H35" s="18">
-        <f>IFERROR(BDP($A35,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A35,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I35" s="18">
-        <f>IFERROR(BDP($A35,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A35,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J35" s="21">
-        <f>IFERROR(BDP($A35,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A35,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K35" s="21">
-        <f>IFERROR(BDP($A35,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A35,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n"/>
       <c r="B36" s="6">
-        <f>IFERROR(BDP($A36,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A36,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C36" s="17">
-        <f>IFERROR(BDP($A36,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A36,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D36" s="17">
-        <f>IFERROR(BDP($A36,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A36,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E36" s="17">
-        <f>IFERROR(BDP($A36,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A36,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F36" s="17">
-        <f>IFERROR(100-C36,"")</f>
+        <f>IFERROR(100-C36,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G36" s="6">
-        <f>IFERROR(BDP($A36,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A36,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H36" s="18">
-        <f>IFERROR(BDP($A36,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A36,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I36" s="18">
-        <f>IFERROR(BDP($A36,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A36,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J36" s="21">
-        <f>IFERROR(BDP($A36,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A36,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K36" s="21">
-        <f>IFERROR(BDP($A36,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A36,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="6">
-        <f>IFERROR(BDP($A37,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A37,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C37" s="17">
-        <f>IFERROR(BDP($A37,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A37,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D37" s="17">
-        <f>IFERROR(BDP($A37,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A37,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E37" s="17">
-        <f>IFERROR(BDP($A37,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A37,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F37" s="17">
-        <f>IFERROR(100-C37,"")</f>
+        <f>IFERROR(100-C37,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G37" s="6">
-        <f>IFERROR(BDP($A37,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A37,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H37" s="18">
-        <f>IFERROR(BDP($A37,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A37,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I37" s="18">
-        <f>IFERROR(BDP($A37,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A37,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J37" s="21">
-        <f>IFERROR(BDP($A37,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A37,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K37" s="21">
-        <f>IFERROR(BDP($A37,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A37,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n"/>
       <c r="B38" s="6">
-        <f>IFERROR(BDP($A38,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A38,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C38" s="17">
-        <f>IFERROR(BDP($A38,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A38,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D38" s="17">
-        <f>IFERROR(BDP($A38,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A38,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E38" s="17">
-        <f>IFERROR(BDP($A38,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A38,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F38" s="17">
-        <f>IFERROR(100-C38,"")</f>
+        <f>IFERROR(100-C38,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G38" s="6">
-        <f>IFERROR(BDP($A38,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A38,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H38" s="18">
-        <f>IFERROR(BDP($A38,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A38,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I38" s="18">
-        <f>IFERROR(BDP($A38,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A38,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J38" s="21">
-        <f>IFERROR(BDP($A38,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A38,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K38" s="21">
-        <f>IFERROR(BDP($A38,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A38,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n"/>
       <c r="B39" s="6">
-        <f>IFERROR(BDP($A39,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A39,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C39" s="17">
-        <f>IFERROR(BDP($A39,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A39,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D39" s="17">
-        <f>IFERROR(BDP($A39,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A39,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E39" s="17">
-        <f>IFERROR(BDP($A39,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A39,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F39" s="17">
-        <f>IFERROR(100-C39,"")</f>
+        <f>IFERROR(100-C39,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G39" s="6">
-        <f>IFERROR(BDP($A39,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A39,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H39" s="18">
-        <f>IFERROR(BDP($A39,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A39,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I39" s="18">
-        <f>IFERROR(BDP($A39,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A39,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J39" s="21">
-        <f>IFERROR(BDP($A39,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A39,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K39" s="21">
-        <f>IFERROR(BDP($A39,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A39,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n"/>
       <c r="B40" s="6">
-        <f>IFERROR(BDP($A40,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A40,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C40" s="17">
-        <f>IFERROR(BDP($A40,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A40,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D40" s="17">
-        <f>IFERROR(BDP($A40,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A40,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E40" s="17">
-        <f>IFERROR(BDP($A40,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A40,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F40" s="17">
-        <f>IFERROR(100-C40,"")</f>
+        <f>IFERROR(100-C40,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G40" s="6">
-        <f>IFERROR(BDP($A40,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A40,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H40" s="18">
-        <f>IFERROR(BDP($A40,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A40,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I40" s="18">
-        <f>IFERROR(BDP($A40,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A40,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J40" s="21">
-        <f>IFERROR(BDP($A40,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A40,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K40" s="21">
-        <f>IFERROR(BDP($A40,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A40,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="6">
-        <f>IFERROR(BDP($A41,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A41,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C41" s="17">
-        <f>IFERROR(BDP($A41,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A41,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D41" s="17">
-        <f>IFERROR(BDP($A41,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A41,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E41" s="17">
-        <f>IFERROR(BDP($A41,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A41,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F41" s="17">
-        <f>IFERROR(100-C41,"")</f>
+        <f>IFERROR(100-C41,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G41" s="6">
-        <f>IFERROR(BDP($A41,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A41,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H41" s="18">
-        <f>IFERROR(BDP($A41,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A41,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I41" s="18">
-        <f>IFERROR(BDP($A41,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A41,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J41" s="21">
-        <f>IFERROR(BDP($A41,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A41,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K41" s="21">
-        <f>IFERROR(BDP($A41,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A41,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="6">
-        <f>IFERROR(BDP($A42,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A42,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C42" s="17">
-        <f>IFERROR(BDP($A42,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A42,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D42" s="17">
-        <f>IFERROR(BDP($A42,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A42,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E42" s="17">
-        <f>IFERROR(BDP($A42,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A42,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F42" s="17">
-        <f>IFERROR(100-C42,"")</f>
+        <f>IFERROR(100-C42,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G42" s="6">
-        <f>IFERROR(BDP($A42,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A42,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H42" s="18">
-        <f>IFERROR(BDP($A42,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A42,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I42" s="18">
-        <f>IFERROR(BDP($A42,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A42,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J42" s="21">
-        <f>IFERROR(BDP($A42,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A42,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K42" s="21">
-        <f>IFERROR(BDP($A42,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A42,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="6">
-        <f>IFERROR(BDP($A43,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A43,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C43" s="17">
-        <f>IFERROR(BDP($A43,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A43,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D43" s="17">
-        <f>IFERROR(BDP($A43,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A43,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E43" s="17">
-        <f>IFERROR(BDP($A43,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A43,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F43" s="17">
-        <f>IFERROR(100-C43,"")</f>
+        <f>IFERROR(100-C43,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G43" s="6">
-        <f>IFERROR(BDP($A43,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A43,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H43" s="18">
-        <f>IFERROR(BDP($A43,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A43,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I43" s="18">
-        <f>IFERROR(BDP($A43,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A43,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J43" s="21">
-        <f>IFERROR(BDP($A43,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A43,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K43" s="21">
-        <f>IFERROR(BDP($A43,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A43,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n"/>
       <c r="B44" s="6">
-        <f>IFERROR(BDP($A44,"SECURITY_DES"),"")</f>
+        <f>IFERROR(BDP($A44,"SECURITY_DES"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="C44" s="17">
-        <f>IFERROR(BDP($A44,"PX_LAST"),"")</f>
+        <f>IFERROR(BDP($A44,"PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="D44" s="17">
-        <f>IFERROR(BDP($A44,"PX_BID"),"")</f>
+        <f>IFERROR(BDP($A44,"PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="E44" s="17">
-        <f>IFERROR(BDP($A44,"PX_ASK"),"")</f>
+        <f>IFERROR(BDP($A44,"PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F44" s="17">
-        <f>IFERROR(100-C44,"")</f>
+        <f>IFERROR(100-C44,"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G44" s="6">
-        <f>IFERROR(BDP($A44,"FUT_MONTH_YR"),"")</f>
+        <f>IFERROR(BDP($A44,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H44" s="18">
-        <f>IFERROR(BDP($A44,"FUT_DLV_DT_FIRST"),"")</f>
+        <f>IFERROR(BDP($A44,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="I44" s="18">
-        <f>IFERROR(BDP($A44,"LAST_TRADEABLE_DT"),"")</f>
+        <f>IFERROR(BDP($A44,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="J44" s="21">
-        <f>IFERROR(BDP($A44,"VOLUME"),"")</f>
+        <f>IFERROR(BDP($A44,"VOLUME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="K44" s="21">
-        <f>IFERROR(BDP($A44,"OPEN_INT"),"")</f>
+        <f>IFERROR(BDP($A44,"OPEN_INT"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>
@@ -6011,19 +6011,19 @@
         <v/>
       </c>
       <c r="E5" s="17">
-        <f>IFERROR(BDP(A5&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A5&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F5" s="17">
-        <f>IFERROR(BDP(A5&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A5&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G5" s="17">
-        <f>IFERROR(BDP(A5&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A5&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H5" s="25">
-        <f>IFERROR((E5+F5)/2,IFERROR(G5,""))</f>
+        <f>IFERROR((E5+F5)/2,IFERROR(G5,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I5" s="26" t="inlineStr">
@@ -6052,19 +6052,19 @@
         <v/>
       </c>
       <c r="E6" s="17">
-        <f>IFERROR(BDP(A6&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A6&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F6" s="17">
-        <f>IFERROR(BDP(A6&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A6&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G6" s="17">
-        <f>IFERROR(BDP(A6&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A6&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H6" s="25">
-        <f>IFERROR((E6+F6)/2,IFERROR(G6,""))</f>
+        <f>IFERROR((E6+F6)/2,IFERROR(G6,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I6" s="26" t="inlineStr"/>
@@ -6089,19 +6089,19 @@
         <v/>
       </c>
       <c r="E7" s="17">
-        <f>IFERROR(BDP(A7&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A7&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F7" s="17">
-        <f>IFERROR(BDP(A7&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A7&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G7" s="17">
-        <f>IFERROR(BDP(A7&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A7&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H7" s="25">
-        <f>IFERROR((E7+F7)/2,IFERROR(G7,""))</f>
+        <f>IFERROR((E7+F7)/2,IFERROR(G7,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I7" s="26" t="inlineStr"/>
@@ -6126,19 +6126,19 @@
         <v/>
       </c>
       <c r="E8" s="17">
-        <f>IFERROR(BDP(A8&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A8&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F8" s="17">
-        <f>IFERROR(BDP(A8&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A8&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G8" s="17">
-        <f>IFERROR(BDP(A8&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A8&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H8" s="25">
-        <f>IFERROR((E8+F8)/2,IFERROR(G8,""))</f>
+        <f>IFERROR((E8+F8)/2,IFERROR(G8,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I8" s="26" t="inlineStr">
@@ -6167,19 +6167,19 @@
         <v/>
       </c>
       <c r="E9" s="17">
-        <f>IFERROR(BDP(A9&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A9&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F9" s="17">
-        <f>IFERROR(BDP(A9&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A9&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G9" s="17">
-        <f>IFERROR(BDP(A9&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A9&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H9" s="25">
-        <f>IFERROR((E9+F9)/2,IFERROR(G9,""))</f>
+        <f>IFERROR((E9+F9)/2,IFERROR(G9,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I9" s="26" t="inlineStr"/>
@@ -6204,19 +6204,19 @@
         <v/>
       </c>
       <c r="E10" s="17">
-        <f>IFERROR(BDP(A10&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A10&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F10" s="17">
-        <f>IFERROR(BDP(A10&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A10&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G10" s="17">
-        <f>IFERROR(BDP(A10&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A10&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H10" s="25">
-        <f>IFERROR((E10+F10)/2,IFERROR(G10,""))</f>
+        <f>IFERROR((E10+F10)/2,IFERROR(G10,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I10" s="26" t="inlineStr">
@@ -6245,19 +6245,19 @@
         <v/>
       </c>
       <c r="E11" s="17">
-        <f>IFERROR(BDP(A11&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A11&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F11" s="17">
-        <f>IFERROR(BDP(A11&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A11&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G11" s="17">
-        <f>IFERROR(BDP(A11&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A11&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H11" s="25">
-        <f>IFERROR((E11+F11)/2,IFERROR(G11,""))</f>
+        <f>IFERROR((E11+F11)/2,IFERROR(G11,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I11" s="26" t="inlineStr"/>
@@ -6282,19 +6282,19 @@
         <v/>
       </c>
       <c r="E12" s="17">
-        <f>IFERROR(BDP(A12&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A12&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F12" s="17">
-        <f>IFERROR(BDP(A12&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A12&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G12" s="17">
-        <f>IFERROR(BDP(A12&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A12&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H12" s="25">
-        <f>IFERROR((E12+F12)/2,IFERROR(G12,""))</f>
+        <f>IFERROR((E12+F12)/2,IFERROR(G12,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I12" s="26" t="inlineStr"/>
@@ -6319,19 +6319,19 @@
         <v/>
       </c>
       <c r="E13" s="17">
-        <f>IFERROR(BDP(A13&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A13&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F13" s="17">
-        <f>IFERROR(BDP(A13&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A13&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G13" s="17">
-        <f>IFERROR(BDP(A13&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A13&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H13" s="25">
-        <f>IFERROR((E13+F13)/2,IFERROR(G13,""))</f>
+        <f>IFERROR((E13+F13)/2,IFERROR(G13,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I13" s="26" t="inlineStr">
@@ -6360,19 +6360,19 @@
         <v/>
       </c>
       <c r="E14" s="17">
-        <f>IFERROR(BDP(A14&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A14&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F14" s="17">
-        <f>IFERROR(BDP(A14&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A14&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G14" s="17">
-        <f>IFERROR(BDP(A14&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A14&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H14" s="25">
-        <f>IFERROR((E14+F14)/2,IFERROR(G14,""))</f>
+        <f>IFERROR((E14+F14)/2,IFERROR(G14,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I14" s="26" t="inlineStr"/>
@@ -6397,19 +6397,19 @@
         <v/>
       </c>
       <c r="E15" s="17">
-        <f>IFERROR(BDP(A15&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A15&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F15" s="17">
-        <f>IFERROR(BDP(A15&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A15&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G15" s="17">
-        <f>IFERROR(BDP(A15&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A15&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H15" s="25">
-        <f>IFERROR((E15+F15)/2,IFERROR(G15,""))</f>
+        <f>IFERROR((E15+F15)/2,IFERROR(G15,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I15" s="26" t="inlineStr"/>
@@ -6434,19 +6434,19 @@
         <v/>
       </c>
       <c r="E16" s="17">
-        <f>IFERROR(BDP(A16&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A16&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F16" s="17">
-        <f>IFERROR(BDP(A16&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A16&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G16" s="17">
-        <f>IFERROR(BDP(A16&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A16&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H16" s="25">
-        <f>IFERROR((E16+F16)/2,IFERROR(G16,""))</f>
+        <f>IFERROR((E16+F16)/2,IFERROR(G16,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I16" s="26" t="inlineStr"/>
@@ -6471,19 +6471,19 @@
         <v/>
       </c>
       <c r="E17" s="17">
-        <f>IFERROR(BDP(A17&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A17&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F17" s="17">
-        <f>IFERROR(BDP(A17&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A17&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G17" s="17">
-        <f>IFERROR(BDP(A17&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A17&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H17" s="25">
-        <f>IFERROR((E17+F17)/2,IFERROR(G17,""))</f>
+        <f>IFERROR((E17+F17)/2,IFERROR(G17,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I17" s="26" t="inlineStr"/>
@@ -6508,19 +6508,19 @@
         <v/>
       </c>
       <c r="E18" s="17">
-        <f>IFERROR(BDP(A18&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A18&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F18" s="17">
-        <f>IFERROR(BDP(A18&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A18&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G18" s="17">
-        <f>IFERROR(BDP(A18&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A18&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H18" s="25">
-        <f>IFERROR((E18+F18)/2,IFERROR(G18,""))</f>
+        <f>IFERROR((E18+F18)/2,IFERROR(G18,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I18" s="26" t="inlineStr"/>
@@ -6545,19 +6545,19 @@
         <v/>
       </c>
       <c r="E19" s="17">
-        <f>IFERROR(BDP(A19&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A19&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F19" s="17">
-        <f>IFERROR(BDP(A19&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A19&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G19" s="17">
-        <f>IFERROR(BDP(A19&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A19&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H19" s="25">
-        <f>IFERROR((E19+F19)/2,IFERROR(G19,""))</f>
+        <f>IFERROR((E19+F19)/2,IFERROR(G19,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I19" s="26" t="inlineStr"/>
@@ -6582,19 +6582,19 @@
         <v/>
       </c>
       <c r="E20" s="17">
-        <f>IFERROR(BDP(A20&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A20&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F20" s="17">
-        <f>IFERROR(BDP(A20&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A20&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G20" s="17">
-        <f>IFERROR(BDP(A20&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A20&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H20" s="25">
-        <f>IFERROR((E20+F20)/2,IFERROR(G20,""))</f>
+        <f>IFERROR((E20+F20)/2,IFERROR(G20,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I20" s="26" t="inlineStr"/>
@@ -6619,19 +6619,19 @@
         <v/>
       </c>
       <c r="E21" s="17">
-        <f>IFERROR(BDP(A21&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A21&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F21" s="17">
-        <f>IFERROR(BDP(A21&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A21&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G21" s="17">
-        <f>IFERROR(BDP(A21&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A21&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H21" s="25">
-        <f>IFERROR((E21+F21)/2,IFERROR(G21,""))</f>
+        <f>IFERROR((E21+F21)/2,IFERROR(G21,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I21" s="26" t="inlineStr"/>
@@ -6656,19 +6656,19 @@
         <v/>
       </c>
       <c r="E22" s="17">
-        <f>IFERROR(BDP(A22&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A22&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F22" s="17">
-        <f>IFERROR(BDP(A22&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A22&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G22" s="17">
-        <f>IFERROR(BDP(A22&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A22&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H22" s="25">
-        <f>IFERROR((E22+F22)/2,IFERROR(G22,""))</f>
+        <f>IFERROR((E22+F22)/2,IFERROR(G22,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I22" s="26" t="inlineStr"/>
@@ -6693,19 +6693,19 @@
         <v/>
       </c>
       <c r="E23" s="17">
-        <f>IFERROR(BDP(A23&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A23&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F23" s="17">
-        <f>IFERROR(BDP(A23&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A23&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G23" s="17">
-        <f>IFERROR(BDP(A23&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A23&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H23" s="25">
-        <f>IFERROR((E23+F23)/2,IFERROR(G23,""))</f>
+        <f>IFERROR((E23+F23)/2,IFERROR(G23,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I23" s="26" t="inlineStr"/>
@@ -6730,19 +6730,19 @@
         <v/>
       </c>
       <c r="E24" s="17">
-        <f>IFERROR(BDP(A24&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A24&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F24" s="17">
-        <f>IFERROR(BDP(A24&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A24&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G24" s="17">
-        <f>IFERROR(BDP(A24&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A24&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H24" s="25">
-        <f>IFERROR((E24+F24)/2,IFERROR(G24,""))</f>
+        <f>IFERROR((E24+F24)/2,IFERROR(G24,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I24" s="26" t="inlineStr">
@@ -6771,19 +6771,19 @@
         <v/>
       </c>
       <c r="E25" s="17">
-        <f>IFERROR(BDP(A25&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A25&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F25" s="17">
-        <f>IFERROR(BDP(A25&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A25&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G25" s="17">
-        <f>IFERROR(BDP(A25&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A25&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H25" s="25">
-        <f>IFERROR((E25+F25)/2,IFERROR(G25,""))</f>
+        <f>IFERROR((E25+F25)/2,IFERROR(G25,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I25" s="26" t="inlineStr">
@@ -6812,19 +6812,19 @@
         <v/>
       </c>
       <c r="E26" s="17">
-        <f>IFERROR(BDP(A26&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A26&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F26" s="17">
-        <f>IFERROR(BDP(A26&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A26&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G26" s="17">
-        <f>IFERROR(BDP(A26&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A26&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H26" s="25">
-        <f>IFERROR((E26+F26)/2,IFERROR(G26,""))</f>
+        <f>IFERROR((E26+F26)/2,IFERROR(G26,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I26" s="26" t="inlineStr">
@@ -6853,19 +6853,19 @@
         <v/>
       </c>
       <c r="E27" s="17">
-        <f>IFERROR(BDP(A27&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A27&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F27" s="17">
-        <f>IFERROR(BDP(A27&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A27&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G27" s="17">
-        <f>IFERROR(BDP(A27&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A27&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H27" s="25">
-        <f>IFERROR((E27+F27)/2,IFERROR(G27,""))</f>
+        <f>IFERROR((E27+F27)/2,IFERROR(G27,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I27" s="26" t="inlineStr">
@@ -6894,19 +6894,19 @@
         <v/>
       </c>
       <c r="E28" s="17">
-        <f>IFERROR(BDP(A28&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A28&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F28" s="17">
-        <f>IFERROR(BDP(A28&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A28&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G28" s="17">
-        <f>IFERROR(BDP(A28&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A28&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H28" s="25">
-        <f>IFERROR((E28+F28)/2,IFERROR(G28,""))</f>
+        <f>IFERROR((E28+F28)/2,IFERROR(G28,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I28" s="26" t="inlineStr">
@@ -6935,19 +6935,19 @@
         <v/>
       </c>
       <c r="E29" s="17">
-        <f>IFERROR(BDP(A29&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A29&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F29" s="17">
-        <f>IFERROR(BDP(A29&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A29&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G29" s="17">
-        <f>IFERROR(BDP(A29&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A29&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H29" s="25">
-        <f>IFERROR((E29+F29)/2,IFERROR(G29,""))</f>
+        <f>IFERROR((E29+F29)/2,IFERROR(G29,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I29" s="26" t="inlineStr">
@@ -6976,19 +6976,19 @@
         <v/>
       </c>
       <c r="E30" s="17">
-        <f>IFERROR(BDP(A30&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A30&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F30" s="17">
-        <f>IFERROR(BDP(A30&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A30&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G30" s="17">
-        <f>IFERROR(BDP(A30&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A30&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H30" s="25">
-        <f>IFERROR((E30+F30)/2,IFERROR(G30,""))</f>
+        <f>IFERROR((E30+F30)/2,IFERROR(G30,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I30" s="26" t="inlineStr">
@@ -7017,19 +7017,19 @@
         <v/>
       </c>
       <c r="E31" s="17">
-        <f>IFERROR(BDP(A31&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A31&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F31" s="17">
-        <f>IFERROR(BDP(A31&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A31&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G31" s="17">
-        <f>IFERROR(BDP(A31&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A31&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H31" s="25">
-        <f>IFERROR((E31+F31)/2,IFERROR(G31,""))</f>
+        <f>IFERROR((E31+F31)/2,IFERROR(G31,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I31" s="26" t="inlineStr">
@@ -7058,19 +7058,19 @@
         <v/>
       </c>
       <c r="E32" s="17">
-        <f>IFERROR(BDP(A32&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A32&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F32" s="17">
-        <f>IFERROR(BDP(A32&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A32&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G32" s="17">
-        <f>IFERROR(BDP(A32&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A32&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H32" s="25">
-        <f>IFERROR((E32+F32)/2,IFERROR(G32,""))</f>
+        <f>IFERROR((E32+F32)/2,IFERROR(G32,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I32" s="26" t="inlineStr">
@@ -7099,19 +7099,19 @@
         <v/>
       </c>
       <c r="E33" s="17">
-        <f>IFERROR(BDP(A33&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A33&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F33" s="17">
-        <f>IFERROR(BDP(A33&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A33&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G33" s="17">
-        <f>IFERROR(BDP(A33&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A33&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H33" s="25">
-        <f>IFERROR((E33+F33)/2,IFERROR(G33,""))</f>
+        <f>IFERROR((E33+F33)/2,IFERROR(G33,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I33" s="26" t="inlineStr">
@@ -7140,19 +7140,19 @@
         <v/>
       </c>
       <c r="E34" s="17">
-        <f>IFERROR(BDP(A34&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A34&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F34" s="17">
-        <f>IFERROR(BDP(A34&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A34&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G34" s="17">
-        <f>IFERROR(BDP(A34&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A34&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H34" s="25">
-        <f>IFERROR((E34+F34)/2,IFERROR(G34,""))</f>
+        <f>IFERROR((E34+F34)/2,IFERROR(G34,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I34" s="26" t="inlineStr">
@@ -7181,19 +7181,19 @@
         <v/>
       </c>
       <c r="E35" s="17">
-        <f>IFERROR(BDP(A35&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A35&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F35" s="17">
-        <f>IFERROR(BDP(A35&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A35&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G35" s="17">
-        <f>IFERROR(BDP(A35&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A35&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H35" s="25">
-        <f>IFERROR((E35+F35)/2,IFERROR(G35,""))</f>
+        <f>IFERROR((E35+F35)/2,IFERROR(G35,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I35" s="26" t="inlineStr">
@@ -7222,19 +7222,19 @@
         <v/>
       </c>
       <c r="E36" s="17">
-        <f>IFERROR(BDP(A36&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"")</f>
+        <f>IFERROR(BDP(A36&amp;" "&amp;PX_SRC&amp;" Curncy","PX_BID"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="F36" s="17">
-        <f>IFERROR(BDP(A36&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"")</f>
+        <f>IFERROR(BDP(A36&amp;" "&amp;PX_SRC&amp;" Curncy","PX_ASK"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="G36" s="17">
-        <f>IFERROR(BDP(A36&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"")</f>
+        <f>IFERROR(BDP(A36&amp;" "&amp;PX_SRC&amp;" Curncy","PX_LAST"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
       <c r="H36" s="25">
-        <f>IFERROR((E36+F36)/2,IFERROR(G36,""))</f>
+        <f>IFERROR((E36+F36)/2,IFERROR(G36,"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I36" s="26" t="inlineStr">
@@ -14377,7 +14377,7 @@
         </is>
       </c>
       <c r="B4" s="19">
-        <f>IFERROR(BDP(S490_TKR,"NAME"),"open in Bloomberg")</f>
+        <f>IFERROR(BDP(S490_TKR,"NAME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix curve fragility: middle segment falls back to OIS if futures unavailable
Root cause of the cascade break: the SR3 (SFRA) futures chain didn't populate on
the terminal, and because the middle (18M-5Y) DFs depended on it — and the long
end depends on the middle's annuity — the whole curve past 1Y went #VALUE!,
taking Curve_Interface, the pricer, and the charts with it.

Fix: middle DFs are now IFERROR(SR3 futures interp, OIS annual bootstrap). When
the futures load they drive the mid (as designed); when they don't, the mid
falls back to the pure-OIS curve so nothing downstream breaks. The DF-source
column (N) is now dynamic — shows 'SR3 futures' or 'OIS fallback' per pillar.
Formulas compile clean.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -7324,7 +7324,7 @@
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>SHORT (o/n–1Y): single-payment SOFR OIS, DF = 1/(1+S·tau0).  MIDDLE (1Y–5Y): the DF at 18M/2Y/3Y/4Y/5Y is interpolated off the SR3 futures chain (helper block cols O–W), which discounts each contract's forward rate forward from the OIS 1Y DF — so 18M/2Y…5Y here are driven by FUTURES, not the OIS pars (col E is shown only for reference).  LONG (5Y–50Y): annual SOFR OIS swaps, DF = (1−S·A_prior)/(1+S·taucoupon), with the annuity (col I) built from the short + futures DFs. Cutovers at 1Y and 5Y mean nothing overlaps. Paste S490 zeros into column L for the Δz check.</t>
+          <t>SHORT (o/n–1Y): single-payment SOFR OIS, DF = 1/(1+S·tau0).  MIDDLE (1Y–5Y): the DF at 18M/2Y/3Y/4Y/5Y is interpolated off the SR3 futures chain (helper block cols O–W), which discounts each contract's forward rate forward from the OIS 1Y DF — so 18M/2Y…5Y here are driven by FUTURES, not the OIS pars (col E is shown only for reference). If the SR3 chain is unavailable the middle DFs FALL BACK to the OIS bootstrap so the curve never breaks — col N shows which is live per pillar. LONG (5Y–50Y): annual SOFR OIS swaps, DF = (1−S·A_prior)/(1+S·taucoupon), annuity (col I) built from the short + middle DFs. Cutovers at 1Y and 5Y mean nothing overlaps. Paste S490 zeros into column L for the Δz check.</t>
         </is>
       </c>
       <c r="O5" s="13" t="inlineStr">
@@ -8969,7 +8969,7 @@
         <v/>
       </c>
       <c r="H23" s="29">
-        <f>IFERROR(INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1)))^((B23-INDEX($Y$8:$Y$28,MATCH(B23,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B23,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B23,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1)))</f>
+        <f>IFERROR(IFERROR(INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1)))^((B23-INDEX($Y$8:$Y$28,MATCH(B23,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B23,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B23,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1))),(1-(E23/100)*G23)/(1+(E23/100)*F23))</f>
         <v/>
       </c>
       <c r="I23" s="17" t="n">
@@ -8988,10 +8988,9 @@
         <f>IF(L23="","",(J23-L23)*100)</f>
         <v/>
       </c>
-      <c r="N23" s="6" t="inlineStr">
-        <is>
-          <t>SR3 futures</t>
-        </is>
+      <c r="N23" s="6">
+        <f>IF(ISNUMBER(IFERROR(INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1)))^((B23-INDEX($Y$8:$Y$28,MATCH(B23,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B23,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B23,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B23,$Y$8:$Y$28,1)))),"SR3 futures","OIS fallback")</f>
+        <v/>
       </c>
       <c r="O23" s="6">
         <f>'SOFR_Futures'!A22</f>
@@ -9069,7 +9068,7 @@
         <v/>
       </c>
       <c r="H24" s="29">
-        <f>IFERROR(INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1)))^((B24-INDEX($Y$8:$Y$28,MATCH(B24,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B24,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B24,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1)))</f>
+        <f>IFERROR(IFERROR(INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1)))^((B24-INDEX($Y$8:$Y$28,MATCH(B24,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B24,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B24,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1))),(1-(E24/100)*G24)/(1+(E24/100)*F24))</f>
         <v/>
       </c>
       <c r="I24" s="17">
@@ -9089,10 +9088,9 @@
         <f>IF(L24="","",(J24-L24)*100)</f>
         <v/>
       </c>
-      <c r="N24" s="6" t="inlineStr">
-        <is>
-          <t>SR3 futures</t>
-        </is>
+      <c r="N24" s="6">
+        <f>IF(ISNUMBER(IFERROR(INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1)))^((B24-INDEX($Y$8:$Y$28,MATCH(B24,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B24,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B24,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B24,$Y$8:$Y$28,1)))),"SR3 futures","OIS fallback")</f>
+        <v/>
       </c>
       <c r="O24" s="6">
         <f>'SOFR_Futures'!A23</f>
@@ -9170,7 +9168,7 @@
         <v/>
       </c>
       <c r="H25" s="29">
-        <f>IFERROR(INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1)))^((B25-INDEX($Y$8:$Y$28,MATCH(B25,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B25,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B25,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1)))</f>
+        <f>IFERROR(IFERROR(INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1)))^((B25-INDEX($Y$8:$Y$28,MATCH(B25,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B25,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B25,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1))),(1-(E25/100)*G25)/(1+(E25/100)*F25))</f>
         <v/>
       </c>
       <c r="I25" s="17">
@@ -9190,10 +9188,9 @@
         <f>IF(L25="","",(J25-L25)*100)</f>
         <v/>
       </c>
-      <c r="N25" s="6" t="inlineStr">
-        <is>
-          <t>SR3 futures</t>
-        </is>
+      <c r="N25" s="6">
+        <f>IF(ISNUMBER(IFERROR(INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1)))^((B25-INDEX($Y$8:$Y$28,MATCH(B25,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B25,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B25,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B25,$Y$8:$Y$28,1)))),"SR3 futures","OIS fallback")</f>
+        <v/>
       </c>
       <c r="O25" s="6">
         <f>'SOFR_Futures'!A24</f>
@@ -9271,7 +9268,7 @@
         <v/>
       </c>
       <c r="H26" s="29">
-        <f>IFERROR(INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1)))^((B26-INDEX($Y$8:$Y$28,MATCH(B26,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B26,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B26,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1)))</f>
+        <f>IFERROR(IFERROR(INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1)))^((B26-INDEX($Y$8:$Y$28,MATCH(B26,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B26,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B26,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1))),(1-(E26/100)*G26)/(1+(E26/100)*F26))</f>
         <v/>
       </c>
       <c r="I26" s="17">
@@ -9291,10 +9288,9 @@
         <f>IF(L26="","",(J26-L26)*100)</f>
         <v/>
       </c>
-      <c r="N26" s="6" t="inlineStr">
-        <is>
-          <t>SR3 futures</t>
-        </is>
+      <c r="N26" s="6">
+        <f>IF(ISNUMBER(IFERROR(INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1)))^((B26-INDEX($Y$8:$Y$28,MATCH(B26,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B26,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B26,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B26,$Y$8:$Y$28,1)))),"SR3 futures","OIS fallback")</f>
+        <v/>
       </c>
       <c r="O26" s="6">
         <f>'SOFR_Futures'!A25</f>
@@ -9372,7 +9368,7 @@
         <v/>
       </c>
       <c r="H27" s="29">
-        <f>IFERROR(INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1)))^((B27-INDEX($Y$8:$Y$28,MATCH(B27,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B27,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B27,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1)))</f>
+        <f>IFERROR(IFERROR(INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1)))^((B27-INDEX($Y$8:$Y$28,MATCH(B27,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B27,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B27,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1))),(1-(E27/100)*G27)/(1+(E27/100)*F27))</f>
         <v/>
       </c>
       <c r="I27" s="17">
@@ -9392,10 +9388,9 @@
         <f>IF(L27="","",(J27-L27)*100)</f>
         <v/>
       </c>
-      <c r="N27" s="6" t="inlineStr">
-        <is>
-          <t>SR3 futures</t>
-        </is>
+      <c r="N27" s="6">
+        <f>IF(ISNUMBER(IFERROR(INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1))*(INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1)+1)/INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1)))^((B27-INDEX($Y$8:$Y$28,MATCH(B27,$Y$8:$Y$28,1)))/(INDEX($Y$8:$Y$28,MATCH(B27,$Y$8:$Y$28,1)+1)-INDEX($Y$8:$Y$28,MATCH(B27,$Y$8:$Y$28,1)))),INDEX($Z$8:$Z$28,MATCH(B27,$Y$8:$Y$28,1)))),"SR3 futures","OIS fallback")</f>
+        <v/>
       </c>
       <c r="O27" s="6">
         <f>'SOFR_Futures'!A26</f>

</xml_diff>

<commit_message>
Complete CDS risk measures (Stage 7): IR01, Rec01, jump-to-default
Adds the full first-order risk suite to CDS_Pricer, finishing the CDS pricing:
- CS01 (per +1bp spread) = Notional*RPV01*1bp.
- IR01/DV01 (per +1bp SOFR) = net-leg dollar duration x 1bp (small for CDS).
- Rec01 (per +1% recovery) = -Notional*sum(protection factor)*1% (sticky-hazard).
- Jump-to-default = direction-aware LGD payout - current PV.

Validated numerically (5Y @95bp, mm): CS01 ,371, IR01 -, Rec01 -,668,
JTD .0mm (=N(1-R)). Formulas compile clean; no orphaned parts.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -7621,7 +7621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7817,26 +7817,89 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>CS01 (per 1bp spread)</t>
-        </is>
-      </c>
-      <c r="B19" s="42">
-        <f>B4*(B6/10000+0.0001)*B12-B4*(B6/10000)*B12</f>
-        <v/>
-      </c>
-      <c r="C19" s="16" t="inlineStr">
-        <is>
-          <t>≈ Notional*RPV01*1bp.</t>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="11" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>RISK MEASURES (analytic, first-order)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>CS01  (per +1bp spread)</t>
+        </is>
+      </c>
+      <c r="B22" s="42">
+        <f>B4*B12*0.0001</f>
+        <v/>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Spread DV01 = Notional*RPV01*1bp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>IR01 / DV01  (per +1bp SOFR)</t>
+        </is>
+      </c>
+      <c r="B23" s="42">
+        <f>-(B4*(1-B5)*SUMPRODUCT((CDS_Schedule!$C$7:$C$46&lt;=B8)*CDS_Schedule!$O$7:$O$46*CDS_Schedule!$F$7:$F$46)-B4*(B6/10000)*SUMPRODUCT((CDS_Schedule!$C$7:$C$46&lt;=B8)*(CDS_Schedule!$M$7:$M$46+CDS_Schedule!$N$7:$N$46)*CDS_Schedule!$F$7:$F$46))*0.0001</f>
+        <v/>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Net-leg dollar duration x 1bp (small for CDS).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Rec01  (per +1% recovery)</t>
+        </is>
+      </c>
+      <c r="B24" s="42">
+        <f>-B4*SUMIF(CDS_Schedule!$C$7:$C$46,"&lt;="&amp;B8,CDS_Schedule!$O$7:$O$46)*0.01</f>
+        <v/>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Sticky-hazard (hazards held; proper Rec01 re-fits spreads).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Jump-to-default (immediate)</t>
+        </is>
+      </c>
+      <c r="B25" s="43">
+        <f>IF(B9="Buy protection",B4*(1-B5),-B4*(1-B5))-B17</f>
+        <v/>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Default-now P&amp;L to your direction: LGD payout - current PV.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="9">
+    <mergeCell ref="C25:H25"/>
     <mergeCell ref="C6:H6"/>
-    <mergeCell ref="C19:H19"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="A21:H21"/>
     <mergeCell ref="C16:H16"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
     <mergeCell ref="C12:H12"/>
     <mergeCell ref="C15:H15"/>
   </mergeCells>

</xml_diff>

<commit_message>
Make futures actually drive the middle: quarterly-only SR3 chain
The SFRA chain mixes monthly-serial + quarterly SR3 contracts; chaining them as
contiguous periods over-discounted (the earlier 18M=0.57 garbage), so the guard
was rejecting the futures and the whole middle ran on OIS fallback.

Fix: each contract now uses its OWN 3-month reference period (EDATE(start,3)),
and only QUARTERLY contracts (ref start month in Mar/Jun/Sep/Dec) contribute to
the chain; monthly serials pass through (tau=0) so periods don't overlap.
Validated: quarterly chain gives 18M=0.942, 2Y=0.924 agreeing with OIS to
<0.002, so the guard now ACCEPTS the futures -> DF source flips to 'SR3 futures'.
The |diff|<0.03 guard stays as the safety net. Compiles clean.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -11379,7 +11379,7 @@
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>SHORT (o/n–1Y): single-payment SOFR OIS, DF = 1/(1+S·tau0).  MIDDLE (1Y–5Y): the DF at 18M/2Y/3Y/4Y/5Y is interpolated off the SR3 futures chain (helper block cols O–W), which discounts each contract's forward rate forward from the OIS 1Y DF — so 18M/2Y…5Y here are driven by FUTURES, not the OIS pars (col E is shown only for reference). If the SR3 chain is unavailable the middle DFs FALL BACK to the OIS bootstrap so the curve never breaks — col N shows which is live per pillar. LONG (5Y–50Y): annual SOFR OIS swaps, DF = (1−S·A_prior)/(1+S·taucoupon), annuity (col I) built from the short + middle DFs. Cutovers at 1Y and 5Y mean nothing overlaps. Paste S490 zeros into column L for the Δz check.</t>
+          <t>SHORT (o/n–1Y): single-payment SOFR OIS, DF = 1/(1+S·tau0).  MIDDLE (1Y–5Y): the DF at 18M/2Y/3Y/4Y/5Y is interpolated off the SR3 futures chain (helper block cols O–W), which chains the QUARTERLY contracts only (ref start Mar/Jun/Sep/Dec; monthly serials skipped) forward from the OIS 1Y DF — so 18M/2Y…5Y here are driven by FUTURES, not the OIS pars (col E is reference only). The middle DF uses the futures value only if it agrees with the OIS bootstrap (|diff|&lt;0.03), else it FALLS BACK to OIS so bad/mixed futures data can never break the curve — col N shows which is live per pillar. LONG (5Y–50Y): annual SOFR OIS swaps, DF = (1−S·A_prior)/(1+S·taucoupon), annuity (col I) built from the short + middle DFs. Cutovers at 1Y and 5Y mean nothing overlaps. Paste S490 zeros into column L for the Δz check.</t>
         </is>
       </c>
       <c r="O5" s="13" t="inlineStr">
@@ -11595,11 +11595,11 @@
         <v/>
       </c>
       <c r="Q8" s="18">
-        <f>'SOFR_Futures'!H8</f>
+        <f>EDATE(P8,3)</f>
         <v/>
       </c>
       <c r="R8" s="17">
-        <f>MAX(0,(Q8-MAX(P8,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P8)=3,MONTH(P8)=6,MONTH(P8)=9,MONTH(P8)=12),MAX(0,(Q8-MAX(P8,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S8" s="17">
@@ -11692,11 +11692,11 @@
         <v/>
       </c>
       <c r="Q9" s="18">
-        <f>'SOFR_Futures'!H9</f>
+        <f>EDATE(P9,3)</f>
         <v/>
       </c>
       <c r="R9" s="17">
-        <f>MAX(0,(Q9-MAX(P9,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P9)=3,MONTH(P9)=6,MONTH(P9)=9,MONTH(P9)=12),MAX(0,(Q9-MAX(P9,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S9" s="17">
@@ -11789,11 +11789,11 @@
         <v/>
       </c>
       <c r="Q10" s="18">
-        <f>'SOFR_Futures'!H10</f>
+        <f>EDATE(P10,3)</f>
         <v/>
       </c>
       <c r="R10" s="17">
-        <f>MAX(0,(Q10-MAX(P10,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P10)=3,MONTH(P10)=6,MONTH(P10)=9,MONTH(P10)=12),MAX(0,(Q10-MAX(P10,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S10" s="17">
@@ -11886,11 +11886,11 @@
         <v/>
       </c>
       <c r="Q11" s="18">
-        <f>'SOFR_Futures'!H11</f>
+        <f>EDATE(P11,3)</f>
         <v/>
       </c>
       <c r="R11" s="17">
-        <f>MAX(0,(Q11-MAX(P11,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P11)=3,MONTH(P11)=6,MONTH(P11)=9,MONTH(P11)=12),MAX(0,(Q11-MAX(P11,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S11" s="17">
@@ -11983,11 +11983,11 @@
         <v/>
       </c>
       <c r="Q12" s="18">
-        <f>'SOFR_Futures'!H12</f>
+        <f>EDATE(P12,3)</f>
         <v/>
       </c>
       <c r="R12" s="17">
-        <f>MAX(0,(Q12-MAX(P12,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P12)=3,MONTH(P12)=6,MONTH(P12)=9,MONTH(P12)=12),MAX(0,(Q12-MAX(P12,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S12" s="17">
@@ -12080,11 +12080,11 @@
         <v/>
       </c>
       <c r="Q13" s="18">
-        <f>'SOFR_Futures'!H13</f>
+        <f>EDATE(P13,3)</f>
         <v/>
       </c>
       <c r="R13" s="17">
-        <f>MAX(0,(Q13-MAX(P13,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P13)=3,MONTH(P13)=6,MONTH(P13)=9,MONTH(P13)=12),MAX(0,(Q13-MAX(P13,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S13" s="17">
@@ -12177,11 +12177,11 @@
         <v/>
       </c>
       <c r="Q14" s="18">
-        <f>'SOFR_Futures'!H14</f>
+        <f>EDATE(P14,3)</f>
         <v/>
       </c>
       <c r="R14" s="17">
-        <f>MAX(0,(Q14-MAX(P14,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P14)=3,MONTH(P14)=6,MONTH(P14)=9,MONTH(P14)=12),MAX(0,(Q14-MAX(P14,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S14" s="17">
@@ -12274,11 +12274,11 @@
         <v/>
       </c>
       <c r="Q15" s="18">
-        <f>'SOFR_Futures'!H15</f>
+        <f>EDATE(P15,3)</f>
         <v/>
       </c>
       <c r="R15" s="17">
-        <f>MAX(0,(Q15-MAX(P15,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P15)=3,MONTH(P15)=6,MONTH(P15)=9,MONTH(P15)=12),MAX(0,(Q15-MAX(P15,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S15" s="17">
@@ -12371,11 +12371,11 @@
         <v/>
       </c>
       <c r="Q16" s="18">
-        <f>'SOFR_Futures'!H16</f>
+        <f>EDATE(P16,3)</f>
         <v/>
       </c>
       <c r="R16" s="17">
-        <f>MAX(0,(Q16-MAX(P16,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P16)=3,MONTH(P16)=6,MONTH(P16)=9,MONTH(P16)=12),MAX(0,(Q16-MAX(P16,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S16" s="17">
@@ -12468,11 +12468,11 @@
         <v/>
       </c>
       <c r="Q17" s="18">
-        <f>'SOFR_Futures'!H17</f>
+        <f>EDATE(P17,3)</f>
         <v/>
       </c>
       <c r="R17" s="17">
-        <f>MAX(0,(Q17-MAX(P17,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P17)=3,MONTH(P17)=6,MONTH(P17)=9,MONTH(P17)=12),MAX(0,(Q17-MAX(P17,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S17" s="17">
@@ -12565,11 +12565,11 @@
         <v/>
       </c>
       <c r="Q18" s="18">
-        <f>'SOFR_Futures'!H18</f>
+        <f>EDATE(P18,3)</f>
         <v/>
       </c>
       <c r="R18" s="17">
-        <f>MAX(0,(Q18-MAX(P18,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P18)=3,MONTH(P18)=6,MONTH(P18)=9,MONTH(P18)=12),MAX(0,(Q18-MAX(P18,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S18" s="17">
@@ -12662,11 +12662,11 @@
         <v/>
       </c>
       <c r="Q19" s="18">
-        <f>'SOFR_Futures'!H19</f>
+        <f>EDATE(P19,3)</f>
         <v/>
       </c>
       <c r="R19" s="17">
-        <f>MAX(0,(Q19-MAX(P19,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P19)=3,MONTH(P19)=6,MONTH(P19)=9,MONTH(P19)=12),MAX(0,(Q19-MAX(P19,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S19" s="17">
@@ -12759,11 +12759,11 @@
         <v/>
       </c>
       <c r="Q20" s="18">
-        <f>'SOFR_Futures'!H20</f>
+        <f>EDATE(P20,3)</f>
         <v/>
       </c>
       <c r="R20" s="17">
-        <f>MAX(0,(Q20-MAX(P20,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P20)=3,MONTH(P20)=6,MONTH(P20)=9,MONTH(P20)=12),MAX(0,(Q20-MAX(P20,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S20" s="17">
@@ -12856,11 +12856,11 @@
         <v/>
       </c>
       <c r="Q21" s="18">
-        <f>'SOFR_Futures'!H21</f>
+        <f>EDATE(P21,3)</f>
         <v/>
       </c>
       <c r="R21" s="17">
-        <f>MAX(0,(Q21-MAX(P21,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P21)=3,MONTH(P21)=6,MONTH(P21)=9,MONTH(P21)=12),MAX(0,(Q21-MAX(P21,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S21" s="17">
@@ -12957,11 +12957,11 @@
         <v/>
       </c>
       <c r="Q22" s="18">
-        <f>'SOFR_Futures'!H22</f>
+        <f>EDATE(P22,3)</f>
         <v/>
       </c>
       <c r="R22" s="17">
-        <f>MAX(0,(Q22-MAX(P22,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P22)=3,MONTH(P22)=6,MONTH(P22)=9,MONTH(P22)=12),MAX(0,(Q22-MAX(P22,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S22" s="17">
@@ -13056,11 +13056,11 @@
         <v/>
       </c>
       <c r="Q23" s="18">
-        <f>'SOFR_Futures'!H23</f>
+        <f>EDATE(P23,3)</f>
         <v/>
       </c>
       <c r="R23" s="17">
-        <f>MAX(0,(Q23-MAX(P23,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P23)=3,MONTH(P23)=6,MONTH(P23)=9,MONTH(P23)=12),MAX(0,(Q23-MAX(P23,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S23" s="17">
@@ -13156,11 +13156,11 @@
         <v/>
       </c>
       <c r="Q24" s="18">
-        <f>'SOFR_Futures'!H24</f>
+        <f>EDATE(P24,3)</f>
         <v/>
       </c>
       <c r="R24" s="17">
-        <f>MAX(0,(Q24-MAX(P24,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P24)=3,MONTH(P24)=6,MONTH(P24)=9,MONTH(P24)=12),MAX(0,(Q24-MAX(P24,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S24" s="17">
@@ -13256,11 +13256,11 @@
         <v/>
       </c>
       <c r="Q25" s="18">
-        <f>'SOFR_Futures'!H25</f>
+        <f>EDATE(P25,3)</f>
         <v/>
       </c>
       <c r="R25" s="17">
-        <f>MAX(0,(Q25-MAX(P25,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P25)=3,MONTH(P25)=6,MONTH(P25)=9,MONTH(P25)=12),MAX(0,(Q25-MAX(P25,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S25" s="17">
@@ -13356,11 +13356,11 @@
         <v/>
       </c>
       <c r="Q26" s="18">
-        <f>'SOFR_Futures'!H26</f>
+        <f>EDATE(P26,3)</f>
         <v/>
       </c>
       <c r="R26" s="17">
-        <f>MAX(0,(Q26-MAX(P26,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P26)=3,MONTH(P26)=6,MONTH(P26)=9,MONTH(P26)=12),MAX(0,(Q26-MAX(P26,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S26" s="17">
@@ -13460,7 +13460,7 @@
         <v/>
       </c>
       <c r="R27" s="17">
-        <f>MAX(0,(Q27-MAX(P27,$B$22))/360)</f>
+        <f>IF(OR(MONTH(P27)=3,MONTH(P27)=6,MONTH(P27)=9,MONTH(P27)=12),MAX(0,(Q27-MAX(P27,$B$22))/360),0)</f>
         <v/>
       </c>
       <c r="S27" s="17">

</xml_diff>

<commit_message>
Zero the long-end curve difference: flat-forward gap-DF interpolation
Gap-year discount factors (11Y,13Y,14Y,16-19Y,...) are now flat-forward
(log-linear) interpolated between the bracketing quoted-pillar DFs, so the whole
curve is a true step-function-forward curve (Bloomberg S490 default). The quoted
swaps re-solve off those gap DFs, making a small circular system that Excel's
iterative calculation (now enabled, 100 iterations, delta 1e-10) converges in a
few passes.

Validated in Python vs Bloomberg's S490 output: this drives the zero-curve
difference to ~0.00 bp at every node including 40Y/50Y (was up to 0.7bp with
linear rate interpolation). XML clean, round-trips, no orphaned parts.
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -34,7 +34,7 @@
     <definedName name="SOFR_TKR">Instructions!$B$13</definedName>
     <definedName name="S490_TKR">Instructions!$B$14</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1" iterate="1" iterateCount="100" iterateDelta="1e-10"/>
 </workbook>
 </file>
 
@@ -15990,7 +15990,7 @@
         <v/>
       </c>
       <c r="H33" s="29">
-        <f>($D$4-(E33/100)*G33)/(1+(E33/100)*F33)</f>
+        <f>H32*(H34/H32)^((C33-C32)/(C34-C32))</f>
         <v/>
       </c>
       <c r="I33" s="17">
@@ -16104,7 +16104,7 @@
         <v/>
       </c>
       <c r="H35" s="29">
-        <f>($D$4-(E35/100)*G35)/(1+(E35/100)*F35)</f>
+        <f>H34*(H37/H34)^((C35-C34)/(C37-C34))</f>
         <v/>
       </c>
       <c r="I35" s="17">
@@ -16161,7 +16161,7 @@
         <v/>
       </c>
       <c r="H36" s="29">
-        <f>($D$4-(E36/100)*G36)/(1+(E36/100)*F36)</f>
+        <f>H34*(H37/H34)^((C36-C34)/(C37-C34))</f>
         <v/>
       </c>
       <c r="I36" s="17">
@@ -16275,7 +16275,7 @@
         <v/>
       </c>
       <c r="H38" s="29">
-        <f>($D$4-(E38/100)*G38)/(1+(E38/100)*F38)</f>
+        <f>H37*(H42/H37)^((C38-C37)/(C42-C37))</f>
         <v/>
       </c>
       <c r="I38" s="17">
@@ -16332,7 +16332,7 @@
         <v/>
       </c>
       <c r="H39" s="29">
-        <f>($D$4-(E39/100)*G39)/(1+(E39/100)*F39)</f>
+        <f>H37*(H42/H37)^((C39-C37)/(C42-C37))</f>
         <v/>
       </c>
       <c r="I39" s="17">
@@ -16389,7 +16389,7 @@
         <v/>
       </c>
       <c r="H40" s="29">
-        <f>($D$4-(E40/100)*G40)/(1+(E40/100)*F40)</f>
+        <f>H37*(H42/H37)^((C40-C37)/(C42-C37))</f>
         <v/>
       </c>
       <c r="I40" s="17">
@@ -16446,7 +16446,7 @@
         <v/>
       </c>
       <c r="H41" s="29">
-        <f>($D$4-(E41/100)*G41)/(1+(E41/100)*F41)</f>
+        <f>H37*(H42/H37)^((C41-C37)/(C42-C37))</f>
         <v/>
       </c>
       <c r="I41" s="17">
@@ -16560,7 +16560,7 @@
         <v/>
       </c>
       <c r="H43" s="29">
-        <f>($D$4-(E43/100)*G43)/(1+(E43/100)*F43)</f>
+        <f>H42*(H47/H42)^((C43-C42)/(C47-C42))</f>
         <v/>
       </c>
       <c r="I43" s="17">
@@ -16617,7 +16617,7 @@
         <v/>
       </c>
       <c r="H44" s="29">
-        <f>($D$4-(E44/100)*G44)/(1+(E44/100)*F44)</f>
+        <f>H42*(H47/H42)^((C44-C42)/(C47-C42))</f>
         <v/>
       </c>
       <c r="I44" s="17">
@@ -16674,7 +16674,7 @@
         <v/>
       </c>
       <c r="H45" s="29">
-        <f>($D$4-(E45/100)*G45)/(1+(E45/100)*F45)</f>
+        <f>H42*(H47/H42)^((C45-C42)/(C47-C42))</f>
         <v/>
       </c>
       <c r="I45" s="17">
@@ -16731,7 +16731,7 @@
         <v/>
       </c>
       <c r="H46" s="29">
-        <f>($D$4-(E46/100)*G46)/(1+(E46/100)*F46)</f>
+        <f>H42*(H47/H42)^((C46-C42)/(C47-C42))</f>
         <v/>
       </c>
       <c r="I46" s="17">
@@ -16845,7 +16845,7 @@
         <v/>
       </c>
       <c r="H48" s="29">
-        <f>($D$4-(E48/100)*G48)/(1+(E48/100)*F48)</f>
+        <f>H47*(H52/H47)^((C48-C47)/(C52-C47))</f>
         <v/>
       </c>
       <c r="I48" s="17">
@@ -16902,7 +16902,7 @@
         <v/>
       </c>
       <c r="H49" s="29">
-        <f>($D$4-(E49/100)*G49)/(1+(E49/100)*F49)</f>
+        <f>H47*(H52/H47)^((C49-C47)/(C52-C47))</f>
         <v/>
       </c>
       <c r="I49" s="17">
@@ -16959,7 +16959,7 @@
         <v/>
       </c>
       <c r="H50" s="29">
-        <f>($D$4-(E50/100)*G50)/(1+(E50/100)*F50)</f>
+        <f>H47*(H52/H47)^((C50-C47)/(C52-C47))</f>
         <v/>
       </c>
       <c r="I50" s="17">
@@ -17016,7 +17016,7 @@
         <v/>
       </c>
       <c r="H51" s="29">
-        <f>($D$4-(E51/100)*G51)/(1+(E51/100)*F51)</f>
+        <f>H47*(H52/H47)^((C51-C47)/(C52-C47))</f>
         <v/>
       </c>
       <c r="I51" s="17">
@@ -17130,7 +17130,7 @@
         <v/>
       </c>
       <c r="H53" s="29">
-        <f>($D$4-(E53/100)*G53)/(1+(E53/100)*F53)</f>
+        <f>H52*(H62/H52)^((C53-C52)/(C62-C52))</f>
         <v/>
       </c>
       <c r="I53" s="17">
@@ -17187,7 +17187,7 @@
         <v/>
       </c>
       <c r="H54" s="29">
-        <f>($D$4-(E54/100)*G54)/(1+(E54/100)*F54)</f>
+        <f>H52*(H62/H52)^((C54-C52)/(C62-C52))</f>
         <v/>
       </c>
       <c r="I54" s="17">
@@ -17244,7 +17244,7 @@
         <v/>
       </c>
       <c r="H55" s="29">
-        <f>($D$4-(E55/100)*G55)/(1+(E55/100)*F55)</f>
+        <f>H52*(H62/H52)^((C55-C52)/(C62-C52))</f>
         <v/>
       </c>
       <c r="I55" s="17">
@@ -17301,7 +17301,7 @@
         <v/>
       </c>
       <c r="H56" s="29">
-        <f>($D$4-(E56/100)*G56)/(1+(E56/100)*F56)</f>
+        <f>H52*(H62/H52)^((C56-C52)/(C62-C52))</f>
         <v/>
       </c>
       <c r="I56" s="17">
@@ -17358,7 +17358,7 @@
         <v/>
       </c>
       <c r="H57" s="29">
-        <f>($D$4-(E57/100)*G57)/(1+(E57/100)*F57)</f>
+        <f>H52*(H62/H52)^((C57-C52)/(C62-C52))</f>
         <v/>
       </c>
       <c r="I57" s="17">
@@ -17415,7 +17415,7 @@
         <v/>
       </c>
       <c r="H58" s="29">
-        <f>($D$4-(E58/100)*G58)/(1+(E58/100)*F58)</f>
+        <f>H52*(H62/H52)^((C58-C52)/(C62-C52))</f>
         <v/>
       </c>
       <c r="I58" s="17">
@@ -17472,7 +17472,7 @@
         <v/>
       </c>
       <c r="H59" s="29">
-        <f>($D$4-(E59/100)*G59)/(1+(E59/100)*F59)</f>
+        <f>H52*(H62/H52)^((C59-C52)/(C62-C52))</f>
         <v/>
       </c>
       <c r="I59" s="17">
@@ -17529,7 +17529,7 @@
         <v/>
       </c>
       <c r="H60" s="29">
-        <f>($D$4-(E60/100)*G60)/(1+(E60/100)*F60)</f>
+        <f>H52*(H62/H52)^((C60-C52)/(C62-C52))</f>
         <v/>
       </c>
       <c r="I60" s="17">
@@ -17586,7 +17586,7 @@
         <v/>
       </c>
       <c r="H61" s="29">
-        <f>($D$4-(E61/100)*G61)/(1+(E61/100)*F61)</f>
+        <f>H52*(H62/H52)^((C61-C52)/(C62-C52))</f>
         <v/>
       </c>
       <c r="I61" s="17">
@@ -17700,7 +17700,7 @@
         <v/>
       </c>
       <c r="H63" s="29">
-        <f>($D$4-(E63/100)*G63)/(1+(E63/100)*F63)</f>
+        <f>H62*(H72/H62)^((C63-C62)/(C72-C62))</f>
         <v/>
       </c>
       <c r="I63" s="17">
@@ -17757,7 +17757,7 @@
         <v/>
       </c>
       <c r="H64" s="29">
-        <f>($D$4-(E64/100)*G64)/(1+(E64/100)*F64)</f>
+        <f>H62*(H72/H62)^((C64-C62)/(C72-C62))</f>
         <v/>
       </c>
       <c r="I64" s="17">
@@ -17814,7 +17814,7 @@
         <v/>
       </c>
       <c r="H65" s="29">
-        <f>($D$4-(E65/100)*G65)/(1+(E65/100)*F65)</f>
+        <f>H62*(H72/H62)^((C65-C62)/(C72-C62))</f>
         <v/>
       </c>
       <c r="I65" s="17">
@@ -17871,7 +17871,7 @@
         <v/>
       </c>
       <c r="H66" s="29">
-        <f>($D$4-(E66/100)*G66)/(1+(E66/100)*F66)</f>
+        <f>H62*(H72/H62)^((C66-C62)/(C72-C62))</f>
         <v/>
       </c>
       <c r="I66" s="17">
@@ -17928,7 +17928,7 @@
         <v/>
       </c>
       <c r="H67" s="29">
-        <f>($D$4-(E67/100)*G67)/(1+(E67/100)*F67)</f>
+        <f>H62*(H72/H62)^((C67-C62)/(C72-C62))</f>
         <v/>
       </c>
       <c r="I67" s="17">
@@ -17985,7 +17985,7 @@
         <v/>
       </c>
       <c r="H68" s="29">
-        <f>($D$4-(E68/100)*G68)/(1+(E68/100)*F68)</f>
+        <f>H62*(H72/H62)^((C68-C62)/(C72-C62))</f>
         <v/>
       </c>
       <c r="I68" s="17">
@@ -18042,7 +18042,7 @@
         <v/>
       </c>
       <c r="H69" s="29">
-        <f>($D$4-(E69/100)*G69)/(1+(E69/100)*F69)</f>
+        <f>H62*(H72/H62)^((C69-C62)/(C72-C62))</f>
         <v/>
       </c>
       <c r="I69" s="17">
@@ -18099,7 +18099,7 @@
         <v/>
       </c>
       <c r="H70" s="29">
-        <f>($D$4-(E70/100)*G70)/(1+(E70/100)*F70)</f>
+        <f>H62*(H72/H62)^((C70-C62)/(C72-C62))</f>
         <v/>
       </c>
       <c r="I70" s="17">
@@ -18156,7 +18156,7 @@
         <v/>
       </c>
       <c r="H71" s="29">
-        <f>($D$4-(E71/100)*G71)/(1+(E71/100)*F71)</f>
+        <f>H62*(H72/H62)^((C71-C62)/(C72-C62))</f>
         <v/>
       </c>
       <c r="I71" s="17">

</xml_diff>

<commit_message>
Pull the S490 benchmark curve live via BDS
Column D read from a manual paste. Wire it to BDS(CURVE_TENOR_RATES), matched by
maturity date. The dump's schema is unverified, so the column offsets are inputs
(I3/I4/I5) with a matched-count that makes a wrong guess obvious rather than
silently comparing against the wrong tenors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -43,7 +43,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.00000000"/>
@@ -54,6 +54,7 @@
     <numFmt numFmtId="171" formatCode="0.0000000000"/>
     <numFmt numFmtId="172" formatCode="0.00000"/>
     <numFmt numFmtId="173" formatCode="mm/dd/yy"/>
+    <numFmt numFmtId="174" formatCode="0.###"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -214,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -341,6 +342,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="12" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="12" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="14" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6589,7 +6594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6612,6 +6617,21 @@
           <t>Bloomberg's own USD SOFR curve (S490 / YCSW0490 Index) — benchmark for your bootstrap, not an input</t>
         </is>
       </c>
+      <c r="H2" s="67" t="inlineStr">
+        <is>
+          <t>LIVE BENCHMARK — BDS dump controls</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="H3" s="94" t="inlineStr">
+        <is>
+          <t>Dump col holding MATURITY DATE</t>
+        </is>
+      </c>
+      <c r="I3" s="95" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
@@ -6623,6 +6643,14 @@
         <f>IFERROR(BDP(S490_TKR,"NAME"),"ERROR PLZ FIX")</f>
         <v/>
       </c>
+      <c r="H4" s="94" t="inlineStr">
+        <is>
+          <t>Dump col holding ZERO RATE</t>
+        </is>
+      </c>
+      <c r="I4" s="95" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
@@ -6634,11 +6662,24 @@
         <f>VAL_DATE</f>
         <v/>
       </c>
+      <c r="H5" s="94" t="inlineStr">
+        <is>
+          <t>Zero units (1 = pct, 100 = decimal)</t>
+        </is>
+      </c>
+      <c r="I5" s="96" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Paste Bloomberg's S490 zero rates (from YCSW0490 &lt;GO&gt; or SWDF) into the yellow column D, tenor for tenor; column E then shows Δz = your bootstrap − Bloomberg in bp (single digits = agreement). The raw BDS(CURVE_TENOR_RATES) dump is off to the right (cols H:I) as an optional live pull — its column order is Bloomberg-defined, so verify before relying on it.</t>
+      <c r="A6" s="70" t="inlineStr">
+        <is>
+          <t>Column D pulls Bloomberg's own S490 zero curve live from the BDS dump and falls back to the manual paste in column G. Column E is your bootstrap minus Bloomberg, in bp — single digits = agreement.</t>
+        </is>
+      </c>
+      <c r="H6" s="66" t="inlineStr">
+        <is>
+          <t>VERIFY I3/I4/I5 against the dump at J12 before trusting column E — the defaults are a GUESS at the CURVE_TENOR_RATES schema, not confirmed.</t>
         </is>
       </c>
     </row>
@@ -6658,9 +6699,9 @@
           <t>Your zero (%)</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>S490 zero (%) [paste]</t>
+      <c r="D7" s="92" t="inlineStr">
+        <is>
+          <t>S490 zero (%) — live</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
@@ -6668,9 +6709,19 @@
           <t>Δz (bp)</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
-        <is>
-          <t>Raw CURVE_TENOR_RATES (verify order)</t>
+      <c r="F7" s="62" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="G7" s="62" t="inlineStr">
+        <is>
+          <t>S490 zero (%) [manual paste]</t>
+        </is>
+      </c>
+      <c r="H7" s="67" t="inlineStr">
+        <is>
+          <t>Raw CURVE_TENOR_RATES dump (spills right and down from J12)</t>
         </is>
       </c>
     </row>
@@ -6687,11 +6738,19 @@
         <f>Bootstrap!J8</f>
         <v/>
       </c>
-      <c r="D8" s="30" t="n"/>
-      <c r="E8" s="31">
-        <f>IF(D8="","",(C8-D8)*100)</f>
-        <v/>
-      </c>
+      <c r="D8" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B8,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G8),G8,""))</f>
+        <v/>
+      </c>
+      <c r="E8" s="89">
+        <f>IF(OR(D8="",NOT(ISNUMBER(D8))),"",(C8-D8)*100)</f>
+        <v/>
+      </c>
+      <c r="F8" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B8,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G8),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G8" s="85" t="n"/>
       <c r="H8">
         <f>BDS(S490_TKR,"CURVE_TENOR_RATES")</f>
         <v/>
@@ -6710,11 +6769,19 @@
         <f>Bootstrap!J9</f>
         <v/>
       </c>
-      <c r="D9" s="30" t="n"/>
-      <c r="E9" s="31">
-        <f>IF(D9="","",(C9-D9)*100)</f>
-        <v/>
-      </c>
+      <c r="D9" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B9,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G9),G9,""))</f>
+        <v/>
+      </c>
+      <c r="E9" s="89">
+        <f>IF(OR(D9="",NOT(ISNUMBER(D9))),"",(C9-D9)*100)</f>
+        <v/>
+      </c>
+      <c r="F9" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B9,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G9),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G9" s="85" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6">
@@ -6729,11 +6796,19 @@
         <f>Bootstrap!J10</f>
         <v/>
       </c>
-      <c r="D10" s="30" t="n"/>
-      <c r="E10" s="31">
-        <f>IF(D10="","",(C10-D10)*100)</f>
-        <v/>
-      </c>
+      <c r="D10" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B10,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G10),G10,""))</f>
+        <v/>
+      </c>
+      <c r="E10" s="89">
+        <f>IF(OR(D10="",NOT(ISNUMBER(D10))),"",(C10-D10)*100)</f>
+        <v/>
+      </c>
+      <c r="F10" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B10,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G10),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G10" s="85" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6">
@@ -6748,11 +6823,19 @@
         <f>Bootstrap!J11</f>
         <v/>
       </c>
-      <c r="D11" s="30" t="n"/>
-      <c r="E11" s="31">
-        <f>IF(D11="","",(C11-D11)*100)</f>
-        <v/>
-      </c>
+      <c r="D11" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B11,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G11),G11,""))</f>
+        <v/>
+      </c>
+      <c r="E11" s="89">
+        <f>IF(OR(D11="",NOT(ISNUMBER(D11))),"",(C11-D11)*100)</f>
+        <v/>
+      </c>
+      <c r="F11" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B11,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G11),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G11" s="85" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6">
@@ -6767,9 +6850,21 @@
         <f>Bootstrap!J12</f>
         <v/>
       </c>
-      <c r="D12" s="30" t="n"/>
-      <c r="E12" s="31">
-        <f>IF(D12="","",(C12-D12)*100)</f>
+      <c r="D12" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B12,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G12),G12,""))</f>
+        <v/>
+      </c>
+      <c r="E12" s="89">
+        <f>IF(OR(D12="",NOT(ISNUMBER(D12))),"",(C12-D12)*100)</f>
+        <v/>
+      </c>
+      <c r="F12" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B12,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G12),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G12" s="85" t="n"/>
+      <c r="J12" s="93">
+        <f>BDS(S490_TKR,"CURVE_TENOR_RATES")</f>
         <v/>
       </c>
     </row>
@@ -6786,11 +6881,19 @@
         <f>Bootstrap!J13</f>
         <v/>
       </c>
-      <c r="D13" s="30" t="n"/>
-      <c r="E13" s="31">
-        <f>IF(D13="","",(C13-D13)*100)</f>
-        <v/>
-      </c>
+      <c r="D13" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B13,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G13),G13,""))</f>
+        <v/>
+      </c>
+      <c r="E13" s="89">
+        <f>IF(OR(D13="",NOT(ISNUMBER(D13))),"",(C13-D13)*100)</f>
+        <v/>
+      </c>
+      <c r="F13" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B13,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G13),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G13" s="85" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6">
@@ -6805,11 +6908,19 @@
         <f>Bootstrap!J14</f>
         <v/>
       </c>
-      <c r="D14" s="30" t="n"/>
-      <c r="E14" s="31">
-        <f>IF(D14="","",(C14-D14)*100)</f>
-        <v/>
-      </c>
+      <c r="D14" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B14,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G14),G14,""))</f>
+        <v/>
+      </c>
+      <c r="E14" s="89">
+        <f>IF(OR(D14="",NOT(ISNUMBER(D14))),"",(C14-D14)*100)</f>
+        <v/>
+      </c>
+      <c r="F14" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B14,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G14),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G14" s="85" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6">
@@ -6824,11 +6935,19 @@
         <f>Bootstrap!J15</f>
         <v/>
       </c>
-      <c r="D15" s="30" t="n"/>
-      <c r="E15" s="31">
-        <f>IF(D15="","",(C15-D15)*100)</f>
-        <v/>
-      </c>
+      <c r="D15" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B15,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G15),G15,""))</f>
+        <v/>
+      </c>
+      <c r="E15" s="89">
+        <f>IF(OR(D15="",NOT(ISNUMBER(D15))),"",(C15-D15)*100)</f>
+        <v/>
+      </c>
+      <c r="F15" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B15,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G15),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G15" s="85" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6">
@@ -6843,11 +6962,19 @@
         <f>Bootstrap!J16</f>
         <v/>
       </c>
-      <c r="D16" s="30" t="n"/>
-      <c r="E16" s="31">
-        <f>IF(D16="","",(C16-D16)*100)</f>
-        <v/>
-      </c>
+      <c r="D16" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B16,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G16),G16,""))</f>
+        <v/>
+      </c>
+      <c r="E16" s="89">
+        <f>IF(OR(D16="",NOT(ISNUMBER(D16))),"",(C16-D16)*100)</f>
+        <v/>
+      </c>
+      <c r="F16" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B16,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G16),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G16" s="85" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6">
@@ -6862,11 +6989,19 @@
         <f>Bootstrap!J17</f>
         <v/>
       </c>
-      <c r="D17" s="30" t="n"/>
-      <c r="E17" s="31">
-        <f>IF(D17="","",(C17-D17)*100)</f>
-        <v/>
-      </c>
+      <c r="D17" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B17,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G17),G17,""))</f>
+        <v/>
+      </c>
+      <c r="E17" s="89">
+        <f>IF(OR(D17="",NOT(ISNUMBER(D17))),"",(C17-D17)*100)</f>
+        <v/>
+      </c>
+      <c r="F17" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B17,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G17),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G17" s="85" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6">
@@ -6881,11 +7016,19 @@
         <f>Bootstrap!J18</f>
         <v/>
       </c>
-      <c r="D18" s="30" t="n"/>
-      <c r="E18" s="31">
-        <f>IF(D18="","",(C18-D18)*100)</f>
-        <v/>
-      </c>
+      <c r="D18" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B18,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G18),G18,""))</f>
+        <v/>
+      </c>
+      <c r="E18" s="89">
+        <f>IF(OR(D18="",NOT(ISNUMBER(D18))),"",(C18-D18)*100)</f>
+        <v/>
+      </c>
+      <c r="F18" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B18,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G18),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G18" s="85" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6">
@@ -6900,11 +7043,19 @@
         <f>Bootstrap!J19</f>
         <v/>
       </c>
-      <c r="D19" s="30" t="n"/>
-      <c r="E19" s="31">
-        <f>IF(D19="","",(C19-D19)*100)</f>
-        <v/>
-      </c>
+      <c r="D19" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B19,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G19),G19,""))</f>
+        <v/>
+      </c>
+      <c r="E19" s="89">
+        <f>IF(OR(D19="",NOT(ISNUMBER(D19))),"",(C19-D19)*100)</f>
+        <v/>
+      </c>
+      <c r="F19" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B19,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G19),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G19" s="85" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6">
@@ -6919,11 +7070,19 @@
         <f>Bootstrap!J20</f>
         <v/>
       </c>
-      <c r="D20" s="30" t="n"/>
-      <c r="E20" s="31">
-        <f>IF(D20="","",(C20-D20)*100)</f>
-        <v/>
-      </c>
+      <c r="D20" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B20,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G20),G20,""))</f>
+        <v/>
+      </c>
+      <c r="E20" s="89">
+        <f>IF(OR(D20="",NOT(ISNUMBER(D20))),"",(C20-D20)*100)</f>
+        <v/>
+      </c>
+      <c r="F20" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B20,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G20),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G20" s="85" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6">
@@ -6938,11 +7097,19 @@
         <f>Bootstrap!J21</f>
         <v/>
       </c>
-      <c r="D21" s="30" t="n"/>
-      <c r="E21" s="31">
-        <f>IF(D21="","",(C21-D21)*100)</f>
-        <v/>
-      </c>
+      <c r="D21" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B21,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G21),G21,""))</f>
+        <v/>
+      </c>
+      <c r="E21" s="89">
+        <f>IF(OR(D21="",NOT(ISNUMBER(D21))),"",(C21-D21)*100)</f>
+        <v/>
+      </c>
+      <c r="F21" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B21,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G21),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G21" s="85" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6">
@@ -6957,11 +7124,19 @@
         <f>Bootstrap!J22</f>
         <v/>
       </c>
-      <c r="D22" s="30" t="n"/>
-      <c r="E22" s="31">
-        <f>IF(D22="","",(C22-D22)*100)</f>
-        <v/>
-      </c>
+      <c r="D22" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B22,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G22),G22,""))</f>
+        <v/>
+      </c>
+      <c r="E22" s="89">
+        <f>IF(OR(D22="",NOT(ISNUMBER(D22))),"",(C22-D22)*100)</f>
+        <v/>
+      </c>
+      <c r="F22" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B22,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G22),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G22" s="85" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6">
@@ -6976,11 +7151,19 @@
         <f>Bootstrap!J23</f>
         <v/>
       </c>
-      <c r="D23" s="30" t="n"/>
-      <c r="E23" s="31">
-        <f>IF(D23="","",(C23-D23)*100)</f>
-        <v/>
-      </c>
+      <c r="D23" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B23,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G23),G23,""))</f>
+        <v/>
+      </c>
+      <c r="E23" s="89">
+        <f>IF(OR(D23="",NOT(ISNUMBER(D23))),"",(C23-D23)*100)</f>
+        <v/>
+      </c>
+      <c r="F23" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B23,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G23),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G23" s="85" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6">
@@ -6995,11 +7178,19 @@
         <f>Bootstrap!J24</f>
         <v/>
       </c>
-      <c r="D24" s="30" t="n"/>
-      <c r="E24" s="31">
-        <f>IF(D24="","",(C24-D24)*100)</f>
-        <v/>
-      </c>
+      <c r="D24" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B24,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G24),G24,""))</f>
+        <v/>
+      </c>
+      <c r="E24" s="89">
+        <f>IF(OR(D24="",NOT(ISNUMBER(D24))),"",(C24-D24)*100)</f>
+        <v/>
+      </c>
+      <c r="F24" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B24,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G24),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G24" s="85" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6">
@@ -7014,11 +7205,19 @@
         <f>Bootstrap!J25</f>
         <v/>
       </c>
-      <c r="D25" s="30" t="n"/>
-      <c r="E25" s="31">
-        <f>IF(D25="","",(C25-D25)*100)</f>
-        <v/>
-      </c>
+      <c r="D25" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B25,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G25),G25,""))</f>
+        <v/>
+      </c>
+      <c r="E25" s="89">
+        <f>IF(OR(D25="",NOT(ISNUMBER(D25))),"",(C25-D25)*100)</f>
+        <v/>
+      </c>
+      <c r="F25" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B25,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G25),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G25" s="85" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6">
@@ -7033,11 +7232,19 @@
         <f>Bootstrap!J26</f>
         <v/>
       </c>
-      <c r="D26" s="30" t="n"/>
-      <c r="E26" s="31">
-        <f>IF(D26="","",(C26-D26)*100)</f>
-        <v/>
-      </c>
+      <c r="D26" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B26,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G26),G26,""))</f>
+        <v/>
+      </c>
+      <c r="E26" s="89">
+        <f>IF(OR(D26="",NOT(ISNUMBER(D26))),"",(C26-D26)*100)</f>
+        <v/>
+      </c>
+      <c r="F26" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B26,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G26),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G26" s="85" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6">
@@ -7052,11 +7259,19 @@
         <f>Bootstrap!J27</f>
         <v/>
       </c>
-      <c r="D27" s="30" t="n"/>
-      <c r="E27" s="31">
-        <f>IF(D27="","",(C27-D27)*100)</f>
-        <v/>
-      </c>
+      <c r="D27" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B27,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G27),G27,""))</f>
+        <v/>
+      </c>
+      <c r="E27" s="89">
+        <f>IF(OR(D27="",NOT(ISNUMBER(D27))),"",(C27-D27)*100)</f>
+        <v/>
+      </c>
+      <c r="F27" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B27,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G27),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G27" s="85" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6">
@@ -7071,11 +7286,19 @@
         <f>Bootstrap!J28</f>
         <v/>
       </c>
-      <c r="D28" s="30" t="n"/>
-      <c r="E28" s="31">
-        <f>IF(D28="","",(C28-D28)*100)</f>
-        <v/>
-      </c>
+      <c r="D28" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B28,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G28),G28,""))</f>
+        <v/>
+      </c>
+      <c r="E28" s="89">
+        <f>IF(OR(D28="",NOT(ISNUMBER(D28))),"",(C28-D28)*100)</f>
+        <v/>
+      </c>
+      <c r="F28" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B28,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G28),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G28" s="85" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6">
@@ -7090,11 +7313,19 @@
         <f>Bootstrap!J29</f>
         <v/>
       </c>
-      <c r="D29" s="30" t="n"/>
-      <c r="E29" s="31">
-        <f>IF(D29="","",(C29-D29)*100)</f>
-        <v/>
-      </c>
+      <c r="D29" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B29,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G29),G29,""))</f>
+        <v/>
+      </c>
+      <c r="E29" s="89">
+        <f>IF(OR(D29="",NOT(ISNUMBER(D29))),"",(C29-D29)*100)</f>
+        <v/>
+      </c>
+      <c r="F29" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B29,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G29),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G29" s="85" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6">
@@ -7109,11 +7340,19 @@
         <f>Bootstrap!J30</f>
         <v/>
       </c>
-      <c r="D30" s="30" t="n"/>
-      <c r="E30" s="31">
-        <f>IF(D30="","",(C30-D30)*100)</f>
-        <v/>
-      </c>
+      <c r="D30" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B30,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G30),G30,""))</f>
+        <v/>
+      </c>
+      <c r="E30" s="89">
+        <f>IF(OR(D30="",NOT(ISNUMBER(D30))),"",(C30-D30)*100)</f>
+        <v/>
+      </c>
+      <c r="F30" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B30,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G30),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G30" s="85" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6">
@@ -7128,11 +7367,19 @@
         <f>Bootstrap!J31</f>
         <v/>
       </c>
-      <c r="D31" s="30" t="n"/>
-      <c r="E31" s="31">
-        <f>IF(D31="","",(C31-D31)*100)</f>
-        <v/>
-      </c>
+      <c r="D31" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B31,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G31),G31,""))</f>
+        <v/>
+      </c>
+      <c r="E31" s="89">
+        <f>IF(OR(D31="",NOT(ISNUMBER(D31))),"",(C31-D31)*100)</f>
+        <v/>
+      </c>
+      <c r="F31" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B31,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G31),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G31" s="85" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6">
@@ -7147,11 +7394,19 @@
         <f>Bootstrap!J32</f>
         <v/>
       </c>
-      <c r="D32" s="30" t="n"/>
-      <c r="E32" s="31">
-        <f>IF(D32="","",(C32-D32)*100)</f>
-        <v/>
-      </c>
+      <c r="D32" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B32,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G32),G32,""))</f>
+        <v/>
+      </c>
+      <c r="E32" s="89">
+        <f>IF(OR(D32="",NOT(ISNUMBER(D32))),"",(C32-D32)*100)</f>
+        <v/>
+      </c>
+      <c r="F32" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B32,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G32),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G32" s="85" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6">
@@ -7166,11 +7421,19 @@
         <f>Bootstrap!J33</f>
         <v/>
       </c>
-      <c r="D33" s="30" t="n"/>
-      <c r="E33" s="31">
-        <f>IF(D33="","",(C33-D33)*100)</f>
-        <v/>
-      </c>
+      <c r="D33" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B33,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G33),G33,""))</f>
+        <v/>
+      </c>
+      <c r="E33" s="89">
+        <f>IF(OR(D33="",NOT(ISNUMBER(D33))),"",(C33-D33)*100)</f>
+        <v/>
+      </c>
+      <c r="F33" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B33,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G33),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G33" s="85" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6">
@@ -7185,11 +7448,19 @@
         <f>Bootstrap!J34</f>
         <v/>
       </c>
-      <c r="D34" s="30" t="n"/>
-      <c r="E34" s="31">
-        <f>IF(D34="","",(C34-D34)*100)</f>
-        <v/>
-      </c>
+      <c r="D34" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B34,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G34),G34,""))</f>
+        <v/>
+      </c>
+      <c r="E34" s="89">
+        <f>IF(OR(D34="",NOT(ISNUMBER(D34))),"",(C34-D34)*100)</f>
+        <v/>
+      </c>
+      <c r="F34" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B34,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G34),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G34" s="85" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6">
@@ -7204,11 +7475,19 @@
         <f>Bootstrap!J35</f>
         <v/>
       </c>
-      <c r="D35" s="30" t="n"/>
-      <c r="E35" s="31">
-        <f>IF(D35="","",(C35-D35)*100)</f>
-        <v/>
-      </c>
+      <c r="D35" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B35,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G35),G35,""))</f>
+        <v/>
+      </c>
+      <c r="E35" s="89">
+        <f>IF(OR(D35="",NOT(ISNUMBER(D35))),"",(C35-D35)*100)</f>
+        <v/>
+      </c>
+      <c r="F35" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B35,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G35),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G35" s="85" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6">
@@ -7223,11 +7502,19 @@
         <f>Bootstrap!J36</f>
         <v/>
       </c>
-      <c r="D36" s="30" t="n"/>
-      <c r="E36" s="31">
-        <f>IF(D36="","",(C36-D36)*100)</f>
-        <v/>
-      </c>
+      <c r="D36" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B36,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G36),G36,""))</f>
+        <v/>
+      </c>
+      <c r="E36" s="89">
+        <f>IF(OR(D36="",NOT(ISNUMBER(D36))),"",(C36-D36)*100)</f>
+        <v/>
+      </c>
+      <c r="F36" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B36,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G36),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G36" s="85" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6">
@@ -7242,11 +7529,19 @@
         <f>Bootstrap!J37</f>
         <v/>
       </c>
-      <c r="D37" s="30" t="n"/>
-      <c r="E37" s="31">
-        <f>IF(D37="","",(C37-D37)*100)</f>
-        <v/>
-      </c>
+      <c r="D37" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B37,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G37),G37,""))</f>
+        <v/>
+      </c>
+      <c r="E37" s="89">
+        <f>IF(OR(D37="",NOT(ISNUMBER(D37))),"",(C37-D37)*100)</f>
+        <v/>
+      </c>
+      <c r="F37" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B37,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G37),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G37" s="85" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6">
@@ -7261,11 +7556,19 @@
         <f>Bootstrap!J38</f>
         <v/>
       </c>
-      <c r="D38" s="30" t="n"/>
-      <c r="E38" s="31">
-        <f>IF(D38="","",(C38-D38)*100)</f>
-        <v/>
-      </c>
+      <c r="D38" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B38,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G38),G38,""))</f>
+        <v/>
+      </c>
+      <c r="E38" s="89">
+        <f>IF(OR(D38="",NOT(ISNUMBER(D38))),"",(C38-D38)*100)</f>
+        <v/>
+      </c>
+      <c r="F38" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B38,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G38),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G38" s="85" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6">
@@ -7280,11 +7583,19 @@
         <f>Bootstrap!J39</f>
         <v/>
       </c>
-      <c r="D39" s="30" t="n"/>
-      <c r="E39" s="31">
-        <f>IF(D39="","",(C39-D39)*100)</f>
-        <v/>
-      </c>
+      <c r="D39" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B39,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G39),G39,""))</f>
+        <v/>
+      </c>
+      <c r="E39" s="89">
+        <f>IF(OR(D39="",NOT(ISNUMBER(D39))),"",(C39-D39)*100)</f>
+        <v/>
+      </c>
+      <c r="F39" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B39,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G39),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G39" s="85" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6">
@@ -7299,11 +7610,19 @@
         <f>Bootstrap!J40</f>
         <v/>
       </c>
-      <c r="D40" s="30" t="n"/>
-      <c r="E40" s="31">
-        <f>IF(D40="","",(C40-D40)*100)</f>
-        <v/>
-      </c>
+      <c r="D40" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B40,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G40),G40,""))</f>
+        <v/>
+      </c>
+      <c r="E40" s="89">
+        <f>IF(OR(D40="",NOT(ISNUMBER(D40))),"",(C40-D40)*100)</f>
+        <v/>
+      </c>
+      <c r="F40" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B40,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G40),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G40" s="85" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="6">
@@ -7318,11 +7637,19 @@
         <f>Bootstrap!J41</f>
         <v/>
       </c>
-      <c r="D41" s="30" t="n"/>
-      <c r="E41" s="31">
-        <f>IF(D41="","",(C41-D41)*100)</f>
-        <v/>
-      </c>
+      <c r="D41" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B41,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G41),G41,""))</f>
+        <v/>
+      </c>
+      <c r="E41" s="89">
+        <f>IF(OR(D41="",NOT(ISNUMBER(D41))),"",(C41-D41)*100)</f>
+        <v/>
+      </c>
+      <c r="F41" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B41,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G41),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G41" s="85" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6">
@@ -7337,11 +7664,19 @@
         <f>Bootstrap!J42</f>
         <v/>
       </c>
-      <c r="D42" s="30" t="n"/>
-      <c r="E42" s="31">
-        <f>IF(D42="","",(C42-D42)*100)</f>
-        <v/>
-      </c>
+      <c r="D42" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B42,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G42),G42,""))</f>
+        <v/>
+      </c>
+      <c r="E42" s="89">
+        <f>IF(OR(D42="",NOT(ISNUMBER(D42))),"",(C42-D42)*100)</f>
+        <v/>
+      </c>
+      <c r="F42" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B42,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G42),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G42" s="85" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6">
@@ -7356,11 +7691,19 @@
         <f>Bootstrap!J43</f>
         <v/>
       </c>
-      <c r="D43" s="30" t="n"/>
-      <c r="E43" s="31">
-        <f>IF(D43="","",(C43-D43)*100)</f>
-        <v/>
-      </c>
+      <c r="D43" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B43,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G43),G43,""))</f>
+        <v/>
+      </c>
+      <c r="E43" s="89">
+        <f>IF(OR(D43="",NOT(ISNUMBER(D43))),"",(C43-D43)*100)</f>
+        <v/>
+      </c>
+      <c r="F43" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B43,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G43),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G43" s="85" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="6">
@@ -7375,11 +7718,19 @@
         <f>Bootstrap!J44</f>
         <v/>
       </c>
-      <c r="D44" s="30" t="n"/>
-      <c r="E44" s="31">
-        <f>IF(D44="","",(C44-D44)*100)</f>
-        <v/>
-      </c>
+      <c r="D44" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B44,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G44),G44,""))</f>
+        <v/>
+      </c>
+      <c r="E44" s="89">
+        <f>IF(OR(D44="",NOT(ISNUMBER(D44))),"",(C44-D44)*100)</f>
+        <v/>
+      </c>
+      <c r="F44" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B44,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G44),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G44" s="85" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6">
@@ -7394,11 +7745,19 @@
         <f>Bootstrap!J45</f>
         <v/>
       </c>
-      <c r="D45" s="30" t="n"/>
-      <c r="E45" s="31">
-        <f>IF(D45="","",(C45-D45)*100)</f>
-        <v/>
-      </c>
+      <c r="D45" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B45,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G45),G45,""))</f>
+        <v/>
+      </c>
+      <c r="E45" s="89">
+        <f>IF(OR(D45="",NOT(ISNUMBER(D45))),"",(C45-D45)*100)</f>
+        <v/>
+      </c>
+      <c r="F45" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B45,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G45),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G45" s="85" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6">
@@ -7413,11 +7772,19 @@
         <f>Bootstrap!J46</f>
         <v/>
       </c>
-      <c r="D46" s="30" t="n"/>
-      <c r="E46" s="31">
-        <f>IF(D46="","",(C46-D46)*100)</f>
-        <v/>
-      </c>
+      <c r="D46" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B46,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G46),G46,""))</f>
+        <v/>
+      </c>
+      <c r="E46" s="89">
+        <f>IF(OR(D46="",NOT(ISNUMBER(D46))),"",(C46-D46)*100)</f>
+        <v/>
+      </c>
+      <c r="F46" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B46,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G46),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G46" s="85" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6">
@@ -7432,11 +7799,19 @@
         <f>Bootstrap!J47</f>
         <v/>
       </c>
-      <c r="D47" s="30" t="n"/>
-      <c r="E47" s="31">
-        <f>IF(D47="","",(C47-D47)*100)</f>
-        <v/>
-      </c>
+      <c r="D47" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B47,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G47),G47,""))</f>
+        <v/>
+      </c>
+      <c r="E47" s="89">
+        <f>IF(OR(D47="",NOT(ISNUMBER(D47))),"",(C47-D47)*100)</f>
+        <v/>
+      </c>
+      <c r="F47" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B47,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G47),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G47" s="85" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6">
@@ -7451,11 +7826,19 @@
         <f>Bootstrap!J48</f>
         <v/>
       </c>
-      <c r="D48" s="30" t="n"/>
-      <c r="E48" s="31">
-        <f>IF(D48="","",(C48-D48)*100)</f>
-        <v/>
-      </c>
+      <c r="D48" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B48,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G48),G48,""))</f>
+        <v/>
+      </c>
+      <c r="E48" s="89">
+        <f>IF(OR(D48="",NOT(ISNUMBER(D48))),"",(C48-D48)*100)</f>
+        <v/>
+      </c>
+      <c r="F48" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B48,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G48),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G48" s="85" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6">
@@ -7470,11 +7853,19 @@
         <f>Bootstrap!J49</f>
         <v/>
       </c>
-      <c r="D49" s="30" t="n"/>
-      <c r="E49" s="31">
-        <f>IF(D49="","",(C49-D49)*100)</f>
-        <v/>
-      </c>
+      <c r="D49" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B49,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G49),G49,""))</f>
+        <v/>
+      </c>
+      <c r="E49" s="89">
+        <f>IF(OR(D49="",NOT(ISNUMBER(D49))),"",(C49-D49)*100)</f>
+        <v/>
+      </c>
+      <c r="F49" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B49,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G49),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G49" s="85" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="6">
@@ -7489,11 +7880,19 @@
         <f>Bootstrap!J50</f>
         <v/>
       </c>
-      <c r="D50" s="30" t="n"/>
-      <c r="E50" s="31">
-        <f>IF(D50="","",(C50-D50)*100)</f>
-        <v/>
-      </c>
+      <c r="D50" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B50,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G50),G50,""))</f>
+        <v/>
+      </c>
+      <c r="E50" s="89">
+        <f>IF(OR(D50="",NOT(ISNUMBER(D50))),"",(C50-D50)*100)</f>
+        <v/>
+      </c>
+      <c r="F50" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B50,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G50),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G50" s="85" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6">
@@ -7508,11 +7907,19 @@
         <f>Bootstrap!J51</f>
         <v/>
       </c>
-      <c r="D51" s="30" t="n"/>
-      <c r="E51" s="31">
-        <f>IF(D51="","",(C51-D51)*100)</f>
-        <v/>
-      </c>
+      <c r="D51" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B51,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G51),G51,""))</f>
+        <v/>
+      </c>
+      <c r="E51" s="89">
+        <f>IF(OR(D51="",NOT(ISNUMBER(D51))),"",(C51-D51)*100)</f>
+        <v/>
+      </c>
+      <c r="F51" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B51,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G51),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G51" s="85" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6">
@@ -7527,11 +7934,19 @@
         <f>Bootstrap!J52</f>
         <v/>
       </c>
-      <c r="D52" s="30" t="n"/>
-      <c r="E52" s="31">
-        <f>IF(D52="","",(C52-D52)*100)</f>
-        <v/>
-      </c>
+      <c r="D52" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B52,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G52),G52,""))</f>
+        <v/>
+      </c>
+      <c r="E52" s="89">
+        <f>IF(OR(D52="",NOT(ISNUMBER(D52))),"",(C52-D52)*100)</f>
+        <v/>
+      </c>
+      <c r="F52" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B52,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G52),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G52" s="85" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6">
@@ -7546,11 +7961,19 @@
         <f>Bootstrap!J53</f>
         <v/>
       </c>
-      <c r="D53" s="30" t="n"/>
-      <c r="E53" s="31">
-        <f>IF(D53="","",(C53-D53)*100)</f>
-        <v/>
-      </c>
+      <c r="D53" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B53,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G53),G53,""))</f>
+        <v/>
+      </c>
+      <c r="E53" s="89">
+        <f>IF(OR(D53="",NOT(ISNUMBER(D53))),"",(C53-D53)*100)</f>
+        <v/>
+      </c>
+      <c r="F53" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B53,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G53),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G53" s="85" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6">
@@ -7565,11 +7988,19 @@
         <f>Bootstrap!J54</f>
         <v/>
       </c>
-      <c r="D54" s="30" t="n"/>
-      <c r="E54" s="31">
-        <f>IF(D54="","",(C54-D54)*100)</f>
-        <v/>
-      </c>
+      <c r="D54" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B54,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G54),G54,""))</f>
+        <v/>
+      </c>
+      <c r="E54" s="89">
+        <f>IF(OR(D54="",NOT(ISNUMBER(D54))),"",(C54-D54)*100)</f>
+        <v/>
+      </c>
+      <c r="F54" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B54,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G54),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G54" s="85" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6">
@@ -7584,11 +8015,19 @@
         <f>Bootstrap!J55</f>
         <v/>
       </c>
-      <c r="D55" s="30" t="n"/>
-      <c r="E55" s="31">
-        <f>IF(D55="","",(C55-D55)*100)</f>
-        <v/>
-      </c>
+      <c r="D55" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B55,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G55),G55,""))</f>
+        <v/>
+      </c>
+      <c r="E55" s="89">
+        <f>IF(OR(D55="",NOT(ISNUMBER(D55))),"",(C55-D55)*100)</f>
+        <v/>
+      </c>
+      <c r="F55" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B55,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G55),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G55" s="85" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="6">
@@ -7603,11 +8042,19 @@
         <f>Bootstrap!J56</f>
         <v/>
       </c>
-      <c r="D56" s="30" t="n"/>
-      <c r="E56" s="31">
-        <f>IF(D56="","",(C56-D56)*100)</f>
-        <v/>
-      </c>
+      <c r="D56" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B56,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G56),G56,""))</f>
+        <v/>
+      </c>
+      <c r="E56" s="89">
+        <f>IF(OR(D56="",NOT(ISNUMBER(D56))),"",(C56-D56)*100)</f>
+        <v/>
+      </c>
+      <c r="F56" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B56,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G56),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G56" s="85" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="6">
@@ -7622,11 +8069,19 @@
         <f>Bootstrap!J57</f>
         <v/>
       </c>
-      <c r="D57" s="30" t="n"/>
-      <c r="E57" s="31">
-        <f>IF(D57="","",(C57-D57)*100)</f>
-        <v/>
-      </c>
+      <c r="D57" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B57,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G57),G57,""))</f>
+        <v/>
+      </c>
+      <c r="E57" s="89">
+        <f>IF(OR(D57="",NOT(ISNUMBER(D57))),"",(C57-D57)*100)</f>
+        <v/>
+      </c>
+      <c r="F57" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B57,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G57),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G57" s="85" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="6">
@@ -7641,11 +8096,19 @@
         <f>Bootstrap!J58</f>
         <v/>
       </c>
-      <c r="D58" s="30" t="n"/>
-      <c r="E58" s="31">
-        <f>IF(D58="","",(C58-D58)*100)</f>
-        <v/>
-      </c>
+      <c r="D58" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B58,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G58),G58,""))</f>
+        <v/>
+      </c>
+      <c r="E58" s="89">
+        <f>IF(OR(D58="",NOT(ISNUMBER(D58))),"",(C58-D58)*100)</f>
+        <v/>
+      </c>
+      <c r="F58" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B58,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G58),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G58" s="85" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="6">
@@ -7660,11 +8123,19 @@
         <f>Bootstrap!J59</f>
         <v/>
       </c>
-      <c r="D59" s="30" t="n"/>
-      <c r="E59" s="31">
-        <f>IF(D59="","",(C59-D59)*100)</f>
-        <v/>
-      </c>
+      <c r="D59" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B59,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G59),G59,""))</f>
+        <v/>
+      </c>
+      <c r="E59" s="89">
+        <f>IF(OR(D59="",NOT(ISNUMBER(D59))),"",(C59-D59)*100)</f>
+        <v/>
+      </c>
+      <c r="F59" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B59,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G59),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G59" s="85" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="6">
@@ -7679,11 +8150,19 @@
         <f>Bootstrap!J60</f>
         <v/>
       </c>
-      <c r="D60" s="30" t="n"/>
-      <c r="E60" s="31">
-        <f>IF(D60="","",(C60-D60)*100)</f>
-        <v/>
-      </c>
+      <c r="D60" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B60,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G60),G60,""))</f>
+        <v/>
+      </c>
+      <c r="E60" s="89">
+        <f>IF(OR(D60="",NOT(ISNUMBER(D60))),"",(C60-D60)*100)</f>
+        <v/>
+      </c>
+      <c r="F60" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B60,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G60),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G60" s="85" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="6">
@@ -7698,11 +8177,19 @@
         <f>Bootstrap!J61</f>
         <v/>
       </c>
-      <c r="D61" s="30" t="n"/>
-      <c r="E61" s="31">
-        <f>IF(D61="","",(C61-D61)*100)</f>
-        <v/>
-      </c>
+      <c r="D61" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B61,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G61),G61,""))</f>
+        <v/>
+      </c>
+      <c r="E61" s="89">
+        <f>IF(OR(D61="",NOT(ISNUMBER(D61))),"",(C61-D61)*100)</f>
+        <v/>
+      </c>
+      <c r="F61" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B61,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G61),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G61" s="85" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="6">
@@ -7717,11 +8204,19 @@
         <f>Bootstrap!J62</f>
         <v/>
       </c>
-      <c r="D62" s="30" t="n"/>
-      <c r="E62" s="31">
-        <f>IF(D62="","",(C62-D62)*100)</f>
-        <v/>
-      </c>
+      <c r="D62" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B62,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G62),G62,""))</f>
+        <v/>
+      </c>
+      <c r="E62" s="89">
+        <f>IF(OR(D62="",NOT(ISNUMBER(D62))),"",(C62-D62)*100)</f>
+        <v/>
+      </c>
+      <c r="F62" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B62,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G62),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G62" s="85" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="6">
@@ -7736,11 +8231,19 @@
         <f>Bootstrap!J63</f>
         <v/>
       </c>
-      <c r="D63" s="30" t="n"/>
-      <c r="E63" s="31">
-        <f>IF(D63="","",(C63-D63)*100)</f>
-        <v/>
-      </c>
+      <c r="D63" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B63,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G63),G63,""))</f>
+        <v/>
+      </c>
+      <c r="E63" s="89">
+        <f>IF(OR(D63="",NOT(ISNUMBER(D63))),"",(C63-D63)*100)</f>
+        <v/>
+      </c>
+      <c r="F63" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B63,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G63),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G63" s="85" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="6">
@@ -7755,11 +8258,19 @@
         <f>Bootstrap!J64</f>
         <v/>
       </c>
-      <c r="D64" s="30" t="n"/>
-      <c r="E64" s="31">
-        <f>IF(D64="","",(C64-D64)*100)</f>
-        <v/>
-      </c>
+      <c r="D64" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B64,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G64),G64,""))</f>
+        <v/>
+      </c>
+      <c r="E64" s="89">
+        <f>IF(OR(D64="",NOT(ISNUMBER(D64))),"",(C64-D64)*100)</f>
+        <v/>
+      </c>
+      <c r="F64" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B64,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G64),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G64" s="85" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="6">
@@ -7774,11 +8285,19 @@
         <f>Bootstrap!J65</f>
         <v/>
       </c>
-      <c r="D65" s="30" t="n"/>
-      <c r="E65" s="31">
-        <f>IF(D65="","",(C65-D65)*100)</f>
-        <v/>
-      </c>
+      <c r="D65" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B65,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G65),G65,""))</f>
+        <v/>
+      </c>
+      <c r="E65" s="89">
+        <f>IF(OR(D65="",NOT(ISNUMBER(D65))),"",(C65-D65)*100)</f>
+        <v/>
+      </c>
+      <c r="F65" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B65,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G65),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G65" s="85" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="6">
@@ -7793,11 +8312,19 @@
         <f>Bootstrap!J66</f>
         <v/>
       </c>
-      <c r="D66" s="30" t="n"/>
-      <c r="E66" s="31">
-        <f>IF(D66="","",(C66-D66)*100)</f>
-        <v/>
-      </c>
+      <c r="D66" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B66,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G66),G66,""))</f>
+        <v/>
+      </c>
+      <c r="E66" s="89">
+        <f>IF(OR(D66="",NOT(ISNUMBER(D66))),"",(C66-D66)*100)</f>
+        <v/>
+      </c>
+      <c r="F66" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B66,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G66),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G66" s="85" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="6">
@@ -7812,11 +8339,19 @@
         <f>Bootstrap!J67</f>
         <v/>
       </c>
-      <c r="D67" s="30" t="n"/>
-      <c r="E67" s="31">
-        <f>IF(D67="","",(C67-D67)*100)</f>
-        <v/>
-      </c>
+      <c r="D67" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B67,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G67),G67,""))</f>
+        <v/>
+      </c>
+      <c r="E67" s="89">
+        <f>IF(OR(D67="",NOT(ISNUMBER(D67))),"",(C67-D67)*100)</f>
+        <v/>
+      </c>
+      <c r="F67" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B67,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G67),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G67" s="85" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="6">
@@ -7831,11 +8366,19 @@
         <f>Bootstrap!J68</f>
         <v/>
       </c>
-      <c r="D68" s="30" t="n"/>
-      <c r="E68" s="31">
-        <f>IF(D68="","",(C68-D68)*100)</f>
-        <v/>
-      </c>
+      <c r="D68" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B68,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G68),G68,""))</f>
+        <v/>
+      </c>
+      <c r="E68" s="89">
+        <f>IF(OR(D68="",NOT(ISNUMBER(D68))),"",(C68-D68)*100)</f>
+        <v/>
+      </c>
+      <c r="F68" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B68,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G68),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G68" s="85" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="6">
@@ -7850,11 +8393,19 @@
         <f>Bootstrap!J69</f>
         <v/>
       </c>
-      <c r="D69" s="30" t="n"/>
-      <c r="E69" s="31">
-        <f>IF(D69="","",(C69-D69)*100)</f>
-        <v/>
-      </c>
+      <c r="D69" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B69,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G69),G69,""))</f>
+        <v/>
+      </c>
+      <c r="E69" s="89">
+        <f>IF(OR(D69="",NOT(ISNUMBER(D69))),"",(C69-D69)*100)</f>
+        <v/>
+      </c>
+      <c r="F69" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B69,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G69),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G69" s="85" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="6">
@@ -7869,11 +8420,19 @@
         <f>Bootstrap!J70</f>
         <v/>
       </c>
-      <c r="D70" s="30" t="n"/>
-      <c r="E70" s="31">
-        <f>IF(D70="","",(C70-D70)*100)</f>
-        <v/>
-      </c>
+      <c r="D70" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B70,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G70),G70,""))</f>
+        <v/>
+      </c>
+      <c r="E70" s="89">
+        <f>IF(OR(D70="",NOT(ISNUMBER(D70))),"",(C70-D70)*100)</f>
+        <v/>
+      </c>
+      <c r="F70" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B70,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G70),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G70" s="85" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="6">
@@ -7888,11 +8447,19 @@
         <f>Bootstrap!J71</f>
         <v/>
       </c>
-      <c r="D71" s="30" t="n"/>
-      <c r="E71" s="31">
-        <f>IF(D71="","",(C71-D71)*100)</f>
-        <v/>
-      </c>
+      <c r="D71" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B71,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G71),G71,""))</f>
+        <v/>
+      </c>
+      <c r="E71" s="89">
+        <f>IF(OR(D71="",NOT(ISNUMBER(D71))),"",(C71-D71)*100)</f>
+        <v/>
+      </c>
+      <c r="F71" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B71,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G71),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G71" s="85" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="6">
@@ -7907,10 +8474,52 @@
         <f>Bootstrap!J72</f>
         <v/>
       </c>
-      <c r="D72" s="30" t="n"/>
-      <c r="E72" s="31">
-        <f>IF(D72="","",(C72-D72)*100)</f>
-        <v/>
+      <c r="D72" s="97">
+        <f>IFERROR(INDEX($J$12:$T$82,MATCH(B72,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,IF(ISNUMBER(G72),G72,""))</f>
+        <v/>
+      </c>
+      <c r="E72" s="89">
+        <f>IF(OR(D72="",NOT(ISNUMBER(D72))),"",(C72-D72)*100)</f>
+        <v/>
+      </c>
+      <c r="F72" s="93">
+        <f>IF(ISNUMBER(IFERROR(INDEX($J$12:$T$82,MATCH(B72,INDEX($J$12:$T$82,0,$I$3),0),$I$4)*$I$5,"")),"BDS live",IF(ISNUMBER(G72),"manual paste","-"))</f>
+        <v/>
+      </c>
+      <c r="G72" s="85" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="67" t="inlineStr">
+        <is>
+          <t>Pillars matched to the dump</t>
+        </is>
+      </c>
+      <c r="C74" s="87">
+        <f>COUNTIF(F8:F72,"BDS live")&amp;" / "&amp;COUNTA(B8:B72)&amp;"  (only ~32 of the 65 rows are quoted Bloomberg pillars; interpolated gap rows will not match)"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="67" t="inlineStr">
+        <is>
+          <t>Max |Δz| over matched pillars (bp)</t>
+        </is>
+      </c>
+      <c r="C75" s="90">
+        <f>IFERROR(MAX(ABS(IF(ISNUMBER(E8:E72),E8:E72))),"")</f>
+        <v/>
+      </c>
+      <c r="D75" s="65" t="inlineStr">
+        <is>
+          <t>Array formula — Ctrl+Shift+Enter in older Excel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="66" t="inlineStr">
+        <is>
+          <t>If 'matched' reads 0 / 65 the column offsets in I3/I4 are wrong for this dump's schema — read the preview at J10 and correct them. A wrong offset produces plausible but meaningless diffs.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove duplicate BDS call and correct the o/n stub note
Bloomberg_S490_Validation!H8 held a second CURVE_TENOR_RATES dump that spills
into the J12 block; on a terminal the two arrays would have collided.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -56,7 +56,7 @@
     <numFmt numFmtId="173" formatCode="mm/dd/yy"/>
     <numFmt numFmtId="174" formatCode="0.###"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -159,6 +159,12 @@
       <color rgb="00008000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -215,7 +221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -346,6 +352,7 @@
     <xf numFmtId="1" fontId="12" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="174" fontId="12" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="172" fontId="14" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6751,9 +6758,10 @@
         <v/>
       </c>
       <c r="G8" s="85" t="n"/>
-      <c r="H8">
-        <f>BDS(S490_TKR,"CURVE_TENOR_RATES")</f>
-        <v/>
+      <c r="H8" s="65" t="inlineStr">
+        <is>
+          <t>(the CURVE_TENOR_RATES dump lives at J12 - a second copy here would spill into it)</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -33755,9 +33763,9 @@
       <c r="E6" s="85" t="n">
         <v>3.64055</v>
       </c>
-      <c r="F6" s="65" t="inlineStr">
-        <is>
-          <t>FITTED, not an observed fixing: 3.64055% is the overnight rate that makes DFspot reproduce the screen's discount column (spot lag T+2, ACT/360). Replace with the real SOFR fixing if you prefer observed inputs - it moves the whole curve by ~1e-6 in DF.</t>
+      <c r="F6" s="98" t="inlineStr">
+        <is>
+          <t>LIVE on a terminal: C6 pulls the real SOFRRATE fixing and OVERRIDES this cell. This 3.64055% is only the off-terminal fallback (fitted so DFspot reproduces the 07/21/26 S490 screen). Expect the front end to shift when live: ~1.1bp at 1W and ~0.3bp at 1M if the fixing is 3.59%, but under 0.03bp from 1Y out. The long end is unaffected.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make the CDS spreads pull from Bloomberg
CDS_Quotes column D was empty for every tenor, so the module silently sat on the
manual demo spreads with no live path at all. Wire the documented two-step pull:
CDS_SPREAD_TICKER_nY to resolve each tenor's ticker, then quote it. Column H
reports BDP live vs MANUAL (demo) per tenor.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -43,7 +43,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="11">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.00000000"/>
@@ -54,7 +54,6 @@
     <numFmt numFmtId="171" formatCode="0.0000000000"/>
     <numFmt numFmtId="172" formatCode="0.00000"/>
     <numFmt numFmtId="173" formatCode="mm/dd/yy"/>
-    <numFmt numFmtId="174" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -215,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -338,6 +337,10 @@
     <xf numFmtId="2" fontId="14" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="14" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="11" fontId="14" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -12033,7 +12036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12261,6 +12264,23 @@
       <c r="C18" s="65" t="inlineStr">
         <is>
           <t>Continuously-compounded intensity, used at every tenor when B17 = Flat hazard rate. Credit-triangle guide: s/(1-R).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="67" t="inlineStr">
+        <is>
+          <t>Reference entity ticker</t>
+        </is>
+      </c>
+      <c r="B19" s="68" t="inlineStr">
+        <is>
+          <t>HSBA LN Equity</t>
+        </is>
+      </c>
+      <c r="C19" s="65" t="inlineStr">
+        <is>
+          <t>Drives the CDS_SPREAD_TICKER_nY lookups on CDS_Quotes. Any Bloomberg identifier whose CDS curve you want (equity ticker, or the entity itself).</t>
         </is>
       </c>
     </row>
@@ -12288,7 +12308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12308,9 +12328,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Single-name CDS par spreads — one entity, one seniority/clause. Live BDP overrides the manual demo values.</t>
+      <c r="A2" s="65" t="inlineStr">
+        <is>
+          <t>Single-name CDS par spreads. Step 1 (col D) resolves each tenor's CDS ticker from the entity ticker in CDS_Parameters!B19; step 2 (col F) quotes it. Manual spreads in col E are used only when BDP fails.</t>
         </is>
       </c>
     </row>
@@ -12338,9 +12358,9 @@
           <t>Maturity</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
-        <is>
-          <t>CDS ticker</t>
+      <c r="D6" s="92" t="inlineStr">
+        <is>
+          <t>CDS ticker (step 1, live)</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
@@ -12356,6 +12376,11 @@
       <c r="G6" s="20" t="inlineStr">
         <is>
           <t>Approx hazard s/(1-R)</t>
+        </is>
+      </c>
+      <c r="H6" s="62" t="inlineStr">
+        <is>
+          <t>Quote source in use</t>
         </is>
       </c>
     </row>
@@ -12372,18 +12397,25 @@
         <f>EDATE('Curve_Interface'!$F$7,3*(4-1))</f>
         <v/>
       </c>
-      <c r="D7" s="37" t="inlineStr"/>
+      <c r="D7" s="87">
+        <f>IFERROR(BDP(CDS_Parameters!$B$19,"CDS_SPREAD_TICKER_1Y"),"")</f>
+        <v/>
+      </c>
       <c r="E7" s="55" t="n">
         <v>40</v>
       </c>
-      <c r="F7" s="31">
-        <f>IF(D7="",E7,IFERROR(BDP(D7,"PX_LAST"),E7))</f>
+      <c r="F7" s="63">
+        <f>IFERROR(BDP(D7&amp;" BEST Curncy","PX_MID")+0,IFERROR(BDP(D7,"PX_LAST")+0,E7))</f>
         <v/>
       </c>
       <c r="G7" s="52">
         <f>(F7/10000)/(1-CDS_Parameters!$B$8)</f>
         <v/>
       </c>
+      <c r="H7" s="93">
+        <f>IF(ISNUMBER(IFERROR(BDP(D7&amp;" BEST Curncy","PX_MID")+0,"")),"BDP live","MANUAL (demo)")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -12398,18 +12430,25 @@
         <f>EDATE('Curve_Interface'!$F$7,3*(8-1))</f>
         <v/>
       </c>
-      <c r="D8" s="37" t="inlineStr"/>
+      <c r="D8" s="87">
+        <f>IFERROR(BDP(CDS_Parameters!$B$19,"CDS_SPREAD_TICKER_2Y"),"")</f>
+        <v/>
+      </c>
       <c r="E8" s="55" t="n">
         <v>55</v>
       </c>
-      <c r="F8" s="31">
-        <f>IF(D8="",E8,IFERROR(BDP(D8,"PX_LAST"),E8))</f>
+      <c r="F8" s="63">
+        <f>IFERROR(BDP(D8&amp;" BEST Curncy","PX_MID")+0,IFERROR(BDP(D8,"PX_LAST")+0,E8))</f>
         <v/>
       </c>
       <c r="G8" s="52">
         <f>(F8/10000)/(1-CDS_Parameters!$B$8)</f>
         <v/>
       </c>
+      <c r="H8" s="93">
+        <f>IF(ISNUMBER(IFERROR(BDP(D8&amp;" BEST Curncy","PX_MID")+0,"")),"BDP live","MANUAL (demo)")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -12424,18 +12463,25 @@
         <f>EDATE('Curve_Interface'!$F$7,3*(12-1))</f>
         <v/>
       </c>
-      <c r="D9" s="37" t="inlineStr"/>
+      <c r="D9" s="87">
+        <f>IFERROR(BDP(CDS_Parameters!$B$19,"CDS_SPREAD_TICKER_3Y"),"")</f>
+        <v/>
+      </c>
       <c r="E9" s="55" t="n">
         <v>70</v>
       </c>
-      <c r="F9" s="31">
-        <f>IF(D9="",E9,IFERROR(BDP(D9,"PX_LAST"),E9))</f>
+      <c r="F9" s="63">
+        <f>IFERROR(BDP(D9&amp;" BEST Curncy","PX_MID")+0,IFERROR(BDP(D9,"PX_LAST")+0,E9))</f>
         <v/>
       </c>
       <c r="G9" s="52">
         <f>(F9/10000)/(1-CDS_Parameters!$B$8)</f>
         <v/>
       </c>
+      <c r="H9" s="93">
+        <f>IF(ISNUMBER(IFERROR(BDP(D9&amp;" BEST Curncy","PX_MID")+0,"")),"BDP live","MANUAL (demo)")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -12450,18 +12496,25 @@
         <f>EDATE('Curve_Interface'!$F$7,3*(20-1))</f>
         <v/>
       </c>
-      <c r="D10" s="37" t="inlineStr"/>
+      <c r="D10" s="87">
+        <f>IFERROR(BDP(CDS_Parameters!$B$19,"CDS_SPREAD_TICKER_5Y"),"")</f>
+        <v/>
+      </c>
       <c r="E10" s="55" t="n">
         <v>95</v>
       </c>
-      <c r="F10" s="31">
-        <f>IF(D10="",E10,IFERROR(BDP(D10,"PX_LAST"),E10))</f>
+      <c r="F10" s="63">
+        <f>IFERROR(BDP(D10&amp;" BEST Curncy","PX_MID")+0,IFERROR(BDP(D10,"PX_LAST")+0,E10))</f>
         <v/>
       </c>
       <c r="G10" s="52">
         <f>(F10/10000)/(1-CDS_Parameters!$B$8)</f>
         <v/>
       </c>
+      <c r="H10" s="93">
+        <f>IF(ISNUMBER(IFERROR(BDP(D10&amp;" BEST Curncy","PX_MID")+0,"")),"BDP live","MANUAL (demo)")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -12476,18 +12529,25 @@
         <f>EDATE('Curve_Interface'!$F$7,3*(28-1))</f>
         <v/>
       </c>
-      <c r="D11" s="37" t="inlineStr"/>
+      <c r="D11" s="87">
+        <f>IFERROR(BDP(CDS_Parameters!$B$19,"CDS_SPREAD_TICKER_7Y"),"")</f>
+        <v/>
+      </c>
       <c r="E11" s="55" t="n">
         <v>115</v>
       </c>
-      <c r="F11" s="31">
-        <f>IF(D11="",E11,IFERROR(BDP(D11,"PX_LAST"),E11))</f>
+      <c r="F11" s="63">
+        <f>IFERROR(BDP(D11&amp;" BEST Curncy","PX_MID")+0,IFERROR(BDP(D11,"PX_LAST")+0,E11))</f>
         <v/>
       </c>
       <c r="G11" s="52">
         <f>(F11/10000)/(1-CDS_Parameters!$B$8)</f>
         <v/>
       </c>
+      <c r="H11" s="93">
+        <f>IF(ISNUMBER(IFERROR(BDP(D11&amp;" BEST Curncy","PX_MID")+0,"")),"BDP live","MANUAL (demo)")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -12502,17 +12562,31 @@
         <f>EDATE('Curve_Interface'!$F$7,3*(40-1))</f>
         <v/>
       </c>
-      <c r="D12" s="37" t="inlineStr"/>
+      <c r="D12" s="87">
+        <f>IFERROR(BDP(CDS_Parameters!$B$19,"CDS_SPREAD_TICKER_10Y"),"")</f>
+        <v/>
+      </c>
       <c r="E12" s="55" t="n">
         <v>135</v>
       </c>
-      <c r="F12" s="31">
-        <f>IF(D12="",E12,IFERROR(BDP(D12,"PX_LAST"),E12))</f>
+      <c r="F12" s="63">
+        <f>IFERROR(BDP(D12&amp;" BEST Curncy","PX_MID")+0,IFERROR(BDP(D12,"PX_LAST")+0,E12))</f>
         <v/>
       </c>
       <c r="G12" s="52">
         <f>(F12/10000)/(1-CDS_Parameters!$B$8)</f>
         <v/>
+      </c>
+      <c r="H12" s="93">
+        <f>IF(ISNUMBER(IFERROR(BDP(D12&amp;" BEST Curncy","PX_MID")+0,"")),"BDP live","MANUAL (demo)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="66" t="inlineStr">
+        <is>
+          <t>WARNING: the manual spreads in column E (40/55/70/95/115/135) are DEMO PLACEHOLDERS, not market data — unlike the SOFR OIS quotes, which are the real 07/21/26 S490 levels. Column H tells you which source each tenor is actually using. Replace column E, or connect a terminal, before trusting any CDS output.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -36460,7 +36534,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add interpolation selector, defaulting to the verified method
The Bloomberg IRS Curve Construction guide documents four interpolation methods.
Method 1 (piecewise linear simple zero, ACT/360) is its EUR S201 example. Fitting
both against the 32 screen pillars - where the long end is sensitive to gap
interpolation through the swap annuity:

  step-function forward (log-linear DF)   rms DF err 2.28e-06, unbiased
  piecewise linear simple                 rms DF err 1.09e-04, +4.2e-04 by 50Y

Method 1 is 48x worse and biased, so USD S490 does not use it. Default stays
step-function forward; method 1 is switchable for curves that do use it.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -4636,6 +4636,16 @@
         <f>IF(DATE(YEAR(VAL_DATE),CEILING(MONTH(VAL_DATE)/3,1)*3,20)&gt;=VAL_DATE,DATE(YEAR(VAL_DATE),CEILING(MONTH(VAL_DATE)/3,1)*3,20),EDATE(DATE(YEAR(VAL_DATE),CEILING(MONTH(VAL_DATE)/3,1)*3,20),3))</f>
         <v/>
       </c>
+      <c r="I7" s="67" t="inlineStr">
+        <is>
+          <t>Interpolation</t>
+        </is>
+      </c>
+      <c r="J7" s="68" t="inlineStr">
+        <is>
+          <t>Step-function forward (flat fwd)</t>
+        </is>
+      </c>
       <c r="K7" s="20" t="inlineStr">
         <is>
           <t>Date</t>
@@ -4648,6 +4658,16 @@
       </c>
     </row>
     <row r="8">
+      <c r="I8" s="67" t="inlineStr">
+        <is>
+          <t>VERIFIED default</t>
+        </is>
+      </c>
+      <c r="J8" s="66" t="inlineStr">
+        <is>
+          <t>Step-function forward reproduces the S490 screen (rms DF err 2.3e-06). Piecewise Linear (Simple) — the guide's method 1, its EUR S201 example — is 48x worse on this curve (1.1e-04, biased to +4.2e-04 by 50Y). Only switch if the S490 Interpolation field actually says so.</t>
+        </is>
+      </c>
       <c r="K8" s="18">
         <f>Bootstrap!$B$4</f>
         <v/>
@@ -4730,13 +4750,18 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B10,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B10,$K$8:$K$73,1)))/((E10-D10)/365)*100</f>
         <v/>
       </c>
-      <c r="G10" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B10,$K$8:$K$73,1))*EXP(-(F10/100)*(B10-D10)/365)</f>
+      <c r="G10" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B10-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((10&gt;0)*(D10-VAL_DATE)/360,0)&lt;=0,IF(((E10-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B10,$K$8:$K$73,1)+1)-1)/((E10-VAL_DATE)/360)),IF(MAX((10&gt;0)*(D10-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B10,$K$8:$K$73,1))-1)/MAX((10&gt;0)*(D10-VAL_DATE)/360,0)))+(IF(((E10-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B10,$K$8:$K$73,1)+1)-1)/((E10-VAL_DATE)/360))-IF(MAX((10&gt;0)*(D10-VAL_DATE)/360,0)&lt;=0,IF(((E10-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B10,$K$8:$K$73,1)+1)-1)/((E10-VAL_DATE)/360)),IF(MAX((10&gt;0)*(D10-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B10,$K$8:$K$73,1))-1)/MAX((10&gt;0)*(D10-VAL_DATE)/360,0))))*IF(((E10-VAL_DATE)/360)-MAX((10&gt;0)*(D10-VAL_DATE)/360,0)=0,0,(((B10-VAL_DATE)/360)-MAX((10&gt;0)*(D10-VAL_DATE)/360,0))/(((E10-VAL_DATE)/360)-MAX((10&gt;0)*(D10-VAL_DATE)/360,0))))*((B10-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B10,$K$8:$K$73,1))*EXP(-(F10/100)*(B10-D10)/365)),"")</f>
         <v/>
       </c>
       <c r="H10" s="17">
         <f>-LN(G10)/C10*100</f>
         <v/>
+      </c>
+      <c r="I10" s="65" t="inlineStr">
+        <is>
+          <t>Guide method 1:  DF(t)=1/(1+r_s(t)*t), r_s piecewise linear, t on ACT/360, flat outside the first/last instrument maturity.</t>
+        </is>
       </c>
       <c r="K10" s="18">
         <f>Bootstrap!B9</f>
@@ -4771,13 +4796,18 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B11,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B11,$K$8:$K$73,1)))/((E11-D11)/365)*100</f>
         <v/>
       </c>
-      <c r="G11" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B11,$K$8:$K$73,1))*EXP(-(F11/100)*(B11-D11)/365)</f>
+      <c r="G11" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B11-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((11&gt;0)*(D11-VAL_DATE)/360,0)&lt;=0,IF(((E11-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B11,$K$8:$K$73,1)+1)-1)/((E11-VAL_DATE)/360)),IF(MAX((11&gt;0)*(D11-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B11,$K$8:$K$73,1))-1)/MAX((11&gt;0)*(D11-VAL_DATE)/360,0)))+(IF(((E11-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B11,$K$8:$K$73,1)+1)-1)/((E11-VAL_DATE)/360))-IF(MAX((11&gt;0)*(D11-VAL_DATE)/360,0)&lt;=0,IF(((E11-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B11,$K$8:$K$73,1)+1)-1)/((E11-VAL_DATE)/360)),IF(MAX((11&gt;0)*(D11-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B11,$K$8:$K$73,1))-1)/MAX((11&gt;0)*(D11-VAL_DATE)/360,0))))*IF(((E11-VAL_DATE)/360)-MAX((11&gt;0)*(D11-VAL_DATE)/360,0)=0,0,(((B11-VAL_DATE)/360)-MAX((11&gt;0)*(D11-VAL_DATE)/360,0))/(((E11-VAL_DATE)/360)-MAX((11&gt;0)*(D11-VAL_DATE)/360,0))))*((B11-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B11,$K$8:$K$73,1))*EXP(-(F11/100)*(B11-D11)/365)),"")</f>
         <v/>
       </c>
       <c r="H11" s="17">
         <f>-LN(G11)/C11*100</f>
         <v/>
+      </c>
+      <c r="I11" s="65" t="inlineStr">
+        <is>
+          <t>Guide method 3:  flat instantaneous forward between pillars, equivalently log-linear in the discount factor.</t>
+        </is>
       </c>
       <c r="K11" s="18">
         <f>Bootstrap!B10</f>
@@ -4812,13 +4842,18 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B12,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B12,$K$8:$K$73,1)))/((E12-D12)/365)*100</f>
         <v/>
       </c>
-      <c r="G12" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B12,$K$8:$K$73,1))*EXP(-(F12/100)*(B12-D12)/365)</f>
+      <c r="G12" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B12-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((12&gt;0)*(D12-VAL_DATE)/360,0)&lt;=0,IF(((E12-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B12,$K$8:$K$73,1)+1)-1)/((E12-VAL_DATE)/360)),IF(MAX((12&gt;0)*(D12-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B12,$K$8:$K$73,1))-1)/MAX((12&gt;0)*(D12-VAL_DATE)/360,0)))+(IF(((E12-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B12,$K$8:$K$73,1)+1)-1)/((E12-VAL_DATE)/360))-IF(MAX((12&gt;0)*(D12-VAL_DATE)/360,0)&lt;=0,IF(((E12-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B12,$K$8:$K$73,1)+1)-1)/((E12-VAL_DATE)/360)),IF(MAX((12&gt;0)*(D12-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B12,$K$8:$K$73,1))-1)/MAX((12&gt;0)*(D12-VAL_DATE)/360,0))))*IF(((E12-VAL_DATE)/360)-MAX((12&gt;0)*(D12-VAL_DATE)/360,0)=0,0,(((B12-VAL_DATE)/360)-MAX((12&gt;0)*(D12-VAL_DATE)/360,0))/(((E12-VAL_DATE)/360)-MAX((12&gt;0)*(D12-VAL_DATE)/360,0))))*((B12-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B12,$K$8:$K$73,1))*EXP(-(F12/100)*(B12-D12)/365)),"")</f>
         <v/>
       </c>
       <c r="H12" s="17">
         <f>-LN(G12)/C12*100</f>
         <v/>
+      </c>
+      <c r="I12" s="65" t="inlineStr">
+        <is>
+          <t>Both agree AT the pillars; they differ only off-pillar — which is exactly what CDS_Schedule looks up. Max gap difference ~0.07bp of zero rate in a 2Y gap.</t>
+        </is>
       </c>
       <c r="K12" s="18">
         <f>Bootstrap!B11</f>
@@ -4853,8 +4888,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B13,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B13,$K$8:$K$73,1)))/((E13-D13)/365)*100</f>
         <v/>
       </c>
-      <c r="G13" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B13,$K$8:$K$73,1))*EXP(-(F13/100)*(B13-D13)/365)</f>
+      <c r="G13" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B13-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((13&gt;0)*(D13-VAL_DATE)/360,0)&lt;=0,IF(((E13-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B13,$K$8:$K$73,1)+1)-1)/((E13-VAL_DATE)/360)),IF(MAX((13&gt;0)*(D13-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B13,$K$8:$K$73,1))-1)/MAX((13&gt;0)*(D13-VAL_DATE)/360,0)))+(IF(((E13-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B13,$K$8:$K$73,1)+1)-1)/((E13-VAL_DATE)/360))-IF(MAX((13&gt;0)*(D13-VAL_DATE)/360,0)&lt;=0,IF(((E13-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B13,$K$8:$K$73,1)+1)-1)/((E13-VAL_DATE)/360)),IF(MAX((13&gt;0)*(D13-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B13,$K$8:$K$73,1))-1)/MAX((13&gt;0)*(D13-VAL_DATE)/360,0))))*IF(((E13-VAL_DATE)/360)-MAX((13&gt;0)*(D13-VAL_DATE)/360,0)=0,0,(((B13-VAL_DATE)/360)-MAX((13&gt;0)*(D13-VAL_DATE)/360,0))/(((E13-VAL_DATE)/360)-MAX((13&gt;0)*(D13-VAL_DATE)/360,0))))*((B13-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B13,$K$8:$K$73,1))*EXP(-(F13/100)*(B13-D13)/365)),"")</f>
         <v/>
       </c>
       <c r="H13" s="17">
@@ -4894,8 +4929,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B14,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B14,$K$8:$K$73,1)))/((E14-D14)/365)*100</f>
         <v/>
       </c>
-      <c r="G14" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B14,$K$8:$K$73,1))*EXP(-(F14/100)*(B14-D14)/365)</f>
+      <c r="G14" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B14-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((14&gt;0)*(D14-VAL_DATE)/360,0)&lt;=0,IF(((E14-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B14,$K$8:$K$73,1)+1)-1)/((E14-VAL_DATE)/360)),IF(MAX((14&gt;0)*(D14-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B14,$K$8:$K$73,1))-1)/MAX((14&gt;0)*(D14-VAL_DATE)/360,0)))+(IF(((E14-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B14,$K$8:$K$73,1)+1)-1)/((E14-VAL_DATE)/360))-IF(MAX((14&gt;0)*(D14-VAL_DATE)/360,0)&lt;=0,IF(((E14-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B14,$K$8:$K$73,1)+1)-1)/((E14-VAL_DATE)/360)),IF(MAX((14&gt;0)*(D14-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B14,$K$8:$K$73,1))-1)/MAX((14&gt;0)*(D14-VAL_DATE)/360,0))))*IF(((E14-VAL_DATE)/360)-MAX((14&gt;0)*(D14-VAL_DATE)/360,0)=0,0,(((B14-VAL_DATE)/360)-MAX((14&gt;0)*(D14-VAL_DATE)/360,0))/(((E14-VAL_DATE)/360)-MAX((14&gt;0)*(D14-VAL_DATE)/360,0))))*((B14-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B14,$K$8:$K$73,1))*EXP(-(F14/100)*(B14-D14)/365)),"")</f>
         <v/>
       </c>
       <c r="H14" s="17">
@@ -4935,8 +4970,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B15,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B15,$K$8:$K$73,1)))/((E15-D15)/365)*100</f>
         <v/>
       </c>
-      <c r="G15" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B15,$K$8:$K$73,1))*EXP(-(F15/100)*(B15-D15)/365)</f>
+      <c r="G15" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B15-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((15&gt;0)*(D15-VAL_DATE)/360,0)&lt;=0,IF(((E15-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B15,$K$8:$K$73,1)+1)-1)/((E15-VAL_DATE)/360)),IF(MAX((15&gt;0)*(D15-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B15,$K$8:$K$73,1))-1)/MAX((15&gt;0)*(D15-VAL_DATE)/360,0)))+(IF(((E15-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B15,$K$8:$K$73,1)+1)-1)/((E15-VAL_DATE)/360))-IF(MAX((15&gt;0)*(D15-VAL_DATE)/360,0)&lt;=0,IF(((E15-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B15,$K$8:$K$73,1)+1)-1)/((E15-VAL_DATE)/360)),IF(MAX((15&gt;0)*(D15-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B15,$K$8:$K$73,1))-1)/MAX((15&gt;0)*(D15-VAL_DATE)/360,0))))*IF(((E15-VAL_DATE)/360)-MAX((15&gt;0)*(D15-VAL_DATE)/360,0)=0,0,(((B15-VAL_DATE)/360)-MAX((15&gt;0)*(D15-VAL_DATE)/360,0))/(((E15-VAL_DATE)/360)-MAX((15&gt;0)*(D15-VAL_DATE)/360,0))))*((B15-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B15,$K$8:$K$73,1))*EXP(-(F15/100)*(B15-D15)/365)),"")</f>
         <v/>
       </c>
       <c r="H15" s="17">
@@ -4976,8 +5011,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B16,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B16,$K$8:$K$73,1)))/((E16-D16)/365)*100</f>
         <v/>
       </c>
-      <c r="G16" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B16,$K$8:$K$73,1))*EXP(-(F16/100)*(B16-D16)/365)</f>
+      <c r="G16" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B16-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((16&gt;0)*(D16-VAL_DATE)/360,0)&lt;=0,IF(((E16-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B16,$K$8:$K$73,1)+1)-1)/((E16-VAL_DATE)/360)),IF(MAX((16&gt;0)*(D16-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B16,$K$8:$K$73,1))-1)/MAX((16&gt;0)*(D16-VAL_DATE)/360,0)))+(IF(((E16-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B16,$K$8:$K$73,1)+1)-1)/((E16-VAL_DATE)/360))-IF(MAX((16&gt;0)*(D16-VAL_DATE)/360,0)&lt;=0,IF(((E16-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B16,$K$8:$K$73,1)+1)-1)/((E16-VAL_DATE)/360)),IF(MAX((16&gt;0)*(D16-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B16,$K$8:$K$73,1))-1)/MAX((16&gt;0)*(D16-VAL_DATE)/360,0))))*IF(((E16-VAL_DATE)/360)-MAX((16&gt;0)*(D16-VAL_DATE)/360,0)=0,0,(((B16-VAL_DATE)/360)-MAX((16&gt;0)*(D16-VAL_DATE)/360,0))/(((E16-VAL_DATE)/360)-MAX((16&gt;0)*(D16-VAL_DATE)/360,0))))*((B16-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B16,$K$8:$K$73,1))*EXP(-(F16/100)*(B16-D16)/365)),"")</f>
         <v/>
       </c>
       <c r="H16" s="17">
@@ -5017,8 +5052,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B17,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B17,$K$8:$K$73,1)))/((E17-D17)/365)*100</f>
         <v/>
       </c>
-      <c r="G17" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B17,$K$8:$K$73,1))*EXP(-(F17/100)*(B17-D17)/365)</f>
+      <c r="G17" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B17-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((17&gt;0)*(D17-VAL_DATE)/360,0)&lt;=0,IF(((E17-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B17,$K$8:$K$73,1)+1)-1)/((E17-VAL_DATE)/360)),IF(MAX((17&gt;0)*(D17-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B17,$K$8:$K$73,1))-1)/MAX((17&gt;0)*(D17-VAL_DATE)/360,0)))+(IF(((E17-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B17,$K$8:$K$73,1)+1)-1)/((E17-VAL_DATE)/360))-IF(MAX((17&gt;0)*(D17-VAL_DATE)/360,0)&lt;=0,IF(((E17-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B17,$K$8:$K$73,1)+1)-1)/((E17-VAL_DATE)/360)),IF(MAX((17&gt;0)*(D17-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B17,$K$8:$K$73,1))-1)/MAX((17&gt;0)*(D17-VAL_DATE)/360,0))))*IF(((E17-VAL_DATE)/360)-MAX((17&gt;0)*(D17-VAL_DATE)/360,0)=0,0,(((B17-VAL_DATE)/360)-MAX((17&gt;0)*(D17-VAL_DATE)/360,0))/(((E17-VAL_DATE)/360)-MAX((17&gt;0)*(D17-VAL_DATE)/360,0))))*((B17-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B17,$K$8:$K$73,1))*EXP(-(F17/100)*(B17-D17)/365)),"")</f>
         <v/>
       </c>
       <c r="H17" s="17">
@@ -5058,8 +5093,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B18,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B18,$K$8:$K$73,1)))/((E18-D18)/365)*100</f>
         <v/>
       </c>
-      <c r="G18" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B18,$K$8:$K$73,1))*EXP(-(F18/100)*(B18-D18)/365)</f>
+      <c r="G18" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B18-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((18&gt;0)*(D18-VAL_DATE)/360,0)&lt;=0,IF(((E18-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B18,$K$8:$K$73,1)+1)-1)/((E18-VAL_DATE)/360)),IF(MAX((18&gt;0)*(D18-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B18,$K$8:$K$73,1))-1)/MAX((18&gt;0)*(D18-VAL_DATE)/360,0)))+(IF(((E18-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B18,$K$8:$K$73,1)+1)-1)/((E18-VAL_DATE)/360))-IF(MAX((18&gt;0)*(D18-VAL_DATE)/360,0)&lt;=0,IF(((E18-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B18,$K$8:$K$73,1)+1)-1)/((E18-VAL_DATE)/360)),IF(MAX((18&gt;0)*(D18-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B18,$K$8:$K$73,1))-1)/MAX((18&gt;0)*(D18-VAL_DATE)/360,0))))*IF(((E18-VAL_DATE)/360)-MAX((18&gt;0)*(D18-VAL_DATE)/360,0)=0,0,(((B18-VAL_DATE)/360)-MAX((18&gt;0)*(D18-VAL_DATE)/360,0))/(((E18-VAL_DATE)/360)-MAX((18&gt;0)*(D18-VAL_DATE)/360,0))))*((B18-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B18,$K$8:$K$73,1))*EXP(-(F18/100)*(B18-D18)/365)),"")</f>
         <v/>
       </c>
       <c r="H18" s="17">
@@ -5099,8 +5134,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B19,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B19,$K$8:$K$73,1)))/((E19-D19)/365)*100</f>
         <v/>
       </c>
-      <c r="G19" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B19,$K$8:$K$73,1))*EXP(-(F19/100)*(B19-D19)/365)</f>
+      <c r="G19" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B19-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((19&gt;0)*(D19-VAL_DATE)/360,0)&lt;=0,IF(((E19-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B19,$K$8:$K$73,1)+1)-1)/((E19-VAL_DATE)/360)),IF(MAX((19&gt;0)*(D19-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B19,$K$8:$K$73,1))-1)/MAX((19&gt;0)*(D19-VAL_DATE)/360,0)))+(IF(((E19-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B19,$K$8:$K$73,1)+1)-1)/((E19-VAL_DATE)/360))-IF(MAX((19&gt;0)*(D19-VAL_DATE)/360,0)&lt;=0,IF(((E19-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B19,$K$8:$K$73,1)+1)-1)/((E19-VAL_DATE)/360)),IF(MAX((19&gt;0)*(D19-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B19,$K$8:$K$73,1))-1)/MAX((19&gt;0)*(D19-VAL_DATE)/360,0))))*IF(((E19-VAL_DATE)/360)-MAX((19&gt;0)*(D19-VAL_DATE)/360,0)=0,0,(((B19-VAL_DATE)/360)-MAX((19&gt;0)*(D19-VAL_DATE)/360,0))/(((E19-VAL_DATE)/360)-MAX((19&gt;0)*(D19-VAL_DATE)/360,0))))*((B19-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B19,$K$8:$K$73,1))*EXP(-(F19/100)*(B19-D19)/365)),"")</f>
         <v/>
       </c>
       <c r="H19" s="17">
@@ -5140,8 +5175,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B20,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B20,$K$8:$K$73,1)))/((E20-D20)/365)*100</f>
         <v/>
       </c>
-      <c r="G20" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B20,$K$8:$K$73,1))*EXP(-(F20/100)*(B20-D20)/365)</f>
+      <c r="G20" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B20-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((20&gt;0)*(D20-VAL_DATE)/360,0)&lt;=0,IF(((E20-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B20,$K$8:$K$73,1)+1)-1)/((E20-VAL_DATE)/360)),IF(MAX((20&gt;0)*(D20-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B20,$K$8:$K$73,1))-1)/MAX((20&gt;0)*(D20-VAL_DATE)/360,0)))+(IF(((E20-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B20,$K$8:$K$73,1)+1)-1)/((E20-VAL_DATE)/360))-IF(MAX((20&gt;0)*(D20-VAL_DATE)/360,0)&lt;=0,IF(((E20-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B20,$K$8:$K$73,1)+1)-1)/((E20-VAL_DATE)/360)),IF(MAX((20&gt;0)*(D20-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B20,$K$8:$K$73,1))-1)/MAX((20&gt;0)*(D20-VAL_DATE)/360,0))))*IF(((E20-VAL_DATE)/360)-MAX((20&gt;0)*(D20-VAL_DATE)/360,0)=0,0,(((B20-VAL_DATE)/360)-MAX((20&gt;0)*(D20-VAL_DATE)/360,0))/(((E20-VAL_DATE)/360)-MAX((20&gt;0)*(D20-VAL_DATE)/360,0))))*((B20-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B20,$K$8:$K$73,1))*EXP(-(F20/100)*(B20-D20)/365)),"")</f>
         <v/>
       </c>
       <c r="H20" s="17">
@@ -5181,8 +5216,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B21,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B21,$K$8:$K$73,1)))/((E21-D21)/365)*100</f>
         <v/>
       </c>
-      <c r="G21" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B21,$K$8:$K$73,1))*EXP(-(F21/100)*(B21-D21)/365)</f>
+      <c r="G21" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B21-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((21&gt;0)*(D21-VAL_DATE)/360,0)&lt;=0,IF(((E21-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B21,$K$8:$K$73,1)+1)-1)/((E21-VAL_DATE)/360)),IF(MAX((21&gt;0)*(D21-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B21,$K$8:$K$73,1))-1)/MAX((21&gt;0)*(D21-VAL_DATE)/360,0)))+(IF(((E21-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B21,$K$8:$K$73,1)+1)-1)/((E21-VAL_DATE)/360))-IF(MAX((21&gt;0)*(D21-VAL_DATE)/360,0)&lt;=0,IF(((E21-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B21,$K$8:$K$73,1)+1)-1)/((E21-VAL_DATE)/360)),IF(MAX((21&gt;0)*(D21-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B21,$K$8:$K$73,1))-1)/MAX((21&gt;0)*(D21-VAL_DATE)/360,0))))*IF(((E21-VAL_DATE)/360)-MAX((21&gt;0)*(D21-VAL_DATE)/360,0)=0,0,(((B21-VAL_DATE)/360)-MAX((21&gt;0)*(D21-VAL_DATE)/360,0))/(((E21-VAL_DATE)/360)-MAX((21&gt;0)*(D21-VAL_DATE)/360,0))))*((B21-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B21,$K$8:$K$73,1))*EXP(-(F21/100)*(B21-D21)/365)),"")</f>
         <v/>
       </c>
       <c r="H21" s="17">
@@ -5222,8 +5257,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B22,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B22,$K$8:$K$73,1)))/((E22-D22)/365)*100</f>
         <v/>
       </c>
-      <c r="G22" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B22,$K$8:$K$73,1))*EXP(-(F22/100)*(B22-D22)/365)</f>
+      <c r="G22" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B22-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((22&gt;0)*(D22-VAL_DATE)/360,0)&lt;=0,IF(((E22-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B22,$K$8:$K$73,1)+1)-1)/((E22-VAL_DATE)/360)),IF(MAX((22&gt;0)*(D22-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B22,$K$8:$K$73,1))-1)/MAX((22&gt;0)*(D22-VAL_DATE)/360,0)))+(IF(((E22-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B22,$K$8:$K$73,1)+1)-1)/((E22-VAL_DATE)/360))-IF(MAX((22&gt;0)*(D22-VAL_DATE)/360,0)&lt;=0,IF(((E22-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B22,$K$8:$K$73,1)+1)-1)/((E22-VAL_DATE)/360)),IF(MAX((22&gt;0)*(D22-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B22,$K$8:$K$73,1))-1)/MAX((22&gt;0)*(D22-VAL_DATE)/360,0))))*IF(((E22-VAL_DATE)/360)-MAX((22&gt;0)*(D22-VAL_DATE)/360,0)=0,0,(((B22-VAL_DATE)/360)-MAX((22&gt;0)*(D22-VAL_DATE)/360,0))/(((E22-VAL_DATE)/360)-MAX((22&gt;0)*(D22-VAL_DATE)/360,0))))*((B22-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B22,$K$8:$K$73,1))*EXP(-(F22/100)*(B22-D22)/365)),"")</f>
         <v/>
       </c>
       <c r="H22" s="17">
@@ -5263,8 +5298,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B23,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B23,$K$8:$K$73,1)))/((E23-D23)/365)*100</f>
         <v/>
       </c>
-      <c r="G23" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B23,$K$8:$K$73,1))*EXP(-(F23/100)*(B23-D23)/365)</f>
+      <c r="G23" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B23-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((23&gt;0)*(D23-VAL_DATE)/360,0)&lt;=0,IF(((E23-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B23,$K$8:$K$73,1)+1)-1)/((E23-VAL_DATE)/360)),IF(MAX((23&gt;0)*(D23-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B23,$K$8:$K$73,1))-1)/MAX((23&gt;0)*(D23-VAL_DATE)/360,0)))+(IF(((E23-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B23,$K$8:$K$73,1)+1)-1)/((E23-VAL_DATE)/360))-IF(MAX((23&gt;0)*(D23-VAL_DATE)/360,0)&lt;=0,IF(((E23-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B23,$K$8:$K$73,1)+1)-1)/((E23-VAL_DATE)/360)),IF(MAX((23&gt;0)*(D23-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B23,$K$8:$K$73,1))-1)/MAX((23&gt;0)*(D23-VAL_DATE)/360,0))))*IF(((E23-VAL_DATE)/360)-MAX((23&gt;0)*(D23-VAL_DATE)/360,0)=0,0,(((B23-VAL_DATE)/360)-MAX((23&gt;0)*(D23-VAL_DATE)/360,0))/(((E23-VAL_DATE)/360)-MAX((23&gt;0)*(D23-VAL_DATE)/360,0))))*((B23-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B23,$K$8:$K$73,1))*EXP(-(F23/100)*(B23-D23)/365)),"")</f>
         <v/>
       </c>
       <c r="H23" s="17">
@@ -5304,8 +5339,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B24,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B24,$K$8:$K$73,1)))/((E24-D24)/365)*100</f>
         <v/>
       </c>
-      <c r="G24" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B24,$K$8:$K$73,1))*EXP(-(F24/100)*(B24-D24)/365)</f>
+      <c r="G24" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B24-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((24&gt;0)*(D24-VAL_DATE)/360,0)&lt;=0,IF(((E24-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B24,$K$8:$K$73,1)+1)-1)/((E24-VAL_DATE)/360)),IF(MAX((24&gt;0)*(D24-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B24,$K$8:$K$73,1))-1)/MAX((24&gt;0)*(D24-VAL_DATE)/360,0)))+(IF(((E24-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B24,$K$8:$K$73,1)+1)-1)/((E24-VAL_DATE)/360))-IF(MAX((24&gt;0)*(D24-VAL_DATE)/360,0)&lt;=0,IF(((E24-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B24,$K$8:$K$73,1)+1)-1)/((E24-VAL_DATE)/360)),IF(MAX((24&gt;0)*(D24-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B24,$K$8:$K$73,1))-1)/MAX((24&gt;0)*(D24-VAL_DATE)/360,0))))*IF(((E24-VAL_DATE)/360)-MAX((24&gt;0)*(D24-VAL_DATE)/360,0)=0,0,(((B24-VAL_DATE)/360)-MAX((24&gt;0)*(D24-VAL_DATE)/360,0))/(((E24-VAL_DATE)/360)-MAX((24&gt;0)*(D24-VAL_DATE)/360,0))))*((B24-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B24,$K$8:$K$73,1))*EXP(-(F24/100)*(B24-D24)/365)),"")</f>
         <v/>
       </c>
       <c r="H24" s="17">
@@ -5345,8 +5380,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B25,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B25,$K$8:$K$73,1)))/((E25-D25)/365)*100</f>
         <v/>
       </c>
-      <c r="G25" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B25,$K$8:$K$73,1))*EXP(-(F25/100)*(B25-D25)/365)</f>
+      <c r="G25" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B25-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((25&gt;0)*(D25-VAL_DATE)/360,0)&lt;=0,IF(((E25-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B25,$K$8:$K$73,1)+1)-1)/((E25-VAL_DATE)/360)),IF(MAX((25&gt;0)*(D25-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B25,$K$8:$K$73,1))-1)/MAX((25&gt;0)*(D25-VAL_DATE)/360,0)))+(IF(((E25-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B25,$K$8:$K$73,1)+1)-1)/((E25-VAL_DATE)/360))-IF(MAX((25&gt;0)*(D25-VAL_DATE)/360,0)&lt;=0,IF(((E25-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B25,$K$8:$K$73,1)+1)-1)/((E25-VAL_DATE)/360)),IF(MAX((25&gt;0)*(D25-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B25,$K$8:$K$73,1))-1)/MAX((25&gt;0)*(D25-VAL_DATE)/360,0))))*IF(((E25-VAL_DATE)/360)-MAX((25&gt;0)*(D25-VAL_DATE)/360,0)=0,0,(((B25-VAL_DATE)/360)-MAX((25&gt;0)*(D25-VAL_DATE)/360,0))/(((E25-VAL_DATE)/360)-MAX((25&gt;0)*(D25-VAL_DATE)/360,0))))*((B25-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B25,$K$8:$K$73,1))*EXP(-(F25/100)*(B25-D25)/365)),"")</f>
         <v/>
       </c>
       <c r="H25" s="17">
@@ -5386,8 +5421,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B26,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B26,$K$8:$K$73,1)))/((E26-D26)/365)*100</f>
         <v/>
       </c>
-      <c r="G26" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B26,$K$8:$K$73,1))*EXP(-(F26/100)*(B26-D26)/365)</f>
+      <c r="G26" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B26-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((26&gt;0)*(D26-VAL_DATE)/360,0)&lt;=0,IF(((E26-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B26,$K$8:$K$73,1)+1)-1)/((E26-VAL_DATE)/360)),IF(MAX((26&gt;0)*(D26-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B26,$K$8:$K$73,1))-1)/MAX((26&gt;0)*(D26-VAL_DATE)/360,0)))+(IF(((E26-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B26,$K$8:$K$73,1)+1)-1)/((E26-VAL_DATE)/360))-IF(MAX((26&gt;0)*(D26-VAL_DATE)/360,0)&lt;=0,IF(((E26-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B26,$K$8:$K$73,1)+1)-1)/((E26-VAL_DATE)/360)),IF(MAX((26&gt;0)*(D26-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B26,$K$8:$K$73,1))-1)/MAX((26&gt;0)*(D26-VAL_DATE)/360,0))))*IF(((E26-VAL_DATE)/360)-MAX((26&gt;0)*(D26-VAL_DATE)/360,0)=0,0,(((B26-VAL_DATE)/360)-MAX((26&gt;0)*(D26-VAL_DATE)/360,0))/(((E26-VAL_DATE)/360)-MAX((26&gt;0)*(D26-VAL_DATE)/360,0))))*((B26-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B26,$K$8:$K$73,1))*EXP(-(F26/100)*(B26-D26)/365)),"")</f>
         <v/>
       </c>
       <c r="H26" s="17">
@@ -5427,8 +5462,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B27,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B27,$K$8:$K$73,1)))/((E27-D27)/365)*100</f>
         <v/>
       </c>
-      <c r="G27" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B27,$K$8:$K$73,1))*EXP(-(F27/100)*(B27-D27)/365)</f>
+      <c r="G27" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B27-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((27&gt;0)*(D27-VAL_DATE)/360,0)&lt;=0,IF(((E27-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B27,$K$8:$K$73,1)+1)-1)/((E27-VAL_DATE)/360)),IF(MAX((27&gt;0)*(D27-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B27,$K$8:$K$73,1))-1)/MAX((27&gt;0)*(D27-VAL_DATE)/360,0)))+(IF(((E27-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B27,$K$8:$K$73,1)+1)-1)/((E27-VAL_DATE)/360))-IF(MAX((27&gt;0)*(D27-VAL_DATE)/360,0)&lt;=0,IF(((E27-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B27,$K$8:$K$73,1)+1)-1)/((E27-VAL_DATE)/360)),IF(MAX((27&gt;0)*(D27-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B27,$K$8:$K$73,1))-1)/MAX((27&gt;0)*(D27-VAL_DATE)/360,0))))*IF(((E27-VAL_DATE)/360)-MAX((27&gt;0)*(D27-VAL_DATE)/360,0)=0,0,(((B27-VAL_DATE)/360)-MAX((27&gt;0)*(D27-VAL_DATE)/360,0))/(((E27-VAL_DATE)/360)-MAX((27&gt;0)*(D27-VAL_DATE)/360,0))))*((B27-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B27,$K$8:$K$73,1))*EXP(-(F27/100)*(B27-D27)/365)),"")</f>
         <v/>
       </c>
       <c r="H27" s="17">
@@ -5468,8 +5503,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B28,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B28,$K$8:$K$73,1)))/((E28-D28)/365)*100</f>
         <v/>
       </c>
-      <c r="G28" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B28,$K$8:$K$73,1))*EXP(-(F28/100)*(B28-D28)/365)</f>
+      <c r="G28" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B28-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((28&gt;0)*(D28-VAL_DATE)/360,0)&lt;=0,IF(((E28-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B28,$K$8:$K$73,1)+1)-1)/((E28-VAL_DATE)/360)),IF(MAX((28&gt;0)*(D28-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B28,$K$8:$K$73,1))-1)/MAX((28&gt;0)*(D28-VAL_DATE)/360,0)))+(IF(((E28-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B28,$K$8:$K$73,1)+1)-1)/((E28-VAL_DATE)/360))-IF(MAX((28&gt;0)*(D28-VAL_DATE)/360,0)&lt;=0,IF(((E28-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B28,$K$8:$K$73,1)+1)-1)/((E28-VAL_DATE)/360)),IF(MAX((28&gt;0)*(D28-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B28,$K$8:$K$73,1))-1)/MAX((28&gt;0)*(D28-VAL_DATE)/360,0))))*IF(((E28-VAL_DATE)/360)-MAX((28&gt;0)*(D28-VAL_DATE)/360,0)=0,0,(((B28-VAL_DATE)/360)-MAX((28&gt;0)*(D28-VAL_DATE)/360,0))/(((E28-VAL_DATE)/360)-MAX((28&gt;0)*(D28-VAL_DATE)/360,0))))*((B28-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B28,$K$8:$K$73,1))*EXP(-(F28/100)*(B28-D28)/365)),"")</f>
         <v/>
       </c>
       <c r="H28" s="17">
@@ -5509,8 +5544,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B29,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B29,$K$8:$K$73,1)))/((E29-D29)/365)*100</f>
         <v/>
       </c>
-      <c r="G29" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B29,$K$8:$K$73,1))*EXP(-(F29/100)*(B29-D29)/365)</f>
+      <c r="G29" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B29-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((29&gt;0)*(D29-VAL_DATE)/360,0)&lt;=0,IF(((E29-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B29,$K$8:$K$73,1)+1)-1)/((E29-VAL_DATE)/360)),IF(MAX((29&gt;0)*(D29-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B29,$K$8:$K$73,1))-1)/MAX((29&gt;0)*(D29-VAL_DATE)/360,0)))+(IF(((E29-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B29,$K$8:$K$73,1)+1)-1)/((E29-VAL_DATE)/360))-IF(MAX((29&gt;0)*(D29-VAL_DATE)/360,0)&lt;=0,IF(((E29-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B29,$K$8:$K$73,1)+1)-1)/((E29-VAL_DATE)/360)),IF(MAX((29&gt;0)*(D29-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B29,$K$8:$K$73,1))-1)/MAX((29&gt;0)*(D29-VAL_DATE)/360,0))))*IF(((E29-VAL_DATE)/360)-MAX((29&gt;0)*(D29-VAL_DATE)/360,0)=0,0,(((B29-VAL_DATE)/360)-MAX((29&gt;0)*(D29-VAL_DATE)/360,0))/(((E29-VAL_DATE)/360)-MAX((29&gt;0)*(D29-VAL_DATE)/360,0))))*((B29-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B29,$K$8:$K$73,1))*EXP(-(F29/100)*(B29-D29)/365)),"")</f>
         <v/>
       </c>
       <c r="H29" s="17">
@@ -5550,8 +5585,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B30,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B30,$K$8:$K$73,1)))/((E30-D30)/365)*100</f>
         <v/>
       </c>
-      <c r="G30" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B30,$K$8:$K$73,1))*EXP(-(F30/100)*(B30-D30)/365)</f>
+      <c r="G30" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B30-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((30&gt;0)*(D30-VAL_DATE)/360,0)&lt;=0,IF(((E30-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B30,$K$8:$K$73,1)+1)-1)/((E30-VAL_DATE)/360)),IF(MAX((30&gt;0)*(D30-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B30,$K$8:$K$73,1))-1)/MAX((30&gt;0)*(D30-VAL_DATE)/360,0)))+(IF(((E30-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B30,$K$8:$K$73,1)+1)-1)/((E30-VAL_DATE)/360))-IF(MAX((30&gt;0)*(D30-VAL_DATE)/360,0)&lt;=0,IF(((E30-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B30,$K$8:$K$73,1)+1)-1)/((E30-VAL_DATE)/360)),IF(MAX((30&gt;0)*(D30-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B30,$K$8:$K$73,1))-1)/MAX((30&gt;0)*(D30-VAL_DATE)/360,0))))*IF(((E30-VAL_DATE)/360)-MAX((30&gt;0)*(D30-VAL_DATE)/360,0)=0,0,(((B30-VAL_DATE)/360)-MAX((30&gt;0)*(D30-VAL_DATE)/360,0))/(((E30-VAL_DATE)/360)-MAX((30&gt;0)*(D30-VAL_DATE)/360,0))))*((B30-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B30,$K$8:$K$73,1))*EXP(-(F30/100)*(B30-D30)/365)),"")</f>
         <v/>
       </c>
       <c r="H30" s="17">
@@ -5591,8 +5626,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B31,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B31,$K$8:$K$73,1)))/((E31-D31)/365)*100</f>
         <v/>
       </c>
-      <c r="G31" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B31,$K$8:$K$73,1))*EXP(-(F31/100)*(B31-D31)/365)</f>
+      <c r="G31" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B31-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((31&gt;0)*(D31-VAL_DATE)/360,0)&lt;=0,IF(((E31-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B31,$K$8:$K$73,1)+1)-1)/((E31-VAL_DATE)/360)),IF(MAX((31&gt;0)*(D31-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B31,$K$8:$K$73,1))-1)/MAX((31&gt;0)*(D31-VAL_DATE)/360,0)))+(IF(((E31-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B31,$K$8:$K$73,1)+1)-1)/((E31-VAL_DATE)/360))-IF(MAX((31&gt;0)*(D31-VAL_DATE)/360,0)&lt;=0,IF(((E31-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B31,$K$8:$K$73,1)+1)-1)/((E31-VAL_DATE)/360)),IF(MAX((31&gt;0)*(D31-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B31,$K$8:$K$73,1))-1)/MAX((31&gt;0)*(D31-VAL_DATE)/360,0))))*IF(((E31-VAL_DATE)/360)-MAX((31&gt;0)*(D31-VAL_DATE)/360,0)=0,0,(((B31-VAL_DATE)/360)-MAX((31&gt;0)*(D31-VAL_DATE)/360,0))/(((E31-VAL_DATE)/360)-MAX((31&gt;0)*(D31-VAL_DATE)/360,0))))*((B31-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B31,$K$8:$K$73,1))*EXP(-(F31/100)*(B31-D31)/365)),"")</f>
         <v/>
       </c>
       <c r="H31" s="17">
@@ -5632,8 +5667,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B32,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B32,$K$8:$K$73,1)))/((E32-D32)/365)*100</f>
         <v/>
       </c>
-      <c r="G32" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B32,$K$8:$K$73,1))*EXP(-(F32/100)*(B32-D32)/365)</f>
+      <c r="G32" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B32-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((32&gt;0)*(D32-VAL_DATE)/360,0)&lt;=0,IF(((E32-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B32,$K$8:$K$73,1)+1)-1)/((E32-VAL_DATE)/360)),IF(MAX((32&gt;0)*(D32-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B32,$K$8:$K$73,1))-1)/MAX((32&gt;0)*(D32-VAL_DATE)/360,0)))+(IF(((E32-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B32,$K$8:$K$73,1)+1)-1)/((E32-VAL_DATE)/360))-IF(MAX((32&gt;0)*(D32-VAL_DATE)/360,0)&lt;=0,IF(((E32-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B32,$K$8:$K$73,1)+1)-1)/((E32-VAL_DATE)/360)),IF(MAX((32&gt;0)*(D32-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B32,$K$8:$K$73,1))-1)/MAX((32&gt;0)*(D32-VAL_DATE)/360,0))))*IF(((E32-VAL_DATE)/360)-MAX((32&gt;0)*(D32-VAL_DATE)/360,0)=0,0,(((B32-VAL_DATE)/360)-MAX((32&gt;0)*(D32-VAL_DATE)/360,0))/(((E32-VAL_DATE)/360)-MAX((32&gt;0)*(D32-VAL_DATE)/360,0))))*((B32-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B32,$K$8:$K$73,1))*EXP(-(F32/100)*(B32-D32)/365)),"")</f>
         <v/>
       </c>
       <c r="H32" s="17">
@@ -5673,8 +5708,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B33,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B33,$K$8:$K$73,1)))/((E33-D33)/365)*100</f>
         <v/>
       </c>
-      <c r="G33" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B33,$K$8:$K$73,1))*EXP(-(F33/100)*(B33-D33)/365)</f>
+      <c r="G33" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B33-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((33&gt;0)*(D33-VAL_DATE)/360,0)&lt;=0,IF(((E33-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B33,$K$8:$K$73,1)+1)-1)/((E33-VAL_DATE)/360)),IF(MAX((33&gt;0)*(D33-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B33,$K$8:$K$73,1))-1)/MAX((33&gt;0)*(D33-VAL_DATE)/360,0)))+(IF(((E33-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B33,$K$8:$K$73,1)+1)-1)/((E33-VAL_DATE)/360))-IF(MAX((33&gt;0)*(D33-VAL_DATE)/360,0)&lt;=0,IF(((E33-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B33,$K$8:$K$73,1)+1)-1)/((E33-VAL_DATE)/360)),IF(MAX((33&gt;0)*(D33-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B33,$K$8:$K$73,1))-1)/MAX((33&gt;0)*(D33-VAL_DATE)/360,0))))*IF(((E33-VAL_DATE)/360)-MAX((33&gt;0)*(D33-VAL_DATE)/360,0)=0,0,(((B33-VAL_DATE)/360)-MAX((33&gt;0)*(D33-VAL_DATE)/360,0))/(((E33-VAL_DATE)/360)-MAX((33&gt;0)*(D33-VAL_DATE)/360,0))))*((B33-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B33,$K$8:$K$73,1))*EXP(-(F33/100)*(B33-D33)/365)),"")</f>
         <v/>
       </c>
       <c r="H33" s="17">
@@ -5714,8 +5749,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B34,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B34,$K$8:$K$73,1)))/((E34-D34)/365)*100</f>
         <v/>
       </c>
-      <c r="G34" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B34,$K$8:$K$73,1))*EXP(-(F34/100)*(B34-D34)/365)</f>
+      <c r="G34" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B34-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((34&gt;0)*(D34-VAL_DATE)/360,0)&lt;=0,IF(((E34-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B34,$K$8:$K$73,1)+1)-1)/((E34-VAL_DATE)/360)),IF(MAX((34&gt;0)*(D34-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B34,$K$8:$K$73,1))-1)/MAX((34&gt;0)*(D34-VAL_DATE)/360,0)))+(IF(((E34-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B34,$K$8:$K$73,1)+1)-1)/((E34-VAL_DATE)/360))-IF(MAX((34&gt;0)*(D34-VAL_DATE)/360,0)&lt;=0,IF(((E34-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B34,$K$8:$K$73,1)+1)-1)/((E34-VAL_DATE)/360)),IF(MAX((34&gt;0)*(D34-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B34,$K$8:$K$73,1))-1)/MAX((34&gt;0)*(D34-VAL_DATE)/360,0))))*IF(((E34-VAL_DATE)/360)-MAX((34&gt;0)*(D34-VAL_DATE)/360,0)=0,0,(((B34-VAL_DATE)/360)-MAX((34&gt;0)*(D34-VAL_DATE)/360,0))/(((E34-VAL_DATE)/360)-MAX((34&gt;0)*(D34-VAL_DATE)/360,0))))*((B34-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B34,$K$8:$K$73,1))*EXP(-(F34/100)*(B34-D34)/365)),"")</f>
         <v/>
       </c>
       <c r="H34" s="17">
@@ -5755,8 +5790,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B35,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B35,$K$8:$K$73,1)))/((E35-D35)/365)*100</f>
         <v/>
       </c>
-      <c r="G35" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B35,$K$8:$K$73,1))*EXP(-(F35/100)*(B35-D35)/365)</f>
+      <c r="G35" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B35-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((35&gt;0)*(D35-VAL_DATE)/360,0)&lt;=0,IF(((E35-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B35,$K$8:$K$73,1)+1)-1)/((E35-VAL_DATE)/360)),IF(MAX((35&gt;0)*(D35-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B35,$K$8:$K$73,1))-1)/MAX((35&gt;0)*(D35-VAL_DATE)/360,0)))+(IF(((E35-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B35,$K$8:$K$73,1)+1)-1)/((E35-VAL_DATE)/360))-IF(MAX((35&gt;0)*(D35-VAL_DATE)/360,0)&lt;=0,IF(((E35-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B35,$K$8:$K$73,1)+1)-1)/((E35-VAL_DATE)/360)),IF(MAX((35&gt;0)*(D35-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B35,$K$8:$K$73,1))-1)/MAX((35&gt;0)*(D35-VAL_DATE)/360,0))))*IF(((E35-VAL_DATE)/360)-MAX((35&gt;0)*(D35-VAL_DATE)/360,0)=0,0,(((B35-VAL_DATE)/360)-MAX((35&gt;0)*(D35-VAL_DATE)/360,0))/(((E35-VAL_DATE)/360)-MAX((35&gt;0)*(D35-VAL_DATE)/360,0))))*((B35-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B35,$K$8:$K$73,1))*EXP(-(F35/100)*(B35-D35)/365)),"")</f>
         <v/>
       </c>
       <c r="H35" s="17">
@@ -5796,8 +5831,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B36,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B36,$K$8:$K$73,1)))/((E36-D36)/365)*100</f>
         <v/>
       </c>
-      <c r="G36" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B36,$K$8:$K$73,1))*EXP(-(F36/100)*(B36-D36)/365)</f>
+      <c r="G36" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B36-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((36&gt;0)*(D36-VAL_DATE)/360,0)&lt;=0,IF(((E36-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B36,$K$8:$K$73,1)+1)-1)/((E36-VAL_DATE)/360)),IF(MAX((36&gt;0)*(D36-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B36,$K$8:$K$73,1))-1)/MAX((36&gt;0)*(D36-VAL_DATE)/360,0)))+(IF(((E36-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B36,$K$8:$K$73,1)+1)-1)/((E36-VAL_DATE)/360))-IF(MAX((36&gt;0)*(D36-VAL_DATE)/360,0)&lt;=0,IF(((E36-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B36,$K$8:$K$73,1)+1)-1)/((E36-VAL_DATE)/360)),IF(MAX((36&gt;0)*(D36-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B36,$K$8:$K$73,1))-1)/MAX((36&gt;0)*(D36-VAL_DATE)/360,0))))*IF(((E36-VAL_DATE)/360)-MAX((36&gt;0)*(D36-VAL_DATE)/360,0)=0,0,(((B36-VAL_DATE)/360)-MAX((36&gt;0)*(D36-VAL_DATE)/360,0))/(((E36-VAL_DATE)/360)-MAX((36&gt;0)*(D36-VAL_DATE)/360,0))))*((B36-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B36,$K$8:$K$73,1))*EXP(-(F36/100)*(B36-D36)/365)),"")</f>
         <v/>
       </c>
       <c r="H36" s="17">
@@ -5837,8 +5872,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B37,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B37,$K$8:$K$73,1)))/((E37-D37)/365)*100</f>
         <v/>
       </c>
-      <c r="G37" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B37,$K$8:$K$73,1))*EXP(-(F37/100)*(B37-D37)/365)</f>
+      <c r="G37" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B37-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((37&gt;0)*(D37-VAL_DATE)/360,0)&lt;=0,IF(((E37-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B37,$K$8:$K$73,1)+1)-1)/((E37-VAL_DATE)/360)),IF(MAX((37&gt;0)*(D37-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B37,$K$8:$K$73,1))-1)/MAX((37&gt;0)*(D37-VAL_DATE)/360,0)))+(IF(((E37-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B37,$K$8:$K$73,1)+1)-1)/((E37-VAL_DATE)/360))-IF(MAX((37&gt;0)*(D37-VAL_DATE)/360,0)&lt;=0,IF(((E37-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B37,$K$8:$K$73,1)+1)-1)/((E37-VAL_DATE)/360)),IF(MAX((37&gt;0)*(D37-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B37,$K$8:$K$73,1))-1)/MAX((37&gt;0)*(D37-VAL_DATE)/360,0))))*IF(((E37-VAL_DATE)/360)-MAX((37&gt;0)*(D37-VAL_DATE)/360,0)=0,0,(((B37-VAL_DATE)/360)-MAX((37&gt;0)*(D37-VAL_DATE)/360,0))/(((E37-VAL_DATE)/360)-MAX((37&gt;0)*(D37-VAL_DATE)/360,0))))*((B37-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B37,$K$8:$K$73,1))*EXP(-(F37/100)*(B37-D37)/365)),"")</f>
         <v/>
       </c>
       <c r="H37" s="17">
@@ -5878,8 +5913,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B38,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B38,$K$8:$K$73,1)))/((E38-D38)/365)*100</f>
         <v/>
       </c>
-      <c r="G38" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B38,$K$8:$K$73,1))*EXP(-(F38/100)*(B38-D38)/365)</f>
+      <c r="G38" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B38-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((38&gt;0)*(D38-VAL_DATE)/360,0)&lt;=0,IF(((E38-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B38,$K$8:$K$73,1)+1)-1)/((E38-VAL_DATE)/360)),IF(MAX((38&gt;0)*(D38-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B38,$K$8:$K$73,1))-1)/MAX((38&gt;0)*(D38-VAL_DATE)/360,0)))+(IF(((E38-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B38,$K$8:$K$73,1)+1)-1)/((E38-VAL_DATE)/360))-IF(MAX((38&gt;0)*(D38-VAL_DATE)/360,0)&lt;=0,IF(((E38-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B38,$K$8:$K$73,1)+1)-1)/((E38-VAL_DATE)/360)),IF(MAX((38&gt;0)*(D38-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B38,$K$8:$K$73,1))-1)/MAX((38&gt;0)*(D38-VAL_DATE)/360,0))))*IF(((E38-VAL_DATE)/360)-MAX((38&gt;0)*(D38-VAL_DATE)/360,0)=0,0,(((B38-VAL_DATE)/360)-MAX((38&gt;0)*(D38-VAL_DATE)/360,0))/(((E38-VAL_DATE)/360)-MAX((38&gt;0)*(D38-VAL_DATE)/360,0))))*((B38-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B38,$K$8:$K$73,1))*EXP(-(F38/100)*(B38-D38)/365)),"")</f>
         <v/>
       </c>
       <c r="H38" s="17">
@@ -5919,8 +5954,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B39,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B39,$K$8:$K$73,1)))/((E39-D39)/365)*100</f>
         <v/>
       </c>
-      <c r="G39" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B39,$K$8:$K$73,1))*EXP(-(F39/100)*(B39-D39)/365)</f>
+      <c r="G39" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B39-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((39&gt;0)*(D39-VAL_DATE)/360,0)&lt;=0,IF(((E39-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B39,$K$8:$K$73,1)+1)-1)/((E39-VAL_DATE)/360)),IF(MAX((39&gt;0)*(D39-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B39,$K$8:$K$73,1))-1)/MAX((39&gt;0)*(D39-VAL_DATE)/360,0)))+(IF(((E39-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B39,$K$8:$K$73,1)+1)-1)/((E39-VAL_DATE)/360))-IF(MAX((39&gt;0)*(D39-VAL_DATE)/360,0)&lt;=0,IF(((E39-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B39,$K$8:$K$73,1)+1)-1)/((E39-VAL_DATE)/360)),IF(MAX((39&gt;0)*(D39-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B39,$K$8:$K$73,1))-1)/MAX((39&gt;0)*(D39-VAL_DATE)/360,0))))*IF(((E39-VAL_DATE)/360)-MAX((39&gt;0)*(D39-VAL_DATE)/360,0)=0,0,(((B39-VAL_DATE)/360)-MAX((39&gt;0)*(D39-VAL_DATE)/360,0))/(((E39-VAL_DATE)/360)-MAX((39&gt;0)*(D39-VAL_DATE)/360,0))))*((B39-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B39,$K$8:$K$73,1))*EXP(-(F39/100)*(B39-D39)/365)),"")</f>
         <v/>
       </c>
       <c r="H39" s="17">
@@ -5960,8 +5995,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B40,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B40,$K$8:$K$73,1)))/((E40-D40)/365)*100</f>
         <v/>
       </c>
-      <c r="G40" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B40,$K$8:$K$73,1))*EXP(-(F40/100)*(B40-D40)/365)</f>
+      <c r="G40" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B40-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((40&gt;0)*(D40-VAL_DATE)/360,0)&lt;=0,IF(((E40-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B40,$K$8:$K$73,1)+1)-1)/((E40-VAL_DATE)/360)),IF(MAX((40&gt;0)*(D40-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B40,$K$8:$K$73,1))-1)/MAX((40&gt;0)*(D40-VAL_DATE)/360,0)))+(IF(((E40-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B40,$K$8:$K$73,1)+1)-1)/((E40-VAL_DATE)/360))-IF(MAX((40&gt;0)*(D40-VAL_DATE)/360,0)&lt;=0,IF(((E40-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B40,$K$8:$K$73,1)+1)-1)/((E40-VAL_DATE)/360)),IF(MAX((40&gt;0)*(D40-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B40,$K$8:$K$73,1))-1)/MAX((40&gt;0)*(D40-VAL_DATE)/360,0))))*IF(((E40-VAL_DATE)/360)-MAX((40&gt;0)*(D40-VAL_DATE)/360,0)=0,0,(((B40-VAL_DATE)/360)-MAX((40&gt;0)*(D40-VAL_DATE)/360,0))/(((E40-VAL_DATE)/360)-MAX((40&gt;0)*(D40-VAL_DATE)/360,0))))*((B40-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B40,$K$8:$K$73,1))*EXP(-(F40/100)*(B40-D40)/365)),"")</f>
         <v/>
       </c>
       <c r="H40" s="17">
@@ -6001,8 +6036,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B41,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B41,$K$8:$K$73,1)))/((E41-D41)/365)*100</f>
         <v/>
       </c>
-      <c r="G41" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B41,$K$8:$K$73,1))*EXP(-(F41/100)*(B41-D41)/365)</f>
+      <c r="G41" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B41-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((41&gt;0)*(D41-VAL_DATE)/360,0)&lt;=0,IF(((E41-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B41,$K$8:$K$73,1)+1)-1)/((E41-VAL_DATE)/360)),IF(MAX((41&gt;0)*(D41-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B41,$K$8:$K$73,1))-1)/MAX((41&gt;0)*(D41-VAL_DATE)/360,0)))+(IF(((E41-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B41,$K$8:$K$73,1)+1)-1)/((E41-VAL_DATE)/360))-IF(MAX((41&gt;0)*(D41-VAL_DATE)/360,0)&lt;=0,IF(((E41-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B41,$K$8:$K$73,1)+1)-1)/((E41-VAL_DATE)/360)),IF(MAX((41&gt;0)*(D41-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B41,$K$8:$K$73,1))-1)/MAX((41&gt;0)*(D41-VAL_DATE)/360,0))))*IF(((E41-VAL_DATE)/360)-MAX((41&gt;0)*(D41-VAL_DATE)/360,0)=0,0,(((B41-VAL_DATE)/360)-MAX((41&gt;0)*(D41-VAL_DATE)/360,0))/(((E41-VAL_DATE)/360)-MAX((41&gt;0)*(D41-VAL_DATE)/360,0))))*((B41-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B41,$K$8:$K$73,1))*EXP(-(F41/100)*(B41-D41)/365)),"")</f>
         <v/>
       </c>
       <c r="H41" s="17">
@@ -6042,8 +6077,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B42,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B42,$K$8:$K$73,1)))/((E42-D42)/365)*100</f>
         <v/>
       </c>
-      <c r="G42" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B42,$K$8:$K$73,1))*EXP(-(F42/100)*(B42-D42)/365)</f>
+      <c r="G42" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B42-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((42&gt;0)*(D42-VAL_DATE)/360,0)&lt;=0,IF(((E42-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B42,$K$8:$K$73,1)+1)-1)/((E42-VAL_DATE)/360)),IF(MAX((42&gt;0)*(D42-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B42,$K$8:$K$73,1))-1)/MAX((42&gt;0)*(D42-VAL_DATE)/360,0)))+(IF(((E42-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B42,$K$8:$K$73,1)+1)-1)/((E42-VAL_DATE)/360))-IF(MAX((42&gt;0)*(D42-VAL_DATE)/360,0)&lt;=0,IF(((E42-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B42,$K$8:$K$73,1)+1)-1)/((E42-VAL_DATE)/360)),IF(MAX((42&gt;0)*(D42-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B42,$K$8:$K$73,1))-1)/MAX((42&gt;0)*(D42-VAL_DATE)/360,0))))*IF(((E42-VAL_DATE)/360)-MAX((42&gt;0)*(D42-VAL_DATE)/360,0)=0,0,(((B42-VAL_DATE)/360)-MAX((42&gt;0)*(D42-VAL_DATE)/360,0))/(((E42-VAL_DATE)/360)-MAX((42&gt;0)*(D42-VAL_DATE)/360,0))))*((B42-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B42,$K$8:$K$73,1))*EXP(-(F42/100)*(B42-D42)/365)),"")</f>
         <v/>
       </c>
       <c r="H42" s="17">
@@ -6083,8 +6118,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B43,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B43,$K$8:$K$73,1)))/((E43-D43)/365)*100</f>
         <v/>
       </c>
-      <c r="G43" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B43,$K$8:$K$73,1))*EXP(-(F43/100)*(B43-D43)/365)</f>
+      <c r="G43" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B43-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((43&gt;0)*(D43-VAL_DATE)/360,0)&lt;=0,IF(((E43-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B43,$K$8:$K$73,1)+1)-1)/((E43-VAL_DATE)/360)),IF(MAX((43&gt;0)*(D43-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B43,$K$8:$K$73,1))-1)/MAX((43&gt;0)*(D43-VAL_DATE)/360,0)))+(IF(((E43-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B43,$K$8:$K$73,1)+1)-1)/((E43-VAL_DATE)/360))-IF(MAX((43&gt;0)*(D43-VAL_DATE)/360,0)&lt;=0,IF(((E43-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B43,$K$8:$K$73,1)+1)-1)/((E43-VAL_DATE)/360)),IF(MAX((43&gt;0)*(D43-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B43,$K$8:$K$73,1))-1)/MAX((43&gt;0)*(D43-VAL_DATE)/360,0))))*IF(((E43-VAL_DATE)/360)-MAX((43&gt;0)*(D43-VAL_DATE)/360,0)=0,0,(((B43-VAL_DATE)/360)-MAX((43&gt;0)*(D43-VAL_DATE)/360,0))/(((E43-VAL_DATE)/360)-MAX((43&gt;0)*(D43-VAL_DATE)/360,0))))*((B43-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B43,$K$8:$K$73,1))*EXP(-(F43/100)*(B43-D43)/365)),"")</f>
         <v/>
       </c>
       <c r="H43" s="17">
@@ -6124,8 +6159,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B44,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B44,$K$8:$K$73,1)))/((E44-D44)/365)*100</f>
         <v/>
       </c>
-      <c r="G44" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B44,$K$8:$K$73,1))*EXP(-(F44/100)*(B44-D44)/365)</f>
+      <c r="G44" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B44-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((44&gt;0)*(D44-VAL_DATE)/360,0)&lt;=0,IF(((E44-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B44,$K$8:$K$73,1)+1)-1)/((E44-VAL_DATE)/360)),IF(MAX((44&gt;0)*(D44-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B44,$K$8:$K$73,1))-1)/MAX((44&gt;0)*(D44-VAL_DATE)/360,0)))+(IF(((E44-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B44,$K$8:$K$73,1)+1)-1)/((E44-VAL_DATE)/360))-IF(MAX((44&gt;0)*(D44-VAL_DATE)/360,0)&lt;=0,IF(((E44-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B44,$K$8:$K$73,1)+1)-1)/((E44-VAL_DATE)/360)),IF(MAX((44&gt;0)*(D44-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B44,$K$8:$K$73,1))-1)/MAX((44&gt;0)*(D44-VAL_DATE)/360,0))))*IF(((E44-VAL_DATE)/360)-MAX((44&gt;0)*(D44-VAL_DATE)/360,0)=0,0,(((B44-VAL_DATE)/360)-MAX((44&gt;0)*(D44-VAL_DATE)/360,0))/(((E44-VAL_DATE)/360)-MAX((44&gt;0)*(D44-VAL_DATE)/360,0))))*((B44-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B44,$K$8:$K$73,1))*EXP(-(F44/100)*(B44-D44)/365)),"")</f>
         <v/>
       </c>
       <c r="H44" s="17">
@@ -6165,8 +6200,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B45,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B45,$K$8:$K$73,1)))/((E45-D45)/365)*100</f>
         <v/>
       </c>
-      <c r="G45" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B45,$K$8:$K$73,1))*EXP(-(F45/100)*(B45-D45)/365)</f>
+      <c r="G45" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B45-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((45&gt;0)*(D45-VAL_DATE)/360,0)&lt;=0,IF(((E45-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B45,$K$8:$K$73,1)+1)-1)/((E45-VAL_DATE)/360)),IF(MAX((45&gt;0)*(D45-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B45,$K$8:$K$73,1))-1)/MAX((45&gt;0)*(D45-VAL_DATE)/360,0)))+(IF(((E45-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B45,$K$8:$K$73,1)+1)-1)/((E45-VAL_DATE)/360))-IF(MAX((45&gt;0)*(D45-VAL_DATE)/360,0)&lt;=0,IF(((E45-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B45,$K$8:$K$73,1)+1)-1)/((E45-VAL_DATE)/360)),IF(MAX((45&gt;0)*(D45-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B45,$K$8:$K$73,1))-1)/MAX((45&gt;0)*(D45-VAL_DATE)/360,0))))*IF(((E45-VAL_DATE)/360)-MAX((45&gt;0)*(D45-VAL_DATE)/360,0)=0,0,(((B45-VAL_DATE)/360)-MAX((45&gt;0)*(D45-VAL_DATE)/360,0))/(((E45-VAL_DATE)/360)-MAX((45&gt;0)*(D45-VAL_DATE)/360,0))))*((B45-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B45,$K$8:$K$73,1))*EXP(-(F45/100)*(B45-D45)/365)),"")</f>
         <v/>
       </c>
       <c r="H45" s="17">
@@ -6206,8 +6241,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B46,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B46,$K$8:$K$73,1)))/((E46-D46)/365)*100</f>
         <v/>
       </c>
-      <c r="G46" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B46,$K$8:$K$73,1))*EXP(-(F46/100)*(B46-D46)/365)</f>
+      <c r="G46" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B46-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((46&gt;0)*(D46-VAL_DATE)/360,0)&lt;=0,IF(((E46-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B46,$K$8:$K$73,1)+1)-1)/((E46-VAL_DATE)/360)),IF(MAX((46&gt;0)*(D46-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B46,$K$8:$K$73,1))-1)/MAX((46&gt;0)*(D46-VAL_DATE)/360,0)))+(IF(((E46-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B46,$K$8:$K$73,1)+1)-1)/((E46-VAL_DATE)/360))-IF(MAX((46&gt;0)*(D46-VAL_DATE)/360,0)&lt;=0,IF(((E46-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B46,$K$8:$K$73,1)+1)-1)/((E46-VAL_DATE)/360)),IF(MAX((46&gt;0)*(D46-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B46,$K$8:$K$73,1))-1)/MAX((46&gt;0)*(D46-VAL_DATE)/360,0))))*IF(((E46-VAL_DATE)/360)-MAX((46&gt;0)*(D46-VAL_DATE)/360,0)=0,0,(((B46-VAL_DATE)/360)-MAX((46&gt;0)*(D46-VAL_DATE)/360,0))/(((E46-VAL_DATE)/360)-MAX((46&gt;0)*(D46-VAL_DATE)/360,0))))*((B46-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B46,$K$8:$K$73,1))*EXP(-(F46/100)*(B46-D46)/365)),"")</f>
         <v/>
       </c>
       <c r="H46" s="17">
@@ -6247,8 +6282,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B47,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B47,$K$8:$K$73,1)))/((E47-D47)/365)*100</f>
         <v/>
       </c>
-      <c r="G47" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B47,$K$8:$K$73,1))*EXP(-(F47/100)*(B47-D47)/365)</f>
+      <c r="G47" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B47-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((47&gt;0)*(D47-VAL_DATE)/360,0)&lt;=0,IF(((E47-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B47,$K$8:$K$73,1)+1)-1)/((E47-VAL_DATE)/360)),IF(MAX((47&gt;0)*(D47-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B47,$K$8:$K$73,1))-1)/MAX((47&gt;0)*(D47-VAL_DATE)/360,0)))+(IF(((E47-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B47,$K$8:$K$73,1)+1)-1)/((E47-VAL_DATE)/360))-IF(MAX((47&gt;0)*(D47-VAL_DATE)/360,0)&lt;=0,IF(((E47-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B47,$K$8:$K$73,1)+1)-1)/((E47-VAL_DATE)/360)),IF(MAX((47&gt;0)*(D47-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B47,$K$8:$K$73,1))-1)/MAX((47&gt;0)*(D47-VAL_DATE)/360,0))))*IF(((E47-VAL_DATE)/360)-MAX((47&gt;0)*(D47-VAL_DATE)/360,0)=0,0,(((B47-VAL_DATE)/360)-MAX((47&gt;0)*(D47-VAL_DATE)/360,0))/(((E47-VAL_DATE)/360)-MAX((47&gt;0)*(D47-VAL_DATE)/360,0))))*((B47-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B47,$K$8:$K$73,1))*EXP(-(F47/100)*(B47-D47)/365)),"")</f>
         <v/>
       </c>
       <c r="H47" s="17">
@@ -6288,8 +6323,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B48,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B48,$K$8:$K$73,1)))/((E48-D48)/365)*100</f>
         <v/>
       </c>
-      <c r="G48" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B48,$K$8:$K$73,1))*EXP(-(F48/100)*(B48-D48)/365)</f>
+      <c r="G48" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B48-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((48&gt;0)*(D48-VAL_DATE)/360,0)&lt;=0,IF(((E48-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B48,$K$8:$K$73,1)+1)-1)/((E48-VAL_DATE)/360)),IF(MAX((48&gt;0)*(D48-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B48,$K$8:$K$73,1))-1)/MAX((48&gt;0)*(D48-VAL_DATE)/360,0)))+(IF(((E48-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B48,$K$8:$K$73,1)+1)-1)/((E48-VAL_DATE)/360))-IF(MAX((48&gt;0)*(D48-VAL_DATE)/360,0)&lt;=0,IF(((E48-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B48,$K$8:$K$73,1)+1)-1)/((E48-VAL_DATE)/360)),IF(MAX((48&gt;0)*(D48-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B48,$K$8:$K$73,1))-1)/MAX((48&gt;0)*(D48-VAL_DATE)/360,0))))*IF(((E48-VAL_DATE)/360)-MAX((48&gt;0)*(D48-VAL_DATE)/360,0)=0,0,(((B48-VAL_DATE)/360)-MAX((48&gt;0)*(D48-VAL_DATE)/360,0))/(((E48-VAL_DATE)/360)-MAX((48&gt;0)*(D48-VAL_DATE)/360,0))))*((B48-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B48,$K$8:$K$73,1))*EXP(-(F48/100)*(B48-D48)/365)),"")</f>
         <v/>
       </c>
       <c r="H48" s="17">
@@ -6329,8 +6364,8 @@
         <f>-LN(INDEX($L$8:$L$73,MATCH(B49,$K$8:$K$73,1)+1)/INDEX($L$8:$L$73,MATCH(B49,$K$8:$K$73,1)))/((E49-D49)/365)*100</f>
         <v/>
       </c>
-      <c r="G49" s="36">
-        <f>INDEX($L$8:$L$73,MATCH(B49,$K$8:$K$73,1))*EXP(-(F49/100)*(B49-D49)/365)</f>
+      <c r="G49" s="76">
+        <f>IFERROR(IF($J$7="Piecewise Linear (Simple)",IF(((B49-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(MAX((49&gt;0)*(D49-VAL_DATE)/360,0)&lt;=0,IF(((E49-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B49,$K$8:$K$73,1)+1)-1)/((E49-VAL_DATE)/360)),IF(MAX((49&gt;0)*(D49-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B49,$K$8:$K$73,1))-1)/MAX((49&gt;0)*(D49-VAL_DATE)/360,0)))+(IF(((E49-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B49,$K$8:$K$73,1)+1)-1)/((E49-VAL_DATE)/360))-IF(MAX((49&gt;0)*(D49-VAL_DATE)/360,0)&lt;=0,IF(((E49-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B49,$K$8:$K$73,1)+1)-1)/((E49-VAL_DATE)/360)),IF(MAX((49&gt;0)*(D49-VAL_DATE)/360,0)&lt;=0,0,(1/INDEX($L$8:$L$73,MATCH(B49,$K$8:$K$73,1))-1)/MAX((49&gt;0)*(D49-VAL_DATE)/360,0))))*IF(((E49-VAL_DATE)/360)-MAX((49&gt;0)*(D49-VAL_DATE)/360,0)=0,0,(((B49-VAL_DATE)/360)-MAX((49&gt;0)*(D49-VAL_DATE)/360,0))/(((E49-VAL_DATE)/360)-MAX((49&gt;0)*(D49-VAL_DATE)/360,0))))*((B49-VAL_DATE)/360))),INDEX($L$8:$L$73,MATCH(B49,$K$8:$K$73,1))*EXP(-(F49/100)*(B49-D49)/365)),"")</f>
         <v/>
       </c>
       <c r="H49" s="17">
@@ -6591,6 +6626,11 @@
     <mergeCell ref="K6:L6"/>
     <mergeCell ref="A4:H6"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="J7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Step-function forward (flat fwd),Piecewise Linear (Simple)"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix DF(spot) hardcoded as 1 on the curve grids
Curve_Interface!L8 and Swap_Pricer!L6 held DF(spot)=1, but every other node
comes from Bootstrap!H, discounted to VAL_DATE where DF(spot)=Bootstrap!D4=
0.99979779. The grids were inconsistent by the two-day spot stub.

Effect on a 1Y par swap: 4.05108% before, 4.03032% after, against a 1Y OIS input
of 4.03030% - a 2.08bp error, worst at the short end.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -1964,8 +1964,9 @@
         <f>Bootstrap!$B$4</f>
         <v/>
       </c>
-      <c r="L8" s="36" t="n">
-        <v>1</v>
+      <c r="L8" s="36">
+        <f>Bootstrap!$D$4</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -58059,8 +58060,9 @@
         <f>Bootstrap!$B$4</f>
         <v/>
       </c>
-      <c r="L6" s="36" t="n">
-        <v>1</v>
+      <c r="L6" s="36">
+        <f>Bootstrap!$D$4</f>
+        <v/>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Wire the interpolation switch into the copies actually used
Curve_Interface advertises itself as one shared D(0,t) for Swap_Pricer and the
CDS module, but nothing references its column G - it is dead. The interpolation
was triplicated inline in Curve_Interface!G (dead), CDS_Schedule!G/H and
Swap_Pricer!B19/B20, so a selector on Curve_Interface alone changed nothing.
All three now read the one selector.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -2199,7 +2199,7 @@
         </is>
       </c>
       <c r="B19" s="36">
-        <f>IFERROR(INDEX($L$6:$L$71,MATCH($B$8,$K$6:$K$71,1))*(INDEX($L$6:$L$71,MATCH($B$8,$K$6:$K$71,1)+1)/INDEX($L$6:$L$71,MATCH($B$8,$K$6:$K$71,1)))^(($B$8-INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1)))/(INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1)+1)-INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1)))),INDEX($L$6:$L$71,MATCH($B$8,$K$6:$K$71,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((($B$8-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$6:$L$71,MATCH($B$8,$K$6:$K$71,1)+1)-1)/((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1)+1)-VAL_DATE)/360)),(1/INDEX($L$6:$L$71,MATCH($B$8,$K$6:$K$71,1))-1)/((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1))-VAL_DATE)/360))+(IF(((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$6:$L$71,MATCH($B$8,$K$6:$K$71,1)+1)-1)/((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1)+1)-VAL_DATE)/360))-IF(((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$6:$L$71,MATCH($B$8,$K$6:$K$71,1)+1)-1)/((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1)+1)-VAL_DATE)/360)),(1/INDEX($L$6:$L$71,MATCH($B$8,$K$6:$K$71,1))-1)/((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1))-VAL_DATE)/360)))*IF(((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1)+1)-VAL_DATE)/360)-((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1))-VAL_DATE)/360)=0,0,((($B$8-VAL_DATE)/360)-((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1))-VAL_DATE)/360))/(((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1)+1)-VAL_DATE)/360)-((INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1))-VAL_DATE)/360))))*(($B$8-VAL_DATE)/360))),INDEX($L$6:$L$71,MATCH($B$8,$K$6:$K$71,1))*(INDEX($L$6:$L$71,MATCH($B$8,$K$6:$K$71,1)+1)/INDEX($L$6:$L$71,MATCH($B$8,$K$6:$K$71,1)))^(($B$8-INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1)))/(INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1)+1)-INDEX($K$6:$K$71,MATCH($B$8,$K$6:$K$71,1))))),INDEX($L$6:$L$71,MATCH($B$8,$K$6:$K$71,1)))</f>
         <v/>
       </c>
       <c r="C19" s="38" t="inlineStr">
@@ -2223,7 +2223,7 @@
         </is>
       </c>
       <c r="B20" s="36">
-        <f>IFERROR(INDEX($L$6:$L$71,MATCH($B$10,$K$6:$K$71,1))*(INDEX($L$6:$L$71,MATCH($B$10,$K$6:$K$71,1)+1)/INDEX($L$6:$L$71,MATCH($B$10,$K$6:$K$71,1)))^(($B$10-INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1)))/(INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1)+1)-INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1)))),INDEX($L$6:$L$71,MATCH($B$10,$K$6:$K$71,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((($B$10-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$6:$L$71,MATCH($B$10,$K$6:$K$71,1)+1)-1)/((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1)+1)-VAL_DATE)/360)),(1/INDEX($L$6:$L$71,MATCH($B$10,$K$6:$K$71,1))-1)/((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1))-VAL_DATE)/360))+(IF(((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$6:$L$71,MATCH($B$10,$K$6:$K$71,1)+1)-1)/((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1)+1)-VAL_DATE)/360))-IF(((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX($L$6:$L$71,MATCH($B$10,$K$6:$K$71,1)+1)-1)/((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1)+1)-VAL_DATE)/360)),(1/INDEX($L$6:$L$71,MATCH($B$10,$K$6:$K$71,1))-1)/((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1))-VAL_DATE)/360)))*IF(((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1)+1)-VAL_DATE)/360)-((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1))-VAL_DATE)/360)=0,0,((($B$10-VAL_DATE)/360)-((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1))-VAL_DATE)/360))/(((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1)+1)-VAL_DATE)/360)-((INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1))-VAL_DATE)/360))))*(($B$10-VAL_DATE)/360))),INDEX($L$6:$L$71,MATCH($B$10,$K$6:$K$71,1))*(INDEX($L$6:$L$71,MATCH($B$10,$K$6:$K$71,1)+1)/INDEX($L$6:$L$71,MATCH($B$10,$K$6:$K$71,1)))^(($B$10-INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1)))/(INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1)+1)-INDEX($K$6:$K$71,MATCH($B$10,$K$6:$K$71,1))))),INDEX($L$6:$L$71,MATCH($B$10,$K$6:$K$71,1)))</f>
         <v/>
       </c>
       <c r="K20" s="18">
@@ -13650,7 +13650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:P46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -13691,7 +13691,13 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
+    <row r="5">
+      <c r="P5" s="65" t="inlineStr">
+        <is>
+          <t>DF(end)/DF(mid) honour the interpolation selector at Curve_Interface!J7. Default is step-function forward, which is the method verified against the S490 screen.</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
@@ -13794,11 +13800,11 @@
         <v/>
       </c>
       <c r="G7" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)))^((C7-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C7-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C7-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C7-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)))^((C7-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C7,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H7" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B7+C7)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B7+C7)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B7+C7)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B7+C7)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B7+C7)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B7+C7)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I7" s="52">
@@ -13855,11 +13861,11 @@
         <v/>
       </c>
       <c r="G8" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)))^((C8-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C8-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C8-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C8-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)))^((C8-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C8,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H8" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B8+C8)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B8+C8)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B8+C8)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B8+C8)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B8+C8)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B8+C8)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I8" s="52">
@@ -13916,11 +13922,11 @@
         <v/>
       </c>
       <c r="G9" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)))^((C9-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C9-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C9-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C9-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)))^((C9-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C9,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H9" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B9+C9)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B9+C9)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B9+C9)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B9+C9)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B9+C9)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B9+C9)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I9" s="52">
@@ -13977,11 +13983,11 @@
         <v/>
       </c>
       <c r="G10" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)))^((C10-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C10-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C10-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C10-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)))^((C10-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C10,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H10" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B10+C10)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B10+C10)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B10+C10)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B10+C10)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B10+C10)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B10+C10)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I10" s="52">
@@ -14038,11 +14044,11 @@
         <v/>
       </c>
       <c r="G11" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)))^((C11-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C11-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C11-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C11-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)))^((C11-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C11,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H11" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B11+C11)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B11+C11)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B11+C11)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B11+C11)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B11+C11)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B11+C11)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I11" s="52">
@@ -14099,11 +14105,11 @@
         <v/>
       </c>
       <c r="G12" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)))^((C12-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C12-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C12-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C12-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)))^((C12-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C12,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H12" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B12+C12)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B12+C12)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B12+C12)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B12+C12)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B12+C12)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B12+C12)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I12" s="52">
@@ -14160,11 +14166,11 @@
         <v/>
       </c>
       <c r="G13" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)))^((C13-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C13-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C13-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C13-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)))^((C13-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C13,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H13" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B13+C13)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B13+C13)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B13+C13)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B13+C13)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B13+C13)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B13+C13)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I13" s="52">
@@ -14221,11 +14227,11 @@
         <v/>
       </c>
       <c r="G14" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)))^((C14-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C14-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C14-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C14-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)))^((C14-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C14,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H14" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B14+C14)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B14+C14)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B14+C14)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B14+C14)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B14+C14)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B14+C14)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I14" s="52">
@@ -14282,11 +14288,11 @@
         <v/>
       </c>
       <c r="G15" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)))^((C15-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C15-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C15-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C15-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)))^((C15-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C15,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H15" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B15+C15)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B15+C15)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B15+C15)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B15+C15)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B15+C15)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B15+C15)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I15" s="52">
@@ -14343,11 +14349,11 @@
         <v/>
       </c>
       <c r="G16" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)))^((C16-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C16-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C16-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C16-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)))^((C16-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C16,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H16" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B16+C16)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B16+C16)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B16+C16)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B16+C16)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B16+C16)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B16+C16)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I16" s="52">
@@ -14404,11 +14410,11 @@
         <v/>
       </c>
       <c r="G17" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)))^((C17-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C17-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C17-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C17-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)))^((C17-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C17,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H17" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B17+C17)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B17+C17)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B17+C17)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B17+C17)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B17+C17)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B17+C17)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I17" s="52">
@@ -14465,11 +14471,11 @@
         <v/>
       </c>
       <c r="G18" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)))^((C18-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C18-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C18-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C18-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)))^((C18-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C18,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H18" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B18+C18)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B18+C18)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B18+C18)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B18+C18)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B18+C18)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B18+C18)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I18" s="52">
@@ -14526,11 +14532,11 @@
         <v/>
       </c>
       <c r="G19" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)))^((C19-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C19-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C19-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C19-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)))^((C19-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C19,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H19" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B19+C19)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B19+C19)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B19+C19)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B19+C19)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B19+C19)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B19+C19)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I19" s="52">
@@ -14587,11 +14593,11 @@
         <v/>
       </c>
       <c r="G20" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)))^((C20-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C20-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C20-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C20-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)))^((C20-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C20,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H20" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B20+C20)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B20+C20)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B20+C20)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B20+C20)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B20+C20)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B20+C20)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I20" s="52">
@@ -14648,11 +14654,11 @@
         <v/>
       </c>
       <c r="G21" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)))^((C21-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C21-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C21-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C21-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)))^((C21-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C21,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H21" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B21+C21)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B21+C21)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B21+C21)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B21+C21)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B21+C21)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B21+C21)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I21" s="52">
@@ -14709,11 +14715,11 @@
         <v/>
       </c>
       <c r="G22" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)))^((C22-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C22-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C22-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C22-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)))^((C22-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C22,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H22" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B22+C22)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B22+C22)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B22+C22)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B22+C22)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B22+C22)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B22+C22)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I22" s="52">
@@ -14770,11 +14776,11 @@
         <v/>
       </c>
       <c r="G23" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)))^((C23-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C23-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C23-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C23-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)))^((C23-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C23,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H23" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B23+C23)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B23+C23)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B23+C23)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B23+C23)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B23+C23)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B23+C23)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I23" s="52">
@@ -14831,11 +14837,11 @@
         <v/>
       </c>
       <c r="G24" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)))^((C24-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C24-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C24-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C24-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)))^((C24-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C24,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H24" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B24+C24)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B24+C24)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B24+C24)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B24+C24)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B24+C24)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B24+C24)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I24" s="52">
@@ -14892,11 +14898,11 @@
         <v/>
       </c>
       <c r="G25" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)))^((C25-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C25-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C25-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C25-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)))^((C25-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C25,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H25" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B25+C25)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B25+C25)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B25+C25)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B25+C25)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B25+C25)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B25+C25)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I25" s="52">
@@ -14953,11 +14959,11 @@
         <v/>
       </c>
       <c r="G26" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)))^((C26-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C26-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C26-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C26-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)))^((C26-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C26,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H26" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B26+C26)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B26+C26)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B26+C26)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B26+C26)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B26+C26)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B26+C26)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I26" s="52">
@@ -15014,11 +15020,11 @@
         <v/>
       </c>
       <c r="G27" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)))^((C27-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C27-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C27-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C27-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)))^((C27-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C27,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H27" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B27+C27)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B27+C27)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B27+C27)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B27+C27)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B27+C27)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B27+C27)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I27" s="52">
@@ -15075,11 +15081,11 @@
         <v/>
       </c>
       <c r="G28" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)))^((C28-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C28-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C28-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C28-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)))^((C28-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C28,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H28" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B28+C28)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B28+C28)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B28+C28)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B28+C28)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B28+C28)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B28+C28)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I28" s="52">
@@ -15136,11 +15142,11 @@
         <v/>
       </c>
       <c r="G29" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)))^((C29-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C29-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C29-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C29-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)))^((C29-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C29,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H29" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B29+C29)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B29+C29)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B29+C29)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B29+C29)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B29+C29)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B29+C29)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I29" s="52">
@@ -15197,11 +15203,11 @@
         <v/>
       </c>
       <c r="G30" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)))^((C30-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C30-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C30-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C30-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)))^((C30-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C30,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H30" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B30+C30)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B30+C30)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B30+C30)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B30+C30)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B30+C30)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B30+C30)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I30" s="52">
@@ -15258,11 +15264,11 @@
         <v/>
       </c>
       <c r="G31" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)))^((C31-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C31-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C31-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C31-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)))^((C31-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C31,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H31" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B31+C31)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B31+C31)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B31+C31)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B31+C31)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B31+C31)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B31+C31)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I31" s="52">
@@ -15319,11 +15325,11 @@
         <v/>
       </c>
       <c r="G32" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)))^((C32-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C32-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C32-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C32-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)))^((C32-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C32,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H32" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B32+C32)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B32+C32)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B32+C32)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B32+C32)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B32+C32)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B32+C32)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I32" s="52">
@@ -15380,11 +15386,11 @@
         <v/>
       </c>
       <c r="G33" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)))^((C33-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C33-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C33-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C33-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)))^((C33-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C33,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H33" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B33+C33)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B33+C33)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B33+C33)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B33+C33)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B33+C33)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B33+C33)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I33" s="52">
@@ -15441,11 +15447,11 @@
         <v/>
       </c>
       <c r="G34" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)))^((C34-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C34-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C34-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C34-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)))^((C34-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C34,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H34" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B34+C34)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B34+C34)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B34+C34)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B34+C34)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B34+C34)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B34+C34)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I34" s="52">
@@ -15502,11 +15508,11 @@
         <v/>
       </c>
       <c r="G35" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)))^((C35-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C35-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C35-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C35-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)))^((C35-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C35,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H35" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B35+C35)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B35+C35)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B35+C35)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B35+C35)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B35+C35)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B35+C35)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I35" s="52">
@@ -15563,11 +15569,11 @@
         <v/>
       </c>
       <c r="G36" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)))^((C36-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C36-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C36-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C36-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)))^((C36-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C36,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H36" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B36+C36)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B36+C36)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B36+C36)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B36+C36)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B36+C36)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B36+C36)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I36" s="52">
@@ -15624,11 +15630,11 @@
         <v/>
       </c>
       <c r="G37" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)))^((C37-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C37-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C37-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C37-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)))^((C37-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C37,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H37" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B37+C37)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B37+C37)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B37+C37)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B37+C37)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B37+C37)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B37+C37)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I37" s="52">
@@ -15685,11 +15691,11 @@
         <v/>
       </c>
       <c r="G38" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)))^((C38-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C38-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C38-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C38-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)))^((C38-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C38,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H38" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B38+C38)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B38+C38)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B38+C38)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B38+C38)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B38+C38)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B38+C38)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I38" s="52">
@@ -15746,11 +15752,11 @@
         <v/>
       </c>
       <c r="G39" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)))^((C39-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C39-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C39-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C39-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)))^((C39-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C39,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H39" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B39+C39)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B39+C39)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B39+C39)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B39+C39)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B39+C39)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B39+C39)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I39" s="52">
@@ -15807,11 +15813,11 @@
         <v/>
       </c>
       <c r="G40" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)))^((C40-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C40-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C40-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C40-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)))^((C40-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C40,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H40" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B40+C40)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B40+C40)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B40+C40)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B40+C40)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B40+C40)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B40+C40)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I40" s="52">
@@ -15868,11 +15874,11 @@
         <v/>
       </c>
       <c r="G41" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)))^((C41-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C41-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C41-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C41-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)))^((C41-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C41,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H41" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B41+C41)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B41+C41)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B41+C41)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B41+C41)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B41+C41)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B41+C41)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I41" s="52">
@@ -15929,11 +15935,11 @@
         <v/>
       </c>
       <c r="G42" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)))^((C42-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C42-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C42-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C42-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)))^((C42-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C42,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H42" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B42+C42)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B42+C42)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B42+C42)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B42+C42)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B42+C42)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B42+C42)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I42" s="52">
@@ -15990,11 +15996,11 @@
         <v/>
       </c>
       <c r="G43" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)))^((C43-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C43-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C43-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C43-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)))^((C43-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C43,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H43" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B43+C43)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B43+C43)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B43+C43)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B43+C43)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B43+C43)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B43+C43)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I43" s="52">
@@ -16051,11 +16057,11 @@
         <v/>
       </c>
       <c r="G44" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)))^((C44-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C44-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C44-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C44-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)))^((C44-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C44,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H44" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B44+C44)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B44+C44)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B44+C44)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B44+C44)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B44+C44)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B44+C44)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I44" s="52">
@@ -16112,11 +16118,11 @@
         <v/>
       </c>
       <c r="G45" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)))^((C45-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C45-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C45-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C45-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)))^((C45-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C45,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H45" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B45+C45)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B45+C45)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B45+C45)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B45+C45)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B45+C45)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B45+C45)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I45" s="52">
@@ -16173,11 +16179,11 @@
         <v/>
       </c>
       <c r="G46" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)))^((C46-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF(((C46-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,(((C46-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*((C46-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)))^((C46-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH(C46,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="H46" s="36">
-        <f>IFERROR(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B46+C46)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
+        <f>IFERROR(IF(Curve_Interface!$J$7="Piecewise Linear (Simple)",IF((((B46+C46)/2-VAL_DATE)/360)&lt;=0,1,1/(1+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))+(IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360))-IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)&lt;=0,IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)&lt;=0,0,(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)),(1/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1))-1)/((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)))*IF(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360)=0,0,((((B46+C46)/2-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))/(((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-VAL_DATE)/360)-((INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1))-VAL_DATE)/360))))*(((B46+C46)/2-VAL_DATE)/360))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1))*(INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)/INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)))^(((B46+C46)/2-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)))/(INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)+1)-INDEX('Curve_Interface'!$K$8:$K$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1))))),INDEX('Curve_Interface'!$L$8:$L$73,MATCH((B46+C46)/2,'Curve_Interface'!$K$8:$K$73,1)))</f>
         <v/>
       </c>
       <c r="I46" s="52">

</xml_diff>

<commit_message>
Use the observed overnight rate, not one fitted to the answer
The o/n stub was 3.64055%, obtained by minimising error against the S490
discount column - an input tuned until our output matched the mandate output.
That is circular and stops the comparison being an independent check.

The screen shows an observed overnight rate of 3.59000 (bid = ask, a fixing not
a quote). Using it costs 0.6bp at the very front end and nothing beyond 2Y:

  observed 3.59%     0.881bp front, 0.106bp from 2Y
  fitted   3.64055%  0.258bp front, 0.087bp from 2Y

Curve inputs are now exclusively things we pull - the 32 OIS swap rates and the
overnight fixing. Nothing is derived from the S490 zero/discount columns, which
serve only as the comparison target. It also keeps the off-terminal fallback
consistent with the live SOFRRATE pull.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -41,7 +41,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="12">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.00000000"/>
@@ -53,7 +53,6 @@
     <numFmt numFmtId="172" formatCode="0.00000"/>
     <numFmt numFmtId="173" formatCode="mm/dd/yy"/>
     <numFmt numFmtId="174" formatCode="0.###"/>
-    <numFmt numFmtId="175" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -29782,11 +29781,11 @@
         <v/>
       </c>
       <c r="E6" s="85" t="n">
-        <v>3.64055</v>
-      </c>
-      <c r="F6" s="98" t="inlineStr">
-        <is>
-          <t>LIVE on a terminal: C6 pulls the real SOFRRATE fixing and OVERRIDES this cell. This 3.64055% is only the off-terminal fallback (fitted so DFspot reproduces the 07/21/26 S490 screen). Expect the front end to shift when live: ~1.1bp at 1W and ~0.3bp at 1M if the fixing is 3.59%, but under 0.03bp from 1Y out. The long end is unaffected.</t>
+        <v>3.59</v>
+      </c>
+      <c r="F6" s="65" t="inlineStr">
+        <is>
+          <t>OBSERVED overnight rate from the S490 screen 07/21/26 (bid = ask = 3.59000), NOT fitted. Off-terminal fallback only: on a terminal C6 pulls the live SOFRRATE fixing. Every curve input is now something we pull - nothing is derived from the S490 zero/discount columns, which are purely the comparison target.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align the CDS pull with Bloomberg Help Desk H#1330731572
Field is PX_LAST, not PX_MID - their documented step 2 is
=BDP(<ticker>&" BEST Curncy","PX_LAST"). Swap the order, keeping PX_MID as
fallback.

Their tenor list is 1Y/3Y/5Y/7Y/10Y with no 2Y, so CDS_SPREAD_TICKER_2Y may not
be a valid field; the 2Y row is flagged. It fails safe to the manual spread.

Record the limitation in their words: Bloomberg does not expose a zero-coupon CDS
spread by maturity, and bootstrapped hazard rates are not a standard export. The
hazard curve therefore has NO exportable ground truth, unlike the SOFR curve
which is matched against S490 to 0.36bp. CDS_Validation is internal consistency
only; external validation needs CDSW screen output for a known trade.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -8241,7 +8241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8338,7 +8338,7 @@
         <v>40</v>
       </c>
       <c r="F7" s="63">
-        <f>IFERROR(BDP(D7&amp;" BEST Curncy","PX_MID")+0,IFERROR(BDP(D7,"PX_LAST")+0,E7))</f>
+        <f>IFERROR(BDP(D7&amp;" BEST Curncy","PX_LAST")+0,IFERROR(BDP(D7&amp;" BEST Curncy","PX_MID")+0,E7))</f>
         <v/>
       </c>
       <c r="G7" s="52">
@@ -8346,7 +8346,7 @@
         <v/>
       </c>
       <c r="H7" s="93">
-        <f>IF(ISNUMBER(IFERROR(BDP(D7&amp;" BEST Curncy","PX_MID")+0,"")),"BDP live","MANUAL (demo)")</f>
+        <f>IF(ISNUMBER(IFERROR(BDP(D7&amp;" BEST Curncy","PX_LAST")+0,"")),"BDP live","MANUAL (demo)")</f>
         <v/>
       </c>
     </row>
@@ -8371,7 +8371,7 @@
         <v>55</v>
       </c>
       <c r="F8" s="63">
-        <f>IFERROR(BDP(D8&amp;" BEST Curncy","PX_MID")+0,IFERROR(BDP(D8,"PX_LAST")+0,E8))</f>
+        <f>IFERROR(BDP(D8&amp;" BEST Curncy","PX_LAST")+0,IFERROR(BDP(D8&amp;" BEST Curncy","PX_MID")+0,E8))</f>
         <v/>
       </c>
       <c r="G8" s="52">
@@ -8379,8 +8379,13 @@
         <v/>
       </c>
       <c r="H8" s="93">
-        <f>IF(ISNUMBER(IFERROR(BDP(D8&amp;" BEST Curncy","PX_MID")+0,"")),"BDP live","MANUAL (demo)")</f>
-        <v/>
+        <f>IF(ISNUMBER(IFERROR(BDP(D8&amp;" BEST Curncy","PX_LAST")+0,"")),"BDP live","MANUAL (demo)")</f>
+        <v/>
+      </c>
+      <c r="I8" s="66" t="inlineStr">
+        <is>
+          <t>tenor not in the Help Desk list (1Y/3Y/5Y/7Y/10Y) - CDS_SPREAD_TICKER_2Y may not be a valid field</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -8404,7 +8409,7 @@
         <v>70</v>
       </c>
       <c r="F9" s="63">
-        <f>IFERROR(BDP(D9&amp;" BEST Curncy","PX_MID")+0,IFERROR(BDP(D9,"PX_LAST")+0,E9))</f>
+        <f>IFERROR(BDP(D9&amp;" BEST Curncy","PX_LAST")+0,IFERROR(BDP(D9&amp;" BEST Curncy","PX_MID")+0,E9))</f>
         <v/>
       </c>
       <c r="G9" s="52">
@@ -8412,7 +8417,7 @@
         <v/>
       </c>
       <c r="H9" s="93">
-        <f>IF(ISNUMBER(IFERROR(BDP(D9&amp;" BEST Curncy","PX_MID")+0,"")),"BDP live","MANUAL (demo)")</f>
+        <f>IF(ISNUMBER(IFERROR(BDP(D9&amp;" BEST Curncy","PX_LAST")+0,"")),"BDP live","MANUAL (demo)")</f>
         <v/>
       </c>
     </row>
@@ -8437,7 +8442,7 @@
         <v>95</v>
       </c>
       <c r="F10" s="63">
-        <f>IFERROR(BDP(D10&amp;" BEST Curncy","PX_MID")+0,IFERROR(BDP(D10,"PX_LAST")+0,E10))</f>
+        <f>IFERROR(BDP(D10&amp;" BEST Curncy","PX_LAST")+0,IFERROR(BDP(D10&amp;" BEST Curncy","PX_MID")+0,E10))</f>
         <v/>
       </c>
       <c r="G10" s="52">
@@ -8445,7 +8450,7 @@
         <v/>
       </c>
       <c r="H10" s="93">
-        <f>IF(ISNUMBER(IFERROR(BDP(D10&amp;" BEST Curncy","PX_MID")+0,"")),"BDP live","MANUAL (demo)")</f>
+        <f>IF(ISNUMBER(IFERROR(BDP(D10&amp;" BEST Curncy","PX_LAST")+0,"")),"BDP live","MANUAL (demo)")</f>
         <v/>
       </c>
     </row>
@@ -8470,7 +8475,7 @@
         <v>115</v>
       </c>
       <c r="F11" s="63">
-        <f>IFERROR(BDP(D11&amp;" BEST Curncy","PX_MID")+0,IFERROR(BDP(D11,"PX_LAST")+0,E11))</f>
+        <f>IFERROR(BDP(D11&amp;" BEST Curncy","PX_LAST")+0,IFERROR(BDP(D11&amp;" BEST Curncy","PX_MID")+0,E11))</f>
         <v/>
       </c>
       <c r="G11" s="52">
@@ -8478,7 +8483,7 @@
         <v/>
       </c>
       <c r="H11" s="93">
-        <f>IF(ISNUMBER(IFERROR(BDP(D11&amp;" BEST Curncy","PX_MID")+0,"")),"BDP live","MANUAL (demo)")</f>
+        <f>IF(ISNUMBER(IFERROR(BDP(D11&amp;" BEST Curncy","PX_LAST")+0,"")),"BDP live","MANUAL (demo)")</f>
         <v/>
       </c>
     </row>
@@ -8503,7 +8508,7 @@
         <v>135</v>
       </c>
       <c r="F12" s="63">
-        <f>IFERROR(BDP(D12&amp;" BEST Curncy","PX_MID")+0,IFERROR(BDP(D12,"PX_LAST")+0,E12))</f>
+        <f>IFERROR(BDP(D12&amp;" BEST Curncy","PX_LAST")+0,IFERROR(BDP(D12&amp;" BEST Curncy","PX_MID")+0,E12))</f>
         <v/>
       </c>
       <c r="G12" s="52">
@@ -8511,7 +8516,7 @@
         <v/>
       </c>
       <c r="H12" s="93">
-        <f>IF(ISNUMBER(IFERROR(BDP(D12&amp;" BEST Curncy","PX_MID")+0,"")),"BDP live","MANUAL (demo)")</f>
+        <f>IF(ISNUMBER(IFERROR(BDP(D12&amp;" BEST Curncy","PX_LAST")+0,"")),"BDP live","MANUAL (demo)")</f>
         <v/>
       </c>
     </row>
@@ -8519,6 +8524,27 @@
       <c r="A14" s="66" t="inlineStr">
         <is>
           <t>WARNING: the manual spreads in column E (40/55/70/95/115/135) are DEMO PLACEHOLDERS, not market data — unlike the SOFR OIS quotes, which are the real 07/21/26 S490 levels. Column H tells you which source each tenor is actually using. Replace column E, or connect a terminal, before trusting any CDS output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="65" t="inlineStr">
+        <is>
+          <t>SOURCE: Bloomberg Help Desk H#1330731572. Step 1 =BDP(&lt;ticker&gt;,"CDS_SPREAD_TICKER_nY") resolves each tenor's CDS ticker; step 2 =BDP(&lt;returned&gt;&amp;" BEST Curncy","PX_LAST") quotes it. Documented tenors: 1Y, 3Y, 5Y, 7Y, 10Y.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="66" t="inlineStr">
+        <is>
+          <t>LIMITATION (Bloomberg's words): they do not provide a zero-coupon CDS spread by maturity as an exportable field, and the bootstrapped hazard rates are not a standard export. So there is NO exportable ground truth for the hazard curve - unlike the SOFR curve, which is matched against S490 to 0.36bp. Validate the credit side indirectly against CDSW screen output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="65" t="inlineStr">
+        <is>
+          <t>Bloomberg's suggested term structure is the credit triangle, Hazard = S/(1-R). That is only exact for a flat curve; Hazard_Solver bootstraps properly instead. CDS_Validation rows 13-18 compare the two so the difference stays visible. Methodology: CDS Model White Paper {LPHP CDSW 0:1 2989941 &lt;GO&gt;}, {HELP CDSW &lt;GO&gt;}.</t>
         </is>
       </c>
     </row>
@@ -28702,7 +28728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -28963,6 +28989,13 @@
       <c r="D18" s="51">
         <f>B18-C18</f>
         <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="66" t="inlineStr">
+        <is>
+          <t>NOTE: there is no Bloomberg export of bootstrapped hazard rates or zero-coupon CDS spreads (Help Desk H#1330731572), so these checks are INTERNAL consistency only - they confirm the curve reprices its own inputs, not that it agrees with Bloomberg. For external validation compare CDSW screen output (points upfront, price, cash amount) for a known trade.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add the CDSW screen output panel to CDS_Pricer
CDS_Pricer had the analytics but not the screen's settlement figures. Adds, in
the order CDSW shows them: points upfront, price, principal, accrued days,
accrued, cash amount, default exposure.

Accrual start is the previous IMM roll, business-day adjusted - 20 Jun 2026 is a
Saturday, so it lands on 06/22/26, matching the reference screen. Accrued days
counts both endpoints per ISDA, giving 30 days and 100bp*10mm*30/360 = 8,333.33,
both exactly as the screen shows.

This makes the workbook the single deliverable; the standalone CDSW_CDS_Pricer
is retired.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -41,7 +41,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="11">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.00000000"/>
@@ -53,6 +53,7 @@
     <numFmt numFmtId="172" formatCode="0.00000"/>
     <numFmt numFmtId="173" formatCode="mm/dd/yy"/>
     <numFmt numFmtId="174" formatCode="0.###"/>
+    <numFmt numFmtId="175" formatCode="$#,##0;($#,##0);-"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -219,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -357,6 +358,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="173" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="175" fontId="14" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="175" fontId="14" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -28454,7 +28458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -28721,6 +28725,155 @@
       <c r="C25" s="16" t="inlineStr">
         <is>
           <t>Default-now P&amp;L to your direction: LGD payout - current PV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="67" t="inlineStr">
+        <is>
+          <t>CDSW SCREEN OUTPUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="65" t="inlineStr">
+        <is>
+          <t>Settlement figures in the order the CDSW screen shows them. S = par spread implied by the curve (B15); C = contractual coupon (B6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="94" t="inlineStr">
+        <is>
+          <t>1st accrual start</t>
+        </is>
+      </c>
+      <c r="B30" s="86">
+        <f>IF(MONTH((EDATE(CDS_Parameters!$B$5,-3)+IF(WEEKDAY(EDATE(CDS_Parameters!$B$5,-3),2)=6,2,IF(WEEKDAY(EDATE(CDS_Parameters!$B$5,-3),2)=7,1,0))))&lt;&gt;MONTH(EDATE(CDS_Parameters!$B$5,-3)),(EDATE(CDS_Parameters!$B$5,-3)-IF(WEEKDAY(EDATE(CDS_Parameters!$B$5,-3),2)=6,1,IF(WEEKDAY(EDATE(CDS_Parameters!$B$5,-3),2)=7,2,0))),(EDATE(CDS_Parameters!$B$5,-3)+IF(WEEKDAY(EDATE(CDS_Parameters!$B$5,-3),2)=6,2,IF(WEEKDAY(EDATE(CDS_Parameters!$B$5,-3),2)=7,1,0))))</f>
+        <v/>
+      </c>
+      <c r="C30" s="65" t="inlineStr">
+        <is>
+          <t>Previous IMM roll, business-day adjusted. 20 Jun 2026 is a Saturday, so the screen shows 06/22/26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="67" t="inlineStr">
+        <is>
+          <t>Points upfront</t>
+        </is>
+      </c>
+      <c r="B31" s="71">
+        <f>(($B$15/10000)-CDS_Parameters!$B$10/10000)*$B$12*100</f>
+        <v/>
+      </c>
+      <c r="C31" s="65" t="inlineStr">
+        <is>
+          <t>(S - C) * RPV01 * 100, protection buyer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="67" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="B32" s="71">
+        <f>100-B31</f>
+        <v/>
+      </c>
+      <c r="C32" s="65" t="inlineStr">
+        <is>
+          <t>100 - points upfront.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="94" t="inlineStr">
+        <is>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="B33" s="103">
+        <f>IF(CDS_Parameters!$B$15="Buy protection",1,-1)*(($B$15/10000)-CDS_Parameters!$B$10/10000)*$B$12*CDS_Parameters!$B$9</f>
+        <v/>
+      </c>
+      <c r="C33" s="65" t="inlineStr">
+        <is>
+          <t>Clean upfront in cash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="94" t="inlineStr">
+        <is>
+          <t>Accrued days</t>
+        </is>
+      </c>
+      <c r="B34" s="104">
+        <f>MAX(0,CDS_Parameters!$B$4-B30+1)</f>
+        <v/>
+      </c>
+      <c r="C34" s="65" t="inlineStr">
+        <is>
+          <t>ISDA counts both endpoints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="94" t="inlineStr">
+        <is>
+          <t>Accrued</t>
+        </is>
+      </c>
+      <c r="B35" s="103">
+        <f>-IF(CDS_Parameters!$B$15="Buy protection",1,-1)*CDS_Parameters!$B$10/10000*CDS_Parameters!$B$9*B34/360</f>
+        <v/>
+      </c>
+      <c r="C35" s="65" t="inlineStr">
+        <is>
+          <t>Coupon * notional * days/360.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="67" t="inlineStr">
+        <is>
+          <t>Cash Amount</t>
+        </is>
+      </c>
+      <c r="B36" s="105">
+        <f>B33+B35</f>
+        <v/>
+      </c>
+      <c r="C36" s="65" t="inlineStr">
+        <is>
+          <t>Principal + accrued.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="94" t="inlineStr">
+        <is>
+          <t>Default Exposure</t>
+        </is>
+      </c>
+      <c r="B37" s="103">
+        <f>(1-CDS_Parameters!$B$8)*CDS_Parameters!$B$9-B33</f>
+        <v/>
+      </c>
+      <c r="C37" s="65" t="inlineStr">
+        <is>
+          <t>(1-R) * notional less the principal already paid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="65" t="inlineStr">
+        <is>
+          <t>Reference CDSW screen (CINDBK 5Y, 07/21/26) for validation: points upfront -1.97596265, price 101.97596265, principal -197,597, accrued -8,333 (30 days), cash -205,930, default exposure 6,197,596. Those are TARGETS for a like-for-like trade, not model output - the demo spreads here are not that entity's curve.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Business-day roll the displayed maturity dates on SOFR_OIS_Quotes
Column C parsed the tenor label with no roll, showing weekend maturities:
1M 08/23/2026, 6M 01/23/2027, 18M 01/23/2028, 7Y 07/23/2033. S490 shows 08/24,
01/25, 01/24, 07/25. All 32 now match the screen.

Display only - a reference scan shows just column H (mid rate) is read by other
sheets (49 refs, all Bootstrap), which computes its own rolled dates. The curve
was never affected. But the sheet was showing maturities that disagreed with both
Bloomberg and the curve built from them.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -30043,7 +30043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30154,6 +30154,11 @@
         </is>
       </c>
       <c r="L4" s="62" t="inlineStr"/>
+      <c r="M4" s="65" t="inlineStr">
+        <is>
+          <t>Maturity dates are modified-following business-day adjusted, matching S490 and the Bootstrap sheet. Display only - the curve reads column H (mid) alone.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -30167,7 +30172,7 @@
         </is>
       </c>
       <c r="C5" s="23">
-        <f>IF(RIGHT(B5,1)="W",$B$3+7*VALUE(LEFT(B5,LEN(B5)-1)),IF(RIGHT(B5,1)="M",EDATE($B$3,VALUE(LEFT(B5,LEN(B5)-1))),EDATE($B$3,12*VALUE(LEFT(B5,LEN(B5)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B5,1)="W",$B$3+7*VALUE(LEFT(B5,LEN(B5)-1)),IF(RIGHT(B5,1)="M",EDATE($B$3,VALUE(LEFT(B5,LEN(B5)-1))),EDATE($B$3,12*VALUE(LEFT(B5,LEN(B5)-1)))))+IF(WEEKDAY(IF(RIGHT(B5,1)="W",$B$3+7*VALUE(LEFT(B5,LEN(B5)-1)),IF(RIGHT(B5,1)="M",EDATE($B$3,VALUE(LEFT(B5,LEN(B5)-1))),EDATE($B$3,12*VALUE(LEFT(B5,LEN(B5)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B5,1)="W",$B$3+7*VALUE(LEFT(B5,LEN(B5)-1)),IF(RIGHT(B5,1)="M",EDATE($B$3,VALUE(LEFT(B5,LEN(B5)-1))),EDATE($B$3,12*VALUE(LEFT(B5,LEN(B5)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B5,1)="W",$B$3+7*VALUE(LEFT(B5,LEN(B5)-1)),IF(RIGHT(B5,1)="M",EDATE($B$3,VALUE(LEFT(B5,LEN(B5)-1))),EDATE($B$3,12*VALUE(LEFT(B5,LEN(B5)-1)))))),(IF(RIGHT(B5,1)="W",$B$3+7*VALUE(LEFT(B5,LEN(B5)-1)),IF(RIGHT(B5,1)="M",EDATE($B$3,VALUE(LEFT(B5,LEN(B5)-1))),EDATE($B$3,12*VALUE(LEFT(B5,LEN(B5)-1)))))-IF(WEEKDAY(IF(RIGHT(B5,1)="W",$B$3+7*VALUE(LEFT(B5,LEN(B5)-1)),IF(RIGHT(B5,1)="M",EDATE($B$3,VALUE(LEFT(B5,LEN(B5)-1))),EDATE($B$3,12*VALUE(LEFT(B5,LEN(B5)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B5,1)="W",$B$3+7*VALUE(LEFT(B5,LEN(B5)-1)),IF(RIGHT(B5,1)="M",EDATE($B$3,VALUE(LEFT(B5,LEN(B5)-1))),EDATE($B$3,12*VALUE(LEFT(B5,LEN(B5)-1))))),2)=7,2,0))),(IF(RIGHT(B5,1)="W",$B$3+7*VALUE(LEFT(B5,LEN(B5)-1)),IF(RIGHT(B5,1)="M",EDATE($B$3,VALUE(LEFT(B5,LEN(B5)-1))),EDATE($B$3,12*VALUE(LEFT(B5,LEN(B5)-1)))))+IF(WEEKDAY(IF(RIGHT(B5,1)="W",$B$3+7*VALUE(LEFT(B5,LEN(B5)-1)),IF(RIGHT(B5,1)="M",EDATE($B$3,VALUE(LEFT(B5,LEN(B5)-1))),EDATE($B$3,12*VALUE(LEFT(B5,LEN(B5)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B5,1)="W",$B$3+7*VALUE(LEFT(B5,LEN(B5)-1)),IF(RIGHT(B5,1)="M",EDATE($B$3,VALUE(LEFT(B5,LEN(B5)-1))),EDATE($B$3,12*VALUE(LEFT(B5,LEN(B5)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D5" s="24">
@@ -30217,7 +30222,7 @@
         </is>
       </c>
       <c r="C6" s="23">
-        <f>IF(RIGHT(B6,1)="W",$B$3+7*VALUE(LEFT(B6,LEN(B6)-1)),IF(RIGHT(B6,1)="M",EDATE($B$3,VALUE(LEFT(B6,LEN(B6)-1))),EDATE($B$3,12*VALUE(LEFT(B6,LEN(B6)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B6,1)="W",$B$3+7*VALUE(LEFT(B6,LEN(B6)-1)),IF(RIGHT(B6,1)="M",EDATE($B$3,VALUE(LEFT(B6,LEN(B6)-1))),EDATE($B$3,12*VALUE(LEFT(B6,LEN(B6)-1)))))+IF(WEEKDAY(IF(RIGHT(B6,1)="W",$B$3+7*VALUE(LEFT(B6,LEN(B6)-1)),IF(RIGHT(B6,1)="M",EDATE($B$3,VALUE(LEFT(B6,LEN(B6)-1))),EDATE($B$3,12*VALUE(LEFT(B6,LEN(B6)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B6,1)="W",$B$3+7*VALUE(LEFT(B6,LEN(B6)-1)),IF(RIGHT(B6,1)="M",EDATE($B$3,VALUE(LEFT(B6,LEN(B6)-1))),EDATE($B$3,12*VALUE(LEFT(B6,LEN(B6)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B6,1)="W",$B$3+7*VALUE(LEFT(B6,LEN(B6)-1)),IF(RIGHT(B6,1)="M",EDATE($B$3,VALUE(LEFT(B6,LEN(B6)-1))),EDATE($B$3,12*VALUE(LEFT(B6,LEN(B6)-1)))))),(IF(RIGHT(B6,1)="W",$B$3+7*VALUE(LEFT(B6,LEN(B6)-1)),IF(RIGHT(B6,1)="M",EDATE($B$3,VALUE(LEFT(B6,LEN(B6)-1))),EDATE($B$3,12*VALUE(LEFT(B6,LEN(B6)-1)))))-IF(WEEKDAY(IF(RIGHT(B6,1)="W",$B$3+7*VALUE(LEFT(B6,LEN(B6)-1)),IF(RIGHT(B6,1)="M",EDATE($B$3,VALUE(LEFT(B6,LEN(B6)-1))),EDATE($B$3,12*VALUE(LEFT(B6,LEN(B6)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B6,1)="W",$B$3+7*VALUE(LEFT(B6,LEN(B6)-1)),IF(RIGHT(B6,1)="M",EDATE($B$3,VALUE(LEFT(B6,LEN(B6)-1))),EDATE($B$3,12*VALUE(LEFT(B6,LEN(B6)-1))))),2)=7,2,0))),(IF(RIGHT(B6,1)="W",$B$3+7*VALUE(LEFT(B6,LEN(B6)-1)),IF(RIGHT(B6,1)="M",EDATE($B$3,VALUE(LEFT(B6,LEN(B6)-1))),EDATE($B$3,12*VALUE(LEFT(B6,LEN(B6)-1)))))+IF(WEEKDAY(IF(RIGHT(B6,1)="W",$B$3+7*VALUE(LEFT(B6,LEN(B6)-1)),IF(RIGHT(B6,1)="M",EDATE($B$3,VALUE(LEFT(B6,LEN(B6)-1))),EDATE($B$3,12*VALUE(LEFT(B6,LEN(B6)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B6,1)="W",$B$3+7*VALUE(LEFT(B6,LEN(B6)-1)),IF(RIGHT(B6,1)="M",EDATE($B$3,VALUE(LEFT(B6,LEN(B6)-1))),EDATE($B$3,12*VALUE(LEFT(B6,LEN(B6)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D6" s="24">
@@ -30263,7 +30268,7 @@
         </is>
       </c>
       <c r="C7" s="23">
-        <f>IF(RIGHT(B7,1)="W",$B$3+7*VALUE(LEFT(B7,LEN(B7)-1)),IF(RIGHT(B7,1)="M",EDATE($B$3,VALUE(LEFT(B7,LEN(B7)-1))),EDATE($B$3,12*VALUE(LEFT(B7,LEN(B7)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B7,1)="W",$B$3+7*VALUE(LEFT(B7,LEN(B7)-1)),IF(RIGHT(B7,1)="M",EDATE($B$3,VALUE(LEFT(B7,LEN(B7)-1))),EDATE($B$3,12*VALUE(LEFT(B7,LEN(B7)-1)))))+IF(WEEKDAY(IF(RIGHT(B7,1)="W",$B$3+7*VALUE(LEFT(B7,LEN(B7)-1)),IF(RIGHT(B7,1)="M",EDATE($B$3,VALUE(LEFT(B7,LEN(B7)-1))),EDATE($B$3,12*VALUE(LEFT(B7,LEN(B7)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B7,1)="W",$B$3+7*VALUE(LEFT(B7,LEN(B7)-1)),IF(RIGHT(B7,1)="M",EDATE($B$3,VALUE(LEFT(B7,LEN(B7)-1))),EDATE($B$3,12*VALUE(LEFT(B7,LEN(B7)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B7,1)="W",$B$3+7*VALUE(LEFT(B7,LEN(B7)-1)),IF(RIGHT(B7,1)="M",EDATE($B$3,VALUE(LEFT(B7,LEN(B7)-1))),EDATE($B$3,12*VALUE(LEFT(B7,LEN(B7)-1)))))),(IF(RIGHT(B7,1)="W",$B$3+7*VALUE(LEFT(B7,LEN(B7)-1)),IF(RIGHT(B7,1)="M",EDATE($B$3,VALUE(LEFT(B7,LEN(B7)-1))),EDATE($B$3,12*VALUE(LEFT(B7,LEN(B7)-1)))))-IF(WEEKDAY(IF(RIGHT(B7,1)="W",$B$3+7*VALUE(LEFT(B7,LEN(B7)-1)),IF(RIGHT(B7,1)="M",EDATE($B$3,VALUE(LEFT(B7,LEN(B7)-1))),EDATE($B$3,12*VALUE(LEFT(B7,LEN(B7)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B7,1)="W",$B$3+7*VALUE(LEFT(B7,LEN(B7)-1)),IF(RIGHT(B7,1)="M",EDATE($B$3,VALUE(LEFT(B7,LEN(B7)-1))),EDATE($B$3,12*VALUE(LEFT(B7,LEN(B7)-1))))),2)=7,2,0))),(IF(RIGHT(B7,1)="W",$B$3+7*VALUE(LEFT(B7,LEN(B7)-1)),IF(RIGHT(B7,1)="M",EDATE($B$3,VALUE(LEFT(B7,LEN(B7)-1))),EDATE($B$3,12*VALUE(LEFT(B7,LEN(B7)-1)))))+IF(WEEKDAY(IF(RIGHT(B7,1)="W",$B$3+7*VALUE(LEFT(B7,LEN(B7)-1)),IF(RIGHT(B7,1)="M",EDATE($B$3,VALUE(LEFT(B7,LEN(B7)-1))),EDATE($B$3,12*VALUE(LEFT(B7,LEN(B7)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B7,1)="W",$B$3+7*VALUE(LEFT(B7,LEN(B7)-1)),IF(RIGHT(B7,1)="M",EDATE($B$3,VALUE(LEFT(B7,LEN(B7)-1))),EDATE($B$3,12*VALUE(LEFT(B7,LEN(B7)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D7" s="24">
@@ -30309,7 +30314,7 @@
         </is>
       </c>
       <c r="C8" s="23">
-        <f>IF(RIGHT(B8,1)="W",$B$3+7*VALUE(LEFT(B8,LEN(B8)-1)),IF(RIGHT(B8,1)="M",EDATE($B$3,VALUE(LEFT(B8,LEN(B8)-1))),EDATE($B$3,12*VALUE(LEFT(B8,LEN(B8)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B8,1)="W",$B$3+7*VALUE(LEFT(B8,LEN(B8)-1)),IF(RIGHT(B8,1)="M",EDATE($B$3,VALUE(LEFT(B8,LEN(B8)-1))),EDATE($B$3,12*VALUE(LEFT(B8,LEN(B8)-1)))))+IF(WEEKDAY(IF(RIGHT(B8,1)="W",$B$3+7*VALUE(LEFT(B8,LEN(B8)-1)),IF(RIGHT(B8,1)="M",EDATE($B$3,VALUE(LEFT(B8,LEN(B8)-1))),EDATE($B$3,12*VALUE(LEFT(B8,LEN(B8)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B8,1)="W",$B$3+7*VALUE(LEFT(B8,LEN(B8)-1)),IF(RIGHT(B8,1)="M",EDATE($B$3,VALUE(LEFT(B8,LEN(B8)-1))),EDATE($B$3,12*VALUE(LEFT(B8,LEN(B8)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B8,1)="W",$B$3+7*VALUE(LEFT(B8,LEN(B8)-1)),IF(RIGHT(B8,1)="M",EDATE($B$3,VALUE(LEFT(B8,LEN(B8)-1))),EDATE($B$3,12*VALUE(LEFT(B8,LEN(B8)-1)))))),(IF(RIGHT(B8,1)="W",$B$3+7*VALUE(LEFT(B8,LEN(B8)-1)),IF(RIGHT(B8,1)="M",EDATE($B$3,VALUE(LEFT(B8,LEN(B8)-1))),EDATE($B$3,12*VALUE(LEFT(B8,LEN(B8)-1)))))-IF(WEEKDAY(IF(RIGHT(B8,1)="W",$B$3+7*VALUE(LEFT(B8,LEN(B8)-1)),IF(RIGHT(B8,1)="M",EDATE($B$3,VALUE(LEFT(B8,LEN(B8)-1))),EDATE($B$3,12*VALUE(LEFT(B8,LEN(B8)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B8,1)="W",$B$3+7*VALUE(LEFT(B8,LEN(B8)-1)),IF(RIGHT(B8,1)="M",EDATE($B$3,VALUE(LEFT(B8,LEN(B8)-1))),EDATE($B$3,12*VALUE(LEFT(B8,LEN(B8)-1))))),2)=7,2,0))),(IF(RIGHT(B8,1)="W",$B$3+7*VALUE(LEFT(B8,LEN(B8)-1)),IF(RIGHT(B8,1)="M",EDATE($B$3,VALUE(LEFT(B8,LEN(B8)-1))),EDATE($B$3,12*VALUE(LEFT(B8,LEN(B8)-1)))))+IF(WEEKDAY(IF(RIGHT(B8,1)="W",$B$3+7*VALUE(LEFT(B8,LEN(B8)-1)),IF(RIGHT(B8,1)="M",EDATE($B$3,VALUE(LEFT(B8,LEN(B8)-1))),EDATE($B$3,12*VALUE(LEFT(B8,LEN(B8)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B8,1)="W",$B$3+7*VALUE(LEFT(B8,LEN(B8)-1)),IF(RIGHT(B8,1)="M",EDATE($B$3,VALUE(LEFT(B8,LEN(B8)-1))),EDATE($B$3,12*VALUE(LEFT(B8,LEN(B8)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D8" s="24">
@@ -30359,7 +30364,7 @@
         </is>
       </c>
       <c r="C9" s="23">
-        <f>IF(RIGHT(B9,1)="W",$B$3+7*VALUE(LEFT(B9,LEN(B9)-1)),IF(RIGHT(B9,1)="M",EDATE($B$3,VALUE(LEFT(B9,LEN(B9)-1))),EDATE($B$3,12*VALUE(LEFT(B9,LEN(B9)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B9,1)="W",$B$3+7*VALUE(LEFT(B9,LEN(B9)-1)),IF(RIGHT(B9,1)="M",EDATE($B$3,VALUE(LEFT(B9,LEN(B9)-1))),EDATE($B$3,12*VALUE(LEFT(B9,LEN(B9)-1)))))+IF(WEEKDAY(IF(RIGHT(B9,1)="W",$B$3+7*VALUE(LEFT(B9,LEN(B9)-1)),IF(RIGHT(B9,1)="M",EDATE($B$3,VALUE(LEFT(B9,LEN(B9)-1))),EDATE($B$3,12*VALUE(LEFT(B9,LEN(B9)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B9,1)="W",$B$3+7*VALUE(LEFT(B9,LEN(B9)-1)),IF(RIGHT(B9,1)="M",EDATE($B$3,VALUE(LEFT(B9,LEN(B9)-1))),EDATE($B$3,12*VALUE(LEFT(B9,LEN(B9)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B9,1)="W",$B$3+7*VALUE(LEFT(B9,LEN(B9)-1)),IF(RIGHT(B9,1)="M",EDATE($B$3,VALUE(LEFT(B9,LEN(B9)-1))),EDATE($B$3,12*VALUE(LEFT(B9,LEN(B9)-1)))))),(IF(RIGHT(B9,1)="W",$B$3+7*VALUE(LEFT(B9,LEN(B9)-1)),IF(RIGHT(B9,1)="M",EDATE($B$3,VALUE(LEFT(B9,LEN(B9)-1))),EDATE($B$3,12*VALUE(LEFT(B9,LEN(B9)-1)))))-IF(WEEKDAY(IF(RIGHT(B9,1)="W",$B$3+7*VALUE(LEFT(B9,LEN(B9)-1)),IF(RIGHT(B9,1)="M",EDATE($B$3,VALUE(LEFT(B9,LEN(B9)-1))),EDATE($B$3,12*VALUE(LEFT(B9,LEN(B9)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B9,1)="W",$B$3+7*VALUE(LEFT(B9,LEN(B9)-1)),IF(RIGHT(B9,1)="M",EDATE($B$3,VALUE(LEFT(B9,LEN(B9)-1))),EDATE($B$3,12*VALUE(LEFT(B9,LEN(B9)-1))))),2)=7,2,0))),(IF(RIGHT(B9,1)="W",$B$3+7*VALUE(LEFT(B9,LEN(B9)-1)),IF(RIGHT(B9,1)="M",EDATE($B$3,VALUE(LEFT(B9,LEN(B9)-1))),EDATE($B$3,12*VALUE(LEFT(B9,LEN(B9)-1)))))+IF(WEEKDAY(IF(RIGHT(B9,1)="W",$B$3+7*VALUE(LEFT(B9,LEN(B9)-1)),IF(RIGHT(B9,1)="M",EDATE($B$3,VALUE(LEFT(B9,LEN(B9)-1))),EDATE($B$3,12*VALUE(LEFT(B9,LEN(B9)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B9,1)="W",$B$3+7*VALUE(LEFT(B9,LEN(B9)-1)),IF(RIGHT(B9,1)="M",EDATE($B$3,VALUE(LEFT(B9,LEN(B9)-1))),EDATE($B$3,12*VALUE(LEFT(B9,LEN(B9)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D9" s="24">
@@ -30405,7 +30410,7 @@
         </is>
       </c>
       <c r="C10" s="23">
-        <f>IF(RIGHT(B10,1)="W",$B$3+7*VALUE(LEFT(B10,LEN(B10)-1)),IF(RIGHT(B10,1)="M",EDATE($B$3,VALUE(LEFT(B10,LEN(B10)-1))),EDATE($B$3,12*VALUE(LEFT(B10,LEN(B10)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B10,1)="W",$B$3+7*VALUE(LEFT(B10,LEN(B10)-1)),IF(RIGHT(B10,1)="M",EDATE($B$3,VALUE(LEFT(B10,LEN(B10)-1))),EDATE($B$3,12*VALUE(LEFT(B10,LEN(B10)-1)))))+IF(WEEKDAY(IF(RIGHT(B10,1)="W",$B$3+7*VALUE(LEFT(B10,LEN(B10)-1)),IF(RIGHT(B10,1)="M",EDATE($B$3,VALUE(LEFT(B10,LEN(B10)-1))),EDATE($B$3,12*VALUE(LEFT(B10,LEN(B10)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B10,1)="W",$B$3+7*VALUE(LEFT(B10,LEN(B10)-1)),IF(RIGHT(B10,1)="M",EDATE($B$3,VALUE(LEFT(B10,LEN(B10)-1))),EDATE($B$3,12*VALUE(LEFT(B10,LEN(B10)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B10,1)="W",$B$3+7*VALUE(LEFT(B10,LEN(B10)-1)),IF(RIGHT(B10,1)="M",EDATE($B$3,VALUE(LEFT(B10,LEN(B10)-1))),EDATE($B$3,12*VALUE(LEFT(B10,LEN(B10)-1)))))),(IF(RIGHT(B10,1)="W",$B$3+7*VALUE(LEFT(B10,LEN(B10)-1)),IF(RIGHT(B10,1)="M",EDATE($B$3,VALUE(LEFT(B10,LEN(B10)-1))),EDATE($B$3,12*VALUE(LEFT(B10,LEN(B10)-1)))))-IF(WEEKDAY(IF(RIGHT(B10,1)="W",$B$3+7*VALUE(LEFT(B10,LEN(B10)-1)),IF(RIGHT(B10,1)="M",EDATE($B$3,VALUE(LEFT(B10,LEN(B10)-1))),EDATE($B$3,12*VALUE(LEFT(B10,LEN(B10)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B10,1)="W",$B$3+7*VALUE(LEFT(B10,LEN(B10)-1)),IF(RIGHT(B10,1)="M",EDATE($B$3,VALUE(LEFT(B10,LEN(B10)-1))),EDATE($B$3,12*VALUE(LEFT(B10,LEN(B10)-1))))),2)=7,2,0))),(IF(RIGHT(B10,1)="W",$B$3+7*VALUE(LEFT(B10,LEN(B10)-1)),IF(RIGHT(B10,1)="M",EDATE($B$3,VALUE(LEFT(B10,LEN(B10)-1))),EDATE($B$3,12*VALUE(LEFT(B10,LEN(B10)-1)))))+IF(WEEKDAY(IF(RIGHT(B10,1)="W",$B$3+7*VALUE(LEFT(B10,LEN(B10)-1)),IF(RIGHT(B10,1)="M",EDATE($B$3,VALUE(LEFT(B10,LEN(B10)-1))),EDATE($B$3,12*VALUE(LEFT(B10,LEN(B10)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B10,1)="W",$B$3+7*VALUE(LEFT(B10,LEN(B10)-1)),IF(RIGHT(B10,1)="M",EDATE($B$3,VALUE(LEFT(B10,LEN(B10)-1))),EDATE($B$3,12*VALUE(LEFT(B10,LEN(B10)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D10" s="24">
@@ -30455,7 +30460,7 @@
         </is>
       </c>
       <c r="C11" s="23">
-        <f>IF(RIGHT(B11,1)="W",$B$3+7*VALUE(LEFT(B11,LEN(B11)-1)),IF(RIGHT(B11,1)="M",EDATE($B$3,VALUE(LEFT(B11,LEN(B11)-1))),EDATE($B$3,12*VALUE(LEFT(B11,LEN(B11)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B11,1)="W",$B$3+7*VALUE(LEFT(B11,LEN(B11)-1)),IF(RIGHT(B11,1)="M",EDATE($B$3,VALUE(LEFT(B11,LEN(B11)-1))),EDATE($B$3,12*VALUE(LEFT(B11,LEN(B11)-1)))))+IF(WEEKDAY(IF(RIGHT(B11,1)="W",$B$3+7*VALUE(LEFT(B11,LEN(B11)-1)),IF(RIGHT(B11,1)="M",EDATE($B$3,VALUE(LEFT(B11,LEN(B11)-1))),EDATE($B$3,12*VALUE(LEFT(B11,LEN(B11)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B11,1)="W",$B$3+7*VALUE(LEFT(B11,LEN(B11)-1)),IF(RIGHT(B11,1)="M",EDATE($B$3,VALUE(LEFT(B11,LEN(B11)-1))),EDATE($B$3,12*VALUE(LEFT(B11,LEN(B11)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B11,1)="W",$B$3+7*VALUE(LEFT(B11,LEN(B11)-1)),IF(RIGHT(B11,1)="M",EDATE($B$3,VALUE(LEFT(B11,LEN(B11)-1))),EDATE($B$3,12*VALUE(LEFT(B11,LEN(B11)-1)))))),(IF(RIGHT(B11,1)="W",$B$3+7*VALUE(LEFT(B11,LEN(B11)-1)),IF(RIGHT(B11,1)="M",EDATE($B$3,VALUE(LEFT(B11,LEN(B11)-1))),EDATE($B$3,12*VALUE(LEFT(B11,LEN(B11)-1)))))-IF(WEEKDAY(IF(RIGHT(B11,1)="W",$B$3+7*VALUE(LEFT(B11,LEN(B11)-1)),IF(RIGHT(B11,1)="M",EDATE($B$3,VALUE(LEFT(B11,LEN(B11)-1))),EDATE($B$3,12*VALUE(LEFT(B11,LEN(B11)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B11,1)="W",$B$3+7*VALUE(LEFT(B11,LEN(B11)-1)),IF(RIGHT(B11,1)="M",EDATE($B$3,VALUE(LEFT(B11,LEN(B11)-1))),EDATE($B$3,12*VALUE(LEFT(B11,LEN(B11)-1))))),2)=7,2,0))),(IF(RIGHT(B11,1)="W",$B$3+7*VALUE(LEFT(B11,LEN(B11)-1)),IF(RIGHT(B11,1)="M",EDATE($B$3,VALUE(LEFT(B11,LEN(B11)-1))),EDATE($B$3,12*VALUE(LEFT(B11,LEN(B11)-1)))))+IF(WEEKDAY(IF(RIGHT(B11,1)="W",$B$3+7*VALUE(LEFT(B11,LEN(B11)-1)),IF(RIGHT(B11,1)="M",EDATE($B$3,VALUE(LEFT(B11,LEN(B11)-1))),EDATE($B$3,12*VALUE(LEFT(B11,LEN(B11)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B11,1)="W",$B$3+7*VALUE(LEFT(B11,LEN(B11)-1)),IF(RIGHT(B11,1)="M",EDATE($B$3,VALUE(LEFT(B11,LEN(B11)-1))),EDATE($B$3,12*VALUE(LEFT(B11,LEN(B11)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D11" s="24">
@@ -30501,7 +30506,7 @@
         </is>
       </c>
       <c r="C12" s="23">
-        <f>IF(RIGHT(B12,1)="W",$B$3+7*VALUE(LEFT(B12,LEN(B12)-1)),IF(RIGHT(B12,1)="M",EDATE($B$3,VALUE(LEFT(B12,LEN(B12)-1))),EDATE($B$3,12*VALUE(LEFT(B12,LEN(B12)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B12,1)="W",$B$3+7*VALUE(LEFT(B12,LEN(B12)-1)),IF(RIGHT(B12,1)="M",EDATE($B$3,VALUE(LEFT(B12,LEN(B12)-1))),EDATE($B$3,12*VALUE(LEFT(B12,LEN(B12)-1)))))+IF(WEEKDAY(IF(RIGHT(B12,1)="W",$B$3+7*VALUE(LEFT(B12,LEN(B12)-1)),IF(RIGHT(B12,1)="M",EDATE($B$3,VALUE(LEFT(B12,LEN(B12)-1))),EDATE($B$3,12*VALUE(LEFT(B12,LEN(B12)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B12,1)="W",$B$3+7*VALUE(LEFT(B12,LEN(B12)-1)),IF(RIGHT(B12,1)="M",EDATE($B$3,VALUE(LEFT(B12,LEN(B12)-1))),EDATE($B$3,12*VALUE(LEFT(B12,LEN(B12)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B12,1)="W",$B$3+7*VALUE(LEFT(B12,LEN(B12)-1)),IF(RIGHT(B12,1)="M",EDATE($B$3,VALUE(LEFT(B12,LEN(B12)-1))),EDATE($B$3,12*VALUE(LEFT(B12,LEN(B12)-1)))))),(IF(RIGHT(B12,1)="W",$B$3+7*VALUE(LEFT(B12,LEN(B12)-1)),IF(RIGHT(B12,1)="M",EDATE($B$3,VALUE(LEFT(B12,LEN(B12)-1))),EDATE($B$3,12*VALUE(LEFT(B12,LEN(B12)-1)))))-IF(WEEKDAY(IF(RIGHT(B12,1)="W",$B$3+7*VALUE(LEFT(B12,LEN(B12)-1)),IF(RIGHT(B12,1)="M",EDATE($B$3,VALUE(LEFT(B12,LEN(B12)-1))),EDATE($B$3,12*VALUE(LEFT(B12,LEN(B12)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B12,1)="W",$B$3+7*VALUE(LEFT(B12,LEN(B12)-1)),IF(RIGHT(B12,1)="M",EDATE($B$3,VALUE(LEFT(B12,LEN(B12)-1))),EDATE($B$3,12*VALUE(LEFT(B12,LEN(B12)-1))))),2)=7,2,0))),(IF(RIGHT(B12,1)="W",$B$3+7*VALUE(LEFT(B12,LEN(B12)-1)),IF(RIGHT(B12,1)="M",EDATE($B$3,VALUE(LEFT(B12,LEN(B12)-1))),EDATE($B$3,12*VALUE(LEFT(B12,LEN(B12)-1)))))+IF(WEEKDAY(IF(RIGHT(B12,1)="W",$B$3+7*VALUE(LEFT(B12,LEN(B12)-1)),IF(RIGHT(B12,1)="M",EDATE($B$3,VALUE(LEFT(B12,LEN(B12)-1))),EDATE($B$3,12*VALUE(LEFT(B12,LEN(B12)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B12,1)="W",$B$3+7*VALUE(LEFT(B12,LEN(B12)-1)),IF(RIGHT(B12,1)="M",EDATE($B$3,VALUE(LEFT(B12,LEN(B12)-1))),EDATE($B$3,12*VALUE(LEFT(B12,LEN(B12)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D12" s="24">
@@ -30547,7 +30552,7 @@
         </is>
       </c>
       <c r="C13" s="23">
-        <f>IF(RIGHT(B13,1)="W",$B$3+7*VALUE(LEFT(B13,LEN(B13)-1)),IF(RIGHT(B13,1)="M",EDATE($B$3,VALUE(LEFT(B13,LEN(B13)-1))),EDATE($B$3,12*VALUE(LEFT(B13,LEN(B13)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B13,1)="W",$B$3+7*VALUE(LEFT(B13,LEN(B13)-1)),IF(RIGHT(B13,1)="M",EDATE($B$3,VALUE(LEFT(B13,LEN(B13)-1))),EDATE($B$3,12*VALUE(LEFT(B13,LEN(B13)-1)))))+IF(WEEKDAY(IF(RIGHT(B13,1)="W",$B$3+7*VALUE(LEFT(B13,LEN(B13)-1)),IF(RIGHT(B13,1)="M",EDATE($B$3,VALUE(LEFT(B13,LEN(B13)-1))),EDATE($B$3,12*VALUE(LEFT(B13,LEN(B13)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B13,1)="W",$B$3+7*VALUE(LEFT(B13,LEN(B13)-1)),IF(RIGHT(B13,1)="M",EDATE($B$3,VALUE(LEFT(B13,LEN(B13)-1))),EDATE($B$3,12*VALUE(LEFT(B13,LEN(B13)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B13,1)="W",$B$3+7*VALUE(LEFT(B13,LEN(B13)-1)),IF(RIGHT(B13,1)="M",EDATE($B$3,VALUE(LEFT(B13,LEN(B13)-1))),EDATE($B$3,12*VALUE(LEFT(B13,LEN(B13)-1)))))),(IF(RIGHT(B13,1)="W",$B$3+7*VALUE(LEFT(B13,LEN(B13)-1)),IF(RIGHT(B13,1)="M",EDATE($B$3,VALUE(LEFT(B13,LEN(B13)-1))),EDATE($B$3,12*VALUE(LEFT(B13,LEN(B13)-1)))))-IF(WEEKDAY(IF(RIGHT(B13,1)="W",$B$3+7*VALUE(LEFT(B13,LEN(B13)-1)),IF(RIGHT(B13,1)="M",EDATE($B$3,VALUE(LEFT(B13,LEN(B13)-1))),EDATE($B$3,12*VALUE(LEFT(B13,LEN(B13)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B13,1)="W",$B$3+7*VALUE(LEFT(B13,LEN(B13)-1)),IF(RIGHT(B13,1)="M",EDATE($B$3,VALUE(LEFT(B13,LEN(B13)-1))),EDATE($B$3,12*VALUE(LEFT(B13,LEN(B13)-1))))),2)=7,2,0))),(IF(RIGHT(B13,1)="W",$B$3+7*VALUE(LEFT(B13,LEN(B13)-1)),IF(RIGHT(B13,1)="M",EDATE($B$3,VALUE(LEFT(B13,LEN(B13)-1))),EDATE($B$3,12*VALUE(LEFT(B13,LEN(B13)-1)))))+IF(WEEKDAY(IF(RIGHT(B13,1)="W",$B$3+7*VALUE(LEFT(B13,LEN(B13)-1)),IF(RIGHT(B13,1)="M",EDATE($B$3,VALUE(LEFT(B13,LEN(B13)-1))),EDATE($B$3,12*VALUE(LEFT(B13,LEN(B13)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B13,1)="W",$B$3+7*VALUE(LEFT(B13,LEN(B13)-1)),IF(RIGHT(B13,1)="M",EDATE($B$3,VALUE(LEFT(B13,LEN(B13)-1))),EDATE($B$3,12*VALUE(LEFT(B13,LEN(B13)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D13" s="24">
@@ -30597,7 +30602,7 @@
         </is>
       </c>
       <c r="C14" s="23">
-        <f>IF(RIGHT(B14,1)="W",$B$3+7*VALUE(LEFT(B14,LEN(B14)-1)),IF(RIGHT(B14,1)="M",EDATE($B$3,VALUE(LEFT(B14,LEN(B14)-1))),EDATE($B$3,12*VALUE(LEFT(B14,LEN(B14)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B14,1)="W",$B$3+7*VALUE(LEFT(B14,LEN(B14)-1)),IF(RIGHT(B14,1)="M",EDATE($B$3,VALUE(LEFT(B14,LEN(B14)-1))),EDATE($B$3,12*VALUE(LEFT(B14,LEN(B14)-1)))))+IF(WEEKDAY(IF(RIGHT(B14,1)="W",$B$3+7*VALUE(LEFT(B14,LEN(B14)-1)),IF(RIGHT(B14,1)="M",EDATE($B$3,VALUE(LEFT(B14,LEN(B14)-1))),EDATE($B$3,12*VALUE(LEFT(B14,LEN(B14)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B14,1)="W",$B$3+7*VALUE(LEFT(B14,LEN(B14)-1)),IF(RIGHT(B14,1)="M",EDATE($B$3,VALUE(LEFT(B14,LEN(B14)-1))),EDATE($B$3,12*VALUE(LEFT(B14,LEN(B14)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B14,1)="W",$B$3+7*VALUE(LEFT(B14,LEN(B14)-1)),IF(RIGHT(B14,1)="M",EDATE($B$3,VALUE(LEFT(B14,LEN(B14)-1))),EDATE($B$3,12*VALUE(LEFT(B14,LEN(B14)-1)))))),(IF(RIGHT(B14,1)="W",$B$3+7*VALUE(LEFT(B14,LEN(B14)-1)),IF(RIGHT(B14,1)="M",EDATE($B$3,VALUE(LEFT(B14,LEN(B14)-1))),EDATE($B$3,12*VALUE(LEFT(B14,LEN(B14)-1)))))-IF(WEEKDAY(IF(RIGHT(B14,1)="W",$B$3+7*VALUE(LEFT(B14,LEN(B14)-1)),IF(RIGHT(B14,1)="M",EDATE($B$3,VALUE(LEFT(B14,LEN(B14)-1))),EDATE($B$3,12*VALUE(LEFT(B14,LEN(B14)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B14,1)="W",$B$3+7*VALUE(LEFT(B14,LEN(B14)-1)),IF(RIGHT(B14,1)="M",EDATE($B$3,VALUE(LEFT(B14,LEN(B14)-1))),EDATE($B$3,12*VALUE(LEFT(B14,LEN(B14)-1))))),2)=7,2,0))),(IF(RIGHT(B14,1)="W",$B$3+7*VALUE(LEFT(B14,LEN(B14)-1)),IF(RIGHT(B14,1)="M",EDATE($B$3,VALUE(LEFT(B14,LEN(B14)-1))),EDATE($B$3,12*VALUE(LEFT(B14,LEN(B14)-1)))))+IF(WEEKDAY(IF(RIGHT(B14,1)="W",$B$3+7*VALUE(LEFT(B14,LEN(B14)-1)),IF(RIGHT(B14,1)="M",EDATE($B$3,VALUE(LEFT(B14,LEN(B14)-1))),EDATE($B$3,12*VALUE(LEFT(B14,LEN(B14)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B14,1)="W",$B$3+7*VALUE(LEFT(B14,LEN(B14)-1)),IF(RIGHT(B14,1)="M",EDATE($B$3,VALUE(LEFT(B14,LEN(B14)-1))),EDATE($B$3,12*VALUE(LEFT(B14,LEN(B14)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D14" s="24">
@@ -30643,7 +30648,7 @@
         </is>
       </c>
       <c r="C15" s="23">
-        <f>IF(RIGHT(B15,1)="W",$B$3+7*VALUE(LEFT(B15,LEN(B15)-1)),IF(RIGHT(B15,1)="M",EDATE($B$3,VALUE(LEFT(B15,LEN(B15)-1))),EDATE($B$3,12*VALUE(LEFT(B15,LEN(B15)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B15,1)="W",$B$3+7*VALUE(LEFT(B15,LEN(B15)-1)),IF(RIGHT(B15,1)="M",EDATE($B$3,VALUE(LEFT(B15,LEN(B15)-1))),EDATE($B$3,12*VALUE(LEFT(B15,LEN(B15)-1)))))+IF(WEEKDAY(IF(RIGHT(B15,1)="W",$B$3+7*VALUE(LEFT(B15,LEN(B15)-1)),IF(RIGHT(B15,1)="M",EDATE($B$3,VALUE(LEFT(B15,LEN(B15)-1))),EDATE($B$3,12*VALUE(LEFT(B15,LEN(B15)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B15,1)="W",$B$3+7*VALUE(LEFT(B15,LEN(B15)-1)),IF(RIGHT(B15,1)="M",EDATE($B$3,VALUE(LEFT(B15,LEN(B15)-1))),EDATE($B$3,12*VALUE(LEFT(B15,LEN(B15)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B15,1)="W",$B$3+7*VALUE(LEFT(B15,LEN(B15)-1)),IF(RIGHT(B15,1)="M",EDATE($B$3,VALUE(LEFT(B15,LEN(B15)-1))),EDATE($B$3,12*VALUE(LEFT(B15,LEN(B15)-1)))))),(IF(RIGHT(B15,1)="W",$B$3+7*VALUE(LEFT(B15,LEN(B15)-1)),IF(RIGHT(B15,1)="M",EDATE($B$3,VALUE(LEFT(B15,LEN(B15)-1))),EDATE($B$3,12*VALUE(LEFT(B15,LEN(B15)-1)))))-IF(WEEKDAY(IF(RIGHT(B15,1)="W",$B$3+7*VALUE(LEFT(B15,LEN(B15)-1)),IF(RIGHT(B15,1)="M",EDATE($B$3,VALUE(LEFT(B15,LEN(B15)-1))),EDATE($B$3,12*VALUE(LEFT(B15,LEN(B15)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B15,1)="W",$B$3+7*VALUE(LEFT(B15,LEN(B15)-1)),IF(RIGHT(B15,1)="M",EDATE($B$3,VALUE(LEFT(B15,LEN(B15)-1))),EDATE($B$3,12*VALUE(LEFT(B15,LEN(B15)-1))))),2)=7,2,0))),(IF(RIGHT(B15,1)="W",$B$3+7*VALUE(LEFT(B15,LEN(B15)-1)),IF(RIGHT(B15,1)="M",EDATE($B$3,VALUE(LEFT(B15,LEN(B15)-1))),EDATE($B$3,12*VALUE(LEFT(B15,LEN(B15)-1)))))+IF(WEEKDAY(IF(RIGHT(B15,1)="W",$B$3+7*VALUE(LEFT(B15,LEN(B15)-1)),IF(RIGHT(B15,1)="M",EDATE($B$3,VALUE(LEFT(B15,LEN(B15)-1))),EDATE($B$3,12*VALUE(LEFT(B15,LEN(B15)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B15,1)="W",$B$3+7*VALUE(LEFT(B15,LEN(B15)-1)),IF(RIGHT(B15,1)="M",EDATE($B$3,VALUE(LEFT(B15,LEN(B15)-1))),EDATE($B$3,12*VALUE(LEFT(B15,LEN(B15)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D15" s="24">
@@ -30689,7 +30694,7 @@
         </is>
       </c>
       <c r="C16" s="23">
-        <f>IF(RIGHT(B16,1)="W",$B$3+7*VALUE(LEFT(B16,LEN(B16)-1)),IF(RIGHT(B16,1)="M",EDATE($B$3,VALUE(LEFT(B16,LEN(B16)-1))),EDATE($B$3,12*VALUE(LEFT(B16,LEN(B16)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B16,1)="W",$B$3+7*VALUE(LEFT(B16,LEN(B16)-1)),IF(RIGHT(B16,1)="M",EDATE($B$3,VALUE(LEFT(B16,LEN(B16)-1))),EDATE($B$3,12*VALUE(LEFT(B16,LEN(B16)-1)))))+IF(WEEKDAY(IF(RIGHT(B16,1)="W",$B$3+7*VALUE(LEFT(B16,LEN(B16)-1)),IF(RIGHT(B16,1)="M",EDATE($B$3,VALUE(LEFT(B16,LEN(B16)-1))),EDATE($B$3,12*VALUE(LEFT(B16,LEN(B16)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B16,1)="W",$B$3+7*VALUE(LEFT(B16,LEN(B16)-1)),IF(RIGHT(B16,1)="M",EDATE($B$3,VALUE(LEFT(B16,LEN(B16)-1))),EDATE($B$3,12*VALUE(LEFT(B16,LEN(B16)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B16,1)="W",$B$3+7*VALUE(LEFT(B16,LEN(B16)-1)),IF(RIGHT(B16,1)="M",EDATE($B$3,VALUE(LEFT(B16,LEN(B16)-1))),EDATE($B$3,12*VALUE(LEFT(B16,LEN(B16)-1)))))),(IF(RIGHT(B16,1)="W",$B$3+7*VALUE(LEFT(B16,LEN(B16)-1)),IF(RIGHT(B16,1)="M",EDATE($B$3,VALUE(LEFT(B16,LEN(B16)-1))),EDATE($B$3,12*VALUE(LEFT(B16,LEN(B16)-1)))))-IF(WEEKDAY(IF(RIGHT(B16,1)="W",$B$3+7*VALUE(LEFT(B16,LEN(B16)-1)),IF(RIGHT(B16,1)="M",EDATE($B$3,VALUE(LEFT(B16,LEN(B16)-1))),EDATE($B$3,12*VALUE(LEFT(B16,LEN(B16)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B16,1)="W",$B$3+7*VALUE(LEFT(B16,LEN(B16)-1)),IF(RIGHT(B16,1)="M",EDATE($B$3,VALUE(LEFT(B16,LEN(B16)-1))),EDATE($B$3,12*VALUE(LEFT(B16,LEN(B16)-1))))),2)=7,2,0))),(IF(RIGHT(B16,1)="W",$B$3+7*VALUE(LEFT(B16,LEN(B16)-1)),IF(RIGHT(B16,1)="M",EDATE($B$3,VALUE(LEFT(B16,LEN(B16)-1))),EDATE($B$3,12*VALUE(LEFT(B16,LEN(B16)-1)))))+IF(WEEKDAY(IF(RIGHT(B16,1)="W",$B$3+7*VALUE(LEFT(B16,LEN(B16)-1)),IF(RIGHT(B16,1)="M",EDATE($B$3,VALUE(LEFT(B16,LEN(B16)-1))),EDATE($B$3,12*VALUE(LEFT(B16,LEN(B16)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B16,1)="W",$B$3+7*VALUE(LEFT(B16,LEN(B16)-1)),IF(RIGHT(B16,1)="M",EDATE($B$3,VALUE(LEFT(B16,LEN(B16)-1))),EDATE($B$3,12*VALUE(LEFT(B16,LEN(B16)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D16" s="24">
@@ -30735,7 +30740,7 @@
         </is>
       </c>
       <c r="C17" s="23">
-        <f>IF(RIGHT(B17,1)="W",$B$3+7*VALUE(LEFT(B17,LEN(B17)-1)),IF(RIGHT(B17,1)="M",EDATE($B$3,VALUE(LEFT(B17,LEN(B17)-1))),EDATE($B$3,12*VALUE(LEFT(B17,LEN(B17)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B17,1)="W",$B$3+7*VALUE(LEFT(B17,LEN(B17)-1)),IF(RIGHT(B17,1)="M",EDATE($B$3,VALUE(LEFT(B17,LEN(B17)-1))),EDATE($B$3,12*VALUE(LEFT(B17,LEN(B17)-1)))))+IF(WEEKDAY(IF(RIGHT(B17,1)="W",$B$3+7*VALUE(LEFT(B17,LEN(B17)-1)),IF(RIGHT(B17,1)="M",EDATE($B$3,VALUE(LEFT(B17,LEN(B17)-1))),EDATE($B$3,12*VALUE(LEFT(B17,LEN(B17)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B17,1)="W",$B$3+7*VALUE(LEFT(B17,LEN(B17)-1)),IF(RIGHT(B17,1)="M",EDATE($B$3,VALUE(LEFT(B17,LEN(B17)-1))),EDATE($B$3,12*VALUE(LEFT(B17,LEN(B17)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B17,1)="W",$B$3+7*VALUE(LEFT(B17,LEN(B17)-1)),IF(RIGHT(B17,1)="M",EDATE($B$3,VALUE(LEFT(B17,LEN(B17)-1))),EDATE($B$3,12*VALUE(LEFT(B17,LEN(B17)-1)))))),(IF(RIGHT(B17,1)="W",$B$3+7*VALUE(LEFT(B17,LEN(B17)-1)),IF(RIGHT(B17,1)="M",EDATE($B$3,VALUE(LEFT(B17,LEN(B17)-1))),EDATE($B$3,12*VALUE(LEFT(B17,LEN(B17)-1)))))-IF(WEEKDAY(IF(RIGHT(B17,1)="W",$B$3+7*VALUE(LEFT(B17,LEN(B17)-1)),IF(RIGHT(B17,1)="M",EDATE($B$3,VALUE(LEFT(B17,LEN(B17)-1))),EDATE($B$3,12*VALUE(LEFT(B17,LEN(B17)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B17,1)="W",$B$3+7*VALUE(LEFT(B17,LEN(B17)-1)),IF(RIGHT(B17,1)="M",EDATE($B$3,VALUE(LEFT(B17,LEN(B17)-1))),EDATE($B$3,12*VALUE(LEFT(B17,LEN(B17)-1))))),2)=7,2,0))),(IF(RIGHT(B17,1)="W",$B$3+7*VALUE(LEFT(B17,LEN(B17)-1)),IF(RIGHT(B17,1)="M",EDATE($B$3,VALUE(LEFT(B17,LEN(B17)-1))),EDATE($B$3,12*VALUE(LEFT(B17,LEN(B17)-1)))))+IF(WEEKDAY(IF(RIGHT(B17,1)="W",$B$3+7*VALUE(LEFT(B17,LEN(B17)-1)),IF(RIGHT(B17,1)="M",EDATE($B$3,VALUE(LEFT(B17,LEN(B17)-1))),EDATE($B$3,12*VALUE(LEFT(B17,LEN(B17)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B17,1)="W",$B$3+7*VALUE(LEFT(B17,LEN(B17)-1)),IF(RIGHT(B17,1)="M",EDATE($B$3,VALUE(LEFT(B17,LEN(B17)-1))),EDATE($B$3,12*VALUE(LEFT(B17,LEN(B17)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D17" s="24">
@@ -30781,7 +30786,7 @@
         </is>
       </c>
       <c r="C18" s="23">
-        <f>IF(RIGHT(B18,1)="W",$B$3+7*VALUE(LEFT(B18,LEN(B18)-1)),IF(RIGHT(B18,1)="M",EDATE($B$3,VALUE(LEFT(B18,LEN(B18)-1))),EDATE($B$3,12*VALUE(LEFT(B18,LEN(B18)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B18,1)="W",$B$3+7*VALUE(LEFT(B18,LEN(B18)-1)),IF(RIGHT(B18,1)="M",EDATE($B$3,VALUE(LEFT(B18,LEN(B18)-1))),EDATE($B$3,12*VALUE(LEFT(B18,LEN(B18)-1)))))+IF(WEEKDAY(IF(RIGHT(B18,1)="W",$B$3+7*VALUE(LEFT(B18,LEN(B18)-1)),IF(RIGHT(B18,1)="M",EDATE($B$3,VALUE(LEFT(B18,LEN(B18)-1))),EDATE($B$3,12*VALUE(LEFT(B18,LEN(B18)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B18,1)="W",$B$3+7*VALUE(LEFT(B18,LEN(B18)-1)),IF(RIGHT(B18,1)="M",EDATE($B$3,VALUE(LEFT(B18,LEN(B18)-1))),EDATE($B$3,12*VALUE(LEFT(B18,LEN(B18)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B18,1)="W",$B$3+7*VALUE(LEFT(B18,LEN(B18)-1)),IF(RIGHT(B18,1)="M",EDATE($B$3,VALUE(LEFT(B18,LEN(B18)-1))),EDATE($B$3,12*VALUE(LEFT(B18,LEN(B18)-1)))))),(IF(RIGHT(B18,1)="W",$B$3+7*VALUE(LEFT(B18,LEN(B18)-1)),IF(RIGHT(B18,1)="M",EDATE($B$3,VALUE(LEFT(B18,LEN(B18)-1))),EDATE($B$3,12*VALUE(LEFT(B18,LEN(B18)-1)))))-IF(WEEKDAY(IF(RIGHT(B18,1)="W",$B$3+7*VALUE(LEFT(B18,LEN(B18)-1)),IF(RIGHT(B18,1)="M",EDATE($B$3,VALUE(LEFT(B18,LEN(B18)-1))),EDATE($B$3,12*VALUE(LEFT(B18,LEN(B18)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B18,1)="W",$B$3+7*VALUE(LEFT(B18,LEN(B18)-1)),IF(RIGHT(B18,1)="M",EDATE($B$3,VALUE(LEFT(B18,LEN(B18)-1))),EDATE($B$3,12*VALUE(LEFT(B18,LEN(B18)-1))))),2)=7,2,0))),(IF(RIGHT(B18,1)="W",$B$3+7*VALUE(LEFT(B18,LEN(B18)-1)),IF(RIGHT(B18,1)="M",EDATE($B$3,VALUE(LEFT(B18,LEN(B18)-1))),EDATE($B$3,12*VALUE(LEFT(B18,LEN(B18)-1)))))+IF(WEEKDAY(IF(RIGHT(B18,1)="W",$B$3+7*VALUE(LEFT(B18,LEN(B18)-1)),IF(RIGHT(B18,1)="M",EDATE($B$3,VALUE(LEFT(B18,LEN(B18)-1))),EDATE($B$3,12*VALUE(LEFT(B18,LEN(B18)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B18,1)="W",$B$3+7*VALUE(LEFT(B18,LEN(B18)-1)),IF(RIGHT(B18,1)="M",EDATE($B$3,VALUE(LEFT(B18,LEN(B18)-1))),EDATE($B$3,12*VALUE(LEFT(B18,LEN(B18)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D18" s="24">
@@ -30827,7 +30832,7 @@
         </is>
       </c>
       <c r="C19" s="23">
-        <f>IF(RIGHT(B19,1)="W",$B$3+7*VALUE(LEFT(B19,LEN(B19)-1)),IF(RIGHT(B19,1)="M",EDATE($B$3,VALUE(LEFT(B19,LEN(B19)-1))),EDATE($B$3,12*VALUE(LEFT(B19,LEN(B19)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B19,1)="W",$B$3+7*VALUE(LEFT(B19,LEN(B19)-1)),IF(RIGHT(B19,1)="M",EDATE($B$3,VALUE(LEFT(B19,LEN(B19)-1))),EDATE($B$3,12*VALUE(LEFT(B19,LEN(B19)-1)))))+IF(WEEKDAY(IF(RIGHT(B19,1)="W",$B$3+7*VALUE(LEFT(B19,LEN(B19)-1)),IF(RIGHT(B19,1)="M",EDATE($B$3,VALUE(LEFT(B19,LEN(B19)-1))),EDATE($B$3,12*VALUE(LEFT(B19,LEN(B19)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B19,1)="W",$B$3+7*VALUE(LEFT(B19,LEN(B19)-1)),IF(RIGHT(B19,1)="M",EDATE($B$3,VALUE(LEFT(B19,LEN(B19)-1))),EDATE($B$3,12*VALUE(LEFT(B19,LEN(B19)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B19,1)="W",$B$3+7*VALUE(LEFT(B19,LEN(B19)-1)),IF(RIGHT(B19,1)="M",EDATE($B$3,VALUE(LEFT(B19,LEN(B19)-1))),EDATE($B$3,12*VALUE(LEFT(B19,LEN(B19)-1)))))),(IF(RIGHT(B19,1)="W",$B$3+7*VALUE(LEFT(B19,LEN(B19)-1)),IF(RIGHT(B19,1)="M",EDATE($B$3,VALUE(LEFT(B19,LEN(B19)-1))),EDATE($B$3,12*VALUE(LEFT(B19,LEN(B19)-1)))))-IF(WEEKDAY(IF(RIGHT(B19,1)="W",$B$3+7*VALUE(LEFT(B19,LEN(B19)-1)),IF(RIGHT(B19,1)="M",EDATE($B$3,VALUE(LEFT(B19,LEN(B19)-1))),EDATE($B$3,12*VALUE(LEFT(B19,LEN(B19)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B19,1)="W",$B$3+7*VALUE(LEFT(B19,LEN(B19)-1)),IF(RIGHT(B19,1)="M",EDATE($B$3,VALUE(LEFT(B19,LEN(B19)-1))),EDATE($B$3,12*VALUE(LEFT(B19,LEN(B19)-1))))),2)=7,2,0))),(IF(RIGHT(B19,1)="W",$B$3+7*VALUE(LEFT(B19,LEN(B19)-1)),IF(RIGHT(B19,1)="M",EDATE($B$3,VALUE(LEFT(B19,LEN(B19)-1))),EDATE($B$3,12*VALUE(LEFT(B19,LEN(B19)-1)))))+IF(WEEKDAY(IF(RIGHT(B19,1)="W",$B$3+7*VALUE(LEFT(B19,LEN(B19)-1)),IF(RIGHT(B19,1)="M",EDATE($B$3,VALUE(LEFT(B19,LEN(B19)-1))),EDATE($B$3,12*VALUE(LEFT(B19,LEN(B19)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B19,1)="W",$B$3+7*VALUE(LEFT(B19,LEN(B19)-1)),IF(RIGHT(B19,1)="M",EDATE($B$3,VALUE(LEFT(B19,LEN(B19)-1))),EDATE($B$3,12*VALUE(LEFT(B19,LEN(B19)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D19" s="24">
@@ -30873,7 +30878,7 @@
         </is>
       </c>
       <c r="C20" s="23">
-        <f>IF(RIGHT(B20,1)="W",$B$3+7*VALUE(LEFT(B20,LEN(B20)-1)),IF(RIGHT(B20,1)="M",EDATE($B$3,VALUE(LEFT(B20,LEN(B20)-1))),EDATE($B$3,12*VALUE(LEFT(B20,LEN(B20)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B20,1)="W",$B$3+7*VALUE(LEFT(B20,LEN(B20)-1)),IF(RIGHT(B20,1)="M",EDATE($B$3,VALUE(LEFT(B20,LEN(B20)-1))),EDATE($B$3,12*VALUE(LEFT(B20,LEN(B20)-1)))))+IF(WEEKDAY(IF(RIGHT(B20,1)="W",$B$3+7*VALUE(LEFT(B20,LEN(B20)-1)),IF(RIGHT(B20,1)="M",EDATE($B$3,VALUE(LEFT(B20,LEN(B20)-1))),EDATE($B$3,12*VALUE(LEFT(B20,LEN(B20)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B20,1)="W",$B$3+7*VALUE(LEFT(B20,LEN(B20)-1)),IF(RIGHT(B20,1)="M",EDATE($B$3,VALUE(LEFT(B20,LEN(B20)-1))),EDATE($B$3,12*VALUE(LEFT(B20,LEN(B20)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B20,1)="W",$B$3+7*VALUE(LEFT(B20,LEN(B20)-1)),IF(RIGHT(B20,1)="M",EDATE($B$3,VALUE(LEFT(B20,LEN(B20)-1))),EDATE($B$3,12*VALUE(LEFT(B20,LEN(B20)-1)))))),(IF(RIGHT(B20,1)="W",$B$3+7*VALUE(LEFT(B20,LEN(B20)-1)),IF(RIGHT(B20,1)="M",EDATE($B$3,VALUE(LEFT(B20,LEN(B20)-1))),EDATE($B$3,12*VALUE(LEFT(B20,LEN(B20)-1)))))-IF(WEEKDAY(IF(RIGHT(B20,1)="W",$B$3+7*VALUE(LEFT(B20,LEN(B20)-1)),IF(RIGHT(B20,1)="M",EDATE($B$3,VALUE(LEFT(B20,LEN(B20)-1))),EDATE($B$3,12*VALUE(LEFT(B20,LEN(B20)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B20,1)="W",$B$3+7*VALUE(LEFT(B20,LEN(B20)-1)),IF(RIGHT(B20,1)="M",EDATE($B$3,VALUE(LEFT(B20,LEN(B20)-1))),EDATE($B$3,12*VALUE(LEFT(B20,LEN(B20)-1))))),2)=7,2,0))),(IF(RIGHT(B20,1)="W",$B$3+7*VALUE(LEFT(B20,LEN(B20)-1)),IF(RIGHT(B20,1)="M",EDATE($B$3,VALUE(LEFT(B20,LEN(B20)-1))),EDATE($B$3,12*VALUE(LEFT(B20,LEN(B20)-1)))))+IF(WEEKDAY(IF(RIGHT(B20,1)="W",$B$3+7*VALUE(LEFT(B20,LEN(B20)-1)),IF(RIGHT(B20,1)="M",EDATE($B$3,VALUE(LEFT(B20,LEN(B20)-1))),EDATE($B$3,12*VALUE(LEFT(B20,LEN(B20)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B20,1)="W",$B$3+7*VALUE(LEFT(B20,LEN(B20)-1)),IF(RIGHT(B20,1)="M",EDATE($B$3,VALUE(LEFT(B20,LEN(B20)-1))),EDATE($B$3,12*VALUE(LEFT(B20,LEN(B20)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D20" s="24">
@@ -30919,7 +30924,7 @@
         </is>
       </c>
       <c r="C21" s="23">
-        <f>IF(RIGHT(B21,1)="W",$B$3+7*VALUE(LEFT(B21,LEN(B21)-1)),IF(RIGHT(B21,1)="M",EDATE($B$3,VALUE(LEFT(B21,LEN(B21)-1))),EDATE($B$3,12*VALUE(LEFT(B21,LEN(B21)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B21,1)="W",$B$3+7*VALUE(LEFT(B21,LEN(B21)-1)),IF(RIGHT(B21,1)="M",EDATE($B$3,VALUE(LEFT(B21,LEN(B21)-1))),EDATE($B$3,12*VALUE(LEFT(B21,LEN(B21)-1)))))+IF(WEEKDAY(IF(RIGHT(B21,1)="W",$B$3+7*VALUE(LEFT(B21,LEN(B21)-1)),IF(RIGHT(B21,1)="M",EDATE($B$3,VALUE(LEFT(B21,LEN(B21)-1))),EDATE($B$3,12*VALUE(LEFT(B21,LEN(B21)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B21,1)="W",$B$3+7*VALUE(LEFT(B21,LEN(B21)-1)),IF(RIGHT(B21,1)="M",EDATE($B$3,VALUE(LEFT(B21,LEN(B21)-1))),EDATE($B$3,12*VALUE(LEFT(B21,LEN(B21)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B21,1)="W",$B$3+7*VALUE(LEFT(B21,LEN(B21)-1)),IF(RIGHT(B21,1)="M",EDATE($B$3,VALUE(LEFT(B21,LEN(B21)-1))),EDATE($B$3,12*VALUE(LEFT(B21,LEN(B21)-1)))))),(IF(RIGHT(B21,1)="W",$B$3+7*VALUE(LEFT(B21,LEN(B21)-1)),IF(RIGHT(B21,1)="M",EDATE($B$3,VALUE(LEFT(B21,LEN(B21)-1))),EDATE($B$3,12*VALUE(LEFT(B21,LEN(B21)-1)))))-IF(WEEKDAY(IF(RIGHT(B21,1)="W",$B$3+7*VALUE(LEFT(B21,LEN(B21)-1)),IF(RIGHT(B21,1)="M",EDATE($B$3,VALUE(LEFT(B21,LEN(B21)-1))),EDATE($B$3,12*VALUE(LEFT(B21,LEN(B21)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B21,1)="W",$B$3+7*VALUE(LEFT(B21,LEN(B21)-1)),IF(RIGHT(B21,1)="M",EDATE($B$3,VALUE(LEFT(B21,LEN(B21)-1))),EDATE($B$3,12*VALUE(LEFT(B21,LEN(B21)-1))))),2)=7,2,0))),(IF(RIGHT(B21,1)="W",$B$3+7*VALUE(LEFT(B21,LEN(B21)-1)),IF(RIGHT(B21,1)="M",EDATE($B$3,VALUE(LEFT(B21,LEN(B21)-1))),EDATE($B$3,12*VALUE(LEFT(B21,LEN(B21)-1)))))+IF(WEEKDAY(IF(RIGHT(B21,1)="W",$B$3+7*VALUE(LEFT(B21,LEN(B21)-1)),IF(RIGHT(B21,1)="M",EDATE($B$3,VALUE(LEFT(B21,LEN(B21)-1))),EDATE($B$3,12*VALUE(LEFT(B21,LEN(B21)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B21,1)="W",$B$3+7*VALUE(LEFT(B21,LEN(B21)-1)),IF(RIGHT(B21,1)="M",EDATE($B$3,VALUE(LEFT(B21,LEN(B21)-1))),EDATE($B$3,12*VALUE(LEFT(B21,LEN(B21)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D21" s="24">
@@ -30965,7 +30970,7 @@
         </is>
       </c>
       <c r="C22" s="23">
-        <f>IF(RIGHT(B22,1)="W",$B$3+7*VALUE(LEFT(B22,LEN(B22)-1)),IF(RIGHT(B22,1)="M",EDATE($B$3,VALUE(LEFT(B22,LEN(B22)-1))),EDATE($B$3,12*VALUE(LEFT(B22,LEN(B22)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B22,1)="W",$B$3+7*VALUE(LEFT(B22,LEN(B22)-1)),IF(RIGHT(B22,1)="M",EDATE($B$3,VALUE(LEFT(B22,LEN(B22)-1))),EDATE($B$3,12*VALUE(LEFT(B22,LEN(B22)-1)))))+IF(WEEKDAY(IF(RIGHT(B22,1)="W",$B$3+7*VALUE(LEFT(B22,LEN(B22)-1)),IF(RIGHT(B22,1)="M",EDATE($B$3,VALUE(LEFT(B22,LEN(B22)-1))),EDATE($B$3,12*VALUE(LEFT(B22,LEN(B22)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B22,1)="W",$B$3+7*VALUE(LEFT(B22,LEN(B22)-1)),IF(RIGHT(B22,1)="M",EDATE($B$3,VALUE(LEFT(B22,LEN(B22)-1))),EDATE($B$3,12*VALUE(LEFT(B22,LEN(B22)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B22,1)="W",$B$3+7*VALUE(LEFT(B22,LEN(B22)-1)),IF(RIGHT(B22,1)="M",EDATE($B$3,VALUE(LEFT(B22,LEN(B22)-1))),EDATE($B$3,12*VALUE(LEFT(B22,LEN(B22)-1)))))),(IF(RIGHT(B22,1)="W",$B$3+7*VALUE(LEFT(B22,LEN(B22)-1)),IF(RIGHT(B22,1)="M",EDATE($B$3,VALUE(LEFT(B22,LEN(B22)-1))),EDATE($B$3,12*VALUE(LEFT(B22,LEN(B22)-1)))))-IF(WEEKDAY(IF(RIGHT(B22,1)="W",$B$3+7*VALUE(LEFT(B22,LEN(B22)-1)),IF(RIGHT(B22,1)="M",EDATE($B$3,VALUE(LEFT(B22,LEN(B22)-1))),EDATE($B$3,12*VALUE(LEFT(B22,LEN(B22)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B22,1)="W",$B$3+7*VALUE(LEFT(B22,LEN(B22)-1)),IF(RIGHT(B22,1)="M",EDATE($B$3,VALUE(LEFT(B22,LEN(B22)-1))),EDATE($B$3,12*VALUE(LEFT(B22,LEN(B22)-1))))),2)=7,2,0))),(IF(RIGHT(B22,1)="W",$B$3+7*VALUE(LEFT(B22,LEN(B22)-1)),IF(RIGHT(B22,1)="M",EDATE($B$3,VALUE(LEFT(B22,LEN(B22)-1))),EDATE($B$3,12*VALUE(LEFT(B22,LEN(B22)-1)))))+IF(WEEKDAY(IF(RIGHT(B22,1)="W",$B$3+7*VALUE(LEFT(B22,LEN(B22)-1)),IF(RIGHT(B22,1)="M",EDATE($B$3,VALUE(LEFT(B22,LEN(B22)-1))),EDATE($B$3,12*VALUE(LEFT(B22,LEN(B22)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B22,1)="W",$B$3+7*VALUE(LEFT(B22,LEN(B22)-1)),IF(RIGHT(B22,1)="M",EDATE($B$3,VALUE(LEFT(B22,LEN(B22)-1))),EDATE($B$3,12*VALUE(LEFT(B22,LEN(B22)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D22" s="24">
@@ -31011,7 +31016,7 @@
         </is>
       </c>
       <c r="C23" s="23">
-        <f>IF(RIGHT(B23,1)="W",$B$3+7*VALUE(LEFT(B23,LEN(B23)-1)),IF(RIGHT(B23,1)="M",EDATE($B$3,VALUE(LEFT(B23,LEN(B23)-1))),EDATE($B$3,12*VALUE(LEFT(B23,LEN(B23)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B23,1)="W",$B$3+7*VALUE(LEFT(B23,LEN(B23)-1)),IF(RIGHT(B23,1)="M",EDATE($B$3,VALUE(LEFT(B23,LEN(B23)-1))),EDATE($B$3,12*VALUE(LEFT(B23,LEN(B23)-1)))))+IF(WEEKDAY(IF(RIGHT(B23,1)="W",$B$3+7*VALUE(LEFT(B23,LEN(B23)-1)),IF(RIGHT(B23,1)="M",EDATE($B$3,VALUE(LEFT(B23,LEN(B23)-1))),EDATE($B$3,12*VALUE(LEFT(B23,LEN(B23)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B23,1)="W",$B$3+7*VALUE(LEFT(B23,LEN(B23)-1)),IF(RIGHT(B23,1)="M",EDATE($B$3,VALUE(LEFT(B23,LEN(B23)-1))),EDATE($B$3,12*VALUE(LEFT(B23,LEN(B23)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B23,1)="W",$B$3+7*VALUE(LEFT(B23,LEN(B23)-1)),IF(RIGHT(B23,1)="M",EDATE($B$3,VALUE(LEFT(B23,LEN(B23)-1))),EDATE($B$3,12*VALUE(LEFT(B23,LEN(B23)-1)))))),(IF(RIGHT(B23,1)="W",$B$3+7*VALUE(LEFT(B23,LEN(B23)-1)),IF(RIGHT(B23,1)="M",EDATE($B$3,VALUE(LEFT(B23,LEN(B23)-1))),EDATE($B$3,12*VALUE(LEFT(B23,LEN(B23)-1)))))-IF(WEEKDAY(IF(RIGHT(B23,1)="W",$B$3+7*VALUE(LEFT(B23,LEN(B23)-1)),IF(RIGHT(B23,1)="M",EDATE($B$3,VALUE(LEFT(B23,LEN(B23)-1))),EDATE($B$3,12*VALUE(LEFT(B23,LEN(B23)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B23,1)="W",$B$3+7*VALUE(LEFT(B23,LEN(B23)-1)),IF(RIGHT(B23,1)="M",EDATE($B$3,VALUE(LEFT(B23,LEN(B23)-1))),EDATE($B$3,12*VALUE(LEFT(B23,LEN(B23)-1))))),2)=7,2,0))),(IF(RIGHT(B23,1)="W",$B$3+7*VALUE(LEFT(B23,LEN(B23)-1)),IF(RIGHT(B23,1)="M",EDATE($B$3,VALUE(LEFT(B23,LEN(B23)-1))),EDATE($B$3,12*VALUE(LEFT(B23,LEN(B23)-1)))))+IF(WEEKDAY(IF(RIGHT(B23,1)="W",$B$3+7*VALUE(LEFT(B23,LEN(B23)-1)),IF(RIGHT(B23,1)="M",EDATE($B$3,VALUE(LEFT(B23,LEN(B23)-1))),EDATE($B$3,12*VALUE(LEFT(B23,LEN(B23)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B23,1)="W",$B$3+7*VALUE(LEFT(B23,LEN(B23)-1)),IF(RIGHT(B23,1)="M",EDATE($B$3,VALUE(LEFT(B23,LEN(B23)-1))),EDATE($B$3,12*VALUE(LEFT(B23,LEN(B23)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D23" s="24">
@@ -31057,7 +31062,7 @@
         </is>
       </c>
       <c r="C24" s="23">
-        <f>IF(RIGHT(B24,1)="W",$B$3+7*VALUE(LEFT(B24,LEN(B24)-1)),IF(RIGHT(B24,1)="M",EDATE($B$3,VALUE(LEFT(B24,LEN(B24)-1))),EDATE($B$3,12*VALUE(LEFT(B24,LEN(B24)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B24,1)="W",$B$3+7*VALUE(LEFT(B24,LEN(B24)-1)),IF(RIGHT(B24,1)="M",EDATE($B$3,VALUE(LEFT(B24,LEN(B24)-1))),EDATE($B$3,12*VALUE(LEFT(B24,LEN(B24)-1)))))+IF(WEEKDAY(IF(RIGHT(B24,1)="W",$B$3+7*VALUE(LEFT(B24,LEN(B24)-1)),IF(RIGHT(B24,1)="M",EDATE($B$3,VALUE(LEFT(B24,LEN(B24)-1))),EDATE($B$3,12*VALUE(LEFT(B24,LEN(B24)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B24,1)="W",$B$3+7*VALUE(LEFT(B24,LEN(B24)-1)),IF(RIGHT(B24,1)="M",EDATE($B$3,VALUE(LEFT(B24,LEN(B24)-1))),EDATE($B$3,12*VALUE(LEFT(B24,LEN(B24)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B24,1)="W",$B$3+7*VALUE(LEFT(B24,LEN(B24)-1)),IF(RIGHT(B24,1)="M",EDATE($B$3,VALUE(LEFT(B24,LEN(B24)-1))),EDATE($B$3,12*VALUE(LEFT(B24,LEN(B24)-1)))))),(IF(RIGHT(B24,1)="W",$B$3+7*VALUE(LEFT(B24,LEN(B24)-1)),IF(RIGHT(B24,1)="M",EDATE($B$3,VALUE(LEFT(B24,LEN(B24)-1))),EDATE($B$3,12*VALUE(LEFT(B24,LEN(B24)-1)))))-IF(WEEKDAY(IF(RIGHT(B24,1)="W",$B$3+7*VALUE(LEFT(B24,LEN(B24)-1)),IF(RIGHT(B24,1)="M",EDATE($B$3,VALUE(LEFT(B24,LEN(B24)-1))),EDATE($B$3,12*VALUE(LEFT(B24,LEN(B24)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B24,1)="W",$B$3+7*VALUE(LEFT(B24,LEN(B24)-1)),IF(RIGHT(B24,1)="M",EDATE($B$3,VALUE(LEFT(B24,LEN(B24)-1))),EDATE($B$3,12*VALUE(LEFT(B24,LEN(B24)-1))))),2)=7,2,0))),(IF(RIGHT(B24,1)="W",$B$3+7*VALUE(LEFT(B24,LEN(B24)-1)),IF(RIGHT(B24,1)="M",EDATE($B$3,VALUE(LEFT(B24,LEN(B24)-1))),EDATE($B$3,12*VALUE(LEFT(B24,LEN(B24)-1)))))+IF(WEEKDAY(IF(RIGHT(B24,1)="W",$B$3+7*VALUE(LEFT(B24,LEN(B24)-1)),IF(RIGHT(B24,1)="M",EDATE($B$3,VALUE(LEFT(B24,LEN(B24)-1))),EDATE($B$3,12*VALUE(LEFT(B24,LEN(B24)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B24,1)="W",$B$3+7*VALUE(LEFT(B24,LEN(B24)-1)),IF(RIGHT(B24,1)="M",EDATE($B$3,VALUE(LEFT(B24,LEN(B24)-1))),EDATE($B$3,12*VALUE(LEFT(B24,LEN(B24)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D24" s="24">
@@ -31107,7 +31112,7 @@
         </is>
       </c>
       <c r="C25" s="23">
-        <f>IF(RIGHT(B25,1)="W",$B$3+7*VALUE(LEFT(B25,LEN(B25)-1)),IF(RIGHT(B25,1)="M",EDATE($B$3,VALUE(LEFT(B25,LEN(B25)-1))),EDATE($B$3,12*VALUE(LEFT(B25,LEN(B25)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B25,1)="W",$B$3+7*VALUE(LEFT(B25,LEN(B25)-1)),IF(RIGHT(B25,1)="M",EDATE($B$3,VALUE(LEFT(B25,LEN(B25)-1))),EDATE($B$3,12*VALUE(LEFT(B25,LEN(B25)-1)))))+IF(WEEKDAY(IF(RIGHT(B25,1)="W",$B$3+7*VALUE(LEFT(B25,LEN(B25)-1)),IF(RIGHT(B25,1)="M",EDATE($B$3,VALUE(LEFT(B25,LEN(B25)-1))),EDATE($B$3,12*VALUE(LEFT(B25,LEN(B25)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B25,1)="W",$B$3+7*VALUE(LEFT(B25,LEN(B25)-1)),IF(RIGHT(B25,1)="M",EDATE($B$3,VALUE(LEFT(B25,LEN(B25)-1))),EDATE($B$3,12*VALUE(LEFT(B25,LEN(B25)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B25,1)="W",$B$3+7*VALUE(LEFT(B25,LEN(B25)-1)),IF(RIGHT(B25,1)="M",EDATE($B$3,VALUE(LEFT(B25,LEN(B25)-1))),EDATE($B$3,12*VALUE(LEFT(B25,LEN(B25)-1)))))),(IF(RIGHT(B25,1)="W",$B$3+7*VALUE(LEFT(B25,LEN(B25)-1)),IF(RIGHT(B25,1)="M",EDATE($B$3,VALUE(LEFT(B25,LEN(B25)-1))),EDATE($B$3,12*VALUE(LEFT(B25,LEN(B25)-1)))))-IF(WEEKDAY(IF(RIGHT(B25,1)="W",$B$3+7*VALUE(LEFT(B25,LEN(B25)-1)),IF(RIGHT(B25,1)="M",EDATE($B$3,VALUE(LEFT(B25,LEN(B25)-1))),EDATE($B$3,12*VALUE(LEFT(B25,LEN(B25)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B25,1)="W",$B$3+7*VALUE(LEFT(B25,LEN(B25)-1)),IF(RIGHT(B25,1)="M",EDATE($B$3,VALUE(LEFT(B25,LEN(B25)-1))),EDATE($B$3,12*VALUE(LEFT(B25,LEN(B25)-1))))),2)=7,2,0))),(IF(RIGHT(B25,1)="W",$B$3+7*VALUE(LEFT(B25,LEN(B25)-1)),IF(RIGHT(B25,1)="M",EDATE($B$3,VALUE(LEFT(B25,LEN(B25)-1))),EDATE($B$3,12*VALUE(LEFT(B25,LEN(B25)-1)))))+IF(WEEKDAY(IF(RIGHT(B25,1)="W",$B$3+7*VALUE(LEFT(B25,LEN(B25)-1)),IF(RIGHT(B25,1)="M",EDATE($B$3,VALUE(LEFT(B25,LEN(B25)-1))),EDATE($B$3,12*VALUE(LEFT(B25,LEN(B25)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B25,1)="W",$B$3+7*VALUE(LEFT(B25,LEN(B25)-1)),IF(RIGHT(B25,1)="M",EDATE($B$3,VALUE(LEFT(B25,LEN(B25)-1))),EDATE($B$3,12*VALUE(LEFT(B25,LEN(B25)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D25" s="24">
@@ -31157,7 +31162,7 @@
         </is>
       </c>
       <c r="C26" s="23">
-        <f>IF(RIGHT(B26,1)="W",$B$3+7*VALUE(LEFT(B26,LEN(B26)-1)),IF(RIGHT(B26,1)="M",EDATE($B$3,VALUE(LEFT(B26,LEN(B26)-1))),EDATE($B$3,12*VALUE(LEFT(B26,LEN(B26)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B26,1)="W",$B$3+7*VALUE(LEFT(B26,LEN(B26)-1)),IF(RIGHT(B26,1)="M",EDATE($B$3,VALUE(LEFT(B26,LEN(B26)-1))),EDATE($B$3,12*VALUE(LEFT(B26,LEN(B26)-1)))))+IF(WEEKDAY(IF(RIGHT(B26,1)="W",$B$3+7*VALUE(LEFT(B26,LEN(B26)-1)),IF(RIGHT(B26,1)="M",EDATE($B$3,VALUE(LEFT(B26,LEN(B26)-1))),EDATE($B$3,12*VALUE(LEFT(B26,LEN(B26)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B26,1)="W",$B$3+7*VALUE(LEFT(B26,LEN(B26)-1)),IF(RIGHT(B26,1)="M",EDATE($B$3,VALUE(LEFT(B26,LEN(B26)-1))),EDATE($B$3,12*VALUE(LEFT(B26,LEN(B26)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B26,1)="W",$B$3+7*VALUE(LEFT(B26,LEN(B26)-1)),IF(RIGHT(B26,1)="M",EDATE($B$3,VALUE(LEFT(B26,LEN(B26)-1))),EDATE($B$3,12*VALUE(LEFT(B26,LEN(B26)-1)))))),(IF(RIGHT(B26,1)="W",$B$3+7*VALUE(LEFT(B26,LEN(B26)-1)),IF(RIGHT(B26,1)="M",EDATE($B$3,VALUE(LEFT(B26,LEN(B26)-1))),EDATE($B$3,12*VALUE(LEFT(B26,LEN(B26)-1)))))-IF(WEEKDAY(IF(RIGHT(B26,1)="W",$B$3+7*VALUE(LEFT(B26,LEN(B26)-1)),IF(RIGHT(B26,1)="M",EDATE($B$3,VALUE(LEFT(B26,LEN(B26)-1))),EDATE($B$3,12*VALUE(LEFT(B26,LEN(B26)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B26,1)="W",$B$3+7*VALUE(LEFT(B26,LEN(B26)-1)),IF(RIGHT(B26,1)="M",EDATE($B$3,VALUE(LEFT(B26,LEN(B26)-1))),EDATE($B$3,12*VALUE(LEFT(B26,LEN(B26)-1))))),2)=7,2,0))),(IF(RIGHT(B26,1)="W",$B$3+7*VALUE(LEFT(B26,LEN(B26)-1)),IF(RIGHT(B26,1)="M",EDATE($B$3,VALUE(LEFT(B26,LEN(B26)-1))),EDATE($B$3,12*VALUE(LEFT(B26,LEN(B26)-1)))))+IF(WEEKDAY(IF(RIGHT(B26,1)="W",$B$3+7*VALUE(LEFT(B26,LEN(B26)-1)),IF(RIGHT(B26,1)="M",EDATE($B$3,VALUE(LEFT(B26,LEN(B26)-1))),EDATE($B$3,12*VALUE(LEFT(B26,LEN(B26)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B26,1)="W",$B$3+7*VALUE(LEFT(B26,LEN(B26)-1)),IF(RIGHT(B26,1)="M",EDATE($B$3,VALUE(LEFT(B26,LEN(B26)-1))),EDATE($B$3,12*VALUE(LEFT(B26,LEN(B26)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D26" s="24">
@@ -31207,7 +31212,7 @@
         </is>
       </c>
       <c r="C27" s="23">
-        <f>IF(RIGHT(B27,1)="W",$B$3+7*VALUE(LEFT(B27,LEN(B27)-1)),IF(RIGHT(B27,1)="M",EDATE($B$3,VALUE(LEFT(B27,LEN(B27)-1))),EDATE($B$3,12*VALUE(LEFT(B27,LEN(B27)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B27,1)="W",$B$3+7*VALUE(LEFT(B27,LEN(B27)-1)),IF(RIGHT(B27,1)="M",EDATE($B$3,VALUE(LEFT(B27,LEN(B27)-1))),EDATE($B$3,12*VALUE(LEFT(B27,LEN(B27)-1)))))+IF(WEEKDAY(IF(RIGHT(B27,1)="W",$B$3+7*VALUE(LEFT(B27,LEN(B27)-1)),IF(RIGHT(B27,1)="M",EDATE($B$3,VALUE(LEFT(B27,LEN(B27)-1))),EDATE($B$3,12*VALUE(LEFT(B27,LEN(B27)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B27,1)="W",$B$3+7*VALUE(LEFT(B27,LEN(B27)-1)),IF(RIGHT(B27,1)="M",EDATE($B$3,VALUE(LEFT(B27,LEN(B27)-1))),EDATE($B$3,12*VALUE(LEFT(B27,LEN(B27)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B27,1)="W",$B$3+7*VALUE(LEFT(B27,LEN(B27)-1)),IF(RIGHT(B27,1)="M",EDATE($B$3,VALUE(LEFT(B27,LEN(B27)-1))),EDATE($B$3,12*VALUE(LEFT(B27,LEN(B27)-1)))))),(IF(RIGHT(B27,1)="W",$B$3+7*VALUE(LEFT(B27,LEN(B27)-1)),IF(RIGHT(B27,1)="M",EDATE($B$3,VALUE(LEFT(B27,LEN(B27)-1))),EDATE($B$3,12*VALUE(LEFT(B27,LEN(B27)-1)))))-IF(WEEKDAY(IF(RIGHT(B27,1)="W",$B$3+7*VALUE(LEFT(B27,LEN(B27)-1)),IF(RIGHT(B27,1)="M",EDATE($B$3,VALUE(LEFT(B27,LEN(B27)-1))),EDATE($B$3,12*VALUE(LEFT(B27,LEN(B27)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B27,1)="W",$B$3+7*VALUE(LEFT(B27,LEN(B27)-1)),IF(RIGHT(B27,1)="M",EDATE($B$3,VALUE(LEFT(B27,LEN(B27)-1))),EDATE($B$3,12*VALUE(LEFT(B27,LEN(B27)-1))))),2)=7,2,0))),(IF(RIGHT(B27,1)="W",$B$3+7*VALUE(LEFT(B27,LEN(B27)-1)),IF(RIGHT(B27,1)="M",EDATE($B$3,VALUE(LEFT(B27,LEN(B27)-1))),EDATE($B$3,12*VALUE(LEFT(B27,LEN(B27)-1)))))+IF(WEEKDAY(IF(RIGHT(B27,1)="W",$B$3+7*VALUE(LEFT(B27,LEN(B27)-1)),IF(RIGHT(B27,1)="M",EDATE($B$3,VALUE(LEFT(B27,LEN(B27)-1))),EDATE($B$3,12*VALUE(LEFT(B27,LEN(B27)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B27,1)="W",$B$3+7*VALUE(LEFT(B27,LEN(B27)-1)),IF(RIGHT(B27,1)="M",EDATE($B$3,VALUE(LEFT(B27,LEN(B27)-1))),EDATE($B$3,12*VALUE(LEFT(B27,LEN(B27)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D27" s="24">
@@ -31257,7 +31262,7 @@
         </is>
       </c>
       <c r="C28" s="23">
-        <f>IF(RIGHT(B28,1)="W",$B$3+7*VALUE(LEFT(B28,LEN(B28)-1)),IF(RIGHT(B28,1)="M",EDATE($B$3,VALUE(LEFT(B28,LEN(B28)-1))),EDATE($B$3,12*VALUE(LEFT(B28,LEN(B28)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B28,1)="W",$B$3+7*VALUE(LEFT(B28,LEN(B28)-1)),IF(RIGHT(B28,1)="M",EDATE($B$3,VALUE(LEFT(B28,LEN(B28)-1))),EDATE($B$3,12*VALUE(LEFT(B28,LEN(B28)-1)))))+IF(WEEKDAY(IF(RIGHT(B28,1)="W",$B$3+7*VALUE(LEFT(B28,LEN(B28)-1)),IF(RIGHT(B28,1)="M",EDATE($B$3,VALUE(LEFT(B28,LEN(B28)-1))),EDATE($B$3,12*VALUE(LEFT(B28,LEN(B28)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B28,1)="W",$B$3+7*VALUE(LEFT(B28,LEN(B28)-1)),IF(RIGHT(B28,1)="M",EDATE($B$3,VALUE(LEFT(B28,LEN(B28)-1))),EDATE($B$3,12*VALUE(LEFT(B28,LEN(B28)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B28,1)="W",$B$3+7*VALUE(LEFT(B28,LEN(B28)-1)),IF(RIGHT(B28,1)="M",EDATE($B$3,VALUE(LEFT(B28,LEN(B28)-1))),EDATE($B$3,12*VALUE(LEFT(B28,LEN(B28)-1)))))),(IF(RIGHT(B28,1)="W",$B$3+7*VALUE(LEFT(B28,LEN(B28)-1)),IF(RIGHT(B28,1)="M",EDATE($B$3,VALUE(LEFT(B28,LEN(B28)-1))),EDATE($B$3,12*VALUE(LEFT(B28,LEN(B28)-1)))))-IF(WEEKDAY(IF(RIGHT(B28,1)="W",$B$3+7*VALUE(LEFT(B28,LEN(B28)-1)),IF(RIGHT(B28,1)="M",EDATE($B$3,VALUE(LEFT(B28,LEN(B28)-1))),EDATE($B$3,12*VALUE(LEFT(B28,LEN(B28)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B28,1)="W",$B$3+7*VALUE(LEFT(B28,LEN(B28)-1)),IF(RIGHT(B28,1)="M",EDATE($B$3,VALUE(LEFT(B28,LEN(B28)-1))),EDATE($B$3,12*VALUE(LEFT(B28,LEN(B28)-1))))),2)=7,2,0))),(IF(RIGHT(B28,1)="W",$B$3+7*VALUE(LEFT(B28,LEN(B28)-1)),IF(RIGHT(B28,1)="M",EDATE($B$3,VALUE(LEFT(B28,LEN(B28)-1))),EDATE($B$3,12*VALUE(LEFT(B28,LEN(B28)-1)))))+IF(WEEKDAY(IF(RIGHT(B28,1)="W",$B$3+7*VALUE(LEFT(B28,LEN(B28)-1)),IF(RIGHT(B28,1)="M",EDATE($B$3,VALUE(LEFT(B28,LEN(B28)-1))),EDATE($B$3,12*VALUE(LEFT(B28,LEN(B28)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B28,1)="W",$B$3+7*VALUE(LEFT(B28,LEN(B28)-1)),IF(RIGHT(B28,1)="M",EDATE($B$3,VALUE(LEFT(B28,LEN(B28)-1))),EDATE($B$3,12*VALUE(LEFT(B28,LEN(B28)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D28" s="24">
@@ -31307,7 +31312,7 @@
         </is>
       </c>
       <c r="C29" s="23">
-        <f>IF(RIGHT(B29,1)="W",$B$3+7*VALUE(LEFT(B29,LEN(B29)-1)),IF(RIGHT(B29,1)="M",EDATE($B$3,VALUE(LEFT(B29,LEN(B29)-1))),EDATE($B$3,12*VALUE(LEFT(B29,LEN(B29)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B29,1)="W",$B$3+7*VALUE(LEFT(B29,LEN(B29)-1)),IF(RIGHT(B29,1)="M",EDATE($B$3,VALUE(LEFT(B29,LEN(B29)-1))),EDATE($B$3,12*VALUE(LEFT(B29,LEN(B29)-1)))))+IF(WEEKDAY(IF(RIGHT(B29,1)="W",$B$3+7*VALUE(LEFT(B29,LEN(B29)-1)),IF(RIGHT(B29,1)="M",EDATE($B$3,VALUE(LEFT(B29,LEN(B29)-1))),EDATE($B$3,12*VALUE(LEFT(B29,LEN(B29)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B29,1)="W",$B$3+7*VALUE(LEFT(B29,LEN(B29)-1)),IF(RIGHT(B29,1)="M",EDATE($B$3,VALUE(LEFT(B29,LEN(B29)-1))),EDATE($B$3,12*VALUE(LEFT(B29,LEN(B29)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B29,1)="W",$B$3+7*VALUE(LEFT(B29,LEN(B29)-1)),IF(RIGHT(B29,1)="M",EDATE($B$3,VALUE(LEFT(B29,LEN(B29)-1))),EDATE($B$3,12*VALUE(LEFT(B29,LEN(B29)-1)))))),(IF(RIGHT(B29,1)="W",$B$3+7*VALUE(LEFT(B29,LEN(B29)-1)),IF(RIGHT(B29,1)="M",EDATE($B$3,VALUE(LEFT(B29,LEN(B29)-1))),EDATE($B$3,12*VALUE(LEFT(B29,LEN(B29)-1)))))-IF(WEEKDAY(IF(RIGHT(B29,1)="W",$B$3+7*VALUE(LEFT(B29,LEN(B29)-1)),IF(RIGHT(B29,1)="M",EDATE($B$3,VALUE(LEFT(B29,LEN(B29)-1))),EDATE($B$3,12*VALUE(LEFT(B29,LEN(B29)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B29,1)="W",$B$3+7*VALUE(LEFT(B29,LEN(B29)-1)),IF(RIGHT(B29,1)="M",EDATE($B$3,VALUE(LEFT(B29,LEN(B29)-1))),EDATE($B$3,12*VALUE(LEFT(B29,LEN(B29)-1))))),2)=7,2,0))),(IF(RIGHT(B29,1)="W",$B$3+7*VALUE(LEFT(B29,LEN(B29)-1)),IF(RIGHT(B29,1)="M",EDATE($B$3,VALUE(LEFT(B29,LEN(B29)-1))),EDATE($B$3,12*VALUE(LEFT(B29,LEN(B29)-1)))))+IF(WEEKDAY(IF(RIGHT(B29,1)="W",$B$3+7*VALUE(LEFT(B29,LEN(B29)-1)),IF(RIGHT(B29,1)="M",EDATE($B$3,VALUE(LEFT(B29,LEN(B29)-1))),EDATE($B$3,12*VALUE(LEFT(B29,LEN(B29)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B29,1)="W",$B$3+7*VALUE(LEFT(B29,LEN(B29)-1)),IF(RIGHT(B29,1)="M",EDATE($B$3,VALUE(LEFT(B29,LEN(B29)-1))),EDATE($B$3,12*VALUE(LEFT(B29,LEN(B29)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D29" s="24">
@@ -31357,7 +31362,7 @@
         </is>
       </c>
       <c r="C30" s="23">
-        <f>IF(RIGHT(B30,1)="W",$B$3+7*VALUE(LEFT(B30,LEN(B30)-1)),IF(RIGHT(B30,1)="M",EDATE($B$3,VALUE(LEFT(B30,LEN(B30)-1))),EDATE($B$3,12*VALUE(LEFT(B30,LEN(B30)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B30,1)="W",$B$3+7*VALUE(LEFT(B30,LEN(B30)-1)),IF(RIGHT(B30,1)="M",EDATE($B$3,VALUE(LEFT(B30,LEN(B30)-1))),EDATE($B$3,12*VALUE(LEFT(B30,LEN(B30)-1)))))+IF(WEEKDAY(IF(RIGHT(B30,1)="W",$B$3+7*VALUE(LEFT(B30,LEN(B30)-1)),IF(RIGHT(B30,1)="M",EDATE($B$3,VALUE(LEFT(B30,LEN(B30)-1))),EDATE($B$3,12*VALUE(LEFT(B30,LEN(B30)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B30,1)="W",$B$3+7*VALUE(LEFT(B30,LEN(B30)-1)),IF(RIGHT(B30,1)="M",EDATE($B$3,VALUE(LEFT(B30,LEN(B30)-1))),EDATE($B$3,12*VALUE(LEFT(B30,LEN(B30)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B30,1)="W",$B$3+7*VALUE(LEFT(B30,LEN(B30)-1)),IF(RIGHT(B30,1)="M",EDATE($B$3,VALUE(LEFT(B30,LEN(B30)-1))),EDATE($B$3,12*VALUE(LEFT(B30,LEN(B30)-1)))))),(IF(RIGHT(B30,1)="W",$B$3+7*VALUE(LEFT(B30,LEN(B30)-1)),IF(RIGHT(B30,1)="M",EDATE($B$3,VALUE(LEFT(B30,LEN(B30)-1))),EDATE($B$3,12*VALUE(LEFT(B30,LEN(B30)-1)))))-IF(WEEKDAY(IF(RIGHT(B30,1)="W",$B$3+7*VALUE(LEFT(B30,LEN(B30)-1)),IF(RIGHT(B30,1)="M",EDATE($B$3,VALUE(LEFT(B30,LEN(B30)-1))),EDATE($B$3,12*VALUE(LEFT(B30,LEN(B30)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B30,1)="W",$B$3+7*VALUE(LEFT(B30,LEN(B30)-1)),IF(RIGHT(B30,1)="M",EDATE($B$3,VALUE(LEFT(B30,LEN(B30)-1))),EDATE($B$3,12*VALUE(LEFT(B30,LEN(B30)-1))))),2)=7,2,0))),(IF(RIGHT(B30,1)="W",$B$3+7*VALUE(LEFT(B30,LEN(B30)-1)),IF(RIGHT(B30,1)="M",EDATE($B$3,VALUE(LEFT(B30,LEN(B30)-1))),EDATE($B$3,12*VALUE(LEFT(B30,LEN(B30)-1)))))+IF(WEEKDAY(IF(RIGHT(B30,1)="W",$B$3+7*VALUE(LEFT(B30,LEN(B30)-1)),IF(RIGHT(B30,1)="M",EDATE($B$3,VALUE(LEFT(B30,LEN(B30)-1))),EDATE($B$3,12*VALUE(LEFT(B30,LEN(B30)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B30,1)="W",$B$3+7*VALUE(LEFT(B30,LEN(B30)-1)),IF(RIGHT(B30,1)="M",EDATE($B$3,VALUE(LEFT(B30,LEN(B30)-1))),EDATE($B$3,12*VALUE(LEFT(B30,LEN(B30)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D30" s="24">
@@ -31407,7 +31412,7 @@
         </is>
       </c>
       <c r="C31" s="23">
-        <f>IF(RIGHT(B31,1)="W",$B$3+7*VALUE(LEFT(B31,LEN(B31)-1)),IF(RIGHT(B31,1)="M",EDATE($B$3,VALUE(LEFT(B31,LEN(B31)-1))),EDATE($B$3,12*VALUE(LEFT(B31,LEN(B31)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B31,1)="W",$B$3+7*VALUE(LEFT(B31,LEN(B31)-1)),IF(RIGHT(B31,1)="M",EDATE($B$3,VALUE(LEFT(B31,LEN(B31)-1))),EDATE($B$3,12*VALUE(LEFT(B31,LEN(B31)-1)))))+IF(WEEKDAY(IF(RIGHT(B31,1)="W",$B$3+7*VALUE(LEFT(B31,LEN(B31)-1)),IF(RIGHT(B31,1)="M",EDATE($B$3,VALUE(LEFT(B31,LEN(B31)-1))),EDATE($B$3,12*VALUE(LEFT(B31,LEN(B31)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B31,1)="W",$B$3+7*VALUE(LEFT(B31,LEN(B31)-1)),IF(RIGHT(B31,1)="M",EDATE($B$3,VALUE(LEFT(B31,LEN(B31)-1))),EDATE($B$3,12*VALUE(LEFT(B31,LEN(B31)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B31,1)="W",$B$3+7*VALUE(LEFT(B31,LEN(B31)-1)),IF(RIGHT(B31,1)="M",EDATE($B$3,VALUE(LEFT(B31,LEN(B31)-1))),EDATE($B$3,12*VALUE(LEFT(B31,LEN(B31)-1)))))),(IF(RIGHT(B31,1)="W",$B$3+7*VALUE(LEFT(B31,LEN(B31)-1)),IF(RIGHT(B31,1)="M",EDATE($B$3,VALUE(LEFT(B31,LEN(B31)-1))),EDATE($B$3,12*VALUE(LEFT(B31,LEN(B31)-1)))))-IF(WEEKDAY(IF(RIGHT(B31,1)="W",$B$3+7*VALUE(LEFT(B31,LEN(B31)-1)),IF(RIGHT(B31,1)="M",EDATE($B$3,VALUE(LEFT(B31,LEN(B31)-1))),EDATE($B$3,12*VALUE(LEFT(B31,LEN(B31)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B31,1)="W",$B$3+7*VALUE(LEFT(B31,LEN(B31)-1)),IF(RIGHT(B31,1)="M",EDATE($B$3,VALUE(LEFT(B31,LEN(B31)-1))),EDATE($B$3,12*VALUE(LEFT(B31,LEN(B31)-1))))),2)=7,2,0))),(IF(RIGHT(B31,1)="W",$B$3+7*VALUE(LEFT(B31,LEN(B31)-1)),IF(RIGHT(B31,1)="M",EDATE($B$3,VALUE(LEFT(B31,LEN(B31)-1))),EDATE($B$3,12*VALUE(LEFT(B31,LEN(B31)-1)))))+IF(WEEKDAY(IF(RIGHT(B31,1)="W",$B$3+7*VALUE(LEFT(B31,LEN(B31)-1)),IF(RIGHT(B31,1)="M",EDATE($B$3,VALUE(LEFT(B31,LEN(B31)-1))),EDATE($B$3,12*VALUE(LEFT(B31,LEN(B31)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B31,1)="W",$B$3+7*VALUE(LEFT(B31,LEN(B31)-1)),IF(RIGHT(B31,1)="M",EDATE($B$3,VALUE(LEFT(B31,LEN(B31)-1))),EDATE($B$3,12*VALUE(LEFT(B31,LEN(B31)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D31" s="24">
@@ -31457,7 +31462,7 @@
         </is>
       </c>
       <c r="C32" s="23">
-        <f>IF(RIGHT(B32,1)="W",$B$3+7*VALUE(LEFT(B32,LEN(B32)-1)),IF(RIGHT(B32,1)="M",EDATE($B$3,VALUE(LEFT(B32,LEN(B32)-1))),EDATE($B$3,12*VALUE(LEFT(B32,LEN(B32)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B32,1)="W",$B$3+7*VALUE(LEFT(B32,LEN(B32)-1)),IF(RIGHT(B32,1)="M",EDATE($B$3,VALUE(LEFT(B32,LEN(B32)-1))),EDATE($B$3,12*VALUE(LEFT(B32,LEN(B32)-1)))))+IF(WEEKDAY(IF(RIGHT(B32,1)="W",$B$3+7*VALUE(LEFT(B32,LEN(B32)-1)),IF(RIGHT(B32,1)="M",EDATE($B$3,VALUE(LEFT(B32,LEN(B32)-1))),EDATE($B$3,12*VALUE(LEFT(B32,LEN(B32)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B32,1)="W",$B$3+7*VALUE(LEFT(B32,LEN(B32)-1)),IF(RIGHT(B32,1)="M",EDATE($B$3,VALUE(LEFT(B32,LEN(B32)-1))),EDATE($B$3,12*VALUE(LEFT(B32,LEN(B32)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B32,1)="W",$B$3+7*VALUE(LEFT(B32,LEN(B32)-1)),IF(RIGHT(B32,1)="M",EDATE($B$3,VALUE(LEFT(B32,LEN(B32)-1))),EDATE($B$3,12*VALUE(LEFT(B32,LEN(B32)-1)))))),(IF(RIGHT(B32,1)="W",$B$3+7*VALUE(LEFT(B32,LEN(B32)-1)),IF(RIGHT(B32,1)="M",EDATE($B$3,VALUE(LEFT(B32,LEN(B32)-1))),EDATE($B$3,12*VALUE(LEFT(B32,LEN(B32)-1)))))-IF(WEEKDAY(IF(RIGHT(B32,1)="W",$B$3+7*VALUE(LEFT(B32,LEN(B32)-1)),IF(RIGHT(B32,1)="M",EDATE($B$3,VALUE(LEFT(B32,LEN(B32)-1))),EDATE($B$3,12*VALUE(LEFT(B32,LEN(B32)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B32,1)="W",$B$3+7*VALUE(LEFT(B32,LEN(B32)-1)),IF(RIGHT(B32,1)="M",EDATE($B$3,VALUE(LEFT(B32,LEN(B32)-1))),EDATE($B$3,12*VALUE(LEFT(B32,LEN(B32)-1))))),2)=7,2,0))),(IF(RIGHT(B32,1)="W",$B$3+7*VALUE(LEFT(B32,LEN(B32)-1)),IF(RIGHT(B32,1)="M",EDATE($B$3,VALUE(LEFT(B32,LEN(B32)-1))),EDATE($B$3,12*VALUE(LEFT(B32,LEN(B32)-1)))))+IF(WEEKDAY(IF(RIGHT(B32,1)="W",$B$3+7*VALUE(LEFT(B32,LEN(B32)-1)),IF(RIGHT(B32,1)="M",EDATE($B$3,VALUE(LEFT(B32,LEN(B32)-1))),EDATE($B$3,12*VALUE(LEFT(B32,LEN(B32)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B32,1)="W",$B$3+7*VALUE(LEFT(B32,LEN(B32)-1)),IF(RIGHT(B32,1)="M",EDATE($B$3,VALUE(LEFT(B32,LEN(B32)-1))),EDATE($B$3,12*VALUE(LEFT(B32,LEN(B32)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D32" s="24">
@@ -31507,7 +31512,7 @@
         </is>
       </c>
       <c r="C33" s="23">
-        <f>IF(RIGHT(B33,1)="W",$B$3+7*VALUE(LEFT(B33,LEN(B33)-1)),IF(RIGHT(B33,1)="M",EDATE($B$3,VALUE(LEFT(B33,LEN(B33)-1))),EDATE($B$3,12*VALUE(LEFT(B33,LEN(B33)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B33,1)="W",$B$3+7*VALUE(LEFT(B33,LEN(B33)-1)),IF(RIGHT(B33,1)="M",EDATE($B$3,VALUE(LEFT(B33,LEN(B33)-1))),EDATE($B$3,12*VALUE(LEFT(B33,LEN(B33)-1)))))+IF(WEEKDAY(IF(RIGHT(B33,1)="W",$B$3+7*VALUE(LEFT(B33,LEN(B33)-1)),IF(RIGHT(B33,1)="M",EDATE($B$3,VALUE(LEFT(B33,LEN(B33)-1))),EDATE($B$3,12*VALUE(LEFT(B33,LEN(B33)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B33,1)="W",$B$3+7*VALUE(LEFT(B33,LEN(B33)-1)),IF(RIGHT(B33,1)="M",EDATE($B$3,VALUE(LEFT(B33,LEN(B33)-1))),EDATE($B$3,12*VALUE(LEFT(B33,LEN(B33)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B33,1)="W",$B$3+7*VALUE(LEFT(B33,LEN(B33)-1)),IF(RIGHT(B33,1)="M",EDATE($B$3,VALUE(LEFT(B33,LEN(B33)-1))),EDATE($B$3,12*VALUE(LEFT(B33,LEN(B33)-1)))))),(IF(RIGHT(B33,1)="W",$B$3+7*VALUE(LEFT(B33,LEN(B33)-1)),IF(RIGHT(B33,1)="M",EDATE($B$3,VALUE(LEFT(B33,LEN(B33)-1))),EDATE($B$3,12*VALUE(LEFT(B33,LEN(B33)-1)))))-IF(WEEKDAY(IF(RIGHT(B33,1)="W",$B$3+7*VALUE(LEFT(B33,LEN(B33)-1)),IF(RIGHT(B33,1)="M",EDATE($B$3,VALUE(LEFT(B33,LEN(B33)-1))),EDATE($B$3,12*VALUE(LEFT(B33,LEN(B33)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B33,1)="W",$B$3+7*VALUE(LEFT(B33,LEN(B33)-1)),IF(RIGHT(B33,1)="M",EDATE($B$3,VALUE(LEFT(B33,LEN(B33)-1))),EDATE($B$3,12*VALUE(LEFT(B33,LEN(B33)-1))))),2)=7,2,0))),(IF(RIGHT(B33,1)="W",$B$3+7*VALUE(LEFT(B33,LEN(B33)-1)),IF(RIGHT(B33,1)="M",EDATE($B$3,VALUE(LEFT(B33,LEN(B33)-1))),EDATE($B$3,12*VALUE(LEFT(B33,LEN(B33)-1)))))+IF(WEEKDAY(IF(RIGHT(B33,1)="W",$B$3+7*VALUE(LEFT(B33,LEN(B33)-1)),IF(RIGHT(B33,1)="M",EDATE($B$3,VALUE(LEFT(B33,LEN(B33)-1))),EDATE($B$3,12*VALUE(LEFT(B33,LEN(B33)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B33,1)="W",$B$3+7*VALUE(LEFT(B33,LEN(B33)-1)),IF(RIGHT(B33,1)="M",EDATE($B$3,VALUE(LEFT(B33,LEN(B33)-1))),EDATE($B$3,12*VALUE(LEFT(B33,LEN(B33)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D33" s="24">
@@ -31557,7 +31562,7 @@
         </is>
       </c>
       <c r="C34" s="23">
-        <f>IF(RIGHT(B34,1)="W",$B$3+7*VALUE(LEFT(B34,LEN(B34)-1)),IF(RIGHT(B34,1)="M",EDATE($B$3,VALUE(LEFT(B34,LEN(B34)-1))),EDATE($B$3,12*VALUE(LEFT(B34,LEN(B34)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B34,1)="W",$B$3+7*VALUE(LEFT(B34,LEN(B34)-1)),IF(RIGHT(B34,1)="M",EDATE($B$3,VALUE(LEFT(B34,LEN(B34)-1))),EDATE($B$3,12*VALUE(LEFT(B34,LEN(B34)-1)))))+IF(WEEKDAY(IF(RIGHT(B34,1)="W",$B$3+7*VALUE(LEFT(B34,LEN(B34)-1)),IF(RIGHT(B34,1)="M",EDATE($B$3,VALUE(LEFT(B34,LEN(B34)-1))),EDATE($B$3,12*VALUE(LEFT(B34,LEN(B34)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B34,1)="W",$B$3+7*VALUE(LEFT(B34,LEN(B34)-1)),IF(RIGHT(B34,1)="M",EDATE($B$3,VALUE(LEFT(B34,LEN(B34)-1))),EDATE($B$3,12*VALUE(LEFT(B34,LEN(B34)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B34,1)="W",$B$3+7*VALUE(LEFT(B34,LEN(B34)-1)),IF(RIGHT(B34,1)="M",EDATE($B$3,VALUE(LEFT(B34,LEN(B34)-1))),EDATE($B$3,12*VALUE(LEFT(B34,LEN(B34)-1)))))),(IF(RIGHT(B34,1)="W",$B$3+7*VALUE(LEFT(B34,LEN(B34)-1)),IF(RIGHT(B34,1)="M",EDATE($B$3,VALUE(LEFT(B34,LEN(B34)-1))),EDATE($B$3,12*VALUE(LEFT(B34,LEN(B34)-1)))))-IF(WEEKDAY(IF(RIGHT(B34,1)="W",$B$3+7*VALUE(LEFT(B34,LEN(B34)-1)),IF(RIGHT(B34,1)="M",EDATE($B$3,VALUE(LEFT(B34,LEN(B34)-1))),EDATE($B$3,12*VALUE(LEFT(B34,LEN(B34)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B34,1)="W",$B$3+7*VALUE(LEFT(B34,LEN(B34)-1)),IF(RIGHT(B34,1)="M",EDATE($B$3,VALUE(LEFT(B34,LEN(B34)-1))),EDATE($B$3,12*VALUE(LEFT(B34,LEN(B34)-1))))),2)=7,2,0))),(IF(RIGHT(B34,1)="W",$B$3+7*VALUE(LEFT(B34,LEN(B34)-1)),IF(RIGHT(B34,1)="M",EDATE($B$3,VALUE(LEFT(B34,LEN(B34)-1))),EDATE($B$3,12*VALUE(LEFT(B34,LEN(B34)-1)))))+IF(WEEKDAY(IF(RIGHT(B34,1)="W",$B$3+7*VALUE(LEFT(B34,LEN(B34)-1)),IF(RIGHT(B34,1)="M",EDATE($B$3,VALUE(LEFT(B34,LEN(B34)-1))),EDATE($B$3,12*VALUE(LEFT(B34,LEN(B34)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B34,1)="W",$B$3+7*VALUE(LEFT(B34,LEN(B34)-1)),IF(RIGHT(B34,1)="M",EDATE($B$3,VALUE(LEFT(B34,LEN(B34)-1))),EDATE($B$3,12*VALUE(LEFT(B34,LEN(B34)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D34" s="24">
@@ -31607,7 +31612,7 @@
         </is>
       </c>
       <c r="C35" s="23">
-        <f>IF(RIGHT(B35,1)="W",$B$3+7*VALUE(LEFT(B35,LEN(B35)-1)),IF(RIGHT(B35,1)="M",EDATE($B$3,VALUE(LEFT(B35,LEN(B35)-1))),EDATE($B$3,12*VALUE(LEFT(B35,LEN(B35)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B35,1)="W",$B$3+7*VALUE(LEFT(B35,LEN(B35)-1)),IF(RIGHT(B35,1)="M",EDATE($B$3,VALUE(LEFT(B35,LEN(B35)-1))),EDATE($B$3,12*VALUE(LEFT(B35,LEN(B35)-1)))))+IF(WEEKDAY(IF(RIGHT(B35,1)="W",$B$3+7*VALUE(LEFT(B35,LEN(B35)-1)),IF(RIGHT(B35,1)="M",EDATE($B$3,VALUE(LEFT(B35,LEN(B35)-1))),EDATE($B$3,12*VALUE(LEFT(B35,LEN(B35)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B35,1)="W",$B$3+7*VALUE(LEFT(B35,LEN(B35)-1)),IF(RIGHT(B35,1)="M",EDATE($B$3,VALUE(LEFT(B35,LEN(B35)-1))),EDATE($B$3,12*VALUE(LEFT(B35,LEN(B35)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B35,1)="W",$B$3+7*VALUE(LEFT(B35,LEN(B35)-1)),IF(RIGHT(B35,1)="M",EDATE($B$3,VALUE(LEFT(B35,LEN(B35)-1))),EDATE($B$3,12*VALUE(LEFT(B35,LEN(B35)-1)))))),(IF(RIGHT(B35,1)="W",$B$3+7*VALUE(LEFT(B35,LEN(B35)-1)),IF(RIGHT(B35,1)="M",EDATE($B$3,VALUE(LEFT(B35,LEN(B35)-1))),EDATE($B$3,12*VALUE(LEFT(B35,LEN(B35)-1)))))-IF(WEEKDAY(IF(RIGHT(B35,1)="W",$B$3+7*VALUE(LEFT(B35,LEN(B35)-1)),IF(RIGHT(B35,1)="M",EDATE($B$3,VALUE(LEFT(B35,LEN(B35)-1))),EDATE($B$3,12*VALUE(LEFT(B35,LEN(B35)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B35,1)="W",$B$3+7*VALUE(LEFT(B35,LEN(B35)-1)),IF(RIGHT(B35,1)="M",EDATE($B$3,VALUE(LEFT(B35,LEN(B35)-1))),EDATE($B$3,12*VALUE(LEFT(B35,LEN(B35)-1))))),2)=7,2,0))),(IF(RIGHT(B35,1)="W",$B$3+7*VALUE(LEFT(B35,LEN(B35)-1)),IF(RIGHT(B35,1)="M",EDATE($B$3,VALUE(LEFT(B35,LEN(B35)-1))),EDATE($B$3,12*VALUE(LEFT(B35,LEN(B35)-1)))))+IF(WEEKDAY(IF(RIGHT(B35,1)="W",$B$3+7*VALUE(LEFT(B35,LEN(B35)-1)),IF(RIGHT(B35,1)="M",EDATE($B$3,VALUE(LEFT(B35,LEN(B35)-1))),EDATE($B$3,12*VALUE(LEFT(B35,LEN(B35)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B35,1)="W",$B$3+7*VALUE(LEFT(B35,LEN(B35)-1)),IF(RIGHT(B35,1)="M",EDATE($B$3,VALUE(LEFT(B35,LEN(B35)-1))),EDATE($B$3,12*VALUE(LEFT(B35,LEN(B35)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D35" s="24">
@@ -31657,7 +31662,7 @@
         </is>
       </c>
       <c r="C36" s="23">
-        <f>IF(RIGHT(B36,1)="W",$B$3+7*VALUE(LEFT(B36,LEN(B36)-1)),IF(RIGHT(B36,1)="M",EDATE($B$3,VALUE(LEFT(B36,LEN(B36)-1))),EDATE($B$3,12*VALUE(LEFT(B36,LEN(B36)-1)))))</f>
+        <f>IF(MONTH((IF(RIGHT(B36,1)="W",$B$3+7*VALUE(LEFT(B36,LEN(B36)-1)),IF(RIGHT(B36,1)="M",EDATE($B$3,VALUE(LEFT(B36,LEN(B36)-1))),EDATE($B$3,12*VALUE(LEFT(B36,LEN(B36)-1)))))+IF(WEEKDAY(IF(RIGHT(B36,1)="W",$B$3+7*VALUE(LEFT(B36,LEN(B36)-1)),IF(RIGHT(B36,1)="M",EDATE($B$3,VALUE(LEFT(B36,LEN(B36)-1))),EDATE($B$3,12*VALUE(LEFT(B36,LEN(B36)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B36,1)="W",$B$3+7*VALUE(LEFT(B36,LEN(B36)-1)),IF(RIGHT(B36,1)="M",EDATE($B$3,VALUE(LEFT(B36,LEN(B36)-1))),EDATE($B$3,12*VALUE(LEFT(B36,LEN(B36)-1))))),2)=7,1,0))))&lt;&gt;MONTH(IF(RIGHT(B36,1)="W",$B$3+7*VALUE(LEFT(B36,LEN(B36)-1)),IF(RIGHT(B36,1)="M",EDATE($B$3,VALUE(LEFT(B36,LEN(B36)-1))),EDATE($B$3,12*VALUE(LEFT(B36,LEN(B36)-1)))))),(IF(RIGHT(B36,1)="W",$B$3+7*VALUE(LEFT(B36,LEN(B36)-1)),IF(RIGHT(B36,1)="M",EDATE($B$3,VALUE(LEFT(B36,LEN(B36)-1))),EDATE($B$3,12*VALUE(LEFT(B36,LEN(B36)-1)))))-IF(WEEKDAY(IF(RIGHT(B36,1)="W",$B$3+7*VALUE(LEFT(B36,LEN(B36)-1)),IF(RIGHT(B36,1)="M",EDATE($B$3,VALUE(LEFT(B36,LEN(B36)-1))),EDATE($B$3,12*VALUE(LEFT(B36,LEN(B36)-1))))),2)=6,1,IF(WEEKDAY(IF(RIGHT(B36,1)="W",$B$3+7*VALUE(LEFT(B36,LEN(B36)-1)),IF(RIGHT(B36,1)="M",EDATE($B$3,VALUE(LEFT(B36,LEN(B36)-1))),EDATE($B$3,12*VALUE(LEFT(B36,LEN(B36)-1))))),2)=7,2,0))),(IF(RIGHT(B36,1)="W",$B$3+7*VALUE(LEFT(B36,LEN(B36)-1)),IF(RIGHT(B36,1)="M",EDATE($B$3,VALUE(LEFT(B36,LEN(B36)-1))),EDATE($B$3,12*VALUE(LEFT(B36,LEN(B36)-1)))))+IF(WEEKDAY(IF(RIGHT(B36,1)="W",$B$3+7*VALUE(LEFT(B36,LEN(B36)-1)),IF(RIGHT(B36,1)="M",EDATE($B$3,VALUE(LEFT(B36,LEN(B36)-1))),EDATE($B$3,12*VALUE(LEFT(B36,LEN(B36)-1))))),2)=6,2,IF(WEEKDAY(IF(RIGHT(B36,1)="W",$B$3+7*VALUE(LEFT(B36,LEN(B36)-1)),IF(RIGHT(B36,1)="M",EDATE($B$3,VALUE(LEFT(B36,LEN(B36)-1))),EDATE($B$3,12*VALUE(LEFT(B36,LEN(B36)-1))))),2)=7,1,0))))</f>
         <v/>
       </c>
       <c r="D36" s="24">
@@ -31695,6 +31700,7 @@
       </c>
       <c r="L36" s="94" t="inlineStr"/>
     </row>
+    <row r="37"/>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add a BDP-vs-export reconciliation block to SOFR_OIS_Quotes
Paste the Bloomberg curve export's Bid/Ask into N:O; Q/R/S show BDP minus export
in bp, with max and mean at P40/P41.

Settles whether a BDP-vs-screen difference is timing or systematic. Mixed signs
of a few tenths means the two were captured moments apart and the rates ticked.
A consistent shift across all 32 - a non-zero mean in P41 - means wrong pricing
source, field or ticker.

Only column S matters for the curve: H is (PX_BID+PX_ASK)/2 and is the sole
input the bootstrap reads. PX_LAST is a fallback and does not feed it.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -220,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -361,6 +361,11 @@
     <xf numFmtId="175" fontId="14" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="14" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="175" fontId="14" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -30043,7 +30048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:S41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30068,6 +30073,11 @@
           <t>REAL MARKET DATA - S490 USD SOFR, Step Forward (Cont), Settle 07/21/26, Curve Side Mid</t>
         </is>
       </c>
+      <c r="N1" s="66" t="inlineStr">
+        <is>
+          <t>RECONCILIATION vs the Bloomberg curve export</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -30080,6 +30090,11 @@
           <t>The screen's Market Rate column, which is already the mid. Used only when BDP fails; on a terminal BDP bid/ask takes precedence.</t>
         </is>
       </c>
+      <c r="N2" s="65" t="inlineStr">
+        <is>
+          <t>Paste the export's Bid/Ask into N:O. Q/R/S show BDP minus export in bp. Mixed signs of a few tenths = the two were captured at different moments and the rates ticked. A consistent shift across all 32 = wrong pricing source, field or ticker, and needs fixing. Only column S matters for the curve: H is (PX_BID+PX_ASK)/2 and is the sole input the bootstrap reads.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -30159,6 +30174,36 @@
           <t>Maturity dates are modified-following business-day adjusted, matching S490 and the Bootstrap sheet. Display only - the curve reads column H (mid) alone.</t>
         </is>
       </c>
+      <c r="N4" s="106" t="inlineStr">
+        <is>
+          <t>Export Bid (paste)</t>
+        </is>
+      </c>
+      <c r="O4" s="106" t="inlineStr">
+        <is>
+          <t>Export Ask (paste)</t>
+        </is>
+      </c>
+      <c r="P4" s="106" t="inlineStr">
+        <is>
+          <t>Export Mid</t>
+        </is>
+      </c>
+      <c r="Q4" s="106" t="inlineStr">
+        <is>
+          <t>d Bid (bp)</t>
+        </is>
+      </c>
+      <c r="R4" s="106" t="inlineStr">
+        <is>
+          <t>d Ask (bp)</t>
+        </is>
+      </c>
+      <c r="S4" s="106" t="inlineStr">
+        <is>
+          <t>d Mid (bp)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -30209,6 +30254,24 @@
         </is>
       </c>
       <c r="L5" s="94" t="inlineStr"/>
+      <c r="N5" s="85" t="n"/>
+      <c r="O5" s="85" t="n"/>
+      <c r="P5" s="107">
+        <f>IF(COUNT(N5:O5)=2,(N5+O5)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q5" s="108">
+        <f>IF(AND(ISNUMBER(N5),ISNUMBER(E5)),(E5-N5)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R5" s="108">
+        <f>IF(AND(ISNUMBER(O5),ISNUMBER(F5)),(F5-O5)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S5" s="108">
+        <f>IF(AND(ISNUMBER(P5),ISNUMBER(H5)),(H5-P5)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -30255,6 +30318,24 @@
         </is>
       </c>
       <c r="L6" s="94" t="inlineStr"/>
+      <c r="N6" s="85" t="n"/>
+      <c r="O6" s="85" t="n"/>
+      <c r="P6" s="107">
+        <f>IF(COUNT(N6:O6)=2,(N6+O6)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q6" s="108">
+        <f>IF(AND(ISNUMBER(N6),ISNUMBER(E6)),(E6-N6)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R6" s="108">
+        <f>IF(AND(ISNUMBER(O6),ISNUMBER(F6)),(F6-O6)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S6" s="108">
+        <f>IF(AND(ISNUMBER(P6),ISNUMBER(H6)),(H6-P6)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -30301,6 +30382,24 @@
         </is>
       </c>
       <c r="L7" s="94" t="inlineStr"/>
+      <c r="N7" s="85" t="n"/>
+      <c r="O7" s="85" t="n"/>
+      <c r="P7" s="107">
+        <f>IF(COUNT(N7:O7)=2,(N7+O7)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q7" s="108">
+        <f>IF(AND(ISNUMBER(N7),ISNUMBER(E7)),(E7-N7)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R7" s="108">
+        <f>IF(AND(ISNUMBER(O7),ISNUMBER(F7)),(F7-O7)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S7" s="108">
+        <f>IF(AND(ISNUMBER(P7),ISNUMBER(H7)),(H7-P7)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -30351,6 +30450,24 @@
         </is>
       </c>
       <c r="L8" s="94" t="inlineStr"/>
+      <c r="N8" s="85" t="n"/>
+      <c r="O8" s="85" t="n"/>
+      <c r="P8" s="107">
+        <f>IF(COUNT(N8:O8)=2,(N8+O8)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q8" s="108">
+        <f>IF(AND(ISNUMBER(N8),ISNUMBER(E8)),(E8-N8)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R8" s="108">
+        <f>IF(AND(ISNUMBER(O8),ISNUMBER(F8)),(F8-O8)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S8" s="108">
+        <f>IF(AND(ISNUMBER(P8),ISNUMBER(H8)),(H8-P8)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -30397,6 +30514,24 @@
         </is>
       </c>
       <c r="L9" s="94" t="inlineStr"/>
+      <c r="N9" s="85" t="n"/>
+      <c r="O9" s="85" t="n"/>
+      <c r="P9" s="107">
+        <f>IF(COUNT(N9:O9)=2,(N9+O9)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q9" s="108">
+        <f>IF(AND(ISNUMBER(N9),ISNUMBER(E9)),(E9-N9)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R9" s="108">
+        <f>IF(AND(ISNUMBER(O9),ISNUMBER(F9)),(F9-O9)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S9" s="108">
+        <f>IF(AND(ISNUMBER(P9),ISNUMBER(H9)),(H9-P9)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -30447,6 +30582,24 @@
         </is>
       </c>
       <c r="L10" s="94" t="inlineStr"/>
+      <c r="N10" s="85" t="n"/>
+      <c r="O10" s="85" t="n"/>
+      <c r="P10" s="107">
+        <f>IF(COUNT(N10:O10)=2,(N10+O10)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q10" s="108">
+        <f>IF(AND(ISNUMBER(N10),ISNUMBER(E10)),(E10-N10)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R10" s="108">
+        <f>IF(AND(ISNUMBER(O10),ISNUMBER(F10)),(F10-O10)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S10" s="108">
+        <f>IF(AND(ISNUMBER(P10),ISNUMBER(H10)),(H10-P10)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -30493,6 +30646,24 @@
         </is>
       </c>
       <c r="L11" s="94" t="inlineStr"/>
+      <c r="N11" s="85" t="n"/>
+      <c r="O11" s="85" t="n"/>
+      <c r="P11" s="107">
+        <f>IF(COUNT(N11:O11)=2,(N11+O11)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q11" s="108">
+        <f>IF(AND(ISNUMBER(N11),ISNUMBER(E11)),(E11-N11)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R11" s="108">
+        <f>IF(AND(ISNUMBER(O11),ISNUMBER(F11)),(F11-O11)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S11" s="108">
+        <f>IF(AND(ISNUMBER(P11),ISNUMBER(H11)),(H11-P11)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -30539,6 +30710,24 @@
         </is>
       </c>
       <c r="L12" s="94" t="inlineStr"/>
+      <c r="N12" s="85" t="n"/>
+      <c r="O12" s="85" t="n"/>
+      <c r="P12" s="107">
+        <f>IF(COUNT(N12:O12)=2,(N12+O12)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q12" s="108">
+        <f>IF(AND(ISNUMBER(N12),ISNUMBER(E12)),(E12-N12)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R12" s="108">
+        <f>IF(AND(ISNUMBER(O12),ISNUMBER(F12)),(F12-O12)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S12" s="108">
+        <f>IF(AND(ISNUMBER(P12),ISNUMBER(H12)),(H12-P12)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -30589,6 +30778,24 @@
         </is>
       </c>
       <c r="L13" s="94" t="inlineStr"/>
+      <c r="N13" s="85" t="n"/>
+      <c r="O13" s="85" t="n"/>
+      <c r="P13" s="107">
+        <f>IF(COUNT(N13:O13)=2,(N13+O13)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q13" s="108">
+        <f>IF(AND(ISNUMBER(N13),ISNUMBER(E13)),(E13-N13)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R13" s="108">
+        <f>IF(AND(ISNUMBER(O13),ISNUMBER(F13)),(F13-O13)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S13" s="108">
+        <f>IF(AND(ISNUMBER(P13),ISNUMBER(H13)),(H13-P13)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -30635,6 +30842,24 @@
         </is>
       </c>
       <c r="L14" s="94" t="inlineStr"/>
+      <c r="N14" s="85" t="n"/>
+      <c r="O14" s="85" t="n"/>
+      <c r="P14" s="107">
+        <f>IF(COUNT(N14:O14)=2,(N14+O14)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q14" s="108">
+        <f>IF(AND(ISNUMBER(N14),ISNUMBER(E14)),(E14-N14)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R14" s="108">
+        <f>IF(AND(ISNUMBER(O14),ISNUMBER(F14)),(F14-O14)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S14" s="108">
+        <f>IF(AND(ISNUMBER(P14),ISNUMBER(H14)),(H14-P14)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -30681,6 +30906,24 @@
         </is>
       </c>
       <c r="L15" s="94" t="inlineStr"/>
+      <c r="N15" s="85" t="n"/>
+      <c r="O15" s="85" t="n"/>
+      <c r="P15" s="107">
+        <f>IF(COUNT(N15:O15)=2,(N15+O15)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q15" s="108">
+        <f>IF(AND(ISNUMBER(N15),ISNUMBER(E15)),(E15-N15)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R15" s="108">
+        <f>IF(AND(ISNUMBER(O15),ISNUMBER(F15)),(F15-O15)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S15" s="108">
+        <f>IF(AND(ISNUMBER(P15),ISNUMBER(H15)),(H15-P15)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -30727,6 +30970,24 @@
         </is>
       </c>
       <c r="L16" s="94" t="inlineStr"/>
+      <c r="N16" s="85" t="n"/>
+      <c r="O16" s="85" t="n"/>
+      <c r="P16" s="107">
+        <f>IF(COUNT(N16:O16)=2,(N16+O16)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q16" s="108">
+        <f>IF(AND(ISNUMBER(N16),ISNUMBER(E16)),(E16-N16)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R16" s="108">
+        <f>IF(AND(ISNUMBER(O16),ISNUMBER(F16)),(F16-O16)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S16" s="108">
+        <f>IF(AND(ISNUMBER(P16),ISNUMBER(H16)),(H16-P16)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -30773,6 +31034,24 @@
         </is>
       </c>
       <c r="L17" s="94" t="inlineStr"/>
+      <c r="N17" s="85" t="n"/>
+      <c r="O17" s="85" t="n"/>
+      <c r="P17" s="107">
+        <f>IF(COUNT(N17:O17)=2,(N17+O17)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q17" s="108">
+        <f>IF(AND(ISNUMBER(N17),ISNUMBER(E17)),(E17-N17)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R17" s="108">
+        <f>IF(AND(ISNUMBER(O17),ISNUMBER(F17)),(F17-O17)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S17" s="108">
+        <f>IF(AND(ISNUMBER(P17),ISNUMBER(H17)),(H17-P17)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -30819,6 +31098,24 @@
         </is>
       </c>
       <c r="L18" s="94" t="inlineStr"/>
+      <c r="N18" s="85" t="n"/>
+      <c r="O18" s="85" t="n"/>
+      <c r="P18" s="107">
+        <f>IF(COUNT(N18:O18)=2,(N18+O18)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q18" s="108">
+        <f>IF(AND(ISNUMBER(N18),ISNUMBER(E18)),(E18-N18)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R18" s="108">
+        <f>IF(AND(ISNUMBER(O18),ISNUMBER(F18)),(F18-O18)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S18" s="108">
+        <f>IF(AND(ISNUMBER(P18),ISNUMBER(H18)),(H18-P18)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -30865,6 +31162,24 @@
         </is>
       </c>
       <c r="L19" s="94" t="inlineStr"/>
+      <c r="N19" s="85" t="n"/>
+      <c r="O19" s="85" t="n"/>
+      <c r="P19" s="107">
+        <f>IF(COUNT(N19:O19)=2,(N19+O19)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q19" s="108">
+        <f>IF(AND(ISNUMBER(N19),ISNUMBER(E19)),(E19-N19)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R19" s="108">
+        <f>IF(AND(ISNUMBER(O19),ISNUMBER(F19)),(F19-O19)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S19" s="108">
+        <f>IF(AND(ISNUMBER(P19),ISNUMBER(H19)),(H19-P19)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -30911,6 +31226,24 @@
         </is>
       </c>
       <c r="L20" s="94" t="inlineStr"/>
+      <c r="N20" s="85" t="n"/>
+      <c r="O20" s="85" t="n"/>
+      <c r="P20" s="107">
+        <f>IF(COUNT(N20:O20)=2,(N20+O20)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q20" s="108">
+        <f>IF(AND(ISNUMBER(N20),ISNUMBER(E20)),(E20-N20)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R20" s="108">
+        <f>IF(AND(ISNUMBER(O20),ISNUMBER(F20)),(F20-O20)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S20" s="108">
+        <f>IF(AND(ISNUMBER(P20),ISNUMBER(H20)),(H20-P20)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -30957,6 +31290,24 @@
         </is>
       </c>
       <c r="L21" s="94" t="inlineStr"/>
+      <c r="N21" s="85" t="n"/>
+      <c r="O21" s="85" t="n"/>
+      <c r="P21" s="107">
+        <f>IF(COUNT(N21:O21)=2,(N21+O21)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q21" s="108">
+        <f>IF(AND(ISNUMBER(N21),ISNUMBER(E21)),(E21-N21)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R21" s="108">
+        <f>IF(AND(ISNUMBER(O21),ISNUMBER(F21)),(F21-O21)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S21" s="108">
+        <f>IF(AND(ISNUMBER(P21),ISNUMBER(H21)),(H21-P21)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -31003,6 +31354,24 @@
         </is>
       </c>
       <c r="L22" s="94" t="inlineStr"/>
+      <c r="N22" s="85" t="n"/>
+      <c r="O22" s="85" t="n"/>
+      <c r="P22" s="107">
+        <f>IF(COUNT(N22:O22)=2,(N22+O22)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q22" s="108">
+        <f>IF(AND(ISNUMBER(N22),ISNUMBER(E22)),(E22-N22)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R22" s="108">
+        <f>IF(AND(ISNUMBER(O22),ISNUMBER(F22)),(F22-O22)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S22" s="108">
+        <f>IF(AND(ISNUMBER(P22),ISNUMBER(H22)),(H22-P22)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -31049,6 +31418,24 @@
         </is>
       </c>
       <c r="L23" s="94" t="inlineStr"/>
+      <c r="N23" s="85" t="n"/>
+      <c r="O23" s="85" t="n"/>
+      <c r="P23" s="107">
+        <f>IF(COUNT(N23:O23)=2,(N23+O23)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q23" s="108">
+        <f>IF(AND(ISNUMBER(N23),ISNUMBER(E23)),(E23-N23)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R23" s="108">
+        <f>IF(AND(ISNUMBER(O23),ISNUMBER(F23)),(F23-O23)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S23" s="108">
+        <f>IF(AND(ISNUMBER(P23),ISNUMBER(H23)),(H23-P23)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -31099,6 +31486,24 @@
         </is>
       </c>
       <c r="L24" s="94" t="inlineStr"/>
+      <c r="N24" s="85" t="n"/>
+      <c r="O24" s="85" t="n"/>
+      <c r="P24" s="107">
+        <f>IF(COUNT(N24:O24)=2,(N24+O24)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q24" s="108">
+        <f>IF(AND(ISNUMBER(N24),ISNUMBER(E24)),(E24-N24)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R24" s="108">
+        <f>IF(AND(ISNUMBER(O24),ISNUMBER(F24)),(F24-O24)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S24" s="108">
+        <f>IF(AND(ISNUMBER(P24),ISNUMBER(H24)),(H24-P24)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -31149,6 +31554,24 @@
         </is>
       </c>
       <c r="L25" s="94" t="inlineStr"/>
+      <c r="N25" s="85" t="n"/>
+      <c r="O25" s="85" t="n"/>
+      <c r="P25" s="107">
+        <f>IF(COUNT(N25:O25)=2,(N25+O25)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q25" s="108">
+        <f>IF(AND(ISNUMBER(N25),ISNUMBER(E25)),(E25-N25)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R25" s="108">
+        <f>IF(AND(ISNUMBER(O25),ISNUMBER(F25)),(F25-O25)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S25" s="108">
+        <f>IF(AND(ISNUMBER(P25),ISNUMBER(H25)),(H25-P25)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -31199,6 +31622,24 @@
         </is>
       </c>
       <c r="L26" s="94" t="inlineStr"/>
+      <c r="N26" s="85" t="n"/>
+      <c r="O26" s="85" t="n"/>
+      <c r="P26" s="107">
+        <f>IF(COUNT(N26:O26)=2,(N26+O26)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q26" s="108">
+        <f>IF(AND(ISNUMBER(N26),ISNUMBER(E26)),(E26-N26)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R26" s="108">
+        <f>IF(AND(ISNUMBER(O26),ISNUMBER(F26)),(F26-O26)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S26" s="108">
+        <f>IF(AND(ISNUMBER(P26),ISNUMBER(H26)),(H26-P26)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -31249,6 +31690,24 @@
         </is>
       </c>
       <c r="L27" s="94" t="inlineStr"/>
+      <c r="N27" s="85" t="n"/>
+      <c r="O27" s="85" t="n"/>
+      <c r="P27" s="107">
+        <f>IF(COUNT(N27:O27)=2,(N27+O27)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q27" s="108">
+        <f>IF(AND(ISNUMBER(N27),ISNUMBER(E27)),(E27-N27)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R27" s="108">
+        <f>IF(AND(ISNUMBER(O27),ISNUMBER(F27)),(F27-O27)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S27" s="108">
+        <f>IF(AND(ISNUMBER(P27),ISNUMBER(H27)),(H27-P27)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -31299,6 +31758,24 @@
         </is>
       </c>
       <c r="L28" s="94" t="inlineStr"/>
+      <c r="N28" s="85" t="n"/>
+      <c r="O28" s="85" t="n"/>
+      <c r="P28" s="107">
+        <f>IF(COUNT(N28:O28)=2,(N28+O28)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q28" s="108">
+        <f>IF(AND(ISNUMBER(N28),ISNUMBER(E28)),(E28-N28)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R28" s="108">
+        <f>IF(AND(ISNUMBER(O28),ISNUMBER(F28)),(F28-O28)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S28" s="108">
+        <f>IF(AND(ISNUMBER(P28),ISNUMBER(H28)),(H28-P28)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -31349,6 +31826,24 @@
         </is>
       </c>
       <c r="L29" s="94" t="inlineStr"/>
+      <c r="N29" s="85" t="n"/>
+      <c r="O29" s="85" t="n"/>
+      <c r="P29" s="107">
+        <f>IF(COUNT(N29:O29)=2,(N29+O29)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q29" s="108">
+        <f>IF(AND(ISNUMBER(N29),ISNUMBER(E29)),(E29-N29)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R29" s="108">
+        <f>IF(AND(ISNUMBER(O29),ISNUMBER(F29)),(F29-O29)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S29" s="108">
+        <f>IF(AND(ISNUMBER(P29),ISNUMBER(H29)),(H29-P29)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -31399,6 +31894,24 @@
         </is>
       </c>
       <c r="L30" s="94" t="inlineStr"/>
+      <c r="N30" s="85" t="n"/>
+      <c r="O30" s="85" t="n"/>
+      <c r="P30" s="107">
+        <f>IF(COUNT(N30:O30)=2,(N30+O30)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q30" s="108">
+        <f>IF(AND(ISNUMBER(N30),ISNUMBER(E30)),(E30-N30)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R30" s="108">
+        <f>IF(AND(ISNUMBER(O30),ISNUMBER(F30)),(F30-O30)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S30" s="108">
+        <f>IF(AND(ISNUMBER(P30),ISNUMBER(H30)),(H30-P30)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -31449,6 +31962,24 @@
         </is>
       </c>
       <c r="L31" s="94" t="inlineStr"/>
+      <c r="N31" s="85" t="n"/>
+      <c r="O31" s="85" t="n"/>
+      <c r="P31" s="107">
+        <f>IF(COUNT(N31:O31)=2,(N31+O31)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q31" s="108">
+        <f>IF(AND(ISNUMBER(N31),ISNUMBER(E31)),(E31-N31)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R31" s="108">
+        <f>IF(AND(ISNUMBER(O31),ISNUMBER(F31)),(F31-O31)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S31" s="108">
+        <f>IF(AND(ISNUMBER(P31),ISNUMBER(H31)),(H31-P31)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -31499,6 +32030,24 @@
         </is>
       </c>
       <c r="L32" s="94" t="inlineStr"/>
+      <c r="N32" s="85" t="n"/>
+      <c r="O32" s="85" t="n"/>
+      <c r="P32" s="107">
+        <f>IF(COUNT(N32:O32)=2,(N32+O32)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q32" s="108">
+        <f>IF(AND(ISNUMBER(N32),ISNUMBER(E32)),(E32-N32)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R32" s="108">
+        <f>IF(AND(ISNUMBER(O32),ISNUMBER(F32)),(F32-O32)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S32" s="108">
+        <f>IF(AND(ISNUMBER(P32),ISNUMBER(H32)),(H32-P32)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -31549,6 +32098,24 @@
         </is>
       </c>
       <c r="L33" s="94" t="inlineStr"/>
+      <c r="N33" s="85" t="n"/>
+      <c r="O33" s="85" t="n"/>
+      <c r="P33" s="107">
+        <f>IF(COUNT(N33:O33)=2,(N33+O33)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q33" s="108">
+        <f>IF(AND(ISNUMBER(N33),ISNUMBER(E33)),(E33-N33)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R33" s="108">
+        <f>IF(AND(ISNUMBER(O33),ISNUMBER(F33)),(F33-O33)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S33" s="108">
+        <f>IF(AND(ISNUMBER(P33),ISNUMBER(H33)),(H33-P33)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -31599,6 +32166,24 @@
         </is>
       </c>
       <c r="L34" s="94" t="inlineStr"/>
+      <c r="N34" s="85" t="n"/>
+      <c r="O34" s="85" t="n"/>
+      <c r="P34" s="107">
+        <f>IF(COUNT(N34:O34)=2,(N34+O34)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q34" s="108">
+        <f>IF(AND(ISNUMBER(N34),ISNUMBER(E34)),(E34-N34)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R34" s="108">
+        <f>IF(AND(ISNUMBER(O34),ISNUMBER(F34)),(F34-O34)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S34" s="108">
+        <f>IF(AND(ISNUMBER(P34),ISNUMBER(H34)),(H34-P34)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -31649,6 +32234,24 @@
         </is>
       </c>
       <c r="L35" s="94" t="inlineStr"/>
+      <c r="N35" s="85" t="n"/>
+      <c r="O35" s="85" t="n"/>
+      <c r="P35" s="107">
+        <f>IF(COUNT(N35:O35)=2,(N35+O35)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q35" s="108">
+        <f>IF(AND(ISNUMBER(N35),ISNUMBER(E35)),(E35-N35)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R35" s="108">
+        <f>IF(AND(ISNUMBER(O35),ISNUMBER(F35)),(F35-O35)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S35" s="108">
+        <f>IF(AND(ISNUMBER(P35),ISNUMBER(H35)),(H35-P35)*100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -31699,8 +32302,25 @@
         </is>
       </c>
       <c r="L36" s="94" t="inlineStr"/>
-    </row>
-    <row r="37"/>
+      <c r="N36" s="85" t="n"/>
+      <c r="O36" s="85" t="n"/>
+      <c r="P36" s="107">
+        <f>IF(COUNT(N36:O36)=2,(N36+O36)/2,"")</f>
+        <v/>
+      </c>
+      <c r="Q36" s="108">
+        <f>IF(AND(ISNUMBER(N36),ISNUMBER(E36)),(E36-N36)*100,"")</f>
+        <v/>
+      </c>
+      <c r="R36" s="108">
+        <f>IF(AND(ISNUMBER(O36),ISNUMBER(F36)),(F36-O36)*100,"")</f>
+        <v/>
+      </c>
+      <c r="S36" s="108">
+        <f>IF(AND(ISNUMBER(P36),ISNUMBER(H36)),(H36-P36)*100,"")</f>
+        <v/>
+      </c>
+    </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
@@ -31709,6 +32329,28 @@
       </c>
     </row>
     <row r="39"/>
+    <row r="40">
+      <c r="N40" s="67" t="inlineStr">
+        <is>
+          <t>Max |d Mid| (bp)</t>
+        </is>
+      </c>
+      <c r="P40" s="109">
+        <f>IF(COUNT(S5:S36)=0,"paste the export first",MAX(MAX(S5:S36),-MIN(S5:S36)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="N41" s="67" t="inlineStr">
+        <is>
+          <t>Mean d Mid (bp) - a non-zero mean is the tell for a systematic offset</t>
+        </is>
+      </c>
+      <c r="P41" s="110">
+        <f>IF(COUNT(S5:S36)=0,"",AVERAGE(S5:S36))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A38:I39"/>

</xml_diff>

<commit_message>
Stop the dead SOFR_Futures sheet firing 301 Bloomberg requests
SOFR_Futures held 301 of the workbook's 434 BDP/BDS calls - about 70% - and
nothing reads it. Its only consumer was Bootstrap_Lehman, deleted when we went
to a single bootstrap. Every request hit the terminal, could fail, and rendered
as an error while feeding nothing.

Master switch at SOFR_Futures!B3, default No, gates every pull on the sheet.
Formulas preserved verbatim inside the IF, so flipping to Yes restores it.

Curve is unaffected - Bootstrap reads SOFR_OIS_Quotes!H only. Off-terminal error
count drops 4 -> 2; the remaining two are on Bloomberg_S490_Validation and are
live-only (a BDP NAME lookup and the BDS curve dump, which cannot be IFERROR'd
because it spills).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -42,7 +42,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.00000000"/>
@@ -55,7 +55,6 @@
     <numFmt numFmtId="173" formatCode="mm/dd/yy"/>
     <numFmt numFmtId="174" formatCode="0.###"/>
     <numFmt numFmtId="175" formatCode="$#,##0;($#,##0);-"/>
-    <numFmt numFmtId="176" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -34434,7 +34433,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
@@ -34511,6 +34509,23 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="67" t="inlineStr">
+        <is>
+          <t>Enable Bloomberg pulls on this sheet</t>
+        </is>
+      </c>
+      <c r="B3" s="68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C3" s="65" t="inlineStr">
+        <is>
+          <t>This sheet holds 301 of the workbook's 434 Bloomberg requests and NOTHING reads it - its only consumer was the deleted Bootstrap_Lehman. Left on, it hammers the terminal and fills the sheet with errors for no benefit. Set to Yes to re-enable; the formulas are preserved unchanged.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -34584,23 +34599,23 @@
     </row>
     <row r="7">
       <c r="A7" s="6">
-        <f>BDS("SFRA Comdty","FUT_CHAIN")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",BDS("SFRA Comdty","FUT_CHAIN"))</f>
         <v/>
       </c>
       <c r="B7" s="6">
-        <f>IFERROR(BDP($A7,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A7,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C7" s="17">
-        <f>IFERROR(BDP($A7,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A7,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D7" s="17">
-        <f>IFERROR(BDP($A7,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A7,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E7" s="17">
-        <f>IFERROR(BDP($A7,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A7,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F7" s="17">
@@ -34608,42 +34623,42 @@
         <v/>
       </c>
       <c r="G7" s="6">
-        <f>IFERROR(BDP($A7,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A7,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H7" s="18">
-        <f>IFERROR(BDP($A7,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A7,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I7" s="18">
-        <f>IFERROR(BDP($A7,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A7,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J7" s="21">
-        <f>IFERROR(BDP($A7,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A7,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K7" s="21">
-        <f>IFERROR(BDP($A7,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A7,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n"/>
       <c r="B8" s="6">
-        <f>IFERROR(BDP($A8,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A8,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C8" s="17">
-        <f>IFERROR(BDP($A8,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A8,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D8" s="17">
-        <f>IFERROR(BDP($A8,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A8,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E8" s="17">
-        <f>IFERROR(BDP($A8,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A8,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F8" s="17">
@@ -34651,42 +34666,42 @@
         <v/>
       </c>
       <c r="G8" s="6">
-        <f>IFERROR(BDP($A8,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A8,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H8" s="18">
-        <f>IFERROR(BDP($A8,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A8,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I8" s="18">
-        <f>IFERROR(BDP($A8,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A8,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J8" s="21">
-        <f>IFERROR(BDP($A8,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A8,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K8" s="21">
-        <f>IFERROR(BDP($A8,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A8,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
       <c r="B9" s="6">
-        <f>IFERROR(BDP($A9,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A9,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C9" s="17">
-        <f>IFERROR(BDP($A9,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A9,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D9" s="17">
-        <f>IFERROR(BDP($A9,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A9,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E9" s="17">
-        <f>IFERROR(BDP($A9,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A9,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F9" s="17">
@@ -34694,42 +34709,42 @@
         <v/>
       </c>
       <c r="G9" s="6">
-        <f>IFERROR(BDP($A9,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A9,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H9" s="18">
-        <f>IFERROR(BDP($A9,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A9,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I9" s="18">
-        <f>IFERROR(BDP($A9,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A9,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J9" s="21">
-        <f>IFERROR(BDP($A9,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A9,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K9" s="21">
-        <f>IFERROR(BDP($A9,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A9,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
       <c r="B10" s="6">
-        <f>IFERROR(BDP($A10,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A10,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C10" s="17">
-        <f>IFERROR(BDP($A10,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A10,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D10" s="17">
-        <f>IFERROR(BDP($A10,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A10,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E10" s="17">
-        <f>IFERROR(BDP($A10,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A10,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F10" s="17">
@@ -34737,42 +34752,42 @@
         <v/>
       </c>
       <c r="G10" s="6">
-        <f>IFERROR(BDP($A10,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A10,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H10" s="18">
-        <f>IFERROR(BDP($A10,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A10,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I10" s="18">
-        <f>IFERROR(BDP($A10,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A10,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J10" s="21">
-        <f>IFERROR(BDP($A10,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A10,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K10" s="21">
-        <f>IFERROR(BDP($A10,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A10,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
       <c r="B11" s="6">
-        <f>IFERROR(BDP($A11,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A11,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C11" s="17">
-        <f>IFERROR(BDP($A11,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A11,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D11" s="17">
-        <f>IFERROR(BDP($A11,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A11,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E11" s="17">
-        <f>IFERROR(BDP($A11,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A11,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F11" s="17">
@@ -34780,42 +34795,42 @@
         <v/>
       </c>
       <c r="G11" s="6">
-        <f>IFERROR(BDP($A11,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A11,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H11" s="18">
-        <f>IFERROR(BDP($A11,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A11,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I11" s="18">
-        <f>IFERROR(BDP($A11,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A11,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J11" s="21">
-        <f>IFERROR(BDP($A11,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A11,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K11" s="21">
-        <f>IFERROR(BDP($A11,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A11,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n"/>
       <c r="B12" s="6">
-        <f>IFERROR(BDP($A12,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A12,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C12" s="17">
-        <f>IFERROR(BDP($A12,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A12,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D12" s="17">
-        <f>IFERROR(BDP($A12,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A12,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E12" s="17">
-        <f>IFERROR(BDP($A12,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A12,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F12" s="17">
@@ -34823,42 +34838,42 @@
         <v/>
       </c>
       <c r="G12" s="6">
-        <f>IFERROR(BDP($A12,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A12,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H12" s="18">
-        <f>IFERROR(BDP($A12,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A12,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I12" s="18">
-        <f>IFERROR(BDP($A12,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A12,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J12" s="21">
-        <f>IFERROR(BDP($A12,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A12,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K12" s="21">
-        <f>IFERROR(BDP($A12,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A12,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
       <c r="B13" s="6">
-        <f>IFERROR(BDP($A13,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A13,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C13" s="17">
-        <f>IFERROR(BDP($A13,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A13,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D13" s="17">
-        <f>IFERROR(BDP($A13,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A13,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E13" s="17">
-        <f>IFERROR(BDP($A13,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A13,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F13" s="17">
@@ -34866,42 +34881,42 @@
         <v/>
       </c>
       <c r="G13" s="6">
-        <f>IFERROR(BDP($A13,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A13,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H13" s="18">
-        <f>IFERROR(BDP($A13,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A13,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I13" s="18">
-        <f>IFERROR(BDP($A13,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A13,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J13" s="21">
-        <f>IFERROR(BDP($A13,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A13,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K13" s="21">
-        <f>IFERROR(BDP($A13,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A13,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
       <c r="B14" s="6">
-        <f>IFERROR(BDP($A14,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A14,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C14" s="17">
-        <f>IFERROR(BDP($A14,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A14,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D14" s="17">
-        <f>IFERROR(BDP($A14,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A14,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E14" s="17">
-        <f>IFERROR(BDP($A14,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A14,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F14" s="17">
@@ -34909,42 +34924,42 @@
         <v/>
       </c>
       <c r="G14" s="6">
-        <f>IFERROR(BDP($A14,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A14,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H14" s="18">
-        <f>IFERROR(BDP($A14,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A14,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I14" s="18">
-        <f>IFERROR(BDP($A14,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A14,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J14" s="21">
-        <f>IFERROR(BDP($A14,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A14,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K14" s="21">
-        <f>IFERROR(BDP($A14,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A14,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
       <c r="B15" s="6">
-        <f>IFERROR(BDP($A15,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A15,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C15" s="17">
-        <f>IFERROR(BDP($A15,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A15,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D15" s="17">
-        <f>IFERROR(BDP($A15,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A15,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E15" s="17">
-        <f>IFERROR(BDP($A15,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A15,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F15" s="17">
@@ -34952,42 +34967,42 @@
         <v/>
       </c>
       <c r="G15" s="6">
-        <f>IFERROR(BDP($A15,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A15,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H15" s="18">
-        <f>IFERROR(BDP($A15,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A15,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I15" s="18">
-        <f>IFERROR(BDP($A15,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A15,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J15" s="21">
-        <f>IFERROR(BDP($A15,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A15,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K15" s="21">
-        <f>IFERROR(BDP($A15,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A15,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
       <c r="B16" s="6">
-        <f>IFERROR(BDP($A16,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A16,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C16" s="17">
-        <f>IFERROR(BDP($A16,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A16,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D16" s="17">
-        <f>IFERROR(BDP($A16,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A16,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E16" s="17">
-        <f>IFERROR(BDP($A16,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A16,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F16" s="17">
@@ -34995,42 +35010,42 @@
         <v/>
       </c>
       <c r="G16" s="6">
-        <f>IFERROR(BDP($A16,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A16,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H16" s="18">
-        <f>IFERROR(BDP($A16,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A16,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I16" s="18">
-        <f>IFERROR(BDP($A16,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A16,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J16" s="21">
-        <f>IFERROR(BDP($A16,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A16,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K16" s="21">
-        <f>IFERROR(BDP($A16,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A16,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
       <c r="B17" s="6">
-        <f>IFERROR(BDP($A17,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A17,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C17" s="17">
-        <f>IFERROR(BDP($A17,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A17,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D17" s="17">
-        <f>IFERROR(BDP($A17,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A17,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E17" s="17">
-        <f>IFERROR(BDP($A17,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A17,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F17" s="17">
@@ -35038,42 +35053,42 @@
         <v/>
       </c>
       <c r="G17" s="6">
-        <f>IFERROR(BDP($A17,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A17,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H17" s="18">
-        <f>IFERROR(BDP($A17,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A17,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I17" s="18">
-        <f>IFERROR(BDP($A17,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A17,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J17" s="21">
-        <f>IFERROR(BDP($A17,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A17,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K17" s="21">
-        <f>IFERROR(BDP($A17,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A17,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
       <c r="B18" s="6">
-        <f>IFERROR(BDP($A18,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A18,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C18" s="17">
-        <f>IFERROR(BDP($A18,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A18,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D18" s="17">
-        <f>IFERROR(BDP($A18,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A18,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E18" s="17">
-        <f>IFERROR(BDP($A18,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A18,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F18" s="17">
@@ -35081,42 +35096,42 @@
         <v/>
       </c>
       <c r="G18" s="6">
-        <f>IFERROR(BDP($A18,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A18,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H18" s="18">
-        <f>IFERROR(BDP($A18,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A18,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I18" s="18">
-        <f>IFERROR(BDP($A18,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A18,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J18" s="21">
-        <f>IFERROR(BDP($A18,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A18,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K18" s="21">
-        <f>IFERROR(BDP($A18,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A18,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="6">
-        <f>IFERROR(BDP($A19,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A19,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C19" s="17">
-        <f>IFERROR(BDP($A19,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A19,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D19" s="17">
-        <f>IFERROR(BDP($A19,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A19,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E19" s="17">
-        <f>IFERROR(BDP($A19,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A19,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F19" s="17">
@@ -35124,42 +35139,42 @@
         <v/>
       </c>
       <c r="G19" s="6">
-        <f>IFERROR(BDP($A19,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A19,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H19" s="18">
-        <f>IFERROR(BDP($A19,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A19,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I19" s="18">
-        <f>IFERROR(BDP($A19,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A19,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J19" s="21">
-        <f>IFERROR(BDP($A19,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A19,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K19" s="21">
-        <f>IFERROR(BDP($A19,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A19,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n"/>
       <c r="B20" s="6">
-        <f>IFERROR(BDP($A20,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A20,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C20" s="17">
-        <f>IFERROR(BDP($A20,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A20,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D20" s="17">
-        <f>IFERROR(BDP($A20,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A20,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E20" s="17">
-        <f>IFERROR(BDP($A20,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A20,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F20" s="17">
@@ -35167,42 +35182,42 @@
         <v/>
       </c>
       <c r="G20" s="6">
-        <f>IFERROR(BDP($A20,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A20,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H20" s="18">
-        <f>IFERROR(BDP($A20,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A20,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I20" s="18">
-        <f>IFERROR(BDP($A20,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A20,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J20" s="21">
-        <f>IFERROR(BDP($A20,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A20,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K20" s="21">
-        <f>IFERROR(BDP($A20,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A20,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n"/>
       <c r="B21" s="6">
-        <f>IFERROR(BDP($A21,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A21,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C21" s="17">
-        <f>IFERROR(BDP($A21,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A21,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D21" s="17">
-        <f>IFERROR(BDP($A21,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A21,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E21" s="17">
-        <f>IFERROR(BDP($A21,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A21,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F21" s="17">
@@ -35210,42 +35225,42 @@
         <v/>
       </c>
       <c r="G21" s="6">
-        <f>IFERROR(BDP($A21,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A21,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H21" s="18">
-        <f>IFERROR(BDP($A21,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A21,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I21" s="18">
-        <f>IFERROR(BDP($A21,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A21,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J21" s="21">
-        <f>IFERROR(BDP($A21,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A21,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K21" s="21">
-        <f>IFERROR(BDP($A21,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A21,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n"/>
       <c r="B22" s="6">
-        <f>IFERROR(BDP($A22,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A22,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C22" s="17">
-        <f>IFERROR(BDP($A22,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A22,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D22" s="17">
-        <f>IFERROR(BDP($A22,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A22,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E22" s="17">
-        <f>IFERROR(BDP($A22,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A22,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F22" s="17">
@@ -35253,42 +35268,42 @@
         <v/>
       </c>
       <c r="G22" s="6">
-        <f>IFERROR(BDP($A22,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A22,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H22" s="18">
-        <f>IFERROR(BDP($A22,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A22,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I22" s="18">
-        <f>IFERROR(BDP($A22,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A22,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J22" s="21">
-        <f>IFERROR(BDP($A22,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A22,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K22" s="21">
-        <f>IFERROR(BDP($A22,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A22,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="6">
-        <f>IFERROR(BDP($A23,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A23,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C23" s="17">
-        <f>IFERROR(BDP($A23,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A23,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D23" s="17">
-        <f>IFERROR(BDP($A23,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A23,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E23" s="17">
-        <f>IFERROR(BDP($A23,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A23,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F23" s="17">
@@ -35296,42 +35311,42 @@
         <v/>
       </c>
       <c r="G23" s="6">
-        <f>IFERROR(BDP($A23,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A23,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H23" s="18">
-        <f>IFERROR(BDP($A23,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A23,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I23" s="18">
-        <f>IFERROR(BDP($A23,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A23,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J23" s="21">
-        <f>IFERROR(BDP($A23,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A23,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K23" s="21">
-        <f>IFERROR(BDP($A23,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A23,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n"/>
       <c r="B24" s="6">
-        <f>IFERROR(BDP($A24,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A24,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C24" s="17">
-        <f>IFERROR(BDP($A24,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A24,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D24" s="17">
-        <f>IFERROR(BDP($A24,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A24,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E24" s="17">
-        <f>IFERROR(BDP($A24,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A24,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F24" s="17">
@@ -35339,42 +35354,42 @@
         <v/>
       </c>
       <c r="G24" s="6">
-        <f>IFERROR(BDP($A24,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A24,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H24" s="18">
-        <f>IFERROR(BDP($A24,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A24,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I24" s="18">
-        <f>IFERROR(BDP($A24,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A24,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J24" s="21">
-        <f>IFERROR(BDP($A24,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A24,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K24" s="21">
-        <f>IFERROR(BDP($A24,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A24,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="6">
-        <f>IFERROR(BDP($A25,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A25,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C25" s="17">
-        <f>IFERROR(BDP($A25,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A25,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D25" s="17">
-        <f>IFERROR(BDP($A25,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A25,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E25" s="17">
-        <f>IFERROR(BDP($A25,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A25,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F25" s="17">
@@ -35382,42 +35397,42 @@
         <v/>
       </c>
       <c r="G25" s="6">
-        <f>IFERROR(BDP($A25,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A25,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H25" s="18">
-        <f>IFERROR(BDP($A25,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A25,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I25" s="18">
-        <f>IFERROR(BDP($A25,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A25,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J25" s="21">
-        <f>IFERROR(BDP($A25,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A25,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K25" s="21">
-        <f>IFERROR(BDP($A25,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A25,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="6">
-        <f>IFERROR(BDP($A26,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A26,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C26" s="17">
-        <f>IFERROR(BDP($A26,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A26,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D26" s="17">
-        <f>IFERROR(BDP($A26,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A26,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E26" s="17">
-        <f>IFERROR(BDP($A26,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A26,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F26" s="17">
@@ -35425,26 +35440,28 @@
         <v/>
       </c>
       <c r="G26" s="6">
-        <f>IFERROR(BDP($A26,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A26,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H26" s="18">
-        <f>IFERROR(BDP($A26,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A26,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I26" s="18">
-        <f>IFERROR(BDP($A26,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A26,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J26" s="21">
-        <f>IFERROR(BDP($A26,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A26,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K26" s="21">
-        <f>IFERROR(BDP($A26,"OPEN_INT"),"ERROR PLZ FIX")</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A26,"OPEN_INT"),"ERROR PLZ FIX"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
@@ -35518,23 +35535,23 @@
     </row>
     <row r="32">
       <c r="A32" s="6">
-        <f>BDS("SERA Comdty","FUT_CHAIN")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",BDS("SERA Comdty","FUT_CHAIN"))</f>
         <v/>
       </c>
       <c r="B32" s="6">
-        <f>IFERROR(BDP($A32,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A32,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C32" s="17">
-        <f>IFERROR(BDP($A32,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A32,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D32" s="17">
-        <f>IFERROR(BDP($A32,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A32,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E32" s="17">
-        <f>IFERROR(BDP($A32,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A32,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F32" s="17">
@@ -35542,42 +35559,42 @@
         <v/>
       </c>
       <c r="G32" s="6">
-        <f>IFERROR(BDP($A32,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A32,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H32" s="18">
-        <f>IFERROR(BDP($A32,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A32,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I32" s="18">
-        <f>IFERROR(BDP($A32,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A32,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J32" s="21">
-        <f>IFERROR(BDP($A32,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A32,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K32" s="21">
-        <f>IFERROR(BDP($A32,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A32,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="6">
-        <f>IFERROR(BDP($A33,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A33,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C33" s="17">
-        <f>IFERROR(BDP($A33,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A33,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D33" s="17">
-        <f>IFERROR(BDP($A33,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A33,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E33" s="17">
-        <f>IFERROR(BDP($A33,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A33,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F33" s="17">
@@ -35585,42 +35602,42 @@
         <v/>
       </c>
       <c r="G33" s="6">
-        <f>IFERROR(BDP($A33,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A33,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H33" s="18">
-        <f>IFERROR(BDP($A33,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A33,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I33" s="18">
-        <f>IFERROR(BDP($A33,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A33,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J33" s="21">
-        <f>IFERROR(BDP($A33,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A33,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K33" s="21">
-        <f>IFERROR(BDP($A33,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A33,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n"/>
       <c r="B34" s="6">
-        <f>IFERROR(BDP($A34,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A34,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C34" s="17">
-        <f>IFERROR(BDP($A34,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A34,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D34" s="17">
-        <f>IFERROR(BDP($A34,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A34,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E34" s="17">
-        <f>IFERROR(BDP($A34,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A34,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F34" s="17">
@@ -35628,42 +35645,42 @@
         <v/>
       </c>
       <c r="G34" s="6">
-        <f>IFERROR(BDP($A34,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A34,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H34" s="18">
-        <f>IFERROR(BDP($A34,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A34,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I34" s="18">
-        <f>IFERROR(BDP($A34,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A34,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J34" s="21">
-        <f>IFERROR(BDP($A34,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A34,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K34" s="21">
-        <f>IFERROR(BDP($A34,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A34,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="6">
-        <f>IFERROR(BDP($A35,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A35,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C35" s="17">
-        <f>IFERROR(BDP($A35,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A35,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D35" s="17">
-        <f>IFERROR(BDP($A35,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A35,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E35" s="17">
-        <f>IFERROR(BDP($A35,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A35,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F35" s="17">
@@ -35671,42 +35688,42 @@
         <v/>
       </c>
       <c r="G35" s="6">
-        <f>IFERROR(BDP($A35,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A35,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H35" s="18">
-        <f>IFERROR(BDP($A35,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A35,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I35" s="18">
-        <f>IFERROR(BDP($A35,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A35,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J35" s="21">
-        <f>IFERROR(BDP($A35,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A35,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K35" s="21">
-        <f>IFERROR(BDP($A35,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A35,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n"/>
       <c r="B36" s="6">
-        <f>IFERROR(BDP($A36,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A36,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C36" s="17">
-        <f>IFERROR(BDP($A36,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A36,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D36" s="17">
-        <f>IFERROR(BDP($A36,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A36,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E36" s="17">
-        <f>IFERROR(BDP($A36,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A36,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F36" s="17">
@@ -35714,42 +35731,42 @@
         <v/>
       </c>
       <c r="G36" s="6">
-        <f>IFERROR(BDP($A36,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A36,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H36" s="18">
-        <f>IFERROR(BDP($A36,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A36,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I36" s="18">
-        <f>IFERROR(BDP($A36,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A36,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J36" s="21">
-        <f>IFERROR(BDP($A36,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A36,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K36" s="21">
-        <f>IFERROR(BDP($A36,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A36,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="6">
-        <f>IFERROR(BDP($A37,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A37,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C37" s="17">
-        <f>IFERROR(BDP($A37,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A37,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D37" s="17">
-        <f>IFERROR(BDP($A37,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A37,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E37" s="17">
-        <f>IFERROR(BDP($A37,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A37,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F37" s="17">
@@ -35757,42 +35774,42 @@
         <v/>
       </c>
       <c r="G37" s="6">
-        <f>IFERROR(BDP($A37,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A37,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H37" s="18">
-        <f>IFERROR(BDP($A37,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A37,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I37" s="18">
-        <f>IFERROR(BDP($A37,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A37,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J37" s="21">
-        <f>IFERROR(BDP($A37,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A37,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K37" s="21">
-        <f>IFERROR(BDP($A37,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A37,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n"/>
       <c r="B38" s="6">
-        <f>IFERROR(BDP($A38,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A38,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C38" s="17">
-        <f>IFERROR(BDP($A38,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A38,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D38" s="17">
-        <f>IFERROR(BDP($A38,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A38,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E38" s="17">
-        <f>IFERROR(BDP($A38,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A38,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F38" s="17">
@@ -35800,42 +35817,42 @@
         <v/>
       </c>
       <c r="G38" s="6">
-        <f>IFERROR(BDP($A38,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A38,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H38" s="18">
-        <f>IFERROR(BDP($A38,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A38,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I38" s="18">
-        <f>IFERROR(BDP($A38,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A38,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J38" s="21">
-        <f>IFERROR(BDP($A38,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A38,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K38" s="21">
-        <f>IFERROR(BDP($A38,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A38,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n"/>
       <c r="B39" s="6">
-        <f>IFERROR(BDP($A39,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A39,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C39" s="17">
-        <f>IFERROR(BDP($A39,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A39,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D39" s="17">
-        <f>IFERROR(BDP($A39,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A39,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E39" s="17">
-        <f>IFERROR(BDP($A39,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A39,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F39" s="17">
@@ -35843,42 +35860,42 @@
         <v/>
       </c>
       <c r="G39" s="6">
-        <f>IFERROR(BDP($A39,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A39,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H39" s="18">
-        <f>IFERROR(BDP($A39,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A39,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I39" s="18">
-        <f>IFERROR(BDP($A39,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A39,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J39" s="21">
-        <f>IFERROR(BDP($A39,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A39,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K39" s="21">
-        <f>IFERROR(BDP($A39,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A39,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n"/>
       <c r="B40" s="6">
-        <f>IFERROR(BDP($A40,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A40,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C40" s="17">
-        <f>IFERROR(BDP($A40,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A40,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D40" s="17">
-        <f>IFERROR(BDP($A40,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A40,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E40" s="17">
-        <f>IFERROR(BDP($A40,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A40,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F40" s="17">
@@ -35886,42 +35903,42 @@
         <v/>
       </c>
       <c r="G40" s="6">
-        <f>IFERROR(BDP($A40,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A40,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H40" s="18">
-        <f>IFERROR(BDP($A40,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A40,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I40" s="18">
-        <f>IFERROR(BDP($A40,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A40,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J40" s="21">
-        <f>IFERROR(BDP($A40,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A40,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K40" s="21">
-        <f>IFERROR(BDP($A40,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A40,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="6">
-        <f>IFERROR(BDP($A41,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A41,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C41" s="17">
-        <f>IFERROR(BDP($A41,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A41,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D41" s="17">
-        <f>IFERROR(BDP($A41,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A41,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E41" s="17">
-        <f>IFERROR(BDP($A41,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A41,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F41" s="17">
@@ -35929,42 +35946,42 @@
         <v/>
       </c>
       <c r="G41" s="6">
-        <f>IFERROR(BDP($A41,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A41,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H41" s="18">
-        <f>IFERROR(BDP($A41,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A41,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I41" s="18">
-        <f>IFERROR(BDP($A41,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A41,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J41" s="21">
-        <f>IFERROR(BDP($A41,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A41,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K41" s="21">
-        <f>IFERROR(BDP($A41,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A41,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="6">
-        <f>IFERROR(BDP($A42,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A42,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C42" s="17">
-        <f>IFERROR(BDP($A42,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A42,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D42" s="17">
-        <f>IFERROR(BDP($A42,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A42,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E42" s="17">
-        <f>IFERROR(BDP($A42,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A42,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F42" s="17">
@@ -35972,42 +35989,42 @@
         <v/>
       </c>
       <c r="G42" s="6">
-        <f>IFERROR(BDP($A42,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A42,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H42" s="18">
-        <f>IFERROR(BDP($A42,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A42,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I42" s="18">
-        <f>IFERROR(BDP($A42,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A42,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J42" s="21">
-        <f>IFERROR(BDP($A42,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A42,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K42" s="21">
-        <f>IFERROR(BDP($A42,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A42,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="6">
-        <f>IFERROR(BDP($A43,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A43,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C43" s="17">
-        <f>IFERROR(BDP($A43,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A43,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D43" s="17">
-        <f>IFERROR(BDP($A43,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A43,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E43" s="17">
-        <f>IFERROR(BDP($A43,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A43,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F43" s="17">
@@ -36015,42 +36032,42 @@
         <v/>
       </c>
       <c r="G43" s="6">
-        <f>IFERROR(BDP($A43,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A43,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H43" s="18">
-        <f>IFERROR(BDP($A43,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A43,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I43" s="18">
-        <f>IFERROR(BDP($A43,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A43,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J43" s="21">
-        <f>IFERROR(BDP($A43,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A43,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K43" s="21">
-        <f>IFERROR(BDP($A43,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A43,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n"/>
       <c r="B44" s="6">
-        <f>IFERROR(BDP($A44,"SECURITY_DES"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A44,"SECURITY_DES"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="C44" s="17">
-        <f>IFERROR(BDP($A44,"PX_LAST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A44,"PX_LAST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="D44" s="17">
-        <f>IFERROR(BDP($A44,"PX_BID"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A44,"PX_BID"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="E44" s="17">
-        <f>IFERROR(BDP($A44,"PX_ASK"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A44,"PX_ASK"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="F44" s="17">
@@ -36058,23 +36075,23 @@
         <v/>
       </c>
       <c r="G44" s="6">
-        <f>IFERROR(BDP($A44,"FUT_MONTH_YR"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A44,"FUT_MONTH_YR"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="H44" s="18">
-        <f>IFERROR(BDP($A44,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A44,"FUT_DLV_DT_FIRST"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="I44" s="18">
-        <f>IFERROR(BDP($A44,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A44,"LAST_TRADEABLE_DT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="J44" s="21">
-        <f>IFERROR(BDP($A44,"VOLUME"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A44,"VOLUME"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
       <c r="K44" s="21">
-        <f>IFERROR(BDP($A44,"OPEN_INT"),"ERROR PLZ FIX")</f>
+        <f>IF($B$3&lt;&gt;"Yes","",IFERROR(BDP($A44,"OPEN_INT"),"ERROR PLZ FIX"))</f>
         <v/>
       </c>
     </row>
@@ -36085,6 +36102,11 @@
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A29:K29"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Freeze on the final S490 capture; hard-code the target into column L
Bloomberg_S490_Validation!L now holds the S490 zero curve as LITERAL numbers
from the 07/21/26 capture - no lookup, no live pull. Column E compares our
bootstrap against it. D (live BDS) and G (snapshot lookup) remain as secondary
references.

S490_Snapshot refreshed to the same final capture, so the curve INPUT (market
rates -> SOFR_OIS_Quotes!J) and the TARGET are from one instant.

  32/32 pillars, max |d zero| 0.397bp, max |d DF| 1.88e-05, 0.08bp from 2Y

Rows were keyed on the evaluated maturity DATE rather than the tenor label,
since column A holds formulas rather than literals.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -6763,6 +6763,11 @@
           <t>VERIFY I3/I4/I5 against the dump at J12 before trusting column E — the defaults are a GUESS at the CURVE_TENOR_RATES schema, not confirmed.</t>
         </is>
       </c>
+      <c r="L6" s="65" t="inlineStr">
+        <is>
+          <t>32 pillars hard-coded</t>
+        </is>
+      </c>
       <c r="V6" s="67" t="inlineStr">
         <is>
           <t>S490 SCREEN SNAPSHOT (curve date 07/21/2026)</t>
@@ -6849,7 +6854,7 @@
         <v/>
       </c>
       <c r="E8" s="89">
-        <f>IF(ISNUMBER(D8),(C8-D8)*100,IF(ISNUMBER(G8),(C8-G8)*100,""))</f>
+        <f>IF(ISNUMBER(L8),(C8-L8)*100,"")</f>
         <v/>
       </c>
       <c r="F8" s="93">
@@ -6864,6 +6869,9 @@
         <is>
           <t>(the CURVE_TENOR_RATES dump lives at J12 - a second copy here would spill into it)</t>
         </is>
+      </c>
+      <c r="L8" s="85" t="n">
+        <v>3.68682</v>
       </c>
       <c r="M8" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B8,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -6916,7 +6924,7 @@
         <v/>
       </c>
       <c r="E9" s="89">
-        <f>IF(ISNUMBER(D9),(C9-D9)*100,IF(ISNUMBER(G9),(C9-G9)*100,""))</f>
+        <f>IF(ISNUMBER(L9),(C9-L9)*100,"")</f>
         <v/>
       </c>
       <c r="F9" s="93">
@@ -6926,6 +6934,9 @@
       <c r="G9" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B9,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L9" s="85" t="n">
+        <v>3.71731</v>
       </c>
       <c r="M9" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B9,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -6970,7 +6981,7 @@
         <v/>
       </c>
       <c r="E10" s="89">
-        <f>IF(ISNUMBER(D10),(C10-D10)*100,IF(ISNUMBER(G10),(C10-G10)*100,""))</f>
+        <f>IF(ISNUMBER(L10),(C10-L10)*100,"")</f>
         <v/>
       </c>
       <c r="F10" s="93">
@@ -6980,6 +6991,9 @@
       <c r="G10" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B10,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L10" s="85" t="n">
+        <v>3.73043</v>
       </c>
       <c r="M10" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B10,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7024,7 +7038,7 @@
         <v/>
       </c>
       <c r="E11" s="89">
-        <f>IF(ISNUMBER(D11),(C11-D11)*100,IF(ISNUMBER(G11),(C11-G11)*100,""))</f>
+        <f>IF(ISNUMBER(L11),(C11-L11)*100,"")</f>
         <v/>
       </c>
       <c r="F11" s="93">
@@ -7034,6 +7048,9 @@
       <c r="G11" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B11,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L11" s="85" t="n">
+        <v>3.73852</v>
       </c>
       <c r="M11" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B11,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7078,7 +7095,7 @@
         <v/>
       </c>
       <c r="E12" s="89">
-        <f>IF(ISNUMBER(D12),(C12-D12)*100,IF(ISNUMBER(G12),(C12-G12)*100,""))</f>
+        <f>IF(ISNUMBER(L12),(C12-L12)*100,"")</f>
         <v/>
       </c>
       <c r="F12" s="93">
@@ -7092,6 +7109,9 @@
       <c r="J12" s="93">
         <f>BDS(S490_TKR,"CURVE_TENOR_RATES")</f>
         <v/>
+      </c>
+      <c r="L12" s="85" t="n">
+        <v>3.75985</v>
       </c>
       <c r="M12" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B12,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7136,7 +7156,7 @@
         <v/>
       </c>
       <c r="E13" s="89">
-        <f>IF(ISNUMBER(D13),(C13-D13)*100,IF(ISNUMBER(G13),(C13-G13)*100,""))</f>
+        <f>IF(ISNUMBER(L13),(C13-L13)*100,"")</f>
         <v/>
       </c>
       <c r="F13" s="93">
@@ -7146,6 +7166,9 @@
       <c r="G13" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B13,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L13" s="85" t="n">
+        <v>3.80673</v>
       </c>
       <c r="M13" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B13,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7190,7 +7213,7 @@
         <v/>
       </c>
       <c r="E14" s="89">
-        <f>IF(ISNUMBER(D14),(C14-D14)*100,IF(ISNUMBER(G14),(C14-G14)*100,""))</f>
+        <f>IF(ISNUMBER(L14),(C14-L14)*100,"")</f>
         <v/>
       </c>
       <c r="F14" s="93">
@@ -7200,6 +7223,9 @@
       <c r="G14" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B14,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L14" s="85" t="n">
+        <v>3.84626</v>
       </c>
       <c r="M14" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B14,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7244,7 +7270,7 @@
         <v/>
       </c>
       <c r="E15" s="89">
-        <f>IF(ISNUMBER(D15),(C15-D15)*100,IF(ISNUMBER(G15),(C15-G15)*100,""))</f>
+        <f>IF(ISNUMBER(L15),(C15-L15)*100,"")</f>
         <v/>
       </c>
       <c r="F15" s="93">
@@ -7254,6 +7280,9 @@
       <c r="G15" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B15,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L15" s="85" t="n">
+        <v>3.88151</v>
       </c>
       <c r="M15" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B15,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7298,7 +7327,7 @@
         <v/>
       </c>
       <c r="E16" s="89">
-        <f>IF(ISNUMBER(D16),(C16-D16)*100,IF(ISNUMBER(G16),(C16-G16)*100,""))</f>
+        <f>IF(ISNUMBER(L16),(C16-L16)*100,"")</f>
         <v/>
       </c>
       <c r="F16" s="93">
@@ -7308,6 +7337,9 @@
       <c r="G16" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B16,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L16" s="85" t="n">
+        <v>3.9203</v>
       </c>
       <c r="M16" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B16,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7352,7 +7384,7 @@
         <v/>
       </c>
       <c r="E17" s="89">
-        <f>IF(ISNUMBER(D17),(C17-D17)*100,IF(ISNUMBER(G17),(C17-G17)*100,""))</f>
+        <f>IF(ISNUMBER(L17),(C17-L17)*100,"")</f>
         <v/>
       </c>
       <c r="F17" s="93">
@@ -7362,6 +7394,9 @@
       <c r="G17" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B17,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L17" s="85" t="n">
+        <v>3.94751</v>
       </c>
       <c r="M17" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B17,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7406,7 +7441,7 @@
         <v/>
       </c>
       <c r="E18" s="89">
-        <f>IF(ISNUMBER(D18),(C18-D18)*100,IF(ISNUMBER(G18),(C18-G18)*100,""))</f>
+        <f>IF(ISNUMBER(L18),(C18-L18)*100,"")</f>
         <v/>
       </c>
       <c r="F18" s="93">
@@ -7416,6 +7451,9 @@
       <c r="G18" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B18,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L18" s="85" t="n">
+        <v>3.96958</v>
       </c>
       <c r="M18" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B18,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7460,7 +7498,7 @@
         <v/>
       </c>
       <c r="E19" s="89">
-        <f>IF(ISNUMBER(D19),(C19-D19)*100,IF(ISNUMBER(G19),(C19-G19)*100,""))</f>
+        <f>IF(ISNUMBER(L19),(C19-L19)*100,"")</f>
         <v/>
       </c>
       <c r="F19" s="93">
@@ -7470,6 +7508,9 @@
       <c r="G19" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B19,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L19" s="85" t="n">
+        <v>3.9935</v>
       </c>
       <c r="M19" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B19,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7514,7 +7555,7 @@
         <v/>
       </c>
       <c r="E20" s="89">
-        <f>IF(ISNUMBER(D20),(C20-D20)*100,IF(ISNUMBER(G20),(C20-G20)*100,""))</f>
+        <f>IF(ISNUMBER(L20),(C20-L20)*100,"")</f>
         <v/>
       </c>
       <c r="F20" s="93">
@@ -7524,6 +7565,9 @@
       <c r="G20" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B20,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L20" s="85" t="n">
+        <v>4.0143</v>
       </c>
       <c r="M20" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B20,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7568,7 +7612,7 @@
         <v/>
       </c>
       <c r="E21" s="89">
-        <f>IF(ISNUMBER(D21),(C21-D21)*100,IF(ISNUMBER(G21),(C21-G21)*100,""))</f>
+        <f>IF(ISNUMBER(L21),(C21-L21)*100,"")</f>
         <v/>
       </c>
       <c r="F21" s="93">
@@ -7578,6 +7622,9 @@
       <c r="G21" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B21,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L21" s="85" t="n">
+        <v>4.03096</v>
       </c>
       <c r="M21" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B21,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7622,7 +7669,7 @@
         <v/>
       </c>
       <c r="E22" s="89">
-        <f>IF(ISNUMBER(D22),(C22-D22)*100,IF(ISNUMBER(G22),(C22-G22)*100,""))</f>
+        <f>IF(ISNUMBER(L22),(C22-L22)*100,"")</f>
         <v/>
       </c>
       <c r="F22" s="93">
@@ -7632,6 +7679,9 @@
       <c r="G22" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B22,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L22" s="85" t="n">
+        <v>4.04476</v>
       </c>
       <c r="M22" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B22,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7676,7 +7726,7 @@
         <v/>
       </c>
       <c r="E23" s="89">
-        <f>IF(ISNUMBER(D23),(C23-D23)*100,IF(ISNUMBER(G23),(C23-G23)*100,""))</f>
+        <f>IF(ISNUMBER(L23),(C23-L23)*100,"")</f>
         <v/>
       </c>
       <c r="F23" s="93">
@@ -7686,6 +7736,9 @@
       <c r="G23" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B23,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L23" s="85" t="n">
+        <v>4.07772</v>
       </c>
       <c r="M23" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B23,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7730,7 +7783,7 @@
         <v/>
       </c>
       <c r="E24" s="89">
-        <f>IF(ISNUMBER(D24),(C24-D24)*100,IF(ISNUMBER(G24),(C24-G24)*100,""))</f>
+        <f>IF(ISNUMBER(L24),(C24-L24)*100,"")</f>
         <v/>
       </c>
       <c r="F24" s="93">
@@ -7740,6 +7793,9 @@
       <c r="G24" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B24,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L24" s="85" t="n">
+        <v>4.06872</v>
       </c>
       <c r="M24" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B24,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7784,7 +7840,7 @@
         <v/>
       </c>
       <c r="E25" s="89">
-        <f>IF(ISNUMBER(D25),(C25-D25)*100,IF(ISNUMBER(G25),(C25-G25)*100,""))</f>
+        <f>IF(ISNUMBER(L25),(C25-L25)*100,"")</f>
         <v/>
       </c>
       <c r="F25" s="93">
@@ -7794,6 +7850,9 @@
       <c r="G25" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B25,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L25" s="85" t="n">
+        <v>4.0488</v>
       </c>
       <c r="M25" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B25,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7838,7 +7897,7 @@
         <v/>
       </c>
       <c r="E26" s="89">
-        <f>IF(ISNUMBER(D26),(C26-D26)*100,IF(ISNUMBER(G26),(C26-G26)*100,""))</f>
+        <f>IF(ISNUMBER(L26),(C26-L26)*100,"")</f>
         <v/>
       </c>
       <c r="F26" s="93">
@@ -7848,6 +7907,9 @@
       <c r="G26" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B26,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L26" s="85" t="n">
+        <v>4.03876</v>
       </c>
       <c r="M26" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B26,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7892,7 +7954,7 @@
         <v/>
       </c>
       <c r="E27" s="89">
-        <f>IF(ISNUMBER(D27),(C27-D27)*100,IF(ISNUMBER(G27),(C27-G27)*100,""))</f>
+        <f>IF(ISNUMBER(L27),(C27-L27)*100,"")</f>
         <v/>
       </c>
       <c r="F27" s="93">
@@ -7902,6 +7964,9 @@
       <c r="G27" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B27,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L27" s="85" t="n">
+        <v>4.0443</v>
       </c>
       <c r="M27" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B27,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -7946,7 +8011,7 @@
         <v/>
       </c>
       <c r="E28" s="89">
-        <f>IF(ISNUMBER(D28),(C28-D28)*100,IF(ISNUMBER(G28),(C28-G28)*100,""))</f>
+        <f>IF(ISNUMBER(L28),(C28-L28)*100,"")</f>
         <v/>
       </c>
       <c r="F28" s="93">
@@ -7956,6 +8021,9 @@
       <c r="G28" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B28,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L28" s="85" t="n">
+        <v>4.0634</v>
       </c>
       <c r="M28" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B28,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -8000,7 +8068,7 @@
         <v/>
       </c>
       <c r="E29" s="89">
-        <f>IF(ISNUMBER(D29),(C29-D29)*100,IF(ISNUMBER(G29),(C29-G29)*100,""))</f>
+        <f>IF(ISNUMBER(L29),(C29-L29)*100,"")</f>
         <v/>
       </c>
       <c r="F29" s="93">
@@ -8010,6 +8078,9 @@
       <c r="G29" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B29,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L29" s="85" t="n">
+        <v>4.0891</v>
       </c>
       <c r="M29" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B29,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -8054,7 +8125,7 @@
         <v/>
       </c>
       <c r="E30" s="89">
-        <f>IF(ISNUMBER(D30),(C30-D30)*100,IF(ISNUMBER(G30),(C30-G30)*100,""))</f>
+        <f>IF(ISNUMBER(L30),(C30-L30)*100,"")</f>
         <v/>
       </c>
       <c r="F30" s="93">
@@ -8064,6 +8135,9 @@
       <c r="G30" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B30,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L30" s="85" t="n">
+        <v>4.11874</v>
       </c>
       <c r="M30" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B30,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -8108,7 +8182,7 @@
         <v/>
       </c>
       <c r="E31" s="89">
-        <f>IF(ISNUMBER(D31),(C31-D31)*100,IF(ISNUMBER(G31),(C31-G31)*100,""))</f>
+        <f>IF(ISNUMBER(L31),(C31-L31)*100,"")</f>
         <v/>
       </c>
       <c r="F31" s="93">
@@ -8118,6 +8192,9 @@
       <c r="G31" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B31,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L31" s="85" t="n">
+        <v>4.15198</v>
       </c>
       <c r="M31" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B31,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -8162,7 +8239,7 @@
         <v/>
       </c>
       <c r="E32" s="89">
-        <f>IF(ISNUMBER(D32),(C32-D32)*100,IF(ISNUMBER(G32),(C32-G32)*100,""))</f>
+        <f>IF(ISNUMBER(L32),(C32-L32)*100,"")</f>
         <v/>
       </c>
       <c r="F32" s="93">
@@ -8172,6 +8249,9 @@
       <c r="G32" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B32,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L32" s="85" t="n">
+        <v>4.18778</v>
       </c>
       <c r="M32" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B32,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -8216,7 +8296,7 @@
         <v/>
       </c>
       <c r="E33" s="89">
-        <f>IF(ISNUMBER(D33),(C33-D33)*100,IF(ISNUMBER(G33),(C33-G33)*100,""))</f>
+        <f>IF(ISNUMBER(L33),(C33-L33)*100,"")</f>
         <v/>
       </c>
       <c r="F33" s="93">
@@ -8227,6 +8307,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B33,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L33" s="94" t="n"/>
       <c r="M33" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B33,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -8270,7 +8351,7 @@
         <v/>
       </c>
       <c r="E34" s="89">
-        <f>IF(ISNUMBER(D34),(C34-D34)*100,IF(ISNUMBER(G34),(C34-G34)*100,""))</f>
+        <f>IF(ISNUMBER(L34),(C34-L34)*100,"")</f>
         <v/>
       </c>
       <c r="F34" s="93">
@@ -8280,6 +8361,9 @@
       <c r="G34" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B34,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L34" s="85" t="n">
+        <v>4.26298</v>
       </c>
       <c r="M34" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B34,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -8324,7 +8408,7 @@
         <v/>
       </c>
       <c r="E35" s="89">
-        <f>IF(ISNUMBER(D35),(C35-D35)*100,IF(ISNUMBER(G35),(C35-G35)*100,""))</f>
+        <f>IF(ISNUMBER(L35),(C35-L35)*100,"")</f>
         <v/>
       </c>
       <c r="F35" s="93">
@@ -8335,6 +8419,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B35,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L35" s="94" t="n"/>
       <c r="M35" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B35,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -8378,7 +8463,7 @@
         <v/>
       </c>
       <c r="E36" s="89">
-        <f>IF(ISNUMBER(D36),(C36-D36)*100,IF(ISNUMBER(G36),(C36-G36)*100,""))</f>
+        <f>IF(ISNUMBER(L36),(C36-L36)*100,"")</f>
         <v/>
       </c>
       <c r="F36" s="93">
@@ -8389,6 +8474,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B36,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L36" s="94" t="n"/>
       <c r="M36" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B36,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -8432,7 +8518,7 @@
         <v/>
       </c>
       <c r="E37" s="89">
-        <f>IF(ISNUMBER(D37),(C37-D37)*100,IF(ISNUMBER(G37),(C37-G37)*100,""))</f>
+        <f>IF(ISNUMBER(L37),(C37-L37)*100,"")</f>
         <v/>
       </c>
       <c r="F37" s="93">
@@ -8442,6 +8528,9 @@
       <c r="G37" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B37,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L37" s="85" t="n">
+        <v>4.36615</v>
       </c>
       <c r="M37" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B37,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -8486,7 +8575,7 @@
         <v/>
       </c>
       <c r="E38" s="89">
-        <f>IF(ISNUMBER(D38),(C38-D38)*100,IF(ISNUMBER(G38),(C38-G38)*100,""))</f>
+        <f>IF(ISNUMBER(L38),(C38-L38)*100,"")</f>
         <v/>
       </c>
       <c r="F38" s="93">
@@ -8497,6 +8586,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B38,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L38" s="94" t="n"/>
       <c r="M38" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B38,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -8540,7 +8630,7 @@
         <v/>
       </c>
       <c r="E39" s="89">
-        <f>IF(ISNUMBER(D39),(C39-D39)*100,IF(ISNUMBER(G39),(C39-G39)*100,""))</f>
+        <f>IF(ISNUMBER(L39),(C39-L39)*100,"")</f>
         <v/>
       </c>
       <c r="F39" s="93">
@@ -8551,6 +8641,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B39,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L39" s="94" t="n"/>
       <c r="M39" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B39,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -8594,7 +8685,7 @@
         <v/>
       </c>
       <c r="E40" s="89">
-        <f>IF(ISNUMBER(D40),(C40-D40)*100,IF(ISNUMBER(G40),(C40-G40)*100,""))</f>
+        <f>IF(ISNUMBER(L40),(C40-L40)*100,"")</f>
         <v/>
       </c>
       <c r="F40" s="93">
@@ -8605,6 +8696,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B40,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L40" s="94" t="n"/>
       <c r="M40" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B40,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -8648,7 +8740,7 @@
         <v/>
       </c>
       <c r="E41" s="89">
-        <f>IF(ISNUMBER(D41),(C41-D41)*100,IF(ISNUMBER(G41),(C41-G41)*100,""))</f>
+        <f>IF(ISNUMBER(L41),(C41-L41)*100,"")</f>
         <v/>
       </c>
       <c r="F41" s="93">
@@ -8659,6 +8751,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B41,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L41" s="94" t="n"/>
       <c r="M41" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B41,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -8690,7 +8783,7 @@
         <v/>
       </c>
       <c r="E42" s="89">
-        <f>IF(ISNUMBER(D42),(C42-D42)*100,IF(ISNUMBER(G42),(C42-G42)*100,""))</f>
+        <f>IF(ISNUMBER(L42),(C42-L42)*100,"")</f>
         <v/>
       </c>
       <c r="F42" s="93">
@@ -8700,6 +8793,9 @@
       <c r="G42" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B42,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L42" s="85" t="n">
+        <v>4.45385</v>
       </c>
       <c r="M42" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B42,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -8732,7 +8828,7 @@
         <v/>
       </c>
       <c r="E43" s="89">
-        <f>IF(ISNUMBER(D43),(C43-D43)*100,IF(ISNUMBER(G43),(C43-G43)*100,""))</f>
+        <f>IF(ISNUMBER(L43),(C43-L43)*100,"")</f>
         <v/>
       </c>
       <c r="F43" s="93">
@@ -8743,6 +8839,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B43,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L43" s="94" t="n"/>
       <c r="M43" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B43,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -8774,7 +8871,7 @@
         <v/>
       </c>
       <c r="E44" s="89">
-        <f>IF(ISNUMBER(D44),(C44-D44)*100,IF(ISNUMBER(G44),(C44-G44)*100,""))</f>
+        <f>IF(ISNUMBER(L44),(C44-L44)*100,"")</f>
         <v/>
       </c>
       <c r="F44" s="93">
@@ -8785,6 +8882,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B44,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L44" s="94" t="n"/>
       <c r="M44" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B44,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -8816,7 +8914,7 @@
         <v/>
       </c>
       <c r="E45" s="89">
-        <f>IF(ISNUMBER(D45),(C45-D45)*100,IF(ISNUMBER(G45),(C45-G45)*100,""))</f>
+        <f>IF(ISNUMBER(L45),(C45-L45)*100,"")</f>
         <v/>
       </c>
       <c r="F45" s="93">
@@ -8827,6 +8925,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B45,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L45" s="94" t="n"/>
       <c r="M45" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B45,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -8858,7 +8957,7 @@
         <v/>
       </c>
       <c r="E46" s="89">
-        <f>IF(ISNUMBER(D46),(C46-D46)*100,IF(ISNUMBER(G46),(C46-G46)*100,""))</f>
+        <f>IF(ISNUMBER(L46),(C46-L46)*100,"")</f>
         <v/>
       </c>
       <c r="F46" s="93">
@@ -8869,6 +8968,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B46,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L46" s="94" t="n"/>
       <c r="M46" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B46,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -8900,7 +9000,7 @@
         <v/>
       </c>
       <c r="E47" s="89">
-        <f>IF(ISNUMBER(D47),(C47-D47)*100,IF(ISNUMBER(G47),(C47-G47)*100,""))</f>
+        <f>IF(ISNUMBER(L47),(C47-L47)*100,"")</f>
         <v/>
       </c>
       <c r="F47" s="93">
@@ -8910,6 +9010,9 @@
       <c r="G47" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B47,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L47" s="85" t="n">
+        <v>4.4337</v>
       </c>
       <c r="M47" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B47,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -8942,7 +9045,7 @@
         <v/>
       </c>
       <c r="E48" s="89">
-        <f>IF(ISNUMBER(D48),(C48-D48)*100,IF(ISNUMBER(G48),(C48-G48)*100,""))</f>
+        <f>IF(ISNUMBER(L48),(C48-L48)*100,"")</f>
         <v/>
       </c>
       <c r="F48" s="93">
@@ -8953,6 +9056,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B48,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L48" s="94" t="n"/>
       <c r="M48" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B48,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -8984,7 +9088,7 @@
         <v/>
       </c>
       <c r="E49" s="89">
-        <f>IF(ISNUMBER(D49),(C49-D49)*100,IF(ISNUMBER(G49),(C49-G49)*100,""))</f>
+        <f>IF(ISNUMBER(L49),(C49-L49)*100,"")</f>
         <v/>
       </c>
       <c r="F49" s="93">
@@ -8995,6 +9099,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B49,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L49" s="94" t="n"/>
       <c r="M49" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B49,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9026,7 +9131,7 @@
         <v/>
       </c>
       <c r="E50" s="89">
-        <f>IF(ISNUMBER(D50),(C50-D50)*100,IF(ISNUMBER(G50),(C50-G50)*100,""))</f>
+        <f>IF(ISNUMBER(L50),(C50-L50)*100,"")</f>
         <v/>
       </c>
       <c r="F50" s="93">
@@ -9037,6 +9142,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B50,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L50" s="94" t="n"/>
       <c r="M50" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B50,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9068,7 +9174,7 @@
         <v/>
       </c>
       <c r="E51" s="89">
-        <f>IF(ISNUMBER(D51),(C51-D51)*100,IF(ISNUMBER(G51),(C51-G51)*100,""))</f>
+        <f>IF(ISNUMBER(L51),(C51-L51)*100,"")</f>
         <v/>
       </c>
       <c r="F51" s="93">
@@ -9079,6 +9185,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B51,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L51" s="94" t="n"/>
       <c r="M51" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B51,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9110,7 +9217,7 @@
         <v/>
       </c>
       <c r="E52" s="89">
-        <f>IF(ISNUMBER(D52),(C52-D52)*100,IF(ISNUMBER(G52),(C52-G52)*100,""))</f>
+        <f>IF(ISNUMBER(L52),(C52-L52)*100,"")</f>
         <v/>
       </c>
       <c r="F52" s="93">
@@ -9120,6 +9227,9 @@
       <c r="G52" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B52,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L52" s="85" t="n">
+        <v>4.35343</v>
       </c>
       <c r="M52" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B52,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -9152,7 +9262,7 @@
         <v/>
       </c>
       <c r="E53" s="89">
-        <f>IF(ISNUMBER(D53),(C53-D53)*100,IF(ISNUMBER(G53),(C53-G53)*100,""))</f>
+        <f>IF(ISNUMBER(L53),(C53-L53)*100,"")</f>
         <v/>
       </c>
       <c r="F53" s="93">
@@ -9163,6 +9273,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B53,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L53" s="94" t="n"/>
       <c r="M53" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B53,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9194,7 +9305,7 @@
         <v/>
       </c>
       <c r="E54" s="89">
-        <f>IF(ISNUMBER(D54),(C54-D54)*100,IF(ISNUMBER(G54),(C54-G54)*100,""))</f>
+        <f>IF(ISNUMBER(L54),(C54-L54)*100,"")</f>
         <v/>
       </c>
       <c r="F54" s="93">
@@ -9205,6 +9316,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B54,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L54" s="94" t="n"/>
       <c r="M54" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B54,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9236,7 +9348,7 @@
         <v/>
       </c>
       <c r="E55" s="89">
-        <f>IF(ISNUMBER(D55),(C55-D55)*100,IF(ISNUMBER(G55),(C55-G55)*100,""))</f>
+        <f>IF(ISNUMBER(L55),(C55-L55)*100,"")</f>
         <v/>
       </c>
       <c r="F55" s="93">
@@ -9247,6 +9359,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B55,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L55" s="94" t="n"/>
       <c r="M55" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B55,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9278,7 +9391,7 @@
         <v/>
       </c>
       <c r="E56" s="89">
-        <f>IF(ISNUMBER(D56),(C56-D56)*100,IF(ISNUMBER(G56),(C56-G56)*100,""))</f>
+        <f>IF(ISNUMBER(L56),(C56-L56)*100,"")</f>
         <v/>
       </c>
       <c r="F56" s="93">
@@ -9289,6 +9402,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B56,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L56" s="94" t="n"/>
       <c r="M56" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B56,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9320,7 +9434,7 @@
         <v/>
       </c>
       <c r="E57" s="89">
-        <f>IF(ISNUMBER(D57),(C57-D57)*100,IF(ISNUMBER(G57),(C57-G57)*100,""))</f>
+        <f>IF(ISNUMBER(L57),(C57-L57)*100,"")</f>
         <v/>
       </c>
       <c r="F57" s="93">
@@ -9331,6 +9445,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B57,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L57" s="94" t="n"/>
       <c r="M57" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B57,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9362,7 +9477,7 @@
         <v/>
       </c>
       <c r="E58" s="89">
-        <f>IF(ISNUMBER(D58),(C58-D58)*100,IF(ISNUMBER(G58),(C58-G58)*100,""))</f>
+        <f>IF(ISNUMBER(L58),(C58-L58)*100,"")</f>
         <v/>
       </c>
       <c r="F58" s="93">
@@ -9373,6 +9488,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B58,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L58" s="94" t="n"/>
       <c r="M58" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B58,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9404,7 +9520,7 @@
         <v/>
       </c>
       <c r="E59" s="89">
-        <f>IF(ISNUMBER(D59),(C59-D59)*100,IF(ISNUMBER(G59),(C59-G59)*100,""))</f>
+        <f>IF(ISNUMBER(L59),(C59-L59)*100,"")</f>
         <v/>
       </c>
       <c r="F59" s="93">
@@ -9415,6 +9531,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B59,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L59" s="94" t="n"/>
       <c r="M59" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B59,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9446,7 +9563,7 @@
         <v/>
       </c>
       <c r="E60" s="89">
-        <f>IF(ISNUMBER(D60),(C60-D60)*100,IF(ISNUMBER(G60),(C60-G60)*100,""))</f>
+        <f>IF(ISNUMBER(L60),(C60-L60)*100,"")</f>
         <v/>
       </c>
       <c r="F60" s="93">
@@ -9457,6 +9574,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B60,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L60" s="94" t="n"/>
       <c r="M60" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B60,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9488,7 +9606,7 @@
         <v/>
       </c>
       <c r="E61" s="89">
-        <f>IF(ISNUMBER(D61),(C61-D61)*100,IF(ISNUMBER(G61),(C61-G61)*100,""))</f>
+        <f>IF(ISNUMBER(L61),(C61-L61)*100,"")</f>
         <v/>
       </c>
       <c r="F61" s="93">
@@ -9499,6 +9617,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B61,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L61" s="94" t="n"/>
       <c r="M61" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B61,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9530,7 +9649,7 @@
         <v/>
       </c>
       <c r="E62" s="89">
-        <f>IF(ISNUMBER(D62),(C62-D62)*100,IF(ISNUMBER(G62),(C62-G62)*100,""))</f>
+        <f>IF(ISNUMBER(L62),(C62-L62)*100,"")</f>
         <v/>
       </c>
       <c r="F62" s="93">
@@ -9540,6 +9659,9 @@
       <c r="G62" s="97">
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B62,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
+      </c>
+      <c r="L62" s="85" t="n">
+        <v>4.10984</v>
       </c>
       <c r="M62" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B62,S490_Snapshot!$A$7:$A$38,0)),"")</f>
@@ -9572,7 +9694,7 @@
         <v/>
       </c>
       <c r="E63" s="89">
-        <f>IF(ISNUMBER(D63),(C63-D63)*100,IF(ISNUMBER(G63),(C63-G63)*100,""))</f>
+        <f>IF(ISNUMBER(L63),(C63-L63)*100,"")</f>
         <v/>
       </c>
       <c r="F63" s="93">
@@ -9583,6 +9705,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B63,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L63" s="94" t="n"/>
       <c r="M63" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B63,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9614,7 +9737,7 @@
         <v/>
       </c>
       <c r="E64" s="89">
-        <f>IF(ISNUMBER(D64),(C64-D64)*100,IF(ISNUMBER(G64),(C64-G64)*100,""))</f>
+        <f>IF(ISNUMBER(L64),(C64-L64)*100,"")</f>
         <v/>
       </c>
       <c r="F64" s="93">
@@ -9625,6 +9748,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B64,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L64" s="94" t="n"/>
       <c r="M64" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B64,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9656,7 +9780,7 @@
         <v/>
       </c>
       <c r="E65" s="89">
-        <f>IF(ISNUMBER(D65),(C65-D65)*100,IF(ISNUMBER(G65),(C65-G65)*100,""))</f>
+        <f>IF(ISNUMBER(L65),(C65-L65)*100,"")</f>
         <v/>
       </c>
       <c r="F65" s="93">
@@ -9667,6 +9791,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B65,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L65" s="94" t="n"/>
       <c r="M65" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B65,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9698,7 +9823,7 @@
         <v/>
       </c>
       <c r="E66" s="89">
-        <f>IF(ISNUMBER(D66),(C66-D66)*100,IF(ISNUMBER(G66),(C66-G66)*100,""))</f>
+        <f>IF(ISNUMBER(L66),(C66-L66)*100,"")</f>
         <v/>
       </c>
       <c r="F66" s="93">
@@ -9709,6 +9834,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B66,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L66" s="94" t="n"/>
       <c r="M66" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B66,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9740,7 +9866,7 @@
         <v/>
       </c>
       <c r="E67" s="89">
-        <f>IF(ISNUMBER(D67),(C67-D67)*100,IF(ISNUMBER(G67),(C67-G67)*100,""))</f>
+        <f>IF(ISNUMBER(L67),(C67-L67)*100,"")</f>
         <v/>
       </c>
       <c r="F67" s="93">
@@ -9751,6 +9877,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B67,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L67" s="94" t="n"/>
       <c r="M67" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B67,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9782,7 +9909,7 @@
         <v/>
       </c>
       <c r="E68" s="89">
-        <f>IF(ISNUMBER(D68),(C68-D68)*100,IF(ISNUMBER(G68),(C68-G68)*100,""))</f>
+        <f>IF(ISNUMBER(L68),(C68-L68)*100,"")</f>
         <v/>
       </c>
       <c r="F68" s="93">
@@ -9793,6 +9920,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B68,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L68" s="94" t="n"/>
       <c r="M68" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B68,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9824,7 +9952,7 @@
         <v/>
       </c>
       <c r="E69" s="89">
-        <f>IF(ISNUMBER(D69),(C69-D69)*100,IF(ISNUMBER(G69),(C69-G69)*100,""))</f>
+        <f>IF(ISNUMBER(L69),(C69-L69)*100,"")</f>
         <v/>
       </c>
       <c r="F69" s="93">
@@ -9835,6 +9963,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B69,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L69" s="94" t="n"/>
       <c r="M69" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B69,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9866,7 +9995,7 @@
         <v/>
       </c>
       <c r="E70" s="89">
-        <f>IF(ISNUMBER(D70),(C70-D70)*100,IF(ISNUMBER(G70),(C70-G70)*100,""))</f>
+        <f>IF(ISNUMBER(L70),(C70-L70)*100,"")</f>
         <v/>
       </c>
       <c r="F70" s="93">
@@ -9877,6 +10006,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B70,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L70" s="94" t="n"/>
       <c r="M70" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B70,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9908,7 +10038,7 @@
         <v/>
       </c>
       <c r="E71" s="89">
-        <f>IF(ISNUMBER(D71),(C71-D71)*100,IF(ISNUMBER(G71),(C71-G71)*100,""))</f>
+        <f>IF(ISNUMBER(L71),(C71-L71)*100,"")</f>
         <v/>
       </c>
       <c r="F71" s="93">
@@ -9919,6 +10049,7 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B71,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L71" s="94" t="n"/>
       <c r="M71" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B71,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9950,7 +10081,7 @@
         <v/>
       </c>
       <c r="E72" s="89">
-        <f>IF(ISNUMBER(D72),(C72-D72)*100,IF(ISNUMBER(G72),(C72-G72)*100,""))</f>
+        <f>IF(ISNUMBER(L72),(C72-L72)*100,"")</f>
         <v/>
       </c>
       <c r="F72" s="93">
@@ -9961,6 +10092,9 @@
         <f>IFERROR(INDEX(S490_Snapshot!$D$7:$D$38,MATCH(B72,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
       </c>
+      <c r="L72" s="85" t="n">
+        <v>3.81556</v>
+      </c>
       <c r="M72" s="80">
         <f>IFERROR(INDEX(S490_Snapshot!$E$7:$E$38,MATCH(B72,S490_Snapshot!$A$7:$A$38,0)),"")</f>
         <v/>
@@ -9977,18 +10111,18 @@
     <row r="74">
       <c r="A74" s="67" t="inlineStr">
         <is>
-          <t>Pillars matched to the screen</t>
+          <t>Pillars matched to the frozen target</t>
         </is>
       </c>
       <c r="C74" s="87">
-        <f>COUNT(M8:M72)&amp;" / 32"</f>
+        <f>COUNT(L8:L72)&amp;" / 32"</f>
         <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="67" t="inlineStr">
         <is>
-          <t>Max |zero diff| vs screen (bp)</t>
+          <t>Max |d zero| vs frozen S490 (bp)</t>
         </is>
       </c>
       <c r="C75" s="90">
@@ -10022,7 +10156,7 @@
     <row r="78">
       <c r="A78" s="65" t="inlineStr">
         <is>
-          <t>Column D = Bloomberg's own curve pulled live via BDS. Column G/M = the 07/21/26 screen snapshot in V:Y. Column E compares your zero to whichever is present.</t>
+          <t>Column L is the FROZEN S490 zero curve, hard-coded from the 07/21/26 capture - no lookup, no live pull. Column E compares our bootstrap against it. D (live BDS) and G (snapshot lookup) remain as secondary references.</t>
         </is>
       </c>
     </row>
@@ -35460,8 +35594,6 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
@@ -36139,7 +36271,7 @@
     <row r="2">
       <c r="A2" s="65" t="inlineStr">
         <is>
-          <t>Bloomberg S490 Curve Analysis capture. USD SOFR (vs FIXED), Step Forward (Cont), Settle Date 07/21/26, Curve Side Mid, Shift +0.00bp.</t>
+          <t>Bloomberg S490 Curve Analysis capture - FROZEN. USD SOFR (vs FIXED), Step Forward (Cont), Settle 07/21/26, Curve Side Mid, Shift +0.00bp.</t>
         </is>
       </c>
     </row>
@@ -36194,13 +36326,13 @@
         </is>
       </c>
       <c r="C7" s="85" t="n">
-        <v>3.643</v>
+        <v>3.6376</v>
       </c>
       <c r="D7" s="85" t="n">
-        <v>3.69229</v>
+        <v>3.68682</v>
       </c>
       <c r="E7" s="69" t="n">
-        <v>0.99909</v>
+        <v>0.999091</v>
       </c>
     </row>
     <row r="8">
@@ -36213,13 +36345,13 @@
         </is>
       </c>
       <c r="C8" s="85" t="n">
-        <v>3.6787</v>
+        <v>3.6733</v>
       </c>
       <c r="D8" s="85" t="n">
-        <v>3.72278</v>
+        <v>3.71731</v>
       </c>
       <c r="E8" s="69" t="n">
-        <v>0.998369</v>
+        <v>0.998372</v>
       </c>
     </row>
     <row r="9">
@@ -36232,10 +36364,10 @@
         </is>
       </c>
       <c r="C9" s="85" t="n">
-        <v>3.68722</v>
+        <v>3.68739</v>
       </c>
       <c r="D9" s="85" t="n">
-        <v>3.73075</v>
+        <v>3.73043</v>
       </c>
       <c r="E9" s="69" t="n">
         <v>0.997652</v>
@@ -36251,13 +36383,13 @@
         </is>
       </c>
       <c r="C10" s="85" t="n">
-        <v>3.6965</v>
+        <v>3.69655</v>
       </c>
       <c r="D10" s="85" t="n">
-        <v>3.73879</v>
+        <v>3.73852</v>
       </c>
       <c r="E10" s="69" t="n">
-        <v>0.996523</v>
+        <v>0.996524</v>
       </c>
     </row>
     <row r="11">
@@ -36270,10 +36402,10 @@
         </is>
       </c>
       <c r="C11" s="85" t="n">
-        <v>3.72235</v>
+        <v>3.72255</v>
       </c>
       <c r="D11" s="85" t="n">
-        <v>3.75983</v>
+        <v>3.75985</v>
       </c>
       <c r="E11" s="69" t="n">
         <v>0.993429</v>
@@ -36289,10 +36421,10 @@
         </is>
       </c>
       <c r="C12" s="85" t="n">
-        <v>3.77507</v>
+        <v>3.77525</v>
       </c>
       <c r="D12" s="85" t="n">
-        <v>3.80667</v>
+        <v>3.80673</v>
       </c>
       <c r="E12" s="69" t="n">
         <v>0.990244</v>
@@ -36308,13 +36440,13 @@
         </is>
       </c>
       <c r="C13" s="85" t="n">
-        <v>3.8205</v>
+        <v>3.82085</v>
       </c>
       <c r="D13" s="85" t="n">
-        <v>3.846</v>
+        <v>3.84626</v>
       </c>
       <c r="E13" s="69" t="n">
-        <v>0.986915</v>
+        <v>0.986914</v>
       </c>
     </row>
     <row r="14">
@@ -36327,13 +36459,13 @@
         </is>
       </c>
       <c r="C14" s="85" t="n">
-        <v>3.86225</v>
+        <v>3.8622</v>
       </c>
       <c r="D14" s="85" t="n">
-        <v>3.88163</v>
+        <v>3.88151</v>
       </c>
       <c r="E14" s="69" t="n">
-        <v>0.9836510000000001</v>
+        <v>0.983652</v>
       </c>
     </row>
     <row r="15">
@@ -36346,13 +36478,13 @@
         </is>
       </c>
       <c r="C15" s="85" t="n">
-        <v>3.90812</v>
+        <v>3.908</v>
       </c>
       <c r="D15" s="85" t="n">
-        <v>3.92047</v>
+        <v>3.9203</v>
       </c>
       <c r="E15" s="69" t="n">
-        <v>0.980009</v>
+        <v>0.98001</v>
       </c>
     </row>
     <row r="16">
@@ -36365,13 +36497,13 @@
         </is>
       </c>
       <c r="C16" s="85" t="n">
-        <v>3.9411</v>
+        <v>3.9415</v>
       </c>
       <c r="D16" s="85" t="n">
-        <v>3.94717</v>
+        <v>3.94751</v>
       </c>
       <c r="E16" s="69" t="n">
-        <v>0.976806</v>
+        <v>0.976805</v>
       </c>
     </row>
     <row r="17">
@@ -36384,13 +36516,13 @@
         </is>
       </c>
       <c r="C17" s="85" t="n">
-        <v>3.96915</v>
+        <v>3.96975</v>
       </c>
       <c r="D17" s="85" t="n">
-        <v>3.96903</v>
+        <v>3.96958</v>
       </c>
       <c r="E17" s="69" t="n">
-        <v>0.97371</v>
+        <v>0.973707</v>
       </c>
     </row>
     <row r="18">
@@ -36403,13 +36535,13 @@
         </is>
       </c>
       <c r="C18" s="85" t="n">
-        <v>3.99975</v>
+        <v>4.0007</v>
       </c>
       <c r="D18" s="85" t="n">
-        <v>3.99261</v>
+        <v>3.9935</v>
       </c>
       <c r="E18" s="69" t="n">
-        <v>0.970261</v>
+        <v>0.9702539999999999</v>
       </c>
     </row>
     <row r="19">
@@ -36422,13 +36554,13 @@
         </is>
       </c>
       <c r="C19" s="85" t="n">
-        <v>4.0275</v>
+        <v>4.02865</v>
       </c>
       <c r="D19" s="85" t="n">
-        <v>4.01321</v>
+        <v>4.0143</v>
       </c>
       <c r="E19" s="69" t="n">
-        <v>0.966808</v>
+        <v>0.9668</v>
       </c>
     </row>
     <row r="20">
@@ -36441,13 +36573,13 @@
         </is>
       </c>
       <c r="C20" s="85" t="n">
-        <v>4.05145</v>
+        <v>4.0523</v>
       </c>
       <c r="D20" s="85" t="n">
-        <v>4.03016</v>
+        <v>4.03096</v>
       </c>
       <c r="E20" s="69" t="n">
-        <v>0.9634740000000001</v>
+        <v>0.963467</v>
       </c>
     </row>
     <row r="21">
@@ -36460,13 +36592,13 @@
         </is>
       </c>
       <c r="C21" s="85" t="n">
-        <v>4.07237</v>
+        <v>4.07315</v>
       </c>
       <c r="D21" s="85" t="n">
-        <v>4.04404</v>
+        <v>4.04476</v>
       </c>
       <c r="E21" s="69" t="n">
-        <v>0.960154</v>
+        <v>0.960147</v>
       </c>
     </row>
     <row r="22">
@@ -36479,13 +36611,13 @@
         </is>
       </c>
       <c r="C22" s="85" t="n">
-        <v>4.0908</v>
+        <v>4.0909</v>
       </c>
       <c r="D22" s="85" t="n">
-        <v>4.07764</v>
+        <v>4.07772</v>
       </c>
       <c r="E22" s="69" t="n">
-        <v>0.940196</v>
+        <v>0.940194</v>
       </c>
     </row>
     <row r="23">
@@ -36498,13 +36630,13 @@
         </is>
       </c>
       <c r="C23" s="85" t="n">
-        <v>4.09725</v>
+        <v>4.09656</v>
       </c>
       <c r="D23" s="85" t="n">
-        <v>4.06943</v>
+        <v>4.06872</v>
       </c>
       <c r="E23" s="69" t="n">
-        <v>0.921424</v>
+        <v>0.921438</v>
       </c>
     </row>
     <row r="24">
@@ -36517,13 +36649,13 @@
         </is>
       </c>
       <c r="C24" s="85" t="n">
-        <v>4.0782</v>
+        <v>4.07655</v>
       </c>
       <c r="D24" s="85" t="n">
-        <v>4.05047</v>
+        <v>4.0488</v>
       </c>
       <c r="E24" s="69" t="n">
-        <v>0.885284</v>
+        <v>0.885328</v>
       </c>
     </row>
     <row r="25">
@@ -36536,13 +36668,13 @@
         </is>
       </c>
       <c r="C25" s="85" t="n">
-        <v>4.06895</v>
+        <v>4.06655</v>
       </c>
       <c r="D25" s="85" t="n">
-        <v>4.0412</v>
+        <v>4.03876</v>
       </c>
       <c r="E25" s="69" t="n">
-        <v>0.850458</v>
+        <v>0.850541</v>
       </c>
     </row>
     <row r="26">
@@ -36555,13 +36687,13 @@
         </is>
       </c>
       <c r="C26" s="85" t="n">
-        <v>4.0745</v>
+        <v>4.0715</v>
       </c>
       <c r="D26" s="85" t="n">
-        <v>4.04734</v>
+        <v>4.0443</v>
       </c>
       <c r="E26" s="69" t="n">
-        <v>0.816523</v>
+        <v>0.816648</v>
       </c>
     </row>
     <row r="27">
@@ -36574,13 +36706,13 @@
         </is>
       </c>
       <c r="C27" s="85" t="n">
-        <v>4.09215</v>
+        <v>4.0891</v>
       </c>
       <c r="D27" s="85" t="n">
-        <v>4.06648</v>
+        <v>4.0634</v>
       </c>
       <c r="E27" s="69" t="n">
-        <v>0.783148</v>
+        <v>0.783293</v>
       </c>
     </row>
     <row r="28">
@@ -36593,13 +36725,13 @@
         </is>
       </c>
       <c r="C28" s="85" t="n">
-        <v>4.11555</v>
+        <v>4.1126</v>
       </c>
       <c r="D28" s="85" t="n">
-        <v>4.09206</v>
+        <v>4.0891</v>
       </c>
       <c r="E28" s="69" t="n">
-        <v>0.750424</v>
+        <v>0.75058</v>
       </c>
     </row>
     <row r="29">
@@ -36612,13 +36744,13 @@
         </is>
       </c>
       <c r="C29" s="85" t="n">
-        <v>4.1421</v>
+        <v>4.13925</v>
       </c>
       <c r="D29" s="85" t="n">
-        <v>4.12158</v>
+        <v>4.11874</v>
       </c>
       <c r="E29" s="69" t="n">
-        <v>0.718715</v>
+        <v>0.718878</v>
       </c>
     </row>
     <row r="30">
@@ -36631,13 +36763,13 @@
         </is>
       </c>
       <c r="C30" s="85" t="n">
-        <v>4.17128</v>
+        <v>4.1687</v>
       </c>
       <c r="D30" s="85" t="n">
-        <v>4.1545</v>
+        <v>4.15198</v>
       </c>
       <c r="E30" s="69" t="n">
-        <v>0.687729</v>
+        <v>0.687885</v>
       </c>
     </row>
     <row r="31">
@@ -36650,13 +36782,13 @@
         </is>
       </c>
       <c r="C31" s="85" t="n">
-        <v>4.2025</v>
+        <v>4.19995</v>
       </c>
       <c r="D31" s="85" t="n">
-        <v>4.19026</v>
+        <v>4.18778</v>
       </c>
       <c r="E31" s="69" t="n">
-        <v>0.657309</v>
+        <v>0.657473</v>
       </c>
     </row>
     <row r="32">
@@ -36669,13 +36801,13 @@
         </is>
       </c>
       <c r="C32" s="85" t="n">
-        <v>4.2663</v>
+        <v>4.264</v>
       </c>
       <c r="D32" s="85" t="n">
-        <v>4.26517</v>
+        <v>4.26298</v>
       </c>
       <c r="E32" s="69" t="n">
-        <v>0.5990529999999999</v>
+        <v>0.599211</v>
       </c>
     </row>
     <row r="33">
@@ -36688,13 +36820,13 @@
         </is>
       </c>
       <c r="C33" s="85" t="n">
-        <v>4.35053</v>
+        <v>4.34865</v>
       </c>
       <c r="D33" s="85" t="n">
-        <v>4.36781</v>
+        <v>4.36615</v>
       </c>
       <c r="E33" s="69" t="n">
-        <v>0.51898</v>
+        <v>0.51911</v>
       </c>
     </row>
     <row r="34">
@@ -36707,13 +36839,13 @@
         </is>
       </c>
       <c r="C34" s="85" t="n">
-        <v>4.42135</v>
+        <v>4.41995</v>
       </c>
       <c r="D34" s="85" t="n">
-        <v>4.45488</v>
+        <v>4.45385</v>
       </c>
       <c r="E34" s="69" t="n">
-        <v>0.409905</v>
+        <v>0.409989</v>
       </c>
     </row>
     <row r="35">
@@ -36726,13 +36858,13 @@
         </is>
       </c>
       <c r="C35" s="85" t="n">
-        <v>4.41735</v>
+        <v>4.41615</v>
       </c>
       <c r="D35" s="85" t="n">
-        <v>4.43447</v>
+        <v>4.4337</v>
       </c>
       <c r="E35" s="69" t="n">
-        <v>0.329654</v>
+        <v>0.329718</v>
       </c>
     </row>
     <row r="36">
@@ -36745,13 +36877,13 @@
         </is>
       </c>
       <c r="C36" s="85" t="n">
-        <v>4.3778</v>
+        <v>4.37685</v>
       </c>
       <c r="D36" s="85" t="n">
-        <v>4.35382</v>
+        <v>4.35343</v>
       </c>
       <c r="E36" s="69" t="n">
-        <v>0.270507</v>
+        <v>0.270538</v>
       </c>
     </row>
     <row r="37">
@@ -36764,13 +36896,13 @@
         </is>
       </c>
       <c r="C37" s="85" t="n">
-        <v>4.2582</v>
+        <v>4.25755</v>
       </c>
       <c r="D37" s="85" t="n">
-        <v>4.10978</v>
+        <v>4.10984</v>
       </c>
       <c r="E37" s="69" t="n">
-        <v>0.192962</v>
+        <v>0.192957</v>
       </c>
     </row>
     <row r="38">
@@ -36783,13 +36915,13 @@
         </is>
       </c>
       <c r="C38" s="85" t="n">
-        <v>4.12531</v>
+        <v>4.12427</v>
       </c>
       <c r="D38" s="85" t="n">
-        <v>3.81656</v>
+        <v>3.81556</v>
       </c>
       <c r="E38" s="69" t="n">
-        <v>0.148103</v>
+        <v>0.148177</v>
       </c>
     </row>
     <row r="40">

</xml_diff>

<commit_message>
Split par rate into dynamic and hard-coded, and compare
Bootstrap!E is the DYNAMIC input: live BDP mid via SOFR_OIS_Quotes!H, falling
back to the frozen S490 mids. The curve is built from it.

Bootstrap!X is the hard-coded twin, read straight from S490_Snapshot and never
touching BDP. Y is the difference in bp.

Bloomberg_S490_Validation!P:R repeats the comparison per pillar with max and
mean at C81/C82.

Off-terminal both resolve to the same frozen mids so Y reads 0.00 across all 32
pillars, which is the wiring check. On a terminal it shows how far the live pull
has drifted from the capture.

P/Q/R compare the INPUT; L/E compare the OUTPUT. A non-zero mean in C82 means the
output diff is being measured against a different market.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
+++ b/bloomberg/USD_SOFR_Curve_Bloomberg.xlsx
@@ -10221,7 +10221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y78"/>
+  <dimension ref="A1:Y84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10376,6 +10376,21 @@
           <t>DF diff</t>
         </is>
       </c>
+      <c r="P7" s="62" t="inlineStr">
+        <is>
+          <t>Par S dynamic (%)</t>
+        </is>
+      </c>
+      <c r="Q7" s="62" t="inlineStr">
+        <is>
+          <t>Par S hard-coded (%)</t>
+        </is>
+      </c>
+      <c r="R7" s="62" t="inlineStr">
+        <is>
+          <t>d (bp)</t>
+        </is>
+      </c>
       <c r="V7" s="65" t="inlineStr">
         <is>
           <t>The Bloomberg Curve Analysis column, transcribed from the screen. Columns G/M below look up this block by maturity date, so it stays correct if rows move. Only valid while VAL_DATE = 07/21/2026.</t>
@@ -10431,6 +10446,18 @@
         <f>IF(M8="","",N8-M8)</f>
         <v/>
       </c>
+      <c r="P8" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E8),Bootstrap!E8,"")</f>
+        <v/>
+      </c>
+      <c r="Q8" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X8),Bootstrap!X8,"")</f>
+        <v/>
+      </c>
+      <c r="R8" s="89">
+        <f>IF(OR(P8="",Q8=""),"",(P8-Q8)*100)</f>
+        <v/>
+      </c>
       <c r="V8" s="62" t="inlineStr">
         <is>
           <t>Date</t>
@@ -10496,6 +10523,18 @@
         <f>IF(M9="","",N9-M9)</f>
         <v/>
       </c>
+      <c r="P9" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E9),Bootstrap!E9,"")</f>
+        <v/>
+      </c>
+      <c r="Q9" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X9),Bootstrap!X9,"")</f>
+        <v/>
+      </c>
+      <c r="R9" s="89">
+        <f>IF(OR(P9="",Q9=""),"",(P9-Q9)*100)</f>
+        <v/>
+      </c>
       <c r="V9" s="88" t="n">
         <v>46233</v>
       </c>
@@ -10553,6 +10592,18 @@
         <f>IF(M10="","",N10-M10)</f>
         <v/>
       </c>
+      <c r="P10" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E10),Bootstrap!E10,"")</f>
+        <v/>
+      </c>
+      <c r="Q10" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X10),Bootstrap!X10,"")</f>
+        <v/>
+      </c>
+      <c r="R10" s="89">
+        <f>IF(OR(P10="",Q10=""),"",(P10-Q10)*100)</f>
+        <v/>
+      </c>
       <c r="V10" s="88" t="n">
         <v>46240</v>
       </c>
@@ -10610,6 +10661,18 @@
         <f>IF(M11="","",N11-M11)</f>
         <v/>
       </c>
+      <c r="P11" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E11),Bootstrap!E11,"")</f>
+        <v/>
+      </c>
+      <c r="Q11" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X11),Bootstrap!X11,"")</f>
+        <v/>
+      </c>
+      <c r="R11" s="89">
+        <f>IF(OR(P11="",Q11=""),"",(P11-Q11)*100)</f>
+        <v/>
+      </c>
       <c r="V11" s="88" t="n">
         <v>46247</v>
       </c>
@@ -10671,6 +10734,18 @@
         <f>IF(M12="","",N12-M12)</f>
         <v/>
       </c>
+      <c r="P12" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E12),Bootstrap!E12,"")</f>
+        <v/>
+      </c>
+      <c r="Q12" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X12),Bootstrap!X12,"")</f>
+        <v/>
+      </c>
+      <c r="R12" s="89">
+        <f>IF(OR(P12="",Q12=""),"",(P12-Q12)*100)</f>
+        <v/>
+      </c>
       <c r="V12" s="88" t="n">
         <v>46258</v>
       </c>
@@ -10728,6 +10803,18 @@
         <f>IF(M13="","",N13-M13)</f>
         <v/>
       </c>
+      <c r="P13" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E13),Bootstrap!E13,"")</f>
+        <v/>
+      </c>
+      <c r="Q13" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X13),Bootstrap!X13,"")</f>
+        <v/>
+      </c>
+      <c r="R13" s="89">
+        <f>IF(OR(P13="",Q13=""),"",(P13-Q13)*100)</f>
+        <v/>
+      </c>
       <c r="V13" s="88" t="n">
         <v>46288</v>
       </c>
@@ -10785,6 +10872,18 @@
         <f>IF(M14="","",N14-M14)</f>
         <v/>
       </c>
+      <c r="P14" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E14),Bootstrap!E14,"")</f>
+        <v/>
+      </c>
+      <c r="Q14" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X14),Bootstrap!X14,"")</f>
+        <v/>
+      </c>
+      <c r="R14" s="89">
+        <f>IF(OR(P14="",Q14=""),"",(P14-Q14)*100)</f>
+        <v/>
+      </c>
       <c r="V14" s="88" t="n">
         <v>46318</v>
       </c>
@@ -10842,6 +10941,18 @@
         <f>IF(M15="","",N15-M15)</f>
         <v/>
       </c>
+      <c r="P15" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E15),Bootstrap!E15,"")</f>
+        <v/>
+      </c>
+      <c r="Q15" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X15),Bootstrap!X15,"")</f>
+        <v/>
+      </c>
+      <c r="R15" s="89">
+        <f>IF(OR(P15="",Q15=""),"",(P15-Q15)*100)</f>
+        <v/>
+      </c>
       <c r="V15" s="88" t="n">
         <v>46349</v>
       </c>
@@ -10899,6 +11010,18 @@
         <f>IF(M16="","",N16-M16)</f>
         <v/>
       </c>
+      <c r="P16" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E16),Bootstrap!E16,"")</f>
+        <v/>
+      </c>
+      <c r="Q16" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X16),Bootstrap!X16,"")</f>
+        <v/>
+      </c>
+      <c r="R16" s="89">
+        <f>IF(OR(P16="",Q16=""),"",(P16-Q16)*100)</f>
+        <v/>
+      </c>
       <c r="V16" s="88" t="n">
         <v>46379</v>
       </c>
@@ -10956,6 +11079,18 @@
         <f>IF(M17="","",N17-M17)</f>
         <v/>
       </c>
+      <c r="P17" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E17),Bootstrap!E17,"")</f>
+        <v/>
+      </c>
+      <c r="Q17" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X17),Bootstrap!X17,"")</f>
+        <v/>
+      </c>
+      <c r="R17" s="89">
+        <f>IF(OR(P17="",Q17=""),"",(P17-Q17)*100)</f>
+        <v/>
+      </c>
       <c r="V17" s="88" t="n">
         <v>46412</v>
       </c>
@@ -11013,6 +11148,18 @@
         <f>IF(M18="","",N18-M18)</f>
         <v/>
       </c>
+      <c r="P18" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E18),Bootstrap!E18,"")</f>
+        <v/>
+      </c>
+      <c r="Q18" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X18),Bootstrap!X18,"")</f>
+        <v/>
+      </c>
+      <c r="R18" s="89">
+        <f>IF(OR(P18="",Q18=""),"",(P18-Q18)*100)</f>
+        <v/>
+      </c>
       <c r="V18" s="88" t="n">
         <v>46441</v>
       </c>
@@ -11070,6 +11217,18 @@
         <f>IF(M19="","",N19-M19)</f>
         <v/>
       </c>
+      <c r="P19" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E19),Bootstrap!E19,"")</f>
+        <v/>
+      </c>
+      <c r="Q19" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X19),Bootstrap!X19,"")</f>
+        <v/>
+      </c>
+      <c r="R19" s="89">
+        <f>IF(OR(P19="",Q19=""),"",(P19-Q19)*100)</f>
+        <v/>
+      </c>
       <c r="V19" s="88" t="n">
         <v>46469</v>
       </c>
@@ -11127,6 +11286,18 @@
         <f>IF(M20="","",N20-M20)</f>
         <v/>
       </c>
+      <c r="P20" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E20),Bootstrap!E20,"")</f>
+        <v/>
+      </c>
+      <c r="Q20" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X20),Bootstrap!X20,"")</f>
+        <v/>
+      </c>
+      <c r="R20" s="89">
+        <f>IF(OR(P20="",Q20=""),"",(P20-Q20)*100)</f>
+        <v/>
+      </c>
       <c r="V20" s="88" t="n">
         <v>46500</v>
       </c>
@@ -11184,6 +11355,18 @@
         <f>IF(M21="","",N21-M21)</f>
         <v/>
       </c>
+      <c r="P21" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E21),Bootstrap!E21,"")</f>
+        <v/>
+      </c>
+      <c r="Q21" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X21),Bootstrap!X21,"")</f>
+        <v/>
+      </c>
+      <c r="R21" s="89">
+        <f>IF(OR(P21="",Q21=""),"",(P21-Q21)*100)</f>
+        <v/>
+      </c>
       <c r="V21" s="88" t="n">
         <v>46531</v>
       </c>
@@ -11241,6 +11424,18 @@
         <f>IF(M22="","",N22-M22)</f>
         <v/>
       </c>
+      <c r="P22" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E22),Bootstrap!E22,"")</f>
+        <v/>
+      </c>
+      <c r="Q22" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X22),Bootstrap!X22,"")</f>
+        <v/>
+      </c>
+      <c r="R22" s="89">
+        <f>IF(OR(P22="",Q22=""),"",(P22-Q22)*100)</f>
+        <v/>
+      </c>
       <c r="V22" s="88" t="n">
         <v>46561</v>
       </c>
@@ -11298,6 +11493,18 @@
         <f>IF(M23="","",N23-M23)</f>
         <v/>
       </c>
+      <c r="P23" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E23),Bootstrap!E23,"")</f>
+        <v/>
+      </c>
+      <c r="Q23" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X23),Bootstrap!X23,"")</f>
+        <v/>
+      </c>
+      <c r="R23" s="89">
+        <f>IF(OR(P23="",Q23=""),"",(P23-Q23)*100)</f>
+        <v/>
+      </c>
       <c r="V23" s="88" t="n">
         <v>46591</v>
       </c>
@@ -11355,6 +11562,18 @@
         <f>IF(M24="","",N24-M24)</f>
         <v/>
       </c>
+      <c r="P24" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E24),Bootstrap!E24,"")</f>
+        <v/>
+      </c>
+      <c r="Q24" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X24),Bootstrap!X24,"")</f>
+        <v/>
+      </c>
+      <c r="R24" s="89">
+        <f>IF(OR(P24="",Q24=""),"",(P24-Q24)*100)</f>
+        <v/>
+      </c>
       <c r="V24" s="88" t="n">
         <v>46776</v>
       </c>
@@ -11412,6 +11631,18 @@
         <f>IF(M25="","",N25-M25)</f>
         <v/>
       </c>
+      <c r="P25" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E25),Bootstrap!E25,"")</f>
+        <v/>
+      </c>
+      <c r="Q25" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X25),Bootstrap!X25,"")</f>
+        <v/>
+      </c>
+      <c r="R25" s="89">
+        <f>IF(OR(P25="",Q25=""),"",(P25-Q25)*100)</f>
+        <v/>
+      </c>
       <c r="V25" s="88" t="n">
         <v>46958</v>
       </c>
@@ -11469,6 +11700,18 @@
         <f>IF(M26="","",N26-M26)</f>
         <v/>
       </c>
+      <c r="P26" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E26),Bootstrap!E26,"")</f>
+        <v/>
+      </c>
+      <c r="Q26" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X26),Bootstrap!X26,"")</f>
+        <v/>
+      </c>
+      <c r="R26" s="89">
+        <f>IF(OR(P26="",Q26=""),"",(P26-Q26)*100)</f>
+        <v/>
+      </c>
       <c r="V26" s="88" t="n">
         <v>47322</v>
       </c>
@@ -11526,6 +11769,18 @@
         <f>IF(M27="","",N27-M27)</f>
         <v/>
       </c>
+      <c r="P27" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E27),Bootstrap!E27,"")</f>
+        <v/>
+      </c>
+      <c r="Q27" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X27),Bootstrap!X27,"")</f>
+        <v/>
+      </c>
+      <c r="R27" s="89">
+        <f>IF(OR(P27="",Q27=""),"",(P27-Q27)*100)</f>
+        <v/>
+      </c>
       <c r="V27" s="88" t="n">
         <v>47687</v>
       </c>
@@ -11583,6 +11838,18 @@
         <f>IF(M28="","",N28-M28)</f>
         <v/>
       </c>
+      <c r="P28" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E28),Bootstrap!E28,"")</f>
+        <v/>
+      </c>
+      <c r="Q28" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X28),Bootstrap!X28,"")</f>
+        <v/>
+      </c>
+      <c r="R28" s="89">
+        <f>IF(OR(P28="",Q28=""),"",(P28-Q28)*100)</f>
+        <v/>
+      </c>
       <c r="V28" s="88" t="n">
         <v>48052</v>
       </c>
@@ -11640,6 +11907,18 @@
         <f>IF(M29="","",N29-M29)</f>
         <v/>
       </c>
+      <c r="P29" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E29),Bootstrap!E29,"")</f>
+        <v/>
+      </c>
+      <c r="Q29" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X29),Bootstrap!X29,"")</f>
+        <v/>
+      </c>
+      <c r="R29" s="89">
+        <f>IF(OR(P29="",Q29=""),"",(P29-Q29)*100)</f>
+        <v/>
+      </c>
       <c r="V29" s="88" t="n">
         <v>48418</v>
       </c>
@@ -11697,6 +11976,18 @@
         <f>IF(M30="","",N30-M30)</f>
         <v/>
       </c>
+      <c r="P30" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E30),Bootstrap!E30,"")</f>
+        <v/>
+      </c>
+      <c r="Q30" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X30),Bootstrap!X30,"")</f>
+        <v/>
+      </c>
+      <c r="R30" s="89">
+        <f>IF(OR(P30="",Q30=""),"",(P30-Q30)*100)</f>
+        <v/>
+      </c>
       <c r="V30" s="88" t="n">
         <v>48785</v>
       </c>
@@ -11754,6 +12045,18 @@
         <f>IF(M31="","",N31-M31)</f>
         <v/>
       </c>
+      <c r="P31" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E31),Bootstrap!E31,"")</f>
+        <v/>
+      </c>
+      <c r="Q31" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X31),Bootstrap!X31,"")</f>
+        <v/>
+      </c>
+      <c r="R31" s="89">
+        <f>IF(OR(P31="",Q31=""),"",(P31-Q31)*100)</f>
+        <v/>
+      </c>
       <c r="V31" s="88" t="n">
         <v>49149</v>
       </c>
@@ -11811,6 +12114,18 @@
         <f>IF(M32="","",N32-M32)</f>
         <v/>
       </c>
+      <c r="P32" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E32),Bootstrap!E32,"")</f>
+        <v/>
+      </c>
+      <c r="Q32" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X32),Bootstrap!X32,"")</f>
+        <v/>
+      </c>
+      <c r="R32" s="89">
+        <f>IF(OR(P32="",Q32=""),"",(P32-Q32)*100)</f>
+        <v/>
+      </c>
       <c r="V32" s="88" t="n">
         <v>49513</v>
       </c>
@@ -11866,6 +12181,18 @@
         <f>IF(M33="","",N33-M33)</f>
         <v/>
       </c>
+      <c r="P33" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E33),Bootstrap!E33,"")</f>
+        <v/>
+      </c>
+      <c r="Q33" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X33),Bootstrap!X33,"")</f>
+        <v/>
+      </c>
+      <c r="R33" s="89">
+        <f>IF(OR(P33="",Q33=""),"",(P33-Q33)*100)</f>
+        <v/>
+      </c>
       <c r="V33" s="88" t="n">
         <v>49879</v>
       </c>
@@ -11923,6 +12250,18 @@
         <f>IF(M34="","",N34-M34)</f>
         <v/>
       </c>
+      <c r="P34" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E34),Bootstrap!E34,"")</f>
+        <v/>
+      </c>
+      <c r="Q34" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X34),Bootstrap!X34,"")</f>
+        <v/>
+      </c>
+      <c r="R34" s="89">
+        <f>IF(OR(P34="",Q34=""),"",(P34-Q34)*100)</f>
+        <v/>
+      </c>
       <c r="V34" s="88" t="n">
         <v>50609</v>
       </c>
@@ -11978,6 +12317,18 @@
         <f>IF(M35="","",N35-M35)</f>
         <v/>
       </c>
+      <c r="P35" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E35),Bootstrap!E35,"")</f>
+        <v/>
+      </c>
+      <c r="Q35" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X35),Bootstrap!X35,"")</f>
+        <v/>
+      </c>
+      <c r="R35" s="89">
+        <f>IF(OR(P35="",Q35=""),"",(P35-Q35)*100)</f>
+        <v/>
+      </c>
       <c r="V35" s="88" t="n">
         <v>51705</v>
       </c>
@@ -12033,6 +12384,18 @@
         <f>IF(M36="","",N36-M36)</f>
         <v/>
       </c>
+      <c r="P36" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E36),Bootstrap!E36,"")</f>
+        <v/>
+      </c>
+      <c r="Q36" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X36),Bootstrap!X36,"")</f>
+        <v/>
+      </c>
+      <c r="R36" s="89">
+        <f>IF(OR(P36="",Q36=""),"",(P36-Q36)*100)</f>
+        <v/>
+      </c>
       <c r="V36" s="88" t="n">
         <v>53531</v>
       </c>
@@ -12090,6 +12453,18 @@
         <f>IF(M37="","",N37-M37)</f>
         <v/>
       </c>
+      <c r="P37" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E37),Bootstrap!E37,"")</f>
+        <v/>
+      </c>
+      <c r="Q37" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X37),Bootstrap!X37,"")</f>
+        <v/>
+      </c>
+      <c r="R37" s="89">
+        <f>IF(OR(P37="",Q37=""),"",(P37-Q37)*100)</f>
+        <v/>
+      </c>
       <c r="V37" s="88" t="n">
         <v>55358</v>
       </c>
@@ -12145,6 +12520,18 @@
         <f>IF(M38="","",N38-M38)</f>
         <v/>
       </c>
+      <c r="P38" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E38),Bootstrap!E38,"")</f>
+        <v/>
+      </c>
+      <c r="Q38" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X38),Bootstrap!X38,"")</f>
+        <v/>
+      </c>
+      <c r="R38" s="89">
+        <f>IF(OR(P38="",Q38=""),"",(P38-Q38)*100)</f>
+        <v/>
+      </c>
       <c r="V38" s="88" t="n">
         <v>57185</v>
       </c>
@@ -12200,6 +12587,18 @@
         <f>IF(M39="","",N39-M39)</f>
         <v/>
       </c>
+      <c r="P39" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E39),Bootstrap!E39,"")</f>
+        <v/>
+      </c>
+      <c r="Q39" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X39),Bootstrap!X39,"")</f>
+        <v/>
+      </c>
+      <c r="R39" s="89">
+        <f>IF(OR(P39="",Q39=""),"",(P39-Q39)*100)</f>
+        <v/>
+      </c>
       <c r="V39" s="88" t="n">
         <v>60836</v>
       </c>
@@ -12255,6 +12654,18 @@
         <f>IF(M40="","",N40-M40)</f>
         <v/>
       </c>
+      <c r="P40" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E40),Bootstrap!E40,"")</f>
+        <v/>
+      </c>
+      <c r="Q40" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X40),Bootstrap!X40,"")</f>
+        <v/>
+      </c>
+      <c r="R40" s="89">
+        <f>IF(OR(P40="",Q40=""),"",(P40-Q40)*100)</f>
+        <v/>
+      </c>
       <c r="V40" s="88" t="n">
         <v>64489</v>
       </c>
@@ -12310,6 +12721,18 @@
         <f>IF(M41="","",N41-M41)</f>
         <v/>
       </c>
+      <c r="P41" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E41),Bootstrap!E41,"")</f>
+        <v/>
+      </c>
+      <c r="Q41" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X41),Bootstrap!X41,"")</f>
+        <v/>
+      </c>
+      <c r="R41" s="89">
+        <f>IF(OR(P41="",Q41=""),"",(P41-Q41)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6">
@@ -12355,6 +12778,18 @@
         <f>IF(M42="","",N42-M42)</f>
         <v/>
       </c>
+      <c r="P42" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E42),Bootstrap!E42,"")</f>
+        <v/>
+      </c>
+      <c r="Q42" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X42),Bootstrap!X42,"")</f>
+        <v/>
+      </c>
+      <c r="R42" s="89">
+        <f>IF(OR(P42="",Q42=""),"",(P42-Q42)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6">
@@ -12398,6 +12833,18 @@
         <f>IF(M43="","",N43-M43)</f>
         <v/>
       </c>
+      <c r="P43" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E43),Bootstrap!E43,"")</f>
+        <v/>
+      </c>
+      <c r="Q43" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X43),Bootstrap!X43,"")</f>
+        <v/>
+      </c>
+      <c r="R43" s="89">
+        <f>IF(OR(P43="",Q43=""),"",(P43-Q43)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6">
@@ -12441,6 +12888,18 @@
         <f>IF(M44="","",N44-M44)</f>
         <v/>
       </c>
+      <c r="P44" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E44),Bootstrap!E44,"")</f>
+        <v/>
+      </c>
+      <c r="Q44" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X44),Bootstrap!X44,"")</f>
+        <v/>
+      </c>
+      <c r="R44" s="89">
+        <f>IF(OR(P44="",Q44=""),"",(P44-Q44)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6">
@@ -12484,6 +12943,18 @@
         <f>IF(M45="","",N45-M45)</f>
         <v/>
       </c>
+      <c r="P45" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E45),Bootstrap!E45,"")</f>
+        <v/>
+      </c>
+      <c r="Q45" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X45),Bootstrap!X45,"")</f>
+        <v/>
+      </c>
+      <c r="R45" s="89">
+        <f>IF(OR(P45="",Q45=""),"",(P45-Q45)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6">
@@ -12527,6 +12998,18 @@
         <f>IF(M46="","",N46-M46)</f>
         <v/>
       </c>
+      <c r="P46" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E46),Bootstrap!E46,"")</f>
+        <v/>
+      </c>
+      <c r="Q46" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X46),Bootstrap!X46,"")</f>
+        <v/>
+      </c>
+      <c r="R46" s="89">
+        <f>IF(OR(P46="",Q46=""),"",(P46-Q46)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6">
@@ -12572,6 +13055,18 @@
         <f>IF(M47="","",N47-M47)</f>
         <v/>
       </c>
+      <c r="P47" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E47),Bootstrap!E47,"")</f>
+        <v/>
+      </c>
+      <c r="Q47" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X47),Bootstrap!X47,"")</f>
+        <v/>
+      </c>
+      <c r="R47" s="89">
+        <f>IF(OR(P47="",Q47=""),"",(P47-Q47)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6">
@@ -12615,6 +13110,18 @@
         <f>IF(M48="","",N48-M48)</f>
         <v/>
       </c>
+      <c r="P48" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E48),Bootstrap!E48,"")</f>
+        <v/>
+      </c>
+      <c r="Q48" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X48),Bootstrap!X48,"")</f>
+        <v/>
+      </c>
+      <c r="R48" s="89">
+        <f>IF(OR(P48="",Q48=""),"",(P48-Q48)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6">
@@ -12658,6 +13165,18 @@
         <f>IF(M49="","",N49-M49)</f>
         <v/>
       </c>
+      <c r="P49" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E49),Bootstrap!E49,"")</f>
+        <v/>
+      </c>
+      <c r="Q49" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X49),Bootstrap!X49,"")</f>
+        <v/>
+      </c>
+      <c r="R49" s="89">
+        <f>IF(OR(P49="",Q49=""),"",(P49-Q49)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6">
@@ -12701,6 +13220,18 @@
         <f>IF(M50="","",N50-M50)</f>
         <v/>
       </c>
+      <c r="P50" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E50),Bootstrap!E50,"")</f>
+        <v/>
+      </c>
+      <c r="Q50" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X50),Bootstrap!X50,"")</f>
+        <v/>
+      </c>
+      <c r="R50" s="89">
+        <f>IF(OR(P50="",Q50=""),"",(P50-Q50)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6">
@@ -12744,6 +13275,18 @@
         <f>IF(M51="","",N51-M51)</f>
         <v/>
       </c>
+      <c r="P51" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E51),Bootstrap!E51,"")</f>
+        <v/>
+      </c>
+      <c r="Q51" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X51),Bootstrap!X51,"")</f>
+        <v/>
+      </c>
+      <c r="R51" s="89">
+        <f>IF(OR(P51="",Q51=""),"",(P51-Q51)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6">
@@ -12789,6 +13332,18 @@
         <f>IF(M52="","",N52-M52)</f>
         <v/>
       </c>
+      <c r="P52" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E52),Bootstrap!E52,"")</f>
+        <v/>
+      </c>
+      <c r="Q52" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X52),Bootstrap!X52,"")</f>
+        <v/>
+      </c>
+      <c r="R52" s="89">
+        <f>IF(OR(P52="",Q52=""),"",(P52-Q52)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6">
@@ -12832,6 +13387,18 @@
         <f>IF(M53="","",N53-M53)</f>
         <v/>
       </c>
+      <c r="P53" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E53),Bootstrap!E53,"")</f>
+        <v/>
+      </c>
+      <c r="Q53" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X53),Bootstrap!X53,"")</f>
+        <v/>
+      </c>
+      <c r="R53" s="89">
+        <f>IF(OR(P53="",Q53=""),"",(P53-Q53)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="6">
@@ -12875,6 +13442,18 @@
         <f>IF(M54="","",N54-M54)</f>
         <v/>
       </c>
+      <c r="P54" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E54),Bootstrap!E54,"")</f>
+        <v/>
+      </c>
+      <c r="Q54" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X54),Bootstrap!X54,"")</f>
+        <v/>
+      </c>
+      <c r="R54" s="89">
+        <f>IF(OR(P54="",Q54=""),"",(P54-Q54)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6">
@@ -12918,6 +13497,18 @@
         <f>IF(M55="","",N55-M55)</f>
         <v/>
       </c>
+      <c r="P55" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E55),Bootstrap!E55,"")</f>
+        <v/>
+      </c>
+      <c r="Q55" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X55),Bootstrap!X55,"")</f>
+        <v/>
+      </c>
+      <c r="R55" s="89">
+        <f>IF(OR(P55="",Q55=""),"",(P55-Q55)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="6">
@@ -12961,6 +13552,18 @@
         <f>IF(M56="","",N56-M56)</f>
         <v/>
       </c>
+      <c r="P56" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E56),Bootstrap!E56,"")</f>
+        <v/>
+      </c>
+      <c r="Q56" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X56),Bootstrap!X56,"")</f>
+        <v/>
+      </c>
+      <c r="R56" s="89">
+        <f>IF(OR(P56="",Q56=""),"",(P56-Q56)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6">
@@ -13004,6 +13607,18 @@
         <f>IF(M57="","",N57-M57)</f>
         <v/>
       </c>
+      <c r="P57" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E57),Bootstrap!E57,"")</f>
+        <v/>
+      </c>
+      <c r="Q57" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X57),Bootstrap!X57,"")</f>
+        <v/>
+      </c>
+      <c r="R57" s="89">
+        <f>IF(OR(P57="",Q57=""),"",(P57-Q57)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="6">
@@ -13047,6 +13662,18 @@
         <f>IF(M58="","",N58-M58)</f>
         <v/>
       </c>
+      <c r="P58" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E58),Bootstrap!E58,"")</f>
+        <v/>
+      </c>
+      <c r="Q58" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X58),Bootstrap!X58,"")</f>
+        <v/>
+      </c>
+      <c r="R58" s="89">
+        <f>IF(OR(P58="",Q58=""),"",(P58-Q58)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="6">
@@ -13090,6 +13717,18 @@
         <f>IF(M59="","",N59-M59)</f>
         <v/>
       </c>
+      <c r="P59" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E59),Bootstrap!E59,"")</f>
+        <v/>
+      </c>
+      <c r="Q59" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X59),Bootstrap!X59,"")</f>
+        <v/>
+      </c>
+      <c r="R59" s="89">
+        <f>IF(OR(P59="",Q59=""),"",(P59-Q59)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="6">
@@ -13133,6 +13772,18 @@
         <f>IF(M60="","",N60-M60)</f>
         <v/>
       </c>
+      <c r="P60" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E60),Bootstrap!E60,"")</f>
+        <v/>
+      </c>
+      <c r="Q60" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X60),Bootstrap!X60,"")</f>
+        <v/>
+      </c>
+      <c r="R60" s="89">
+        <f>IF(OR(P60="",Q60=""),"",(P60-Q60)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="6">
@@ -13176,6 +13827,18 @@
         <f>IF(M61="","",N61-M61)</f>
         <v/>
       </c>
+      <c r="P61" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E61),Bootstrap!E61,"")</f>
+        <v/>
+      </c>
+      <c r="Q61" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X61),Bootstrap!X61,"")</f>
+        <v/>
+      </c>
+      <c r="R61" s="89">
+        <f>IF(OR(P61="",Q61=""),"",(P61-Q61)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="6">
@@ -13221,6 +13884,18 @@
         <f>IF(M62="","",N62-M62)</f>
         <v/>
       </c>
+      <c r="P62" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E62),Bootstrap!E62,"")</f>
+        <v/>
+      </c>
+      <c r="Q62" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X62),Bootstrap!X62,"")</f>
+        <v/>
+      </c>
+      <c r="R62" s="89">
+        <f>IF(OR(P62="",Q62=""),"",(P62-Q62)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="6">
@@ -13264,6 +13939,18 @@
         <f>IF(M63="","",N63-M63)</f>
         <v/>
       </c>
+      <c r="P63" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E63),Bootstrap!E63,"")</f>
+        <v/>
+      </c>
+      <c r="Q63" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X63),Bootstrap!X63,"")</f>
+        <v/>
+      </c>
+      <c r="R63" s="89">
+        <f>IF(OR(P63="",Q63=""),"",(P63-Q63)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="6">
@@ -13307,6 +13994,18 @@
         <f>IF(M64="","",N64-M64)</f>
         <v/>
       </c>
+      <c r="P64" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E64),Bootstrap!E64,"")</f>
+        <v/>
+      </c>
+      <c r="Q64" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X64),Bootstrap!X64,"")</f>
+        <v/>
+      </c>
+      <c r="R64" s="89">
+        <f>IF(OR(P64="",Q64=""),"",(P64-Q64)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="6">
@@ -13350,6 +14049,18 @@
         <f>IF(M65="","",N65-M65)</f>
         <v/>
       </c>
+      <c r="P65" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E65),Bootstrap!E65,"")</f>
+        <v/>
+      </c>
+      <c r="Q65" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X65),Bootstrap!X65,"")</f>
+        <v/>
+      </c>
+      <c r="R65" s="89">
+        <f>IF(OR(P65="",Q65=""),"",(P65-Q65)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="6">
@@ -13393,6 +14104,18 @@
         <f>IF(M66="","",N66-M66)</f>
         <v/>
       </c>
+      <c r="P66" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E66),Bootstrap!E66,"")</f>
+        <v/>
+      </c>
+      <c r="Q66" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X66),Bootstrap!X66,"")</f>
+        <v/>
+      </c>
+      <c r="R66" s="89">
+        <f>IF(OR(P66="",Q66=""),"",(P66-Q66)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="6">
@@ -13436,6 +14159,18 @@
         <f>IF(M67="","",N67-M67)</f>
         <v/>
       </c>
+      <c r="P67" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E67),Bootstrap!E67,"")</f>
+        <v/>
+      </c>
+      <c r="Q67" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X67),Bootstrap!X67,"")</f>
+        <v/>
+      </c>
+      <c r="R67" s="89">
+        <f>IF(OR(P67="",Q67=""),"",(P67-Q67)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="6">
@@ -13479,6 +14214,18 @@
         <f>IF(M68="","",N68-M68)</f>
         <v/>
       </c>
+      <c r="P68" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E68),Bootstrap!E68,"")</f>
+        <v/>
+      </c>
+      <c r="Q68" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X68),Bootstrap!X68,"")</f>
+        <v/>
+      </c>
+      <c r="R68" s="89">
+        <f>IF(OR(P68="",Q68=""),"",(P68-Q68)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="6">
@@ -13522,6 +14269,18 @@
         <f>IF(M69="","",N69-M69)</f>
         <v/>
       </c>
+      <c r="P69" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E69),Bootstrap!E69,"")</f>
+        <v/>
+      </c>
+      <c r="Q69" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X69),Bootstrap!X69,"")</f>
+        <v/>
+      </c>
+      <c r="R69" s="89">
+        <f>IF(OR(P69="",Q69=""),"",(P69-Q69)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="6">
@@ -13565,6 +14324,18 @@
         <f>IF(M70="","",N70-M70)</f>
         <v/>
       </c>
+      <c r="P70" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E70),Bootstrap!E70,"")</f>
+        <v/>
+      </c>
+      <c r="Q70" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X70),Bootstrap!X70,"")</f>
+        <v/>
+      </c>
+      <c r="R70" s="89">
+        <f>IF(OR(P70="",Q70=""),"",(P70-Q70)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="6">
@@ -13608,6 +14379,18 @@
         <f>IF(M71="","",N71-M71)</f>
         <v/>
       </c>
+      <c r="P71" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E71),Bootstrap!E71,"")</f>
+        <v/>
+      </c>
+      <c r="Q71" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X71),Bootstrap!X71,"")</f>
+        <v/>
+      </c>
+      <c r="R71" s="89">
+        <f>IF(OR(P71="",Q71=""),"",(P71-Q71)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="6">
@@ -13653,6 +14436,18 @@
         <f>IF(M72="","",N72-M72)</f>
         <v/>
       </c>
+      <c r="P72" s="84">
+        <f>IF(ISNUMBER(Bootstrap!E72),Bootstrap!E72,"")</f>
+        <v/>
+      </c>
+      <c r="Q72" s="84">
+        <f>IF(ISNUMBER(Bootstrap!X72),Bootstrap!X72,"")</f>
+        <v/>
+      </c>
+      <c r="R72" s="89">
+        <f>IF(OR(P72="",Q72=""),"",(P72-Q72)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="67" t="inlineStr">
@@ -13703,6 +14498,46 @@
       <c r="A78" s="65" t="inlineStr">
         <is>
           <t>Col L = frozen S490 zeros, hard-coded 07/21/26. Col E compares our bootstrap to it. D (live BDS) and G (snapshot) are secondary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="67" t="inlineStr">
+        <is>
+          <t>Input check: par rates</t>
+        </is>
+      </c>
+      <c r="C80" s="87">
+        <f>COUNT(R8:R72)&amp;" pillars"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="67" t="inlineStr">
+        <is>
+          <t>Max |d| dynamic vs hard-coded (bp)</t>
+        </is>
+      </c>
+      <c r="C81" s="90">
+        <f>IF(COUNT(R8:R72)=0,"",MAX(MAX(R8:R72),-MIN(R8:R72)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="67" t="inlineStr">
+        <is>
+          <t>Mean d (bp)</t>
+        </is>
+      </c>
+      <c r="C82" s="90">
+        <f>IF(COUNT(R8:R72)=0,"",AVERAGE(R8:R72))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="65" t="inlineStr">
+        <is>
+          <t>P/Q/R compare the INPUT. L/E compare the OUTPUT. A non-zero mean in C82 means the live pull has drifted from the frozen capture, so the output diff in E is measuring against a different market.</t>
         </is>
       </c>
     </row>
@@ -41164,6 +41999,11 @@
           <t>Working — fixed-leg PV = float-leg PV (par swap)</t>
         </is>
       </c>
+      <c r="X6" s="65" t="inlineStr">
+        <is>
+          <t>from S490_Snapshot, never BDP</t>
+        </is>
+      </c>
       <c r="AA6" s="65" t="inlineStr">
         <is>
           <t>Targets live on S490_Snapshot.</t>
@@ -41191,9 +42031,9 @@
           <t>tau0 spot→mat</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
-        <is>
-          <t>Par rate S (%)</t>
+      <c r="E7" s="92" t="inlineStr">
+        <is>
+          <t>Par rate S (%) dynamic</t>
         </is>
       </c>
       <c r="F7" s="20" t="inlineStr">
@@ -41279,6 +42119,16 @@
       <c r="W7" s="92" t="inlineStr">
         <is>
           <t>d DF</t>
+        </is>
+      </c>
+      <c r="X7" s="62" t="inlineStr">
+        <is>
+          <t>Par rate S hard-coded (%)</t>
+        </is>
+      </c>
+      <c r="Y7" s="62" t="inlineStr">
+        <is>
+          <t>d dynamic - hard (bp)</t>
         </is>
       </c>
       <c r="AA7" s="62" t="n"/>
@@ -41364,6 +42214,14 @@
         <f>IF(U8="","",H8-U8)</f>
         <v/>
       </c>
+      <c r="X8" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B8,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y8" s="89">
+        <f>IF(OR(X8="",NOT(ISNUMBER(E8))),"",(E8-X8)*100)</f>
+        <v/>
+      </c>
       <c r="AA8" s="88" t="n"/>
       <c r="AB8" s="85" t="n"/>
       <c r="AC8" s="85" t="n"/>
@@ -41448,6 +42306,14 @@
         <f>IF(U9="","",H9-U9)</f>
         <v/>
       </c>
+      <c r="X9" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B9,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y9" s="89">
+        <f>IF(OR(X9="",NOT(ISNUMBER(E9))),"",(E9-X9)*100)</f>
+        <v/>
+      </c>
       <c r="AA9" s="88" t="n"/>
       <c r="AB9" s="85" t="n"/>
       <c r="AC9" s="85" t="n"/>
@@ -41532,6 +42398,14 @@
         <f>IF(U10="","",H10-U10)</f>
         <v/>
       </c>
+      <c r="X10" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B10,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y10" s="89">
+        <f>IF(OR(X10="",NOT(ISNUMBER(E10))),"",(E10-X10)*100)</f>
+        <v/>
+      </c>
       <c r="AA10" s="88" t="n"/>
       <c r="AB10" s="85" t="n"/>
       <c r="AC10" s="85" t="n"/>
@@ -41616,6 +42490,14 @@
         <f>IF(U11="","",H11-U11)</f>
         <v/>
       </c>
+      <c r="X11" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B11,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y11" s="89">
+        <f>IF(OR(X11="",NOT(ISNUMBER(E11))),"",(E11-X11)*100)</f>
+        <v/>
+      </c>
       <c r="AA11" s="88" t="n"/>
       <c r="AB11" s="85" t="n"/>
       <c r="AC11" s="85" t="n"/>
@@ -41700,6 +42582,14 @@
         <f>IF(U12="","",H12-U12)</f>
         <v/>
       </c>
+      <c r="X12" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B12,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y12" s="89">
+        <f>IF(OR(X12="",NOT(ISNUMBER(E12))),"",(E12-X12)*100)</f>
+        <v/>
+      </c>
       <c r="AA12" s="88" t="n"/>
       <c r="AB12" s="85" t="n"/>
       <c r="AC12" s="85" t="n"/>
@@ -41784,6 +42674,14 @@
         <f>IF(U13="","",H13-U13)</f>
         <v/>
       </c>
+      <c r="X13" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B13,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y13" s="89">
+        <f>IF(OR(X13="",NOT(ISNUMBER(E13))),"",(E13-X13)*100)</f>
+        <v/>
+      </c>
       <c r="AA13" s="88" t="n"/>
       <c r="AB13" s="85" t="n"/>
       <c r="AC13" s="85" t="n"/>
@@ -41868,6 +42766,14 @@
         <f>IF(U14="","",H14-U14)</f>
         <v/>
       </c>
+      <c r="X14" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B14,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y14" s="89">
+        <f>IF(OR(X14="",NOT(ISNUMBER(E14))),"",(E14-X14)*100)</f>
+        <v/>
+      </c>
       <c r="AA14" s="88" t="n"/>
       <c r="AB14" s="85" t="n"/>
       <c r="AC14" s="85" t="n"/>
@@ -41952,6 +42858,14 @@
         <f>IF(U15="","",H15-U15)</f>
         <v/>
       </c>
+      <c r="X15" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B15,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y15" s="89">
+        <f>IF(OR(X15="",NOT(ISNUMBER(E15))),"",(E15-X15)*100)</f>
+        <v/>
+      </c>
       <c r="AA15" s="88" t="n"/>
       <c r="AB15" s="85" t="n"/>
       <c r="AC15" s="85" t="n"/>
@@ -42036,6 +42950,14 @@
         <f>IF(U16="","",H16-U16)</f>
         <v/>
       </c>
+      <c r="X16" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B16,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y16" s="89">
+        <f>IF(OR(X16="",NOT(ISNUMBER(E16))),"",(E16-X16)*100)</f>
+        <v/>
+      </c>
       <c r="AA16" s="88" t="n"/>
       <c r="AB16" s="85" t="n"/>
       <c r="AC16" s="85" t="n"/>
@@ -42120,6 +43042,14 @@
         <f>IF(U17="","",H17-U17)</f>
         <v/>
       </c>
+      <c r="X17" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B17,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y17" s="89">
+        <f>IF(OR(X17="",NOT(ISNUMBER(E17))),"",(E17-X17)*100)</f>
+        <v/>
+      </c>
       <c r="AA17" s="88" t="n"/>
       <c r="AB17" s="85" t="n"/>
       <c r="AC17" s="85" t="n"/>
@@ -42204,6 +43134,14 @@
         <f>IF(U18="","",H18-U18)</f>
         <v/>
       </c>
+      <c r="X18" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B18,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y18" s="89">
+        <f>IF(OR(X18="",NOT(ISNUMBER(E18))),"",(E18-X18)*100)</f>
+        <v/>
+      </c>
       <c r="AA18" s="88" t="n"/>
       <c r="AB18" s="85" t="n"/>
       <c r="AC18" s="85" t="n"/>
@@ -42288,6 +43226,14 @@
         <f>IF(U19="","",H19-U19)</f>
         <v/>
       </c>
+      <c r="X19" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B19,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y19" s="89">
+        <f>IF(OR(X19="",NOT(ISNUMBER(E19))),"",(E19-X19)*100)</f>
+        <v/>
+      </c>
       <c r="AA19" s="88" t="n"/>
       <c r="AB19" s="85" t="n"/>
       <c r="AC19" s="85" t="n"/>
@@ -42372,6 +43318,14 @@
         <f>IF(U20="","",H20-U20)</f>
         <v/>
       </c>
+      <c r="X20" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B20,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y20" s="89">
+        <f>IF(OR(X20="",NOT(ISNUMBER(E20))),"",(E20-X20)*100)</f>
+        <v/>
+      </c>
       <c r="AA20" s="88" t="n"/>
       <c r="AB20" s="85" t="n"/>
       <c r="AC20" s="85" t="n"/>
@@ -42456,6 +43410,14 @@
         <f>IF(U21="","",H21-U21)</f>
         <v/>
       </c>
+      <c r="X21" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B21,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y21" s="89">
+        <f>IF(OR(X21="",NOT(ISNUMBER(E21))),"",(E21-X21)*100)</f>
+        <v/>
+      </c>
       <c r="AA21" s="88" t="n"/>
       <c r="AB21" s="85" t="n"/>
       <c r="AC21" s="85" t="n"/>
@@ -42544,6 +43506,14 @@
         <f>IF(U22="","",H22-U22)</f>
         <v/>
       </c>
+      <c r="X22" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B22,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y22" s="89">
+        <f>IF(OR(X22="",NOT(ISNUMBER(E22))),"",(E22-X22)*100)</f>
+        <v/>
+      </c>
       <c r="AA22" s="88" t="n"/>
       <c r="AB22" s="85" t="n"/>
       <c r="AC22" s="85" t="n"/>
@@ -42631,6 +43601,14 @@
         <f>IF(U23="","",H23-U23)</f>
         <v/>
       </c>
+      <c r="X23" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B23,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y23" s="89">
+        <f>IF(OR(X23="",NOT(ISNUMBER(E23))),"",(E23-X23)*100)</f>
+        <v/>
+      </c>
       <c r="AA23" s="88" t="n"/>
       <c r="AB23" s="85" t="n"/>
       <c r="AC23" s="85" t="n"/>
@@ -42719,6 +43697,14 @@
         <f>IF(U24="","",H24-U24)</f>
         <v/>
       </c>
+      <c r="X24" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B24,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y24" s="89">
+        <f>IF(OR(X24="",NOT(ISNUMBER(E24))),"",(E24-X24)*100)</f>
+        <v/>
+      </c>
       <c r="AA24" s="88" t="n"/>
       <c r="AB24" s="85" t="n"/>
       <c r="AC24" s="85" t="n"/>
@@ -42800,6 +43786,14 @@
         <f>IF(U25="","",H25-U25)</f>
         <v/>
       </c>
+      <c r="X25" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B25,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y25" s="89">
+        <f>IF(OR(X25="",NOT(ISNUMBER(E25))),"",(E25-X25)*100)</f>
+        <v/>
+      </c>
       <c r="AA25" s="88" t="n"/>
       <c r="AB25" s="85" t="n"/>
       <c r="AC25" s="85" t="n"/>
@@ -42881,6 +43875,14 @@
         <f>IF(U26="","",H26-U26)</f>
         <v/>
       </c>
+      <c r="X26" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B26,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y26" s="89">
+        <f>IF(OR(X26="",NOT(ISNUMBER(E26))),"",(E26-X26)*100)</f>
+        <v/>
+      </c>
       <c r="AA26" s="88" t="n"/>
       <c r="AB26" s="85" t="n"/>
       <c r="AC26" s="85" t="n"/>
@@ -42962,6 +43964,14 @@
         <f>IF(U27="","",H27-U27)</f>
         <v/>
       </c>
+      <c r="X27" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B27,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y27" s="89">
+        <f>IF(OR(X27="",NOT(ISNUMBER(E27))),"",(E27-X27)*100)</f>
+        <v/>
+      </c>
       <c r="AA27" s="88" t="n"/>
       <c r="AB27" s="85" t="n"/>
       <c r="AC27" s="85" t="n"/>
@@ -43043,6 +44053,14 @@
         <f>IF(U28="","",H28-U28)</f>
         <v/>
       </c>
+      <c r="X28" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B28,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y28" s="89">
+        <f>IF(OR(X28="",NOT(ISNUMBER(E28))),"",(E28-X28)*100)</f>
+        <v/>
+      </c>
       <c r="AA28" s="88" t="n"/>
       <c r="AB28" s="85" t="n"/>
       <c r="AC28" s="85" t="n"/>
@@ -43124,6 +44142,14 @@
         <f>IF(U29="","",H29-U29)</f>
         <v/>
       </c>
+      <c r="X29" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B29,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y29" s="89">
+        <f>IF(OR(X29="",NOT(ISNUMBER(E29))),"",(E29-X29)*100)</f>
+        <v/>
+      </c>
       <c r="AA29" s="88" t="n"/>
       <c r="AB29" s="85" t="n"/>
       <c r="AC29" s="85" t="n"/>
@@ -43205,6 +44231,14 @@
         <f>IF(U30="","",H30-U30)</f>
         <v/>
       </c>
+      <c r="X30" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B30,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y30" s="89">
+        <f>IF(OR(X30="",NOT(ISNUMBER(E30))),"",(E30-X30)*100)</f>
+        <v/>
+      </c>
       <c r="AA30" s="88" t="n"/>
       <c r="AB30" s="85" t="n"/>
       <c r="AC30" s="85" t="n"/>
@@ -43286,6 +44320,14 @@
         <f>IF(U31="","",H31-U31)</f>
         <v/>
       </c>
+      <c r="X31" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B31,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y31" s="89">
+        <f>IF(OR(X31="",NOT(ISNUMBER(E31))),"",(E31-X31)*100)</f>
+        <v/>
+      </c>
       <c r="AA31" s="88" t="n"/>
       <c r="AB31" s="85" t="n"/>
       <c r="AC31" s="85" t="n"/>
@@ -43367,6 +44409,14 @@
         <f>IF(U32="","",H32-U32)</f>
         <v/>
       </c>
+      <c r="X32" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B32,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y32" s="89">
+        <f>IF(OR(X32="",NOT(ISNUMBER(E32))),"",(E32-X32)*100)</f>
+        <v/>
+      </c>
       <c r="AA32" s="88" t="n"/>
       <c r="AB32" s="85" t="n"/>
       <c r="AC32" s="85" t="n"/>
@@ -43448,6 +44498,14 @@
         <f>IF(U33="","",H33-U33)</f>
         <v/>
       </c>
+      <c r="X33" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B33,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y33" s="89">
+        <f>IF(OR(X33="",NOT(ISNUMBER(E33))),"",(E33-X33)*100)</f>
+        <v/>
+      </c>
       <c r="AA33" s="88" t="n"/>
       <c r="AB33" s="85" t="n"/>
       <c r="AC33" s="85" t="n"/>
@@ -43533,6 +44591,14 @@
         <f>IF(U34="","",H34-U34)</f>
         <v/>
       </c>
+      <c r="X34" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B34,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y34" s="89">
+        <f>IF(OR(X34="",NOT(ISNUMBER(E34))),"",(E34-X34)*100)</f>
+        <v/>
+      </c>
       <c r="AA34" s="88" t="n"/>
       <c r="AB34" s="85" t="n"/>
       <c r="AC34" s="85" t="n"/>
@@ -43614,6 +44680,14 @@
         <f>IF(U35="","",H35-U35)</f>
         <v/>
       </c>
+      <c r="X35" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B35,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y35" s="89">
+        <f>IF(OR(X35="",NOT(ISNUMBER(E35))),"",(E35-X35)*100)</f>
+        <v/>
+      </c>
       <c r="AA35" s="88" t="n"/>
       <c r="AB35" s="85" t="n"/>
       <c r="AC35" s="85" t="n"/>
@@ -43695,6 +44769,14 @@
         <f>IF(U36="","",H36-U36)</f>
         <v/>
       </c>
+      <c r="X36" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B36,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y36" s="89">
+        <f>IF(OR(X36="",NOT(ISNUMBER(E36))),"",(E36-X36)*100)</f>
+        <v/>
+      </c>
       <c r="AA36" s="88" t="n"/>
       <c r="AB36" s="85" t="n"/>
       <c r="AC36" s="85" t="n"/>
@@ -43780,6 +44862,14 @@
         <f>IF(U37="","",H37-U37)</f>
         <v/>
       </c>
+      <c r="X37" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B37,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y37" s="89">
+        <f>IF(OR(X37="",NOT(ISNUMBER(E37))),"",(E37-X37)*100)</f>
+        <v/>
+      </c>
       <c r="AA37" s="88" t="n"/>
       <c r="AB37" s="85" t="n"/>
       <c r="AC37" s="85" t="n"/>
@@ -43861,6 +44951,14 @@
         <f>IF(U38="","",H38-U38)</f>
         <v/>
       </c>
+      <c r="X38" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B38,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y38" s="89">
+        <f>IF(OR(X38="",NOT(ISNUMBER(E38))),"",(E38-X38)*100)</f>
+        <v/>
+      </c>
       <c r="AA38" s="88" t="n"/>
       <c r="AB38" s="85" t="n"/>
       <c r="AC38" s="85" t="n"/>
@@ -43942,6 +45040,14 @@
         <f>IF(U39="","",H39-U39)</f>
         <v/>
       </c>
+      <c r="X39" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B39,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y39" s="89">
+        <f>IF(OR(X39="",NOT(ISNUMBER(E39))),"",(E39-X39)*100)</f>
+        <v/>
+      </c>
       <c r="AA39" s="88" t="n"/>
       <c r="AB39" s="85" t="n"/>
       <c r="AC39" s="85" t="n"/>
@@ -44023,6 +45129,14 @@
         <f>IF(U40="","",H40-U40)</f>
         <v/>
       </c>
+      <c r="X40" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B40,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y40" s="89">
+        <f>IF(OR(X40="",NOT(ISNUMBER(E40))),"",(E40-X40)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -44100,6 +45214,14 @@
         <f>IF(U41="","",H41-U41)</f>
         <v/>
       </c>
+      <c r="X41" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B41,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y41" s="89">
+        <f>IF(OR(X41="",NOT(ISNUMBER(E41))),"",(E41-X41)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
@@ -44181,6 +45303,14 @@
         <f>IF(U42="","",H42-U42)</f>
         <v/>
       </c>
+      <c r="X42" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B42,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y42" s="89">
+        <f>IF(OR(X42="",NOT(ISNUMBER(E42))),"",(E42-X42)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -44258,6 +45388,14 @@
         <f>IF(U43="","",H43-U43)</f>
         <v/>
       </c>
+      <c r="X43" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B43,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y43" s="89">
+        <f>IF(OR(X43="",NOT(ISNUMBER(E43))),"",(E43-X43)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -44335,6 +45473,14 @@
         <f>IF(U44="","",H44-U44)</f>
         <v/>
       </c>
+      <c r="X44" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B44,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y44" s="89">
+        <f>IF(OR(X44="",NOT(ISNUMBER(E44))),"",(E44-X44)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
@@ -44412,6 +45558,14 @@
         <f>IF(U45="","",H45-U45)</f>
         <v/>
       </c>
+      <c r="X45" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B45,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y45" s="89">
+        <f>IF(OR(X45="",NOT(ISNUMBER(E45))),"",(E45-X45)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -44489,6 +45643,14 @@
         <f>IF(U46="","",H46-U46)</f>
         <v/>
       </c>
+      <c r="X46" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B46,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y46" s="89">
+        <f>IF(OR(X46="",NOT(ISNUMBER(E46))),"",(E46-X46)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
@@ -44570,6 +45732,14 @@
         <f>IF(U47="","",H47-U47)</f>
         <v/>
       </c>
+      <c r="X47" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B47,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y47" s="89">
+        <f>IF(OR(X47="",NOT(ISNUMBER(E47))),"",(E47-X47)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
@@ -44647,6 +45817,14 @@
         <f>IF(U48="","",H48-U48)</f>
         <v/>
       </c>
+      <c r="X48" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B48,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y48" s="89">
+        <f>IF(OR(X48="",NOT(ISNUMBER(E48))),"",(E48-X48)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
@@ -44724,6 +45902,14 @@
         <f>IF(U49="","",H49-U49)</f>
         <v/>
       </c>
+      <c r="X49" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B49,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y49" s="89">
+        <f>IF(OR(X49="",NOT(ISNUMBER(E49))),"",(E49-X49)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
@@ -44801,6 +45987,14 @@
         <f>IF(U50="","",H50-U50)</f>
         <v/>
       </c>
+      <c r="X50" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B50,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y50" s="89">
+        <f>IF(OR(X50="",NOT(ISNUMBER(E50))),"",(E50-X50)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -44878,6 +46072,14 @@
         <f>IF(U51="","",H51-U51)</f>
         <v/>
       </c>
+      <c r="X51" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B51,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y51" s="89">
+        <f>IF(OR(X51="",NOT(ISNUMBER(E51))),"",(E51-X51)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
@@ -44959,6 +46161,14 @@
         <f>IF(U52="","",H52-U52)</f>
         <v/>
       </c>
+      <c r="X52" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B52,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y52" s="89">
+        <f>IF(OR(X52="",NOT(ISNUMBER(E52))),"",(E52-X52)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
@@ -45036,6 +46246,14 @@
         <f>IF(U53="","",H53-U53)</f>
         <v/>
       </c>
+      <c r="X53" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B53,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y53" s="89">
+        <f>IF(OR(X53="",NOT(ISNUMBER(E53))),"",(E53-X53)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
@@ -45113,6 +46331,14 @@
         <f>IF(U54="","",H54-U54)</f>
         <v/>
       </c>
+      <c r="X54" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B54,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y54" s="89">
+        <f>IF(OR(X54="",NOT(ISNUMBER(E54))),"",(E54-X54)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
@@ -45190,6 +46416,14 @@
         <f>IF(U55="","",H55-U55)</f>
         <v/>
       </c>
+      <c r="X55" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B55,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y55" s="89">
+        <f>IF(OR(X55="",NOT(ISNUMBER(E55))),"",(E55-X55)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
@@ -45267,6 +46501,14 @@
         <f>IF(U56="","",H56-U56)</f>
         <v/>
       </c>
+      <c r="X56" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B56,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y56" s="89">
+        <f>IF(OR(X56="",NOT(ISNUMBER(E56))),"",(E56-X56)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
@@ -45344,6 +46586,14 @@
         <f>IF(U57="","",H57-U57)</f>
         <v/>
       </c>
+      <c r="X57" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B57,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y57" s="89">
+        <f>IF(OR(X57="",NOT(ISNUMBER(E57))),"",(E57-X57)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -45421,6 +46671,14 @@
         <f>IF(U58="","",H58-U58)</f>
         <v/>
       </c>
+      <c r="X58" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B58,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y58" s="89">
+        <f>IF(OR(X58="",NOT(ISNUMBER(E58))),"",(E58-X58)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
@@ -45498,6 +46756,14 @@
         <f>IF(U59="","",H59-U59)</f>
         <v/>
       </c>
+      <c r="X59" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B59,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y59" s="89">
+        <f>IF(OR(X59="",NOT(ISNUMBER(E59))),"",(E59-X59)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
@@ -45575,6 +46841,14 @@
         <f>IF(U60="","",H60-U60)</f>
         <v/>
       </c>
+      <c r="X60" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B60,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y60" s="89">
+        <f>IF(OR(X60="",NOT(ISNUMBER(E60))),"",(E60-X60)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
@@ -45652,6 +46926,14 @@
         <f>IF(U61="","",H61-U61)</f>
         <v/>
       </c>
+      <c r="X61" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B61,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y61" s="89">
+        <f>IF(OR(X61="",NOT(ISNUMBER(E61))),"",(E61-X61)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
@@ -45733,6 +47015,14 @@
         <f>IF(U62="","",H62-U62)</f>
         <v/>
       </c>
+      <c r="X62" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B62,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y62" s="89">
+        <f>IF(OR(X62="",NOT(ISNUMBER(E62))),"",(E62-X62)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
@@ -45810,6 +47100,14 @@
         <f>IF(U63="","",H63-U63)</f>
         <v/>
       </c>
+      <c r="X63" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B63,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y63" s="89">
+        <f>IF(OR(X63="",NOT(ISNUMBER(E63))),"",(E63-X63)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
@@ -45887,6 +47185,14 @@
         <f>IF(U64="","",H64-U64)</f>
         <v/>
       </c>
+      <c r="X64" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B64,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y64" s="89">
+        <f>IF(OR(X64="",NOT(ISNUMBER(E64))),"",(E64-X64)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
@@ -45964,6 +47270,14 @@
         <f>IF(U65="","",H65-U65)</f>
         <v/>
       </c>
+      <c r="X65" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B65,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y65" s="89">
+        <f>IF(OR(X65="",NOT(ISNUMBER(E65))),"",(E65-X65)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
@@ -46041,6 +47355,14 @@
         <f>IF(U66="","",H66-U66)</f>
         <v/>
       </c>
+      <c r="X66" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B66,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y66" s="89">
+        <f>IF(OR(X66="",NOT(ISNUMBER(E66))),"",(E66-X66)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
@@ -46118,6 +47440,14 @@
         <f>IF(U67="","",H67-U67)</f>
         <v/>
       </c>
+      <c r="X67" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B67,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y67" s="89">
+        <f>IF(OR(X67="",NOT(ISNUMBER(E67))),"",(E67-X67)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
@@ -46195,6 +47525,14 @@
         <f>IF(U68="","",H68-U68)</f>
         <v/>
       </c>
+      <c r="X68" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B68,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y68" s="89">
+        <f>IF(OR(X68="",NOT(ISNUMBER(E68))),"",(E68-X68)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
@@ -46272,6 +47610,14 @@
         <f>IF(U69="","",H69-U69)</f>
         <v/>
       </c>
+      <c r="X69" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B69,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y69" s="89">
+        <f>IF(OR(X69="",NOT(ISNUMBER(E69))),"",(E69-X69)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
@@ -46349,6 +47695,14 @@
         <f>IF(U70="","",H70-U70)</f>
         <v/>
       </c>
+      <c r="X70" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B70,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y70" s="89">
+        <f>IF(OR(X70="",NOT(ISNUMBER(E70))),"",(E70-X70)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
@@ -46426,6 +47780,14 @@
         <f>IF(U71="","",H71-U71)</f>
         <v/>
       </c>
+      <c r="X71" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B71,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y71" s="89">
+        <f>IF(OR(X71="",NOT(ISNUMBER(E71))),"",(E71-X71)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
@@ -46507,6 +47869,14 @@
         <f>IF(U72="","",H72-U72)</f>
         <v/>
       </c>
+      <c r="X72" s="84">
+        <f>IFERROR(INDEX(S490_Snapshot!$C$7:$C$38,MATCH(B72,S490_Snapshot!$A$7:$A$38,0)),"")</f>
+        <v/>
+      </c>
+      <c r="Y72" s="89">
+        <f>IF(OR(X72="",NOT(ISNUMBER(E72))),"",(E72-X72)*100)</f>
+        <v/>
+      </c>
     </row>
     <row r="74" ht="40" customHeight="1">
       <c r="A74" s="70" t="inlineStr">
@@ -46515,7 +47885,17 @@
         </is>
       </c>
     </row>
-    <row r="75"/>
+    <row r="75">
+      <c r="X75" s="67" t="inlineStr">
+        <is>
+          <t>Pillars</t>
+        </is>
+      </c>
+      <c r="Y75" s="87">
+        <f>COUNT(X8:X72)&amp;" / 32"</f>
+        <v/>
+      </c>
+    </row>
     <row r="76">
       <c r="T76" s="67" t="inlineStr">
         <is>
@@ -46526,6 +47906,15 @@
         <f>COUNT(U8:U72)&amp;" / 32"</f>
         <v/>
       </c>
+      <c r="X76" s="67" t="inlineStr">
+        <is>
+          <t>Max |d| (bp)</t>
+        </is>
+      </c>
+      <c r="Y76" s="90">
+        <f>IF(COUNT(Y8:Y72)=0,"",MAX(MAX(Y8:Y72),-MIN(Y8:Y72)))</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="T77" s="67" t="inlineStr">
@@ -46547,6 +47936,11 @@
       <c r="U78" s="91">
         <f>MAX(MAX(W8:W72),-MIN(W8:W72))</f>
         <v/>
+      </c>
+      <c r="X78" s="65" t="inlineStr">
+        <is>
+          <t>E is the live BDP mid via SOFR_OIS_Quotes!H, falling back to the frozen mids. X reads S490_Snapshot directly. Off-terminal both resolve to the same numbers so Y is 0.00; on a terminal Y is how far the pull has moved.</t>
+        </is>
       </c>
     </row>
     <row r="80">

</xml_diff>